<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-07-10
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -540,13 +540,13 @@
         <v>1143</v>
       </c>
       <c r="D5" t="n">
-        <v>5226.3</v>
+        <v>5169.7</v>
       </c>
       <c r="E5" t="n">
-        <v>5745.8</v>
+        <v>5729.1</v>
       </c>
       <c r="F5" t="n">
-        <v>6182.3</v>
+        <v>6172.3</v>
       </c>
     </row>
     <row r="6">
@@ -561,16 +561,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4595</v>
+        <v>4571</v>
       </c>
       <c r="D6" t="n">
-        <v>17022</v>
+        <v>17063.8</v>
       </c>
       <c r="E6" t="n">
-        <v>23376.2</v>
+        <v>23491.7</v>
       </c>
       <c r="F6" t="n">
-        <v>29031.6</v>
+        <v>29523.5</v>
       </c>
     </row>
     <row r="7">
@@ -633,16 +633,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27876</v>
+        <v>27949</v>
       </c>
       <c r="D9" t="n">
-        <v>101573</v>
+        <v>102265.5</v>
       </c>
       <c r="E9" t="n">
-        <v>112196.6</v>
+        <v>113377.6</v>
       </c>
       <c r="F9" t="n">
-        <v>119873.2</v>
+        <v>121044.4</v>
       </c>
     </row>
     <row r="10">
@@ -657,16 +657,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>648227</v>
+        <v>650541</v>
       </c>
       <c r="D10" t="n">
-        <v>2753991.7</v>
+        <v>2767812.5</v>
       </c>
       <c r="E10" t="n">
-        <v>4062358</v>
+        <v>4043634.6</v>
       </c>
       <c r="F10" t="n">
-        <v>4025636.2</v>
+        <v>3939915.6</v>
       </c>
     </row>
     <row r="11">
@@ -705,16 +705,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8068</v>
+        <v>8312</v>
       </c>
       <c r="D12" t="n">
-        <v>30130.8</v>
+        <v>30345.1</v>
       </c>
       <c r="E12" t="n">
-        <v>32790.8</v>
+        <v>32907.2</v>
       </c>
       <c r="F12" t="n">
-        <v>33660.7</v>
+        <v>33721.5</v>
       </c>
     </row>
     <row r="13">
@@ -729,16 +729,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14338</v>
+        <v>14500</v>
       </c>
       <c r="D13" t="n">
-        <v>55023.3</v>
+        <v>56369.3</v>
       </c>
       <c r="E13" t="n">
-        <v>67091.3</v>
+        <v>69187.3</v>
       </c>
       <c r="F13" t="n">
-        <v>71796.7</v>
+        <v>72135</v>
       </c>
     </row>
     <row r="14">
@@ -801,16 +801,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>505</v>
+        <v>513</v>
       </c>
       <c r="D16" t="n">
-        <v>1449.8</v>
+        <v>1452.7</v>
       </c>
       <c r="E16" t="n">
-        <v>2000.7</v>
+        <v>2000.3</v>
       </c>
       <c r="F16" t="n">
-        <v>2027.6</v>
+        <v>2036.9</v>
       </c>
     </row>
     <row r="17">
@@ -849,13 +849,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>10486.2</v>
+        <v>10434.4</v>
       </c>
       <c r="E18" t="n">
-        <v>12287.3</v>
+        <v>12149.2</v>
       </c>
       <c r="F18" t="n">
-        <v>13453.6</v>
+        <v>13426.9</v>
       </c>
     </row>
     <row r="19">
@@ -960,16 +960,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1769</v>
+        <v>1767</v>
       </c>
       <c r="D23" t="n">
-        <v>7263.8</v>
+        <v>7269.1</v>
       </c>
       <c r="E23" t="n">
-        <v>8698.200000000001</v>
+        <v>8732.5</v>
       </c>
       <c r="F23" t="n">
-        <v>10234.5</v>
+        <v>10306.5</v>
       </c>
     </row>
     <row r="24">
@@ -1032,16 +1032,16 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>273</v>
+        <v>284</v>
       </c>
       <c r="D26" t="n">
-        <v>956.5</v>
+        <v>955.3</v>
       </c>
       <c r="E26" t="n">
-        <v>1664.6</v>
+        <v>1620.8</v>
       </c>
       <c r="F26" t="n">
-        <v>2918.6</v>
+        <v>2823.6</v>
       </c>
     </row>
     <row r="27">
@@ -1080,16 +1080,16 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1112</v>
+        <v>1038</v>
       </c>
       <c r="D28" t="n">
-        <v>4633.6</v>
+        <v>4357.2</v>
       </c>
       <c r="E28" t="n">
-        <v>7872.2</v>
+        <v>7439.7</v>
       </c>
       <c r="F28" t="n">
-        <v>8809.299999999999</v>
+        <v>8169.2</v>
       </c>
     </row>
     <row r="29">
@@ -1104,16 +1104,16 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1494</v>
+        <v>1502</v>
       </c>
       <c r="D29" t="n">
-        <v>7586.8</v>
+        <v>7610.5</v>
       </c>
       <c r="E29" t="n">
-        <v>8482.799999999999</v>
+        <v>8508.299999999999</v>
       </c>
       <c r="F29" t="n">
-        <v>8927.5</v>
+        <v>8956</v>
       </c>
     </row>
     <row r="30">
@@ -1176,16 +1176,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>622</v>
+        <v>631</v>
       </c>
       <c r="D32" t="n">
-        <v>2128.8</v>
+        <v>2130.5</v>
       </c>
       <c r="E32" t="n">
-        <v>2358.5</v>
+        <v>2350.3</v>
       </c>
       <c r="F32" t="n">
-        <v>2496.2</v>
+        <v>2458.2</v>
       </c>
     </row>
     <row r="33">
@@ -1200,16 +1200,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>31627</v>
+        <v>31377</v>
       </c>
       <c r="D33" t="n">
-        <v>118832.8</v>
+        <v>119102.2</v>
       </c>
       <c r="E33" t="n">
-        <v>133309.8</v>
+        <v>133173.4</v>
       </c>
       <c r="F33" t="n">
-        <v>146139.6</v>
+        <v>145756.5</v>
       </c>
     </row>
     <row r="34">
@@ -1224,16 +1224,16 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>7553</v>
+        <v>7489</v>
       </c>
       <c r="D34" t="n">
-        <v>32017.8</v>
+        <v>31736.7</v>
       </c>
       <c r="E34" t="n">
-        <v>40240.6</v>
+        <v>40076.2</v>
       </c>
       <c r="F34" t="n">
-        <v>45668.3</v>
+        <v>45608.8</v>
       </c>
     </row>
     <row r="35">
@@ -1251,13 +1251,13 @@
         <v>5604</v>
       </c>
       <c r="D35" t="n">
-        <v>21007.1</v>
+        <v>21132.5</v>
       </c>
       <c r="E35" t="n">
-        <v>23515.9</v>
+        <v>23517.5</v>
       </c>
       <c r="F35" t="n">
-        <v>25014.6</v>
+        <v>25037.6</v>
       </c>
     </row>
     <row r="36">
@@ -1275,10 +1275,10 @@
         <v>1344</v>
       </c>
       <c r="D36" t="n">
-        <v>4617.1</v>
+        <v>4617</v>
       </c>
       <c r="E36" t="n">
-        <v>5073.7</v>
+        <v>5073.1</v>
       </c>
       <c r="F36" t="n">
         <v>5900.8</v>
@@ -1299,13 +1299,13 @@
         <v>850494</v>
       </c>
       <c r="D37" t="n">
-        <v>3742869.5</v>
+        <v>3832403.5</v>
       </c>
       <c r="E37" t="n">
-        <v>5264743.6</v>
+        <v>5422607.5</v>
       </c>
       <c r="F37" t="n">
-        <v>5106293</v>
+        <v>5327749.5</v>
       </c>
     </row>
     <row r="38">
@@ -1320,16 +1320,16 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>5910</v>
+        <v>6107</v>
       </c>
       <c r="D38" t="n">
-        <v>21482.1</v>
+        <v>21714.4</v>
       </c>
       <c r="E38" t="n">
-        <v>19537.1</v>
+        <v>19715.2</v>
       </c>
       <c r="F38" t="n">
-        <v>19834.1</v>
+        <v>19922.1</v>
       </c>
     </row>
     <row r="39">
@@ -1371,13 +1371,13 @@
         <v>4406</v>
       </c>
       <c r="D40" t="n">
-        <v>16669.4</v>
+        <v>16669</v>
       </c>
       <c r="E40" t="n">
-        <v>18989.7</v>
+        <v>18990.1</v>
       </c>
       <c r="F40" t="n">
-        <v>21819.4</v>
+        <v>21819.9</v>
       </c>
     </row>
     <row r="41">
@@ -1416,16 +1416,16 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>-619</v>
+        <v>-523</v>
       </c>
       <c r="D42" t="n">
-        <v>-119.5</v>
+        <v>82.7</v>
       </c>
       <c r="E42" t="n">
-        <v>14700.9</v>
+        <v>14829.6</v>
       </c>
       <c r="F42" t="n">
-        <v>25631.2</v>
+        <v>25291.6</v>
       </c>
     </row>
     <row r="43">
@@ -1464,16 +1464,16 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>17794</v>
+        <v>18359</v>
       </c>
       <c r="D44" t="n">
-        <v>40427.4</v>
+        <v>41243</v>
       </c>
       <c r="E44" t="n">
-        <v>26644.7</v>
+        <v>26789.7</v>
       </c>
       <c r="F44" t="n">
-        <v>27547.9</v>
+        <v>27554.5</v>
       </c>
     </row>
     <row r="45">
@@ -1488,16 +1488,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1013</v>
+        <v>1019</v>
       </c>
       <c r="D45" t="n">
-        <v>3464.6</v>
+        <v>3474.3</v>
       </c>
       <c r="E45" t="n">
-        <v>3725.5</v>
+        <v>3735.5</v>
       </c>
       <c r="F45" t="n">
-        <v>3888.4</v>
+        <v>3891.1</v>
       </c>
     </row>
     <row r="46">
@@ -1539,13 +1539,13 @@
         <v>742</v>
       </c>
       <c r="D47" t="n">
-        <v>3232.2</v>
+        <v>3244.5</v>
       </c>
       <c r="E47" t="n">
-        <v>4451.1</v>
+        <v>4495.9</v>
       </c>
       <c r="F47" t="n">
-        <v>5509.4</v>
+        <v>5694.8</v>
       </c>
     </row>
     <row r="48">
@@ -1581,13 +1581,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="D49" t="n">
-        <v>1749.9</v>
+        <v>1760.9</v>
       </c>
       <c r="E49" t="n">
-        <v>2239.5</v>
+        <v>2249.2</v>
       </c>
       <c r="F49" t="n">
         <v>2685.3</v>
@@ -1605,16 +1605,16 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3938</v>
+        <v>4015</v>
       </c>
       <c r="D50" t="n">
-        <v>16321.6</v>
+        <v>16524.3</v>
       </c>
       <c r="E50" t="n">
-        <v>29922.4</v>
+        <v>31390.1</v>
       </c>
       <c r="F50" t="n">
-        <v>45557.4</v>
+        <v>49657.5</v>
       </c>
     </row>
     <row r="51">
@@ -1629,13 +1629,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D51" t="n">
-        <v>359.5</v>
+        <v>379.5</v>
       </c>
       <c r="E51" t="n">
-        <v>440</v>
+        <v>441.7</v>
       </c>
       <c r="F51" t="n">
         <v>581.3</v>
@@ -1680,13 +1680,13 @@
         <v>14211</v>
       </c>
       <c r="D53" t="n">
-        <v>56430.5</v>
+        <v>56417.8</v>
       </c>
       <c r="E53" t="n">
-        <v>67800.5</v>
+        <v>67968.8</v>
       </c>
       <c r="F53" t="n">
-        <v>78345</v>
+        <v>78474.8</v>
       </c>
     </row>
     <row r="54">
@@ -1725,16 +1725,16 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1257</v>
+        <v>1213</v>
       </c>
       <c r="D55" t="n">
-        <v>3843.6</v>
+        <v>3751.4</v>
       </c>
       <c r="E55" t="n">
-        <v>5392.3</v>
+        <v>5370.1</v>
       </c>
       <c r="F55" t="n">
-        <v>6613.2</v>
+        <v>6603.2</v>
       </c>
     </row>
     <row r="56">
@@ -1797,16 +1797,16 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3933</v>
+        <v>3902</v>
       </c>
       <c r="D58" t="n">
-        <v>15077.2</v>
+        <v>14993.6</v>
       </c>
       <c r="E58" t="n">
-        <v>20347</v>
+        <v>20241</v>
       </c>
       <c r="F58" t="n">
-        <v>23773.6</v>
+        <v>23704.1</v>
       </c>
     </row>
     <row r="59">
@@ -1821,16 +1821,16 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>9345</v>
+        <v>9415</v>
       </c>
       <c r="D59" t="n">
-        <v>35195.9</v>
+        <v>35619.5</v>
       </c>
       <c r="E59" t="n">
-        <v>24390.5</v>
+        <v>24566.4</v>
       </c>
       <c r="F59" t="n">
-        <v>22463.2</v>
+        <v>22576.3</v>
       </c>
     </row>
     <row r="60">
@@ -1845,16 +1845,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1709</v>
+        <v>1803</v>
       </c>
       <c r="D60" t="n">
-        <v>11487.2</v>
+        <v>11679.8</v>
       </c>
       <c r="E60" t="n">
-        <v>13573.3</v>
+        <v>13870.9</v>
       </c>
       <c r="F60" t="n">
-        <v>15312.2</v>
+        <v>15782.4</v>
       </c>
     </row>
     <row r="61">
@@ -1869,16 +1869,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>968</v>
+        <v>1380</v>
       </c>
       <c r="D61" t="n">
-        <v>785.3</v>
+        <v>1671</v>
       </c>
       <c r="E61" t="n">
-        <v>2720.4</v>
+        <v>2610.4</v>
       </c>
       <c r="F61" t="n">
-        <v>4923.2</v>
+        <v>4783.5</v>
       </c>
     </row>
     <row r="62">
@@ -1893,16 +1893,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3152</v>
+        <v>3182</v>
       </c>
       <c r="D62" t="n">
-        <v>11253.4</v>
+        <v>11608</v>
       </c>
       <c r="E62" t="n">
-        <v>8457.200000000001</v>
+        <v>8554.9</v>
       </c>
       <c r="F62" t="n">
-        <v>8962.799999999999</v>
+        <v>9030.200000000001</v>
       </c>
     </row>
     <row r="63">
@@ -1917,16 +1917,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>598</v>
+        <v>576</v>
       </c>
       <c r="D63" t="n">
-        <v>2344.7</v>
+        <v>2314.2</v>
       </c>
       <c r="E63" t="n">
-        <v>2917.7</v>
+        <v>2836.9</v>
       </c>
       <c r="F63" t="n">
-        <v>3226.4</v>
+        <v>3126.8</v>
       </c>
     </row>
     <row r="64">
@@ -1941,16 +1941,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1302</v>
+        <v>1401</v>
       </c>
       <c r="D64" t="n">
-        <v>3738.1</v>
+        <v>3904.6</v>
       </c>
       <c r="E64" t="n">
-        <v>4289.7</v>
+        <v>4430.3</v>
       </c>
       <c r="F64" t="n">
-        <v>4739.6</v>
+        <v>4902.9</v>
       </c>
     </row>
     <row r="65">
@@ -1989,16 +1989,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>9106</v>
+        <v>9114</v>
       </c>
       <c r="D66" t="n">
-        <v>37138</v>
+        <v>37203.2</v>
       </c>
       <c r="E66" t="n">
-        <v>42446.2</v>
+        <v>42456.2</v>
       </c>
       <c r="F66" t="n">
-        <v>46417.6</v>
+        <v>46498.1</v>
       </c>
     </row>
     <row r="67">
@@ -2013,16 +2013,16 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>10249</v>
+        <v>10170</v>
       </c>
       <c r="D67" t="n">
-        <v>42579.6</v>
+        <v>42629.6</v>
       </c>
       <c r="E67" t="n">
-        <v>54915.1</v>
+        <v>54900.1</v>
       </c>
       <c r="F67" t="n">
-        <v>61734.6</v>
+        <v>61729.9</v>
       </c>
     </row>
     <row r="68">
@@ -2061,16 +2061,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D69" t="n">
-        <v>1869.5</v>
+        <v>1879.9</v>
       </c>
       <c r="E69" t="n">
-        <v>2366.9</v>
+        <v>2386.1</v>
       </c>
       <c r="F69" t="n">
-        <v>3050.1</v>
+        <v>3072.4</v>
       </c>
     </row>
     <row r="70">
@@ -2109,16 +2109,16 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>5958</v>
+        <v>6159</v>
       </c>
       <c r="D71" t="n">
-        <v>22124.8</v>
+        <v>22401.3</v>
       </c>
       <c r="E71" t="n">
-        <v>20517.6</v>
+        <v>20758.2</v>
       </c>
       <c r="F71" t="n">
-        <v>20670.3</v>
+        <v>20808.3</v>
       </c>
     </row>
     <row r="72">
@@ -2133,16 +2133,16 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>5271</v>
+        <v>5290</v>
       </c>
       <c r="D72" t="n">
-        <v>19110.6</v>
+        <v>19147.2</v>
       </c>
       <c r="E72" t="n">
-        <v>20293.2</v>
+        <v>20290.9</v>
       </c>
       <c r="F72" t="n">
-        <v>21534.7</v>
+        <v>21493</v>
       </c>
     </row>
     <row r="73">
@@ -2159,12 +2159,6 @@
       <c r="C73" t="n">
         <v>578</v>
       </c>
-      <c r="D73" t="n">
-        <v>2307</v>
-      </c>
-      <c r="E73" t="n">
-        <v>2674</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2202,16 +2196,16 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2293</v>
+        <v>2330</v>
       </c>
       <c r="D75" t="n">
-        <v>8321.200000000001</v>
+        <v>8358.200000000001</v>
       </c>
       <c r="E75" t="n">
-        <v>10627.7</v>
+        <v>10647.7</v>
       </c>
       <c r="F75" t="n">
-        <v>11783.6</v>
+        <v>11831.3</v>
       </c>
     </row>
     <row r="76">
@@ -2226,16 +2220,16 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1092</v>
+        <v>1095</v>
       </c>
       <c r="D76" t="n">
-        <v>4276.4</v>
+        <v>4279.2</v>
       </c>
       <c r="E76" t="n">
-        <v>4995.8</v>
+        <v>4997.4</v>
       </c>
       <c r="F76" t="n">
-        <v>5791.9</v>
+        <v>5789.7</v>
       </c>
     </row>
     <row r="77">
@@ -2250,16 +2244,16 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2652</v>
+        <v>2682</v>
       </c>
       <c r="D77" t="n">
-        <v>9987</v>
+        <v>10136.5</v>
       </c>
       <c r="E77" t="n">
-        <v>11412.8</v>
+        <v>11688.8</v>
       </c>
       <c r="F77" t="n">
-        <v>12195.3</v>
+        <v>12472.5</v>
       </c>
     </row>
     <row r="78">
@@ -2274,13 +2268,13 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1099</v>
+        <v>1104</v>
       </c>
       <c r="D78" t="n">
-        <v>8024.1</v>
+        <v>8034.7</v>
       </c>
       <c r="E78" t="n">
-        <v>8607.299999999999</v>
+        <v>8618.5</v>
       </c>
       <c r="F78" t="n">
         <v>9113.799999999999</v>
@@ -2298,16 +2292,16 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>9540</v>
+        <v>9437</v>
       </c>
       <c r="D79" t="n">
-        <v>37032.5</v>
+        <v>37054.8</v>
       </c>
       <c r="E79" t="n">
-        <v>39694.8</v>
+        <v>39842.8</v>
       </c>
       <c r="F79" t="n">
-        <v>42426.6</v>
+        <v>42556.9</v>
       </c>
     </row>
     <row r="80">
@@ -2322,16 +2316,16 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2188</v>
+        <v>2179</v>
       </c>
       <c r="D80" t="n">
-        <v>8858.799999999999</v>
+        <v>8839.6</v>
       </c>
       <c r="E80" t="n">
-        <v>10346.4</v>
+        <v>10306.5</v>
       </c>
       <c r="F80" t="n">
-        <v>11488.3</v>
+        <v>11529.4</v>
       </c>
     </row>
     <row r="81">
@@ -2370,16 +2364,16 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1462</v>
+        <v>1495</v>
       </c>
       <c r="D82" t="n">
-        <v>5779.2</v>
+        <v>5839.5</v>
       </c>
       <c r="E82" t="n">
-        <v>6028.2</v>
+        <v>6010.8</v>
       </c>
       <c r="F82" t="n">
-        <v>6313.5</v>
+        <v>6274.3</v>
       </c>
     </row>
     <row r="83">
@@ -2418,16 +2412,16 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="D84" t="n">
-        <v>3348.2</v>
+        <v>3339.9</v>
       </c>
       <c r="E84" t="n">
-        <v>3651.5</v>
+        <v>3636.7</v>
       </c>
       <c r="F84" t="n">
-        <v>3717.2</v>
+        <v>3692.6</v>
       </c>
     </row>
     <row r="85">
@@ -2442,16 +2436,16 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>6136</v>
+        <v>6133</v>
       </c>
       <c r="D85" t="n">
-        <v>20737.3</v>
+        <v>20721.3</v>
       </c>
       <c r="E85" t="n">
-        <v>22559</v>
+        <v>22526.8</v>
       </c>
       <c r="F85" t="n">
-        <v>23920.2</v>
+        <v>23847.4</v>
       </c>
     </row>
     <row r="86">
@@ -2466,16 +2460,16 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>3067</v>
+        <v>3062</v>
       </c>
       <c r="D86" t="n">
-        <v>11140</v>
+        <v>11111.1</v>
       </c>
       <c r="E86" t="n">
-        <v>11942.1</v>
+        <v>11959</v>
       </c>
       <c r="F86" t="n">
-        <v>12702.2</v>
+        <v>12715.1</v>
       </c>
     </row>
     <row r="87">
@@ -2490,7 +2484,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>10545</v>
+        <v>10237</v>
       </c>
       <c r="D87" t="n">
         <v>33019.2</v>
@@ -2514,16 +2508,16 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3830</v>
+        <v>3843</v>
       </c>
       <c r="D88" t="n">
-        <v>15061.6</v>
+        <v>15067.6</v>
       </c>
       <c r="E88" t="n">
         <v>16299.9</v>
       </c>
       <c r="F88" t="n">
-        <v>17235</v>
+        <v>17227</v>
       </c>
     </row>
     <row r="89">
@@ -2586,13 +2580,13 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>504</v>
+        <v>498</v>
       </c>
       <c r="D91" t="n">
-        <v>1860.2</v>
+        <v>1856.2</v>
       </c>
       <c r="E91" t="n">
-        <v>2235.7</v>
+        <v>2235.1</v>
       </c>
       <c r="F91" t="n">
         <v>2456</v>
@@ -2610,7 +2604,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>24552</v>
+        <v>24551</v>
       </c>
       <c r="D92" t="n">
         <v>98678.39999999999</v>
@@ -2658,16 +2652,16 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>5717</v>
+        <v>5693</v>
       </c>
       <c r="D94" t="n">
-        <v>24009.3</v>
+        <v>23970.7</v>
       </c>
       <c r="E94" t="n">
-        <v>27681.3</v>
+        <v>27661</v>
       </c>
       <c r="F94" t="n">
-        <v>31261.7</v>
+        <v>31280.1</v>
       </c>
     </row>
     <row r="95">
@@ -2682,16 +2676,16 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2234</v>
+        <v>2226</v>
       </c>
       <c r="D95" t="n">
-        <v>9356.9</v>
+        <v>9376.9</v>
       </c>
       <c r="E95" t="n">
-        <v>10898.9</v>
+        <v>10913.1</v>
       </c>
       <c r="F95" t="n">
-        <v>12550.9</v>
+        <v>12611.7</v>
       </c>
     </row>
     <row r="96">
@@ -2730,16 +2724,16 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1264</v>
+        <v>1266</v>
       </c>
       <c r="D97" t="n">
-        <v>5044</v>
+        <v>5021.2</v>
       </c>
       <c r="E97" t="n">
-        <v>5934.2</v>
+        <v>5888.8</v>
       </c>
       <c r="F97" t="n">
-        <v>6107.5</v>
+        <v>6011.7</v>
       </c>
     </row>
     <row r="98">
@@ -2754,16 +2748,16 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>5746</v>
+        <v>6257</v>
       </c>
       <c r="D98" t="n">
-        <v>21122.5</v>
+        <v>21724.8</v>
       </c>
       <c r="E98" t="n">
-        <v>20023.6</v>
+        <v>20349.5</v>
       </c>
       <c r="F98" t="n">
-        <v>20358.3</v>
+        <v>20600.4</v>
       </c>
     </row>
     <row r="99">
@@ -2778,16 +2772,16 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>5006</v>
+        <v>5217</v>
       </c>
       <c r="D99" t="n">
-        <v>18354.6</v>
+        <v>18987.4</v>
       </c>
       <c r="E99" t="n">
-        <v>23361.2</v>
+        <v>23507.6</v>
       </c>
       <c r="F99" t="n">
-        <v>27990.8</v>
+        <v>27892.4</v>
       </c>
     </row>
     <row r="100">
@@ -2826,16 +2820,16 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1481</v>
+        <v>1508</v>
       </c>
       <c r="D101" t="n">
-        <v>6922.8</v>
+        <v>6988.2</v>
       </c>
       <c r="E101" t="n">
-        <v>7217.9</v>
+        <v>7254.8</v>
       </c>
       <c r="F101" t="n">
-        <v>8205.799999999999</v>
+        <v>8244.9</v>
       </c>
     </row>
     <row r="102">
@@ -2853,13 +2847,13 @@
         <v>3517</v>
       </c>
       <c r="D102" t="n">
-        <v>13927.6</v>
+        <v>13940.8</v>
       </c>
       <c r="E102" t="n">
-        <v>15047.8</v>
+        <v>15092.4</v>
       </c>
       <c r="F102" t="n">
-        <v>15748.5</v>
+        <v>15771.5</v>
       </c>
     </row>
     <row r="103">
@@ -2874,16 +2868,16 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1026</v>
+        <v>1002</v>
       </c>
       <c r="D103" t="n">
-        <v>4699.8</v>
+        <v>4679.8</v>
       </c>
       <c r="E103" t="n">
-        <v>6659.8</v>
+        <v>6650.4</v>
       </c>
       <c r="F103" t="n">
-        <v>8069.8</v>
+        <v>8075.1</v>
       </c>
     </row>
     <row r="104">
@@ -2922,16 +2916,16 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>724</v>
+        <v>751</v>
       </c>
       <c r="D105" t="n">
-        <v>3358.1</v>
+        <v>3421.5</v>
       </c>
       <c r="E105" t="n">
-        <v>3999.1</v>
+        <v>3992.5</v>
       </c>
       <c r="F105" t="n">
-        <v>4304.6</v>
+        <v>4283.7</v>
       </c>
     </row>
     <row r="106">
@@ -2946,16 +2940,16 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3535</v>
+        <v>3808</v>
       </c>
       <c r="D106" t="n">
-        <v>14268.5</v>
+        <v>15532.2</v>
       </c>
       <c r="E106" t="n">
-        <v>39453.1</v>
+        <v>42457.5</v>
       </c>
       <c r="F106" t="n">
-        <v>54547.7</v>
+        <v>59569.1</v>
       </c>
     </row>
     <row r="107">
@@ -2994,16 +2988,16 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>22230</v>
+        <v>22193</v>
       </c>
       <c r="D108" t="n">
-        <v>76847.10000000001</v>
+        <v>76844.60000000001</v>
       </c>
       <c r="E108" t="n">
-        <v>81755.10000000001</v>
+        <v>81715.8</v>
       </c>
       <c r="F108" t="n">
-        <v>85200.2</v>
+        <v>85049.5</v>
       </c>
     </row>
     <row r="109">
@@ -3018,16 +3012,16 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="D109" t="n">
-        <v>2496.6</v>
+        <v>2487.6</v>
       </c>
       <c r="E109" t="n">
-        <v>3337</v>
+        <v>3312.3</v>
       </c>
       <c r="F109" t="n">
-        <v>4291</v>
+        <v>4295.2</v>
       </c>
     </row>
     <row r="110">
@@ -3066,16 +3060,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1446</v>
+        <v>1434</v>
       </c>
       <c r="D111" t="n">
-        <v>6174.8</v>
+        <v>6162.8</v>
       </c>
       <c r="E111" t="n">
-        <v>7034.6</v>
+        <v>7022.6</v>
       </c>
       <c r="F111" t="n">
-        <v>7926.7</v>
+        <v>7902.2</v>
       </c>
     </row>
     <row r="112">
@@ -3093,13 +3087,13 @@
         <v>10580</v>
       </c>
       <c r="D112" t="n">
-        <v>39761.6</v>
+        <v>42384.2</v>
       </c>
       <c r="E112" t="n">
-        <v>44047.7</v>
+        <v>45628.6</v>
       </c>
       <c r="F112" t="n">
-        <v>53580.1</v>
+        <v>55174.1</v>
       </c>
     </row>
     <row r="113">
@@ -3114,16 +3108,16 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>486</v>
+        <v>502</v>
       </c>
       <c r="D113" t="n">
-        <v>2436.4</v>
+        <v>2517.9</v>
       </c>
       <c r="E113" t="n">
-        <v>2285.7</v>
+        <v>2311</v>
       </c>
       <c r="F113" t="n">
-        <v>3228.6</v>
+        <v>3257.2</v>
       </c>
     </row>
     <row r="114">
@@ -3141,13 +3135,13 @@
         <v>4017</v>
       </c>
       <c r="D114" t="n">
-        <v>17618.7</v>
+        <v>17705.6</v>
       </c>
       <c r="E114" t="n">
-        <v>20984.4</v>
+        <v>21003.2</v>
       </c>
       <c r="F114" t="n">
-        <v>24698.8</v>
+        <v>24637.2</v>
       </c>
     </row>
     <row r="115">
@@ -3210,16 +3204,16 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>852</v>
+        <v>858</v>
       </c>
       <c r="D117" t="n">
-        <v>4345.3</v>
+        <v>4359.2</v>
       </c>
       <c r="E117" t="n">
-        <v>5236.6</v>
+        <v>5268.4</v>
       </c>
       <c r="F117" t="n">
-        <v>5604.9</v>
+        <v>5649.9</v>
       </c>
     </row>
     <row r="118">
@@ -3234,16 +3228,16 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>9591</v>
+        <v>10145</v>
       </c>
       <c r="D118" t="n">
-        <v>34673.7</v>
+        <v>35060.4</v>
       </c>
       <c r="E118" t="n">
-        <v>31874.9</v>
+        <v>32190.9</v>
       </c>
       <c r="F118" t="n">
-        <v>32317.2</v>
+        <v>32379.5</v>
       </c>
     </row>
     <row r="119">
@@ -3285,13 +3279,13 @@
         <v>355</v>
       </c>
       <c r="D120" t="n">
-        <v>1515.1</v>
+        <v>1522.5</v>
       </c>
       <c r="E120" t="n">
-        <v>2029.4</v>
+        <v>2035.3</v>
       </c>
       <c r="F120" t="n">
-        <v>2509.1</v>
+        <v>2477.5</v>
       </c>
     </row>
     <row r="121">
@@ -3306,16 +3300,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1460</v>
+        <v>1455</v>
       </c>
       <c r="D121" t="n">
-        <v>5764.2</v>
+        <v>5763.7</v>
       </c>
       <c r="E121" t="n">
-        <v>6140.9</v>
+        <v>5993.2</v>
       </c>
       <c r="F121" t="n">
-        <v>6939.2</v>
+        <v>6656.3</v>
       </c>
     </row>
     <row r="122">
@@ -3378,16 +3372,16 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2075</v>
+        <v>2121</v>
       </c>
       <c r="D124" t="n">
-        <v>5590.4</v>
+        <v>5637.1</v>
       </c>
       <c r="E124" t="n">
-        <v>5992.6</v>
+        <v>6005.9</v>
       </c>
       <c r="F124" t="n">
-        <v>6216.9</v>
+        <v>6231.9</v>
       </c>
     </row>
     <row r="125">
@@ -3402,16 +3396,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>604</v>
+        <v>595</v>
       </c>
       <c r="D125" t="n">
-        <v>2442</v>
+        <v>2407.6</v>
       </c>
       <c r="E125" t="n">
-        <v>3678.6</v>
+        <v>3687.6</v>
       </c>
       <c r="F125" t="n">
-        <v>4513.2</v>
+        <v>4521.6</v>
       </c>
     </row>
     <row r="126">
@@ -3429,13 +3423,13 @@
         <v>5218</v>
       </c>
       <c r="D126" t="n">
-        <v>21777.1</v>
+        <v>21784.2</v>
       </c>
       <c r="E126" t="n">
-        <v>23327.9</v>
+        <v>23322.1</v>
       </c>
       <c r="F126" t="n">
-        <v>24468.7</v>
+        <v>24482.1</v>
       </c>
     </row>
     <row r="127">
@@ -3450,16 +3444,16 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>16554</v>
+        <v>16577</v>
       </c>
       <c r="D127" t="n">
-        <v>60316.2</v>
+        <v>60367.7</v>
       </c>
       <c r="E127" t="n">
-        <v>63092.1</v>
+        <v>63117.4</v>
       </c>
       <c r="F127" t="n">
-        <v>66160.60000000001</v>
+        <v>65992.2</v>
       </c>
     </row>
     <row r="128">
@@ -3474,13 +3468,13 @@
         </is>
       </c>
       <c r="D128" t="n">
-        <v>8076.7</v>
+        <v>8132.5</v>
       </c>
       <c r="E128" t="n">
-        <v>9033.6</v>
+        <v>9055.200000000001</v>
       </c>
       <c r="F128" t="n">
-        <v>8843</v>
+        <v>8905.200000000001</v>
       </c>
     </row>
     <row r="129">
@@ -3495,16 +3489,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>973</v>
+        <v>984</v>
       </c>
       <c r="D129" t="n">
-        <v>4613.4</v>
+        <v>4637.6</v>
       </c>
       <c r="E129" t="n">
-        <v>5257.9</v>
+        <v>5278.1</v>
       </c>
       <c r="F129" t="n">
-        <v>5839.2</v>
+        <v>5882.1</v>
       </c>
     </row>
     <row r="130">
@@ -3534,16 +3528,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>13895</v>
+        <v>13980</v>
       </c>
       <c r="D131" t="n">
-        <v>50970.7</v>
+        <v>50950.2</v>
       </c>
       <c r="E131" t="n">
-        <v>31170</v>
+        <v>31187.9</v>
       </c>
       <c r="F131" t="n">
-        <v>34632.2</v>
+        <v>36712.4</v>
       </c>
     </row>
     <row r="132">
@@ -3582,16 +3576,16 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>835</v>
+        <v>831</v>
       </c>
       <c r="D133" t="n">
-        <v>3619.2</v>
+        <v>3617.8</v>
       </c>
       <c r="E133" t="n">
-        <v>3617.9</v>
+        <v>3606.6</v>
       </c>
       <c r="F133" t="n">
-        <v>3995.7</v>
+        <v>3982.7</v>
       </c>
     </row>
     <row r="134">
@@ -3606,16 +3600,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>25205</v>
+        <v>25740</v>
       </c>
       <c r="D134" t="n">
-        <v>92326.8</v>
+        <v>92733.10000000001</v>
       </c>
       <c r="E134" t="n">
-        <v>94131.89999999999</v>
+        <v>94340.8</v>
       </c>
       <c r="F134" t="n">
-        <v>96926.39999999999</v>
+        <v>97139.5</v>
       </c>
     </row>
     <row r="135">
@@ -3657,13 +3651,13 @@
         <v>787</v>
       </c>
       <c r="D136" t="n">
-        <v>3043.3</v>
+        <v>3032.2</v>
       </c>
       <c r="E136" t="n">
-        <v>3524</v>
+        <v>3488.4</v>
       </c>
       <c r="F136" t="n">
-        <v>3360.5</v>
+        <v>3305.5</v>
       </c>
     </row>
     <row r="137">
@@ -3702,16 +3696,16 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>636</v>
+        <v>632</v>
       </c>
       <c r="D138" t="n">
-        <v>2748.8</v>
+        <v>2803.7</v>
       </c>
       <c r="E138" t="n">
-        <v>3104.2</v>
+        <v>3114.5</v>
       </c>
       <c r="F138" t="n">
-        <v>3326.2</v>
+        <v>3340.5</v>
       </c>
     </row>
     <row r="139">
@@ -3750,16 +3744,16 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>3388</v>
+        <v>3328</v>
       </c>
       <c r="D140" t="n">
-        <v>11174.3</v>
+        <v>11090.9</v>
       </c>
       <c r="E140" t="n">
-        <v>12022.1</v>
+        <v>11963.5</v>
       </c>
       <c r="F140" t="n">
-        <v>12739.8</v>
+        <v>12679.9</v>
       </c>
     </row>
     <row r="141">
@@ -3774,16 +3768,16 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2129</v>
+        <v>2101</v>
       </c>
       <c r="D141" t="n">
-        <v>6665.5</v>
+        <v>6646.1</v>
       </c>
       <c r="E141" t="n">
-        <v>7159.7</v>
+        <v>7169.7</v>
       </c>
       <c r="F141" t="n">
-        <v>7616.2</v>
+        <v>7576.4</v>
       </c>
     </row>
     <row r="142">
@@ -3798,13 +3792,13 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>684</v>
+        <v>672</v>
       </c>
       <c r="D142" t="n">
-        <v>5624.7</v>
+        <v>5599.1</v>
       </c>
       <c r="E142" t="n">
-        <v>6565.3</v>
+        <v>6533.8</v>
       </c>
       <c r="F142" t="n">
         <v>7229.4</v>
@@ -3822,16 +3816,16 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>5250</v>
+        <v>5313</v>
       </c>
       <c r="D143" t="n">
-        <v>21343.7</v>
+        <v>21431.1</v>
       </c>
       <c r="E143" t="n">
-        <v>23655.5</v>
+        <v>23669.5</v>
       </c>
       <c r="F143" t="n">
-        <v>25920.6</v>
+        <v>25886.4</v>
       </c>
     </row>
     <row r="144">
@@ -3846,16 +3840,16 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>942</v>
+        <v>953</v>
       </c>
       <c r="D144" t="n">
-        <v>3116.3</v>
+        <v>3148.2</v>
       </c>
       <c r="E144" t="n">
-        <v>3592</v>
+        <v>3633</v>
       </c>
       <c r="F144" t="n">
-        <v>4045.2</v>
+        <v>4096.7</v>
       </c>
     </row>
     <row r="145">
@@ -3870,16 +3864,16 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2846</v>
+        <v>2872</v>
       </c>
       <c r="D145" t="n">
-        <v>10119.9</v>
+        <v>10076.6</v>
       </c>
       <c r="E145" t="n">
-        <v>10878.2</v>
+        <v>10814.8</v>
       </c>
       <c r="F145" t="n">
-        <v>11448</v>
+        <v>11377.3</v>
       </c>
     </row>
     <row r="146">
@@ -3897,13 +3891,13 @@
         <v>210</v>
       </c>
       <c r="D146" t="n">
-        <v>832.5</v>
+        <v>804.6</v>
       </c>
       <c r="E146" t="n">
-        <v>930.3</v>
+        <v>937.8</v>
       </c>
       <c r="F146" t="n">
-        <v>1021</v>
+        <v>1023.2</v>
       </c>
     </row>
     <row r="147">
@@ -3942,16 +3936,16 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="D148" t="n">
-        <v>2326.2</v>
+        <v>2327.5</v>
       </c>
       <c r="E148" t="n">
-        <v>2746.1</v>
+        <v>2766.5</v>
       </c>
       <c r="F148" t="n">
-        <v>3147.5</v>
+        <v>3194</v>
       </c>
     </row>
     <row r="149">
@@ -3966,16 +3960,16 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="D149" t="n">
-        <v>4038.7</v>
+        <v>4028.2</v>
       </c>
       <c r="E149" t="n">
-        <v>4725.9</v>
+        <v>4685.9</v>
       </c>
       <c r="F149" t="n">
-        <v>5271.8</v>
+        <v>5234.6</v>
       </c>
     </row>
     <row r="150">
@@ -3990,7 +3984,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>5982</v>
+        <v>5997</v>
       </c>
       <c r="D150" t="n">
         <v>24946.2</v>
@@ -4014,16 +4008,16 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1905</v>
+        <v>1941</v>
       </c>
       <c r="D151" t="n">
-        <v>7537.3</v>
+        <v>7591.4</v>
       </c>
       <c r="E151" t="n">
-        <v>9145.9</v>
+        <v>9204.1</v>
       </c>
       <c r="F151" t="n">
-        <v>10099.3</v>
+        <v>10163</v>
       </c>
     </row>
     <row r="152">
@@ -4062,16 +4056,16 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>3576</v>
+        <v>3671</v>
       </c>
       <c r="D153" t="n">
-        <v>14624.1</v>
+        <v>14812.8</v>
       </c>
       <c r="E153" t="n">
-        <v>15762.8</v>
+        <v>15832.8</v>
       </c>
       <c r="F153" t="n">
-        <v>17017.6</v>
+        <v>17211.9</v>
       </c>
     </row>
     <row r="154">
@@ -4110,16 +4104,16 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2845</v>
+        <v>2842</v>
       </c>
       <c r="D155" t="n">
-        <v>12451.1</v>
+        <v>12432</v>
       </c>
       <c r="E155" t="n">
-        <v>15397.3</v>
+        <v>15390.2</v>
       </c>
       <c r="F155" t="n">
-        <v>18794.8</v>
+        <v>18811.5</v>
       </c>
     </row>
     <row r="156">
@@ -4134,16 +4128,16 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1940</v>
+        <v>1945</v>
       </c>
       <c r="D156" t="n">
-        <v>6829.1</v>
+        <v>6812.6</v>
       </c>
       <c r="E156" t="n">
-        <v>8533.200000000001</v>
+        <v>8492.700000000001</v>
       </c>
       <c r="F156" t="n">
-        <v>10361.5</v>
+        <v>10354.5</v>
       </c>
     </row>
     <row r="157">
@@ -4161,7 +4155,7 @@
         <v>1376</v>
       </c>
       <c r="D157" t="n">
-        <v>6508</v>
+        <v>6507.6</v>
       </c>
       <c r="E157" t="n">
         <v>7041.8</v>
@@ -4182,13 +4176,13 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>622</v>
+        <v>604</v>
       </c>
       <c r="D158" t="n">
-        <v>2758</v>
+        <v>2744.2</v>
       </c>
       <c r="E158" t="n">
-        <v>4893.2</v>
+        <v>4888.5</v>
       </c>
       <c r="F158" t="n">
         <v>6189.8</v>
@@ -4206,16 +4200,16 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1674</v>
+        <v>1735</v>
       </c>
       <c r="D159" t="n">
-        <v>6868.8</v>
+        <v>7140.1</v>
       </c>
       <c r="E159" t="n">
-        <v>9190.700000000001</v>
+        <v>9637.700000000001</v>
       </c>
       <c r="F159" t="n">
-        <v>11352.8</v>
+        <v>12055.9</v>
       </c>
     </row>
     <row r="160">
@@ -4230,16 +4224,16 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>455</v>
+        <v>461</v>
       </c>
       <c r="D160" t="n">
-        <v>1880.4</v>
+        <v>1888.8</v>
       </c>
       <c r="E160" t="n">
-        <v>2144</v>
+        <v>2153.5</v>
       </c>
       <c r="F160" t="n">
-        <v>2397.4</v>
+        <v>2409.9</v>
       </c>
     </row>
     <row r="161">
@@ -4254,16 +4248,16 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="D161" t="n">
-        <v>2898.9</v>
+        <v>2910.9</v>
       </c>
       <c r="E161" t="n">
-        <v>3183.1</v>
+        <v>3201.2</v>
       </c>
       <c r="F161" t="n">
-        <v>3423.3</v>
+        <v>3447.5</v>
       </c>
     </row>
     <row r="162">
@@ -4302,16 +4296,16 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="D163" t="n">
-        <v>4444.8</v>
+        <v>4462.8</v>
       </c>
       <c r="E163" t="n">
-        <v>5259.2</v>
+        <v>5285.2</v>
       </c>
       <c r="F163" t="n">
-        <v>5628.6</v>
+        <v>5652.6</v>
       </c>
     </row>
     <row r="164">
@@ -4422,16 +4416,16 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>792</v>
+        <v>798</v>
       </c>
       <c r="D168" t="n">
-        <v>2782.4</v>
+        <v>2774.2</v>
       </c>
       <c r="E168" t="n">
-        <v>3700.4</v>
+        <v>3692.2</v>
       </c>
       <c r="F168" t="n">
-        <v>4723.6</v>
+        <v>4669.3</v>
       </c>
     </row>
     <row r="169">
@@ -4446,16 +4440,16 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>12798</v>
+        <v>12888</v>
       </c>
       <c r="D169" t="n">
-        <v>43303.2</v>
+        <v>43419.9</v>
       </c>
       <c r="E169" t="n">
-        <v>47726.6</v>
+        <v>47767.7</v>
       </c>
       <c r="F169" t="n">
-        <v>50690.1</v>
+        <v>50466.5</v>
       </c>
     </row>
     <row r="170">
@@ -4470,13 +4464,13 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1821</v>
+        <v>1829</v>
       </c>
       <c r="D170" t="n">
-        <v>7088.4</v>
+        <v>7092.9</v>
       </c>
       <c r="E170" t="n">
-        <v>8172.6</v>
+        <v>8168.1</v>
       </c>
       <c r="F170" t="n">
         <v>8940.6</v>
@@ -4521,13 +4515,13 @@
         <v>10003</v>
       </c>
       <c r="D172" t="n">
-        <v>38921.6</v>
+        <v>39168.8</v>
       </c>
       <c r="E172" t="n">
-        <v>45762.3</v>
+        <v>46037.2</v>
       </c>
       <c r="F172" t="n">
-        <v>51602.7</v>
+        <v>52136.8</v>
       </c>
     </row>
     <row r="173">
@@ -4542,16 +4536,16 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1480</v>
+        <v>1499</v>
       </c>
       <c r="D173" t="n">
-        <v>2636.4</v>
+        <v>2659.2</v>
       </c>
       <c r="E173" t="n">
-        <v>4927.2</v>
+        <v>4935</v>
       </c>
       <c r="F173" t="n">
-        <v>5503</v>
+        <v>5511.5</v>
       </c>
     </row>
     <row r="174">
@@ -4593,13 +4587,13 @@
         <v>2034</v>
       </c>
       <c r="D175" t="n">
-        <v>11620.7</v>
+        <v>11444.5</v>
       </c>
       <c r="E175" t="n">
-        <v>40233</v>
+        <v>39869.5</v>
       </c>
       <c r="F175" t="n">
-        <v>60285.2</v>
+        <v>61536.8</v>
       </c>
     </row>
     <row r="176">
@@ -4617,10 +4611,10 @@
         <v>1199</v>
       </c>
       <c r="D176" t="n">
-        <v>5086.2</v>
+        <v>5086.1</v>
       </c>
       <c r="E176" t="n">
-        <v>5624.6</v>
+        <v>5624.8</v>
       </c>
       <c r="F176" t="n">
         <v>6159</v>
@@ -4665,10 +4659,10 @@
         <v>969</v>
       </c>
       <c r="D178" t="n">
-        <v>5294.7</v>
+        <v>5294.5</v>
       </c>
       <c r="E178" t="n">
-        <v>5593.2</v>
+        <v>5592.8</v>
       </c>
       <c r="F178" t="n">
         <v>5983.8</v>
@@ -4773,16 +4767,16 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="D183" t="n">
-        <v>1617.9</v>
+        <v>1606.1</v>
       </c>
       <c r="E183" t="n">
-        <v>2200.1</v>
+        <v>2195.5</v>
       </c>
       <c r="F183" t="n">
-        <v>2794</v>
+        <v>2769.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-07-17
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -452,7 +452,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>KOSPI200 영업이익 컨센 · 기준일 2026-07-16 · 전주 2026-07-13</t>
+          <t>KOSPI200 영업이익 컨센 · 기준일 2026-07-17 · 전주 2026-07-13</t>
         </is>
       </c>
     </row>
@@ -669,40 +669,40 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1140</v>
+        <v>1132</v>
       </c>
       <c r="D5" t="n">
         <v>1140</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="F5" t="n">
-        <v>5163</v>
+        <v>5126.3</v>
       </c>
       <c r="G5" t="n">
         <v>5163</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="I5" t="n">
-        <v>5718.2</v>
+        <v>5683.2</v>
       </c>
       <c r="J5" t="n">
         <v>5718.2</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="L5" t="n">
-        <v>6160.5</v>
+        <v>6123.2</v>
       </c>
       <c r="M5" t="n">
         <v>6160.5</v>
       </c>
       <c r="N5" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="O5" t="n">
         <v>72500</v>
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4571</v>
+        <v>4572</v>
       </c>
       <c r="D6" t="n">
         <v>4571</v>
@@ -735,22 +735,22 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>17063.8</v>
+        <v>17032.2</v>
       </c>
       <c r="G6" t="n">
         <v>17063.8</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="I6" t="n">
-        <v>23491.7</v>
+        <v>23515</v>
       </c>
       <c r="J6" t="n">
         <v>23491.7</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L6" t="n">
         <v>29523.5</v>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>27946</v>
+        <v>27935</v>
       </c>
       <c r="D9" t="n">
         <v>27920</v>
@@ -906,31 +906,31 @@
         <v>0.1</v>
       </c>
       <c r="F9" t="n">
-        <v>102821.2</v>
+        <v>102889.3</v>
       </c>
       <c r="G9" t="n">
         <v>102466.9</v>
       </c>
       <c r="H9" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="I9" t="n">
-        <v>113657.1</v>
+        <v>113580.6</v>
       </c>
       <c r="J9" t="n">
         <v>113527.7</v>
       </c>
       <c r="K9" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>119510.4</v>
+        <v>119352.9</v>
       </c>
       <c r="M9" t="n">
         <v>120853.9</v>
       </c>
       <c r="N9" t="n">
-        <v>-1.1</v>
+        <v>-1.2</v>
       </c>
       <c r="O9" t="n">
         <v>149700</v>
@@ -1011,40 +1011,40 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2005</v>
+        <v>2026</v>
       </c>
       <c r="D11" t="n">
         <v>2005</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" t="n">
-        <v>8244.4</v>
+        <v>8280.6</v>
       </c>
       <c r="G11" t="n">
         <v>8244.4</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I11" t="n">
-        <v>11142.2</v>
+        <v>11114.9</v>
       </c>
       <c r="J11" t="n">
         <v>11142.2</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="L11" t="n">
-        <v>13878.5</v>
+        <v>13860.7</v>
       </c>
       <c r="M11" t="n">
         <v>13845.2</v>
       </c>
       <c r="N11" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="O11" t="n">
         <v>99000</v>
@@ -1068,40 +1068,40 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>8669</v>
+        <v>8815</v>
       </c>
       <c r="D12" t="n">
         <v>8312</v>
       </c>
       <c r="E12" t="n">
-        <v>4.3</v>
+        <v>6.1</v>
       </c>
       <c r="F12" t="n">
-        <v>30745.2</v>
+        <v>30870.2</v>
       </c>
       <c r="G12" t="n">
         <v>30345.1</v>
       </c>
       <c r="H12" t="n">
-        <v>1.3</v>
+        <v>1.7</v>
       </c>
       <c r="I12" t="n">
-        <v>33631.5</v>
+        <v>33681.5</v>
       </c>
       <c r="J12" t="n">
         <v>32907.2</v>
       </c>
       <c r="K12" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="L12" t="n">
-        <v>34054.8</v>
+        <v>34114</v>
       </c>
       <c r="M12" t="n">
         <v>33721.5</v>
       </c>
       <c r="N12" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
       <c r="O12" t="n">
         <v>701000</v>
@@ -1152,13 +1152,13 @@
         <v>-1.8</v>
       </c>
       <c r="L13" t="n">
-        <v>72135</v>
+        <v>72448</v>
       </c>
       <c r="M13" t="n">
         <v>72135</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O13" t="n">
         <v>93200</v>
@@ -1296,40 +1296,40 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>516</v>
+        <v>529</v>
       </c>
       <c r="D16" t="n">
         <v>508</v>
       </c>
       <c r="E16" t="n">
-        <v>1.6</v>
+        <v>4.1</v>
       </c>
       <c r="F16" t="n">
-        <v>1504</v>
+        <v>1517.9</v>
       </c>
       <c r="G16" t="n">
         <v>1464.4</v>
       </c>
       <c r="H16" t="n">
-        <v>2.7</v>
+        <v>3.7</v>
       </c>
       <c r="I16" t="n">
-        <v>2024.1</v>
+        <v>1976.6</v>
       </c>
       <c r="J16" t="n">
         <v>2038.9</v>
       </c>
       <c r="K16" t="n">
-        <v>-0.7</v>
+        <v>-3.1</v>
       </c>
       <c r="L16" t="n">
-        <v>2335.4</v>
+        <v>2211.6</v>
       </c>
       <c r="M16" t="n">
         <v>2062.4</v>
       </c>
       <c r="N16" t="n">
-        <v>13.2</v>
+        <v>7.2</v>
       </c>
       <c r="O16" t="n">
         <v>32500</v>
@@ -1410,13 +1410,13 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>10521.3</v>
+        <v>10625.3</v>
       </c>
       <c r="G18" t="n">
         <v>10434.4</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8</v>
+        <v>1.8</v>
       </c>
       <c r="I18" t="n">
         <v>12179.5</v>
@@ -1668,31 +1668,31 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1786</v>
+        <v>1781</v>
       </c>
       <c r="D23" t="n">
         <v>1790</v>
       </c>
       <c r="E23" t="n">
-        <v>-0.2</v>
+        <v>-0.5</v>
       </c>
       <c r="F23" t="n">
-        <v>7296.7</v>
+        <v>7309.6</v>
       </c>
       <c r="G23" t="n">
         <v>7298.4</v>
       </c>
       <c r="H23" t="n">
-        <v>-0</v>
+        <v>0.2</v>
       </c>
       <c r="I23" t="n">
-        <v>8769.6</v>
+        <v>8786.1</v>
       </c>
       <c r="J23" t="n">
         <v>8765.200000000001</v>
       </c>
       <c r="K23" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="L23" t="n">
         <v>10286.4</v>
@@ -2067,31 +2067,31 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="D30" t="n">
         <v>485</v>
       </c>
       <c r="E30" t="n">
-        <v>1.4</v>
+        <v>2.5</v>
       </c>
       <c r="F30" t="n">
-        <v>2144</v>
+        <v>2150.9</v>
       </c>
       <c r="G30" t="n">
         <v>2133.8</v>
       </c>
       <c r="H30" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="I30" t="n">
-        <v>2321.7</v>
+        <v>2328.6</v>
       </c>
       <c r="J30" t="n">
         <v>2307.4</v>
       </c>
       <c r="K30" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="L30" t="n">
         <v>2454.5</v>
@@ -2181,31 +2181,31 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>647</v>
+        <v>639</v>
       </c>
       <c r="D32" t="n">
         <v>651</v>
       </c>
       <c r="E32" t="n">
-        <v>-0.6</v>
+        <v>-1.8</v>
       </c>
       <c r="F32" t="n">
-        <v>2131.6</v>
+        <v>2123.5</v>
       </c>
       <c r="G32" t="n">
         <v>2138.2</v>
       </c>
       <c r="H32" t="n">
-        <v>-0.3</v>
+        <v>-0.7</v>
       </c>
       <c r="I32" t="n">
-        <v>2351.1</v>
+        <v>2342</v>
       </c>
       <c r="J32" t="n">
         <v>2364.6</v>
       </c>
       <c r="K32" t="n">
-        <v>-0.6</v>
+        <v>-1</v>
       </c>
       <c r="L32" t="n">
         <v>2484.3</v>
@@ -2238,40 +2238,40 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>30293</v>
+        <v>30232</v>
       </c>
       <c r="D33" t="n">
         <v>31086</v>
       </c>
       <c r="E33" t="n">
-        <v>-2.6</v>
+        <v>-2.7</v>
       </c>
       <c r="F33" t="n">
-        <v>117983.4</v>
+        <v>117500.2</v>
       </c>
       <c r="G33" t="n">
         <v>118721.8</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.6</v>
+        <v>-1</v>
       </c>
       <c r="I33" t="n">
-        <v>132991</v>
+        <v>132780.2</v>
       </c>
       <c r="J33" t="n">
         <v>133560</v>
       </c>
       <c r="K33" t="n">
-        <v>-0.4</v>
+        <v>-0.6</v>
       </c>
       <c r="L33" t="n">
-        <v>145128.6</v>
+        <v>144868.6</v>
       </c>
       <c r="M33" t="n">
         <v>146466.8</v>
       </c>
       <c r="N33" t="n">
-        <v>-0.9</v>
+        <v>-1.1</v>
       </c>
       <c r="O33" t="n">
         <v>425000</v>
@@ -2295,40 +2295,40 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>7241</v>
+        <v>7299</v>
       </c>
       <c r="D34" t="n">
         <v>7419</v>
       </c>
       <c r="E34" t="n">
-        <v>-2.4</v>
+        <v>-1.6</v>
       </c>
       <c r="F34" t="n">
-        <v>30676.6</v>
+        <v>30875.7</v>
       </c>
       <c r="G34" t="n">
         <v>31078.4</v>
       </c>
       <c r="H34" t="n">
-        <v>-1.3</v>
+        <v>-0.7</v>
       </c>
       <c r="I34" t="n">
-        <v>38245.5</v>
+        <v>38602.4</v>
       </c>
       <c r="J34" t="n">
         <v>38922.9</v>
       </c>
       <c r="K34" t="n">
-        <v>-1.7</v>
+        <v>-0.8</v>
       </c>
       <c r="L34" t="n">
-        <v>44284.7</v>
+        <v>44763.8</v>
       </c>
       <c r="M34" t="n">
         <v>44719.4</v>
       </c>
       <c r="N34" t="n">
-        <v>-1</v>
+        <v>0.1</v>
       </c>
       <c r="O34" t="n">
         <v>311500</v>
@@ -2361,13 +2361,13 @@
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>21293.7</v>
+        <v>21330.6</v>
       </c>
       <c r="G35" t="n">
         <v>21132.5</v>
       </c>
       <c r="H35" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="I35" t="n">
         <v>23130.1</v>
@@ -3198,40 +3198,40 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>4015</v>
+        <v>4043</v>
       </c>
       <c r="D50" t="n">
         <v>4015</v>
       </c>
       <c r="E50" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="F50" t="n">
-        <v>16524.3</v>
+        <v>16599.1</v>
       </c>
       <c r="G50" t="n">
         <v>16524.3</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I50" t="n">
-        <v>31390.1</v>
+        <v>31750.1</v>
       </c>
       <c r="J50" t="n">
         <v>31390.1</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="L50" t="n">
-        <v>49657.5</v>
+        <v>50852.8</v>
       </c>
       <c r="M50" t="n">
         <v>49657.5</v>
       </c>
       <c r="N50" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="O50" t="n">
         <v>1277000</v>
@@ -3654,31 +3654,31 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>3735</v>
+        <v>3744</v>
       </c>
       <c r="D58" t="n">
         <v>3902</v>
       </c>
       <c r="E58" t="n">
-        <v>-4.3</v>
+        <v>-4</v>
       </c>
       <c r="F58" t="n">
-        <v>14605.2</v>
+        <v>14649.6</v>
       </c>
       <c r="G58" t="n">
         <v>14956.6</v>
       </c>
       <c r="H58" t="n">
-        <v>-2.3</v>
+        <v>-2.1</v>
       </c>
       <c r="I58" t="n">
-        <v>20139.2</v>
+        <v>20222.6</v>
       </c>
       <c r="J58" t="n">
         <v>20358</v>
       </c>
       <c r="K58" t="n">
-        <v>-1.1</v>
+        <v>-0.7</v>
       </c>
       <c r="L58" t="n">
         <v>23690.3</v>
@@ -3768,22 +3768,22 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1803</v>
+        <v>1823</v>
       </c>
       <c r="D60" t="n">
         <v>1803</v>
       </c>
       <c r="E60" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="F60" t="n">
-        <v>11679.8</v>
+        <v>11828.4</v>
       </c>
       <c r="G60" t="n">
         <v>11679.8</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="I60" t="n">
         <v>13870.9</v>
@@ -3882,40 +3882,40 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>3275</v>
+        <v>3463</v>
       </c>
       <c r="D62" t="n">
         <v>3182</v>
       </c>
       <c r="E62" t="n">
-        <v>2.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F62" t="n">
-        <v>11807.9</v>
+        <v>12211.1</v>
       </c>
       <c r="G62" t="n">
         <v>11608</v>
       </c>
       <c r="H62" t="n">
-        <v>1.7</v>
+        <v>5.2</v>
       </c>
       <c r="I62" t="n">
-        <v>8617.9</v>
+        <v>8944.6</v>
       </c>
       <c r="J62" t="n">
         <v>8554.9</v>
       </c>
       <c r="K62" t="n">
-        <v>0.7</v>
+        <v>4.6</v>
       </c>
       <c r="L62" t="n">
-        <v>9030.200000000001</v>
+        <v>9046.9</v>
       </c>
       <c r="M62" t="n">
         <v>9030.200000000001</v>
       </c>
       <c r="N62" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O62" t="n">
         <v>20050</v>
@@ -4110,16 +4110,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>9096</v>
+        <v>9075</v>
       </c>
       <c r="D66" t="n">
         <v>9088</v>
       </c>
       <c r="E66" t="n">
-        <v>0.1</v>
+        <v>-0.1</v>
       </c>
       <c r="F66" t="n">
-        <v>37335.7</v>
+        <v>37334.3</v>
       </c>
       <c r="G66" t="n">
         <v>37234.8</v>
@@ -4128,16 +4128,16 @@
         <v>0.3</v>
       </c>
       <c r="I66" t="n">
-        <v>42530.4</v>
+        <v>42519.2</v>
       </c>
       <c r="J66" t="n">
         <v>42459</v>
       </c>
       <c r="K66" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L66" t="n">
-        <v>46497.8</v>
+        <v>46485</v>
       </c>
       <c r="M66" t="n">
         <v>46500.8</v>
@@ -4167,40 +4167,40 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>10025</v>
+        <v>9962</v>
       </c>
       <c r="D67" t="n">
         <v>10136</v>
       </c>
       <c r="E67" t="n">
-        <v>-1.1</v>
+        <v>-1.7</v>
       </c>
       <c r="F67" t="n">
-        <v>42746.8</v>
+        <v>42796.2</v>
       </c>
       <c r="G67" t="n">
         <v>42647.9</v>
       </c>
       <c r="H67" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="I67" t="n">
-        <v>55240.3</v>
+        <v>54920.9</v>
       </c>
       <c r="J67" t="n">
         <v>55103.9</v>
       </c>
       <c r="K67" t="n">
-        <v>0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="L67" t="n">
-        <v>61947.8</v>
+        <v>61626.3</v>
       </c>
       <c r="M67" t="n">
         <v>62256.4</v>
       </c>
       <c r="N67" t="n">
-        <v>-0.5</v>
+        <v>-1</v>
       </c>
       <c r="O67" t="n">
         <v>943000</v>
@@ -4290,31 +4290,31 @@
         <v>1</v>
       </c>
       <c r="F69" t="n">
-        <v>1889.2</v>
+        <v>1886.8</v>
       </c>
       <c r="G69" t="n">
         <v>1879.9</v>
       </c>
       <c r="H69" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="I69" t="n">
-        <v>2374</v>
+        <v>2361</v>
       </c>
       <c r="J69" t="n">
         <v>2386.1</v>
       </c>
       <c r="K69" t="n">
-        <v>-0.5</v>
+        <v>-1.1</v>
       </c>
       <c r="L69" t="n">
-        <v>2982.6</v>
+        <v>2994.7</v>
       </c>
       <c r="M69" t="n">
         <v>3072.4</v>
       </c>
       <c r="N69" t="n">
-        <v>-2.9</v>
+        <v>-2.5</v>
       </c>
       <c r="O69" t="n">
         <v>244500</v>
@@ -4338,40 +4338,40 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>19553</v>
+        <v>20041</v>
       </c>
       <c r="D70" t="n">
         <v>19122</v>
       </c>
       <c r="E70" t="n">
-        <v>2.3</v>
+        <v>4.8</v>
       </c>
       <c r="F70" t="n">
-        <v>98532.2</v>
+        <v>100192.7</v>
       </c>
       <c r="G70" t="n">
         <v>97617.5</v>
       </c>
       <c r="H70" t="n">
-        <v>0.9</v>
+        <v>2.6</v>
       </c>
       <c r="I70" t="n">
-        <v>136740.3</v>
+        <v>139318.5</v>
       </c>
       <c r="J70" t="n">
         <v>134651.3</v>
       </c>
       <c r="K70" t="n">
-        <v>1.6</v>
+        <v>3.5</v>
       </c>
       <c r="L70" t="n">
-        <v>149138.7</v>
+        <v>152635.4</v>
       </c>
       <c r="M70" t="n">
         <v>148583.9</v>
       </c>
       <c r="N70" t="n">
-        <v>0.4</v>
+        <v>2.7</v>
       </c>
       <c r="O70" t="n">
         <v>34050</v>
@@ -4452,40 +4452,40 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>5425</v>
+        <v>5446</v>
       </c>
       <c r="D72" t="n">
         <v>5307</v>
       </c>
       <c r="E72" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="F72" t="n">
-        <v>19372.4</v>
+        <v>19444.4</v>
       </c>
       <c r="G72" t="n">
         <v>19164.7</v>
       </c>
       <c r="H72" t="n">
-        <v>1.1</v>
+        <v>1.5</v>
       </c>
       <c r="I72" t="n">
-        <v>20475.3</v>
+        <v>20548.8</v>
       </c>
       <c r="J72" t="n">
         <v>20300.4</v>
       </c>
       <c r="K72" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="L72" t="n">
-        <v>21634.8</v>
+        <v>21669.4</v>
       </c>
       <c r="M72" t="n">
         <v>21507.9</v>
       </c>
       <c r="N72" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="O72" t="n">
         <v>89700</v>
@@ -4623,40 +4623,40 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D75" t="n">
         <v>1095</v>
       </c>
       <c r="E75" t="n">
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
       <c r="F75" t="n">
-        <v>4287.6</v>
+        <v>4307</v>
       </c>
       <c r="G75" t="n">
         <v>4279.2</v>
       </c>
       <c r="H75" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="I75" t="n">
-        <v>5039.6</v>
+        <v>5064.6</v>
       </c>
       <c r="J75" t="n">
         <v>4997.4</v>
       </c>
       <c r="K75" t="n">
-        <v>0.8</v>
+        <v>1.3</v>
       </c>
       <c r="L75" t="n">
-        <v>5833.9</v>
+        <v>5878.2</v>
       </c>
       <c r="M75" t="n">
         <v>5789.7</v>
       </c>
       <c r="N75" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="O75" t="n">
         <v>3490</v>
@@ -4965,34 +4965,34 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1546</v>
+        <v>1544</v>
       </c>
       <c r="D81" t="n">
         <v>1503</v>
       </c>
       <c r="E81" t="n">
-        <v>2.9</v>
+        <v>2.7</v>
       </c>
       <c r="F81" t="n">
-        <v>5936.6</v>
+        <v>5923</v>
       </c>
       <c r="G81" t="n">
         <v>5854.9</v>
       </c>
       <c r="H81" t="n">
-        <v>1.4</v>
+        <v>1.2</v>
       </c>
       <c r="I81" t="n">
-        <v>6133.7</v>
+        <v>6114.9</v>
       </c>
       <c r="J81" t="n">
         <v>6091.5</v>
       </c>
       <c r="K81" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="L81" t="n">
-        <v>6369.3</v>
+        <v>6369.4</v>
       </c>
       <c r="M81" t="n">
         <v>6368.1</v>
@@ -5136,7 +5136,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>6038</v>
+        <v>6037</v>
       </c>
       <c r="D84" t="n">
         <v>6081</v>
@@ -5145,31 +5145,31 @@
         <v>-0.7</v>
       </c>
       <c r="F84" t="n">
-        <v>20519.3</v>
+        <v>20554.3</v>
       </c>
       <c r="G84" t="n">
         <v>20653.3</v>
       </c>
       <c r="H84" t="n">
-        <v>-0.6</v>
+        <v>-0.5</v>
       </c>
       <c r="I84" t="n">
-        <v>22467.7</v>
+        <v>22489.1</v>
       </c>
       <c r="J84" t="n">
         <v>22502.9</v>
       </c>
       <c r="K84" t="n">
-        <v>-0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="L84" t="n">
-        <v>23804.6</v>
+        <v>23864.3</v>
       </c>
       <c r="M84" t="n">
         <v>23821.8</v>
       </c>
       <c r="N84" t="n">
-        <v>-0.1</v>
+        <v>0.2</v>
       </c>
       <c r="O84" t="n">
         <v>52400</v>
@@ -5193,25 +5193,25 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>3072</v>
+        <v>3087</v>
       </c>
       <c r="D85" t="n">
         <v>3062</v>
       </c>
       <c r="E85" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="F85" t="n">
-        <v>11105.5</v>
+        <v>11108.8</v>
       </c>
       <c r="G85" t="n">
         <v>11111.1</v>
       </c>
       <c r="H85" t="n">
-        <v>-0.1</v>
+        <v>-0</v>
       </c>
       <c r="I85" t="n">
-        <v>11996.9</v>
+        <v>11988.9</v>
       </c>
       <c r="J85" t="n">
         <v>11959</v>
@@ -5220,7 +5220,7 @@
         <v>0.3</v>
       </c>
       <c r="L85" t="n">
-        <v>12762.1</v>
+        <v>12761.4</v>
       </c>
       <c r="M85" t="n">
         <v>12715.1</v>
@@ -5250,22 +5250,22 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>10237</v>
+        <v>10171</v>
       </c>
       <c r="D86" t="n">
         <v>10237</v>
       </c>
       <c r="E86" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="F86" t="n">
-        <v>33019.2</v>
+        <v>33448.1</v>
       </c>
       <c r="G86" t="n">
         <v>33019.2</v>
       </c>
       <c r="H86" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="I86" t="n">
         <v>52718.3</v>
@@ -5307,31 +5307,31 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>3919</v>
+        <v>3937</v>
       </c>
       <c r="D87" t="n">
         <v>3866</v>
       </c>
       <c r="E87" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="F87" t="n">
-        <v>15120.1</v>
+        <v>15140.1</v>
       </c>
       <c r="G87" t="n">
         <v>15108.4</v>
       </c>
       <c r="H87" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I87" t="n">
-        <v>16261.1</v>
+        <v>16276.8</v>
       </c>
       <c r="J87" t="n">
         <v>16302.5</v>
       </c>
       <c r="K87" t="n">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="L87" t="n">
         <v>17211.8</v>
@@ -5478,40 +5478,40 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>488</v>
+        <v>472</v>
       </c>
       <c r="D90" t="n">
         <v>498</v>
       </c>
       <c r="E90" t="n">
-        <v>-2</v>
+        <v>-5.2</v>
       </c>
       <c r="F90" t="n">
-        <v>1844.2</v>
+        <v>1773.4</v>
       </c>
       <c r="G90" t="n">
         <v>1856.2</v>
       </c>
       <c r="H90" t="n">
-        <v>-0.6</v>
+        <v>-4.5</v>
       </c>
       <c r="I90" t="n">
-        <v>2244.1</v>
+        <v>2147.9</v>
       </c>
       <c r="J90" t="n">
         <v>2235.1</v>
       </c>
       <c r="K90" t="n">
-        <v>0.4</v>
+        <v>-3.9</v>
       </c>
       <c r="L90" t="n">
-        <v>2455.1</v>
+        <v>2443.3</v>
       </c>
       <c r="M90" t="n">
         <v>2456</v>
       </c>
       <c r="N90" t="n">
-        <v>-0</v>
+        <v>-0.5</v>
       </c>
       <c r="O90" t="n">
         <v>10190</v>
@@ -5592,40 +5592,40 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D92" t="n">
         <v>489</v>
       </c>
       <c r="E92" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="F92" t="n">
-        <v>2212.7</v>
+        <v>2231.8</v>
       </c>
       <c r="G92" t="n">
         <v>2212.7</v>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="I92" t="n">
-        <v>2287.4</v>
+        <v>2312.7</v>
       </c>
       <c r="J92" t="n">
         <v>2287.4</v>
       </c>
       <c r="K92" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="L92" t="n">
-        <v>2883.4</v>
+        <v>2882</v>
       </c>
       <c r="M92" t="n">
         <v>2883.4</v>
       </c>
       <c r="N92" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="O92" t="n">
         <v>14410</v>
@@ -5667,22 +5667,22 @@
         <v>-0.3</v>
       </c>
       <c r="I93" t="n">
-        <v>27590</v>
+        <v>27632</v>
       </c>
       <c r="J93" t="n">
         <v>27672</v>
       </c>
       <c r="K93" t="n">
-        <v>-0.3</v>
+        <v>-0.1</v>
       </c>
       <c r="L93" t="n">
-        <v>31240.8</v>
+        <v>31373.3</v>
       </c>
       <c r="M93" t="n">
         <v>31358.5</v>
       </c>
       <c r="N93" t="n">
-        <v>-0.4</v>
+        <v>0</v>
       </c>
       <c r="O93" t="n">
         <v>190000</v>
@@ -5820,40 +5820,40 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1284</v>
+        <v>1294</v>
       </c>
       <c r="D96" t="n">
         <v>1270</v>
       </c>
       <c r="E96" t="n">
-        <v>1.1</v>
+        <v>1.9</v>
       </c>
       <c r="F96" t="n">
-        <v>5019.9</v>
+        <v>5051.7</v>
       </c>
       <c r="G96" t="n">
         <v>5026.8</v>
       </c>
       <c r="H96" t="n">
-        <v>-0.1</v>
+        <v>0.5</v>
       </c>
       <c r="I96" t="n">
-        <v>5897.3</v>
+        <v>5877.6</v>
       </c>
       <c r="J96" t="n">
         <v>5876.9</v>
       </c>
       <c r="K96" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="L96" t="n">
-        <v>5924.6</v>
+        <v>5885.7</v>
       </c>
       <c r="M96" t="n">
         <v>5924.6</v>
       </c>
       <c r="N96" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="O96" t="n">
         <v>223000</v>
@@ -5934,31 +5934,31 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>5300</v>
+        <v>5335</v>
       </c>
       <c r="D98" t="n">
         <v>5252</v>
       </c>
       <c r="E98" t="n">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="F98" t="n">
-        <v>19176.2</v>
+        <v>19239.6</v>
       </c>
       <c r="G98" t="n">
         <v>19011.6</v>
       </c>
       <c r="H98" t="n">
-        <v>0.9</v>
+        <v>1.2</v>
       </c>
       <c r="I98" t="n">
-        <v>23327.3</v>
+        <v>23307.3</v>
       </c>
       <c r="J98" t="n">
         <v>23489.7</v>
       </c>
       <c r="K98" t="n">
-        <v>-0.7</v>
+        <v>-0.8</v>
       </c>
       <c r="L98" t="n">
         <v>27375.2</v>
@@ -6105,25 +6105,25 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>3557</v>
+        <v>3601</v>
       </c>
       <c r="D101" t="n">
         <v>3517</v>
       </c>
       <c r="E101" t="n">
-        <v>1.1</v>
+        <v>2.4</v>
       </c>
       <c r="F101" t="n">
-        <v>13991.6</v>
+        <v>14034.5</v>
       </c>
       <c r="G101" t="n">
         <v>13940.8</v>
       </c>
       <c r="H101" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
       <c r="I101" t="n">
-        <v>15191</v>
+        <v>15201.9</v>
       </c>
       <c r="J101" t="n">
         <v>15092.4</v>
@@ -6132,13 +6132,13 @@
         <v>0.7</v>
       </c>
       <c r="L101" t="n">
-        <v>15938.8</v>
+        <v>15932.4</v>
       </c>
       <c r="M101" t="n">
         <v>15771.5</v>
       </c>
       <c r="N101" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="O101" t="n">
         <v>50900</v>
@@ -6162,40 +6162,40 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>951</v>
+        <v>931</v>
       </c>
       <c r="D102" t="n">
         <v>1002</v>
       </c>
       <c r="E102" t="n">
-        <v>-5.1</v>
+        <v>-7.1</v>
       </c>
       <c r="F102" t="n">
-        <v>4564.2</v>
+        <v>4546.9</v>
       </c>
       <c r="G102" t="n">
         <v>4679.8</v>
       </c>
       <c r="H102" t="n">
-        <v>-2.5</v>
+        <v>-2.8</v>
       </c>
       <c r="I102" t="n">
-        <v>6612.7</v>
+        <v>6570.8</v>
       </c>
       <c r="J102" t="n">
         <v>6650.4</v>
       </c>
       <c r="K102" t="n">
-        <v>-0.6</v>
+        <v>-1.2</v>
       </c>
       <c r="L102" t="n">
-        <v>8049.8</v>
+        <v>8017.4</v>
       </c>
       <c r="M102" t="n">
         <v>8075.1</v>
       </c>
       <c r="N102" t="n">
-        <v>-0.3</v>
+        <v>-0.7</v>
       </c>
       <c r="O102" t="n">
         <v>149200</v>
@@ -6561,40 +6561,40 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2725</v>
+        <v>2706</v>
       </c>
       <c r="D109" t="n">
         <v>2768</v>
       </c>
       <c r="E109" t="n">
-        <v>-1.6</v>
+        <v>-2.2</v>
       </c>
       <c r="F109" t="n">
-        <v>11569.8</v>
+        <v>11551.8</v>
       </c>
       <c r="G109" t="n">
         <v>11805.3</v>
       </c>
       <c r="H109" t="n">
-        <v>-2</v>
+        <v>-2.1</v>
       </c>
       <c r="I109" t="n">
-        <v>15181.7</v>
+        <v>15008.9</v>
       </c>
       <c r="J109" t="n">
         <v>15557.9</v>
       </c>
       <c r="K109" t="n">
-        <v>-2.4</v>
+        <v>-3.5</v>
       </c>
       <c r="L109" t="n">
-        <v>18232.4</v>
+        <v>18246.1</v>
       </c>
       <c r="M109" t="n">
         <v>18626.1</v>
       </c>
       <c r="N109" t="n">
-        <v>-2.1</v>
+        <v>-2</v>
       </c>
       <c r="O109" t="n">
         <v>159000</v>
@@ -6732,40 +6732,40 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>491</v>
+        <v>484</v>
       </c>
       <c r="D112" t="n">
         <v>502</v>
       </c>
       <c r="E112" t="n">
-        <v>-2.2</v>
+        <v>-3.6</v>
       </c>
       <c r="F112" t="n">
-        <v>2488</v>
+        <v>2479.7</v>
       </c>
       <c r="G112" t="n">
         <v>2517.9</v>
       </c>
       <c r="H112" t="n">
-        <v>-1.2</v>
+        <v>-1.5</v>
       </c>
       <c r="I112" t="n">
-        <v>2330.9</v>
+        <v>2351.1</v>
       </c>
       <c r="J112" t="n">
         <v>2311</v>
       </c>
       <c r="K112" t="n">
-        <v>0.9</v>
+        <v>1.7</v>
       </c>
       <c r="L112" t="n">
-        <v>3311.8</v>
+        <v>3364.5</v>
       </c>
       <c r="M112" t="n">
         <v>3257.2</v>
       </c>
       <c r="N112" t="n">
-        <v>1.7</v>
+        <v>3.3</v>
       </c>
       <c r="O112" t="n">
         <v>92000</v>
@@ -7416,40 +7416,40 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="D124" t="n">
         <v>595</v>
       </c>
       <c r="E124" t="n">
-        <v>-2.4</v>
+        <v>-2.5</v>
       </c>
       <c r="F124" t="n">
-        <v>2404.7</v>
+        <v>2416.7</v>
       </c>
       <c r="G124" t="n">
         <v>2407.6</v>
       </c>
       <c r="H124" t="n">
-        <v>-0.1</v>
+        <v>0.4</v>
       </c>
       <c r="I124" t="n">
-        <v>3819.7</v>
+        <v>3854</v>
       </c>
       <c r="J124" t="n">
         <v>3687.6</v>
       </c>
       <c r="K124" t="n">
-        <v>3.6</v>
+        <v>4.5</v>
       </c>
       <c r="L124" t="n">
-        <v>4613</v>
+        <v>4707.3</v>
       </c>
       <c r="M124" t="n">
         <v>4521.6</v>
       </c>
       <c r="N124" t="n">
-        <v>2</v>
+        <v>4.1</v>
       </c>
       <c r="O124" t="n">
         <v>46900</v>
@@ -7587,13 +7587,13 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>8267.299999999999</v>
+        <v>8338.200000000001</v>
       </c>
       <c r="G127" t="n">
         <v>8132.5</v>
       </c>
       <c r="H127" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="I127" t="n">
         <v>9144.799999999999</v>
@@ -7722,40 +7722,40 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>14936</v>
+        <v>15727</v>
       </c>
       <c r="D130" t="n">
         <v>14123</v>
       </c>
       <c r="E130" t="n">
-        <v>5.8</v>
+        <v>11.4</v>
       </c>
       <c r="F130" t="n">
-        <v>52816.8</v>
+        <v>54903.6</v>
       </c>
       <c r="G130" t="n">
         <v>50950.2</v>
       </c>
       <c r="H130" t="n">
-        <v>3.7</v>
+        <v>7.8</v>
       </c>
       <c r="I130" t="n">
-        <v>31630.4</v>
+        <v>33584.2</v>
       </c>
       <c r="J130" t="n">
         <v>31187.9</v>
       </c>
       <c r="K130" t="n">
-        <v>1.4</v>
+        <v>7.7</v>
       </c>
       <c r="L130" t="n">
-        <v>37398.4</v>
+        <v>38301.9</v>
       </c>
       <c r="M130" t="n">
         <v>36712.4</v>
       </c>
       <c r="N130" t="n">
-        <v>1.9</v>
+        <v>4.3</v>
       </c>
       <c r="O130" t="n">
         <v>121400</v>
@@ -7779,31 +7779,31 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2779</v>
+        <v>2777</v>
       </c>
       <c r="D131" t="n">
         <v>2773</v>
       </c>
       <c r="E131" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F131" t="n">
-        <v>12844.8</v>
+        <v>12832.5</v>
       </c>
       <c r="G131" t="n">
         <v>12855.1</v>
       </c>
       <c r="H131" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="I131" t="n">
-        <v>14582.7</v>
+        <v>14554.2</v>
       </c>
       <c r="J131" t="n">
         <v>14545.4</v>
       </c>
       <c r="K131" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="L131" t="n">
         <v>16091</v>
@@ -7836,40 +7836,40 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>848</v>
+        <v>819</v>
       </c>
       <c r="D132" t="n">
         <v>831</v>
       </c>
       <c r="E132" t="n">
-        <v>2</v>
+        <v>-1.4</v>
       </c>
       <c r="F132" t="n">
-        <v>3654.7</v>
+        <v>3630.2</v>
       </c>
       <c r="G132" t="n">
         <v>3617.8</v>
       </c>
       <c r="H132" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="I132" t="n">
-        <v>3583.9</v>
+        <v>3537.3</v>
       </c>
       <c r="J132" t="n">
         <v>3606.6</v>
       </c>
       <c r="K132" t="n">
-        <v>-0.6</v>
+        <v>-1.9</v>
       </c>
       <c r="L132" t="n">
-        <v>3961.3</v>
+        <v>3903.7</v>
       </c>
       <c r="M132" t="n">
         <v>3982.7</v>
       </c>
       <c r="N132" t="n">
-        <v>-0.5</v>
+        <v>-2</v>
       </c>
       <c r="O132" t="n">
         <v>62100</v>
@@ -8064,40 +8064,40 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>712</v>
+        <v>726</v>
       </c>
       <c r="D136" t="n">
         <v>712</v>
       </c>
       <c r="E136" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F136" t="n">
-        <v>2243.2</v>
+        <v>2328.2</v>
       </c>
       <c r="G136" t="n">
         <v>2243.2</v>
       </c>
       <c r="H136" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="I136" t="n">
-        <v>2576.2</v>
+        <v>2607.6</v>
       </c>
       <c r="J136" t="n">
         <v>2576.2</v>
       </c>
       <c r="K136" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="L136" t="n">
-        <v>2980.4</v>
+        <v>3037.5</v>
       </c>
       <c r="M136" t="n">
         <v>2981.2</v>
       </c>
       <c r="N136" t="n">
-        <v>-0</v>
+        <v>1.9</v>
       </c>
       <c r="O136" t="n">
         <v>53600</v>
@@ -8121,40 +8121,40 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1042</v>
+        <v>1056</v>
       </c>
       <c r="D137" t="n">
         <v>866</v>
       </c>
       <c r="E137" t="n">
-        <v>20.3</v>
+        <v>21.9</v>
       </c>
       <c r="F137" t="n">
-        <v>3105.6</v>
+        <v>3103.2</v>
       </c>
       <c r="G137" t="n">
         <v>2961.1</v>
       </c>
       <c r="H137" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="I137" t="n">
-        <v>3147.9</v>
+        <v>3164.5</v>
       </c>
       <c r="J137" t="n">
         <v>3106.5</v>
       </c>
       <c r="K137" t="n">
-        <v>1.3</v>
+        <v>1.9</v>
       </c>
       <c r="L137" t="n">
-        <v>3403.1</v>
+        <v>3447.3</v>
       </c>
       <c r="M137" t="n">
         <v>3328.3</v>
       </c>
       <c r="N137" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="O137" t="n">
         <v>386000</v>
@@ -8463,40 +8463,40 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="D143" t="n">
         <v>953</v>
       </c>
       <c r="E143" t="n">
-        <v>-0.6</v>
+        <v>-0.2</v>
       </c>
       <c r="F143" t="n">
-        <v>3146.1</v>
+        <v>3152.6</v>
       </c>
       <c r="G143" t="n">
         <v>3148.2</v>
       </c>
       <c r="H143" t="n">
-        <v>-0.1</v>
+        <v>0.1</v>
       </c>
       <c r="I143" t="n">
-        <v>3638.5</v>
+        <v>3650.9</v>
       </c>
       <c r="J143" t="n">
         <v>3633</v>
       </c>
       <c r="K143" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="L143" t="n">
-        <v>4102.8</v>
+        <v>4118.9</v>
       </c>
       <c r="M143" t="n">
         <v>4096.7</v>
       </c>
       <c r="N143" t="n">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="O143" t="n">
         <v>107600</v>
@@ -8577,40 +8577,40 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="D145" t="n">
         <v>210</v>
       </c>
       <c r="E145" t="n">
-        <v>0</v>
+        <v>-3.8</v>
       </c>
       <c r="F145" t="n">
-        <v>783.8</v>
+        <v>785.8</v>
       </c>
       <c r="G145" t="n">
         <v>804.6</v>
       </c>
       <c r="H145" t="n">
-        <v>-2.6</v>
+        <v>-2.3</v>
       </c>
       <c r="I145" t="n">
-        <v>903.5</v>
+        <v>901.4</v>
       </c>
       <c r="J145" t="n">
         <v>937.8</v>
       </c>
       <c r="K145" t="n">
-        <v>-3.7</v>
+        <v>-3.9</v>
       </c>
       <c r="L145" t="n">
-        <v>988.5</v>
+        <v>984.8</v>
       </c>
       <c r="M145" t="n">
         <v>1023.2</v>
       </c>
       <c r="N145" t="n">
-        <v>-3.4</v>
+        <v>-3.8</v>
       </c>
       <c r="O145" t="n">
         <v>68300</v>
@@ -8691,34 +8691,34 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="D147" t="n">
         <v>695</v>
       </c>
       <c r="E147" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="F147" t="n">
-        <v>2334.6</v>
+        <v>2331.9</v>
       </c>
       <c r="G147" t="n">
         <v>2327.5</v>
       </c>
       <c r="H147" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="I147" t="n">
-        <v>2777.6</v>
+        <v>2774.9</v>
       </c>
       <c r="J147" t="n">
         <v>2766.5</v>
       </c>
       <c r="K147" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L147" t="n">
-        <v>3207.5</v>
+        <v>3206.8</v>
       </c>
       <c r="M147" t="n">
         <v>3194</v>
@@ -8748,25 +8748,25 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1027</v>
+        <v>1022</v>
       </c>
       <c r="D148" t="n">
         <v>1037</v>
       </c>
       <c r="E148" t="n">
-        <v>-1</v>
+        <v>-1.4</v>
       </c>
       <c r="F148" t="n">
-        <v>4032.2</v>
+        <v>4022.1</v>
       </c>
       <c r="G148" t="n">
         <v>4028.2</v>
       </c>
       <c r="H148" t="n">
-        <v>0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="I148" t="n">
-        <v>4689.4</v>
+        <v>4688.9</v>
       </c>
       <c r="J148" t="n">
         <v>4685.9</v>
@@ -8775,13 +8775,13 @@
         <v>0.1</v>
       </c>
       <c r="L148" t="n">
-        <v>5201.8</v>
+        <v>5231.2</v>
       </c>
       <c r="M148" t="n">
         <v>5234.6</v>
       </c>
       <c r="N148" t="n">
-        <v>-0.6</v>
+        <v>-0.1</v>
       </c>
       <c r="O148" t="n">
         <v>44800</v>
@@ -9204,31 +9204,31 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1373</v>
+        <v>1370</v>
       </c>
       <c r="D156" t="n">
         <v>1376</v>
       </c>
       <c r="E156" t="n">
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="F156" t="n">
-        <v>6482.2</v>
+        <v>6487.6</v>
       </c>
       <c r="G156" t="n">
         <v>6507.6</v>
       </c>
       <c r="H156" t="n">
-        <v>-0.4</v>
+        <v>-0.3</v>
       </c>
       <c r="I156" t="n">
-        <v>7020.5</v>
+        <v>7029.8</v>
       </c>
       <c r="J156" t="n">
         <v>7041.8</v>
       </c>
       <c r="K156" t="n">
-        <v>-0.3</v>
+        <v>-0.2</v>
       </c>
       <c r="L156" t="n">
         <v>7523.1</v>
@@ -9375,31 +9375,31 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="D159" t="n">
         <v>461</v>
       </c>
       <c r="E159" t="n">
-        <v>0.7</v>
+        <v>2.4</v>
       </c>
       <c r="F159" t="n">
-        <v>1892.3</v>
+        <v>1902.3</v>
       </c>
       <c r="G159" t="n">
         <v>1888.8</v>
       </c>
       <c r="H159" t="n">
-        <v>0.2</v>
+        <v>0.7</v>
       </c>
       <c r="I159" t="n">
-        <v>2159.4</v>
+        <v>2170.4</v>
       </c>
       <c r="J159" t="n">
         <v>2153.5</v>
       </c>
       <c r="K159" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
       <c r="L159" t="n">
         <v>2398.1</v>
@@ -9546,40 +9546,40 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1279</v>
+        <v>1305</v>
       </c>
       <c r="D162" t="n">
         <v>1279</v>
       </c>
       <c r="E162" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F162" t="n">
-        <v>4462.8</v>
+        <v>4538.8</v>
       </c>
       <c r="G162" t="n">
         <v>4462.8</v>
       </c>
       <c r="H162" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="I162" t="n">
-        <v>5285.2</v>
+        <v>5431.5</v>
       </c>
       <c r="J162" t="n">
         <v>5285.2</v>
       </c>
       <c r="K162" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="L162" t="n">
-        <v>5652.6</v>
+        <v>5773.2</v>
       </c>
       <c r="M162" t="n">
         <v>5652.6</v>
       </c>
       <c r="N162" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="O162" t="n">
         <v>278000</v>
@@ -9603,40 +9603,40 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2806</v>
+        <v>2812</v>
       </c>
       <c r="D163" t="n">
         <v>2845</v>
       </c>
       <c r="E163" t="n">
-        <v>-1.4</v>
+        <v>-1.2</v>
       </c>
       <c r="F163" t="n">
-        <v>10879.9</v>
+        <v>10910.6</v>
       </c>
       <c r="G163" t="n">
         <v>10942.1</v>
       </c>
       <c r="H163" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="I163" t="n">
-        <v>15397.1</v>
+        <v>15413.5</v>
       </c>
       <c r="J163" t="n">
         <v>15477.6</v>
       </c>
       <c r="K163" t="n">
-        <v>-0.5</v>
+        <v>-0.4</v>
       </c>
       <c r="L163" t="n">
-        <v>19657.9</v>
+        <v>20226.6</v>
       </c>
       <c r="M163" t="n">
         <v>19558.8</v>
       </c>
       <c r="N163" t="n">
-        <v>0.5</v>
+        <v>3.4</v>
       </c>
       <c r="O163" t="n">
         <v>2789000</v>
@@ -10059,31 +10059,31 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>9925</v>
+        <v>9910</v>
       </c>
       <c r="D171" t="n">
         <v>9902</v>
       </c>
       <c r="E171" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="F171" t="n">
-        <v>38979</v>
+        <v>38876</v>
       </c>
       <c r="G171" t="n">
         <v>38897.6</v>
       </c>
       <c r="H171" t="n">
-        <v>0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="I171" t="n">
-        <v>45775.8</v>
+        <v>45739.8</v>
       </c>
       <c r="J171" t="n">
         <v>45686.3</v>
       </c>
       <c r="K171" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L171" t="n">
         <v>52641.7</v>
@@ -10287,25 +10287,25 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1222</v>
+        <v>1227</v>
       </c>
       <c r="D175" t="n">
         <v>1199</v>
       </c>
       <c r="E175" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="F175" t="n">
-        <v>5218.5</v>
+        <v>5259.8</v>
       </c>
       <c r="G175" t="n">
         <v>5129.8</v>
       </c>
       <c r="H175" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
       <c r="I175" t="n">
-        <v>5621.3</v>
+        <v>5620.8</v>
       </c>
       <c r="J175" t="n">
         <v>5671.2</v>
@@ -10314,13 +10314,13 @@
         <v>-0.9</v>
       </c>
       <c r="L175" t="n">
-        <v>6108.3</v>
+        <v>6112.2</v>
       </c>
       <c r="M175" t="n">
         <v>6198.3</v>
       </c>
       <c r="N175" t="n">
-        <v>-1.5</v>
+        <v>-1.4</v>
       </c>
       <c r="O175" t="n">
         <v>60200</v>
@@ -10344,13 +10344,13 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="D176" t="n">
         <v>323</v>
       </c>
       <c r="E176" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="F176" t="n">
         <v>1388.2</v>
@@ -10401,16 +10401,16 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="D177" t="n">
         <v>969</v>
       </c>
       <c r="E177" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="F177" t="n">
-        <v>5307.8</v>
+        <v>5308.8</v>
       </c>
       <c r="G177" t="n">
         <v>5294.5</v>
@@ -10419,22 +10419,22 @@
         <v>0.3</v>
       </c>
       <c r="I177" t="n">
-        <v>5622.7</v>
+        <v>5626.7</v>
       </c>
       <c r="J177" t="n">
         <v>5592.8</v>
       </c>
       <c r="K177" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="L177" t="n">
-        <v>6051.2</v>
+        <v>6061.2</v>
       </c>
       <c r="M177" t="n">
         <v>5983.8</v>
       </c>
       <c r="N177" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="O177" t="n">
         <v>79000</v>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-08-02
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -455,7 +455,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-07-31 · 전주 2026-07-26</t>
+          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-08-02 · 전주 2026-07-26</t>
         </is>
       </c>
     </row>
@@ -669,31 +669,31 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>1302.1</v>
+        <v>1276.2</v>
       </c>
       <c r="J4" t="n">
         <v>1302.1</v>
       </c>
       <c r="K4" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L4" t="n">
-        <v>2221.5</v>
+        <v>2057.1</v>
       </c>
       <c r="M4" t="n">
         <v>2221.5</v>
       </c>
       <c r="N4" t="n">
-        <v>0</v>
+        <v>-7.4</v>
       </c>
       <c r="O4" t="n">
-        <v>3051.5</v>
+        <v>2988.6</v>
       </c>
       <c r="P4" t="n">
         <v>3051.5</v>
       </c>
       <c r="Q4" t="n">
-        <v>0</v>
+        <v>-2.1</v>
       </c>
       <c r="R4" t="n">
         <v>73500</v>
@@ -813,31 +813,31 @@
         <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>17753.8</v>
+        <v>18124.9</v>
       </c>
       <c r="J6" t="n">
         <v>17032.2</v>
       </c>
       <c r="K6" t="n">
-        <v>4.2</v>
+        <v>6.4</v>
       </c>
       <c r="L6" t="n">
-        <v>24731.6</v>
+        <v>24845.8</v>
       </c>
       <c r="M6" t="n">
         <v>23515</v>
       </c>
       <c r="N6" t="n">
-        <v>5.2</v>
+        <v>5.7</v>
       </c>
       <c r="O6" t="n">
-        <v>30543</v>
+        <v>30674</v>
       </c>
       <c r="P6" t="n">
         <v>29523.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.5</v>
+        <v>3.9</v>
       </c>
       <c r="R6" t="n">
         <v>1170000</v>
@@ -1101,16 +1101,16 @@
         <v>0</v>
       </c>
       <c r="I10" t="n">
-        <v>2664928.5</v>
+        <v>2660324.5</v>
       </c>
       <c r="J10" t="n">
         <v>2715863.3</v>
       </c>
       <c r="K10" t="n">
-        <v>-1.9</v>
+        <v>-2</v>
       </c>
       <c r="L10" t="n">
-        <v>3924061.4</v>
+        <v>3923981.9</v>
       </c>
       <c r="M10" t="n">
         <v>3981021.3</v>
@@ -1119,7 +1119,7 @@
         <v>-1.4</v>
       </c>
       <c r="O10" t="n">
-        <v>4018350</v>
+        <v>4018476.8</v>
       </c>
       <c r="P10" t="n">
         <v>3964740.9</v>
@@ -1164,13 +1164,13 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2140</v>
+        <v>2119</v>
       </c>
       <c r="G11" t="n">
         <v>2119</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>8321.4</v>
@@ -1533,31 +1533,31 @@
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>1564.9</v>
+        <v>1625.7</v>
       </c>
       <c r="J16" t="n">
         <v>1564.9</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>3.9</v>
       </c>
       <c r="L16" t="n">
-        <v>2069.4</v>
+        <v>2130.2</v>
       </c>
       <c r="M16" t="n">
         <v>2069.4</v>
       </c>
       <c r="N16" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
       <c r="O16" t="n">
-        <v>2404.4</v>
+        <v>2410.9</v>
       </c>
       <c r="P16" t="n">
         <v>2404.4</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="R16" t="n">
         <v>33300</v>
@@ -1605,31 +1605,31 @@
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>1995.6</v>
+        <v>2285.9</v>
       </c>
       <c r="J17" t="n">
         <v>1995.6</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="L17" t="n">
-        <v>2252.9</v>
+        <v>2555.4</v>
       </c>
       <c r="M17" t="n">
         <v>2252.9</v>
       </c>
       <c r="N17" t="n">
-        <v>0</v>
+        <v>13.4</v>
       </c>
       <c r="O17" t="n">
-        <v>2899.4</v>
+        <v>3230</v>
       </c>
       <c r="P17" t="n">
         <v>2899.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>11.4</v>
       </c>
       <c r="R17" t="n">
         <v>23200</v>
@@ -1866,31 +1866,31 @@
         <v>0</v>
       </c>
       <c r="I21" t="n">
-        <v>1747.6</v>
+        <v>1776.7</v>
       </c>
       <c r="J21" t="n">
         <v>1949.2</v>
       </c>
       <c r="K21" t="n">
-        <v>-10.3</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="L21" t="n">
-        <v>2102.3</v>
+        <v>2139.9</v>
       </c>
       <c r="M21" t="n">
         <v>2228</v>
       </c>
       <c r="N21" t="n">
-        <v>-5.6</v>
+        <v>-4</v>
       </c>
       <c r="O21" t="n">
-        <v>2430.5</v>
+        <v>2437.2</v>
       </c>
       <c r="P21" t="n">
         <v>2513.3</v>
       </c>
       <c r="Q21" t="n">
-        <v>-3.3</v>
+        <v>-3</v>
       </c>
       <c r="R21" t="n">
         <v>6180</v>
@@ -2361,40 +2361,40 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>-2377</v>
+        <v>-1901</v>
       </c>
       <c r="G28" t="n">
         <v>-2377</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I28" t="n">
-        <v>11051.5</v>
+        <v>11586.2</v>
       </c>
       <c r="J28" t="n">
         <v>11051.5</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="L28" t="n">
-        <v>22324.6</v>
+        <v>22110.5</v>
       </c>
       <c r="M28" t="n">
         <v>22324.6</v>
       </c>
       <c r="N28" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O28" t="n">
-        <v>26471.7</v>
+        <v>26041.9</v>
       </c>
       <c r="P28" t="n">
         <v>26471.7</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>-1.6</v>
       </c>
       <c r="R28" t="n">
         <v>25900</v>
@@ -2514,31 +2514,31 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>997.3</v>
+        <v>994.8</v>
       </c>
       <c r="J30" t="n">
         <v>997.3</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="L30" t="n">
-        <v>1648.4</v>
+        <v>1786.1</v>
       </c>
       <c r="M30" t="n">
         <v>1648.4</v>
       </c>
       <c r="N30" t="n">
-        <v>0</v>
+        <v>8.4</v>
       </c>
       <c r="O30" t="n">
-        <v>2856.9</v>
+        <v>3034.8</v>
       </c>
       <c r="P30" t="n">
         <v>2856.9</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="R30" t="n">
         <v>137700</v>
@@ -2586,31 +2586,31 @@
         <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>1478.8</v>
+        <v>1558.2</v>
       </c>
       <c r="J31" t="n">
         <v>1440</v>
       </c>
       <c r="K31" t="n">
-        <v>2.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="L31" t="n">
-        <v>1655.8</v>
+        <v>1610.8</v>
       </c>
       <c r="M31" t="n">
         <v>1628.4</v>
       </c>
       <c r="N31" t="n">
-        <v>1.7</v>
+        <v>-1.1</v>
       </c>
       <c r="O31" t="n">
-        <v>1728.5</v>
+        <v>1734</v>
       </c>
       <c r="P31" t="n">
         <v>1748.7</v>
       </c>
       <c r="Q31" t="n">
-        <v>-1.2</v>
+        <v>-0.8</v>
       </c>
       <c r="R31" t="n">
         <v>44650</v>
@@ -3090,31 +3090,31 @@
         <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>30875.7</v>
+        <v>31198.5</v>
       </c>
       <c r="J38" t="n">
         <v>30875.7</v>
       </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
-        <v>38602.4</v>
+        <v>38184.4</v>
       </c>
       <c r="M38" t="n">
         <v>38602.4</v>
       </c>
       <c r="N38" t="n">
-        <v>0</v>
+        <v>-1.1</v>
       </c>
       <c r="O38" t="n">
-        <v>44763.8</v>
+        <v>43978.5</v>
       </c>
       <c r="P38" t="n">
         <v>44763.8</v>
       </c>
       <c r="Q38" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="R38" t="n">
         <v>312500</v>
@@ -3306,31 +3306,31 @@
         <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>3829987</v>
+        <v>3911296.2</v>
       </c>
       <c r="J41" t="n">
         <v>3832416.1</v>
       </c>
       <c r="K41" t="n">
-        <v>-0.1</v>
+        <v>2.1</v>
       </c>
       <c r="L41" t="n">
-        <v>5414963.6</v>
+        <v>5490913</v>
       </c>
       <c r="M41" t="n">
         <v>5422608.6</v>
       </c>
       <c r="N41" t="n">
-        <v>-0.1</v>
+        <v>1.3</v>
       </c>
       <c r="O41" t="n">
-        <v>5340609.5</v>
+        <v>5563316.4</v>
       </c>
       <c r="P41" t="n">
         <v>5327749.5</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.2</v>
+        <v>4.4</v>
       </c>
       <c r="R41" t="n">
         <v>262500</v>
@@ -3738,31 +3738,31 @@
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>855.3</v>
+        <v>3062.9</v>
       </c>
       <c r="J47" t="n">
         <v>509.1</v>
       </c>
       <c r="K47" t="n">
-        <v>68</v>
+        <v>501.6</v>
       </c>
       <c r="L47" t="n">
-        <v>15162.5</v>
+        <v>13976.6</v>
       </c>
       <c r="M47" t="n">
         <v>14952.3</v>
       </c>
       <c r="N47" t="n">
-        <v>1.4</v>
+        <v>-6.5</v>
       </c>
       <c r="O47" t="n">
-        <v>24694.9</v>
+        <v>24303.4</v>
       </c>
       <c r="P47" t="n">
         <v>25566.4</v>
       </c>
       <c r="Q47" t="n">
-        <v>-3.4</v>
+        <v>-4.9</v>
       </c>
       <c r="R47" t="n">
         <v>397000</v>
@@ -3810,31 +3810,31 @@
         <v>0</v>
       </c>
       <c r="I48" t="n">
-        <v>1925</v>
+        <v>1843.8</v>
       </c>
       <c r="J48" t="n">
         <v>1925</v>
       </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>-4.2</v>
       </c>
       <c r="L48" t="n">
-        <v>2254.8</v>
+        <v>2363.5</v>
       </c>
       <c r="M48" t="n">
         <v>2254.8</v>
       </c>
       <c r="N48" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O48" t="n">
-        <v>2472.6</v>
+        <v>2625.8</v>
       </c>
       <c r="P48" t="n">
         <v>2472.6</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
+        <v>6.2</v>
       </c>
       <c r="R48" t="n">
         <v>85500</v>
@@ -4296,13 +4296,13 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>552</v>
+        <v>544</v>
       </c>
       <c r="G55" t="n">
         <v>544</v>
       </c>
       <c r="H55" t="n">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="I55" t="n">
         <v>1884.9</v>
@@ -4377,31 +4377,31 @@
         <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>16675.9</v>
+        <v>19263.6</v>
       </c>
       <c r="J56" t="n">
         <v>16675.9</v>
       </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>15.5</v>
       </c>
       <c r="L56" t="n">
-        <v>31927.6</v>
+        <v>37014.1</v>
       </c>
       <c r="M56" t="n">
         <v>31927.6</v>
       </c>
       <c r="N56" t="n">
-        <v>0</v>
+        <v>15.9</v>
       </c>
       <c r="O56" t="n">
-        <v>51440.2</v>
+        <v>58301.1</v>
       </c>
       <c r="P56" t="n">
         <v>51440.2</v>
       </c>
       <c r="Q56" t="n">
-        <v>0</v>
+        <v>13.3</v>
       </c>
       <c r="R56" t="n">
         <v>1142000</v>
@@ -4593,16 +4593,16 @@
         <v>0</v>
       </c>
       <c r="I59" t="n">
-        <v>59868.3</v>
+        <v>60493.2</v>
       </c>
       <c r="J59" t="n">
         <v>57969.2</v>
       </c>
       <c r="K59" t="n">
-        <v>3.3</v>
+        <v>4.4</v>
       </c>
       <c r="L59" t="n">
-        <v>71478.7</v>
+        <v>71518.3</v>
       </c>
       <c r="M59" t="n">
         <v>69012.2</v>
@@ -4611,13 +4611,13 @@
         <v>3.6</v>
       </c>
       <c r="O59" t="n">
-        <v>83723.10000000001</v>
+        <v>83788</v>
       </c>
       <c r="P59" t="n">
         <v>80641.10000000001</v>
       </c>
       <c r="Q59" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="R59" t="n">
         <v>384500</v>
@@ -4665,31 +4665,31 @@
         <v>0</v>
       </c>
       <c r="I60" t="n">
-        <v>8261.799999999999</v>
+        <v>8068.5</v>
       </c>
       <c r="J60" t="n">
         <v>7641.5</v>
       </c>
       <c r="K60" t="n">
-        <v>8.1</v>
+        <v>5.6</v>
       </c>
       <c r="L60" t="n">
-        <v>11941.1</v>
+        <v>11562.8</v>
       </c>
       <c r="M60" t="n">
         <v>12300.9</v>
       </c>
       <c r="N60" t="n">
-        <v>-2.9</v>
+        <v>-6</v>
       </c>
       <c r="O60" t="n">
-        <v>13974.7</v>
+        <v>13668.4</v>
       </c>
       <c r="P60" t="n">
         <v>15192.5</v>
       </c>
       <c r="Q60" t="n">
-        <v>-8</v>
+        <v>-10</v>
       </c>
       <c r="R60" t="n">
         <v>25500</v>
@@ -5304,40 +5304,40 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>3797</v>
+        <v>3962</v>
       </c>
       <c r="G69" t="n">
         <v>3788</v>
       </c>
       <c r="H69" t="n">
-        <v>0.2</v>
+        <v>4.6</v>
       </c>
       <c r="I69" t="n">
-        <v>13739.3</v>
+        <v>14632.7</v>
       </c>
       <c r="J69" t="n">
         <v>13678.5</v>
       </c>
       <c r="K69" t="n">
-        <v>0.4</v>
+        <v>7</v>
       </c>
       <c r="L69" t="n">
-        <v>9780.200000000001</v>
+        <v>10103.5</v>
       </c>
       <c r="M69" t="n">
         <v>9774.299999999999</v>
       </c>
       <c r="N69" t="n">
-        <v>0.1</v>
+        <v>3.4</v>
       </c>
       <c r="O69" t="n">
-        <v>9794.200000000001</v>
+        <v>10048.4</v>
       </c>
       <c r="P69" t="n">
         <v>9789.200000000001</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.1</v>
+        <v>2.6</v>
       </c>
       <c r="R69" t="n">
         <v>20950</v>
@@ -5673,31 +5673,31 @@
         <v>0</v>
       </c>
       <c r="I74" t="n">
-        <v>37812.3</v>
+        <v>37830.2</v>
       </c>
       <c r="J74" t="n">
         <v>37353.9</v>
       </c>
       <c r="K74" t="n">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
       <c r="L74" t="n">
-        <v>42599.5</v>
+        <v>42606.3</v>
       </c>
       <c r="M74" t="n">
         <v>42626.4</v>
       </c>
       <c r="N74" t="n">
-        <v>-0.1</v>
+        <v>-0</v>
       </c>
       <c r="O74" t="n">
-        <v>46098.4</v>
+        <v>46132.5</v>
       </c>
       <c r="P74" t="n">
         <v>46322.8</v>
       </c>
       <c r="Q74" t="n">
-        <v>-0.5</v>
+        <v>-0.4</v>
       </c>
       <c r="R74" t="n">
         <v>476000</v>
@@ -5736,40 +5736,40 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>9962</v>
+        <v>9970</v>
       </c>
       <c r="G75" t="n">
         <v>9970</v>
       </c>
       <c r="H75" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="I75" t="n">
-        <v>42863.6</v>
+        <v>42800.5</v>
       </c>
       <c r="J75" t="n">
         <v>42852.8</v>
       </c>
       <c r="K75" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="L75" t="n">
-        <v>55046.6</v>
+        <v>55094.4</v>
       </c>
       <c r="M75" t="n">
         <v>54780.9</v>
       </c>
       <c r="N75" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="O75" t="n">
-        <v>61839.9</v>
+        <v>61471.3</v>
       </c>
       <c r="P75" t="n">
         <v>61398</v>
       </c>
       <c r="Q75" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="R75" t="n">
         <v>917000</v>
@@ -6528,31 +6528,31 @@
         <v>0</v>
       </c>
       <c r="I86" t="n">
-        <v>8327.9</v>
+        <v>8304.200000000001</v>
       </c>
       <c r="J86" t="n">
         <v>8379.5</v>
       </c>
       <c r="K86" t="n">
-        <v>-0.6</v>
+        <v>-0.9</v>
       </c>
       <c r="L86" t="n">
-        <v>10685.2</v>
+        <v>10724.8</v>
       </c>
       <c r="M86" t="n">
         <v>10717.4</v>
       </c>
       <c r="N86" t="n">
-        <v>-0.3</v>
+        <v>0.1</v>
       </c>
       <c r="O86" t="n">
-        <v>12003.7</v>
+        <v>11914</v>
       </c>
       <c r="P86" t="n">
         <v>12125.8</v>
       </c>
       <c r="Q86" t="n">
-        <v>-1</v>
+        <v>-1.7</v>
       </c>
       <c r="R86" t="n">
         <v>206000</v>
@@ -6600,31 +6600,31 @@
         <v>0</v>
       </c>
       <c r="I87" t="n">
-        <v>4350.9</v>
+        <v>4325.1</v>
       </c>
       <c r="J87" t="n">
         <v>4350.9</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="L87" t="n">
-        <v>5147.3</v>
+        <v>5038.9</v>
       </c>
       <c r="M87" t="n">
         <v>5147.3</v>
       </c>
       <c r="N87" t="n">
-        <v>0</v>
+        <v>-2.1</v>
       </c>
       <c r="O87" t="n">
-        <v>5926.1</v>
+        <v>5851.9</v>
       </c>
       <c r="P87" t="n">
         <v>5926.1</v>
       </c>
       <c r="Q87" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="R87" t="n">
         <v>3305</v>
@@ -6888,31 +6888,31 @@
         <v>0</v>
       </c>
       <c r="I91" t="n">
-        <v>36858.3</v>
+        <v>37009.7</v>
       </c>
       <c r="J91" t="n">
         <v>36894.8</v>
       </c>
       <c r="K91" t="n">
-        <v>-0.1</v>
+        <v>0.3</v>
       </c>
       <c r="L91" t="n">
-        <v>39741</v>
+        <v>39989.8</v>
       </c>
       <c r="M91" t="n">
         <v>39631.1</v>
       </c>
       <c r="N91" t="n">
-        <v>0.3</v>
+        <v>0.9</v>
       </c>
       <c r="O91" t="n">
-        <v>42158.7</v>
+        <v>42270.6</v>
       </c>
       <c r="P91" t="n">
         <v>42250.5</v>
       </c>
       <c r="Q91" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="R91" t="n">
         <v>20650</v>
@@ -7032,7 +7032,7 @@
         <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>37926.9</v>
+        <v>37916.4</v>
       </c>
       <c r="J93" t="n">
         <v>36427</v>
@@ -7041,22 +7041,22 @@
         <v>4.1</v>
       </c>
       <c r="L93" t="n">
-        <v>43783.1</v>
+        <v>43710</v>
       </c>
       <c r="M93" t="n">
         <v>41311</v>
       </c>
       <c r="N93" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="O93" t="n">
-        <v>47509.5</v>
+        <v>47320.3</v>
       </c>
       <c r="P93" t="n">
         <v>45429.5</v>
       </c>
       <c r="Q93" t="n">
-        <v>4.6</v>
+        <v>4.2</v>
       </c>
       <c r="R93" t="n">
         <v>351500</v>
@@ -7095,13 +7095,13 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>1559</v>
+        <v>1557</v>
       </c>
       <c r="G94" t="n">
         <v>1557</v>
       </c>
       <c r="H94" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="I94" t="n">
         <v>5949.2</v>
@@ -7860,31 +7860,31 @@
         <v>0</v>
       </c>
       <c r="I105" t="n">
-        <v>10077.8</v>
+        <v>9648.9</v>
       </c>
       <c r="J105" t="n">
         <v>10077.8</v>
       </c>
       <c r="K105" t="n">
-        <v>0</v>
+        <v>-4.3</v>
       </c>
       <c r="L105" t="n">
-        <v>14137.8</v>
+        <v>14046</v>
       </c>
       <c r="M105" t="n">
         <v>14137.8</v>
       </c>
       <c r="N105" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="O105" t="n">
-        <v>17103.4</v>
+        <v>17013.4</v>
       </c>
       <c r="P105" t="n">
         <v>17103.4</v>
       </c>
       <c r="Q105" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="R105" t="n">
         <v>9210</v>
@@ -8868,31 +8868,31 @@
         <v>0</v>
       </c>
       <c r="I119" t="n">
-        <v>22291.9</v>
+        <v>22902.4</v>
       </c>
       <c r="J119" t="n">
         <v>22166.6</v>
       </c>
       <c r="K119" t="n">
-        <v>0.6</v>
+        <v>3.3</v>
       </c>
       <c r="L119" t="n">
-        <v>20515.7</v>
+        <v>19494.5</v>
       </c>
       <c r="M119" t="n">
         <v>20465.1</v>
       </c>
       <c r="N119" t="n">
-        <v>0.2</v>
+        <v>-4.7</v>
       </c>
       <c r="O119" t="n">
-        <v>20865.4</v>
+        <v>19779.6</v>
       </c>
       <c r="P119" t="n">
         <v>20751.9</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.5</v>
+        <v>-4.7</v>
       </c>
       <c r="R119" t="n">
         <v>293500</v>
@@ -9300,31 +9300,31 @@
         <v>0</v>
       </c>
       <c r="I125" t="n">
-        <v>14079.3</v>
+        <v>14688.2</v>
       </c>
       <c r="J125" t="n">
         <v>14079.3</v>
       </c>
       <c r="K125" t="n">
-        <v>0</v>
+        <v>4.3</v>
       </c>
       <c r="L125" t="n">
-        <v>15235.2</v>
+        <v>15554.8</v>
       </c>
       <c r="M125" t="n">
         <v>15235.2</v>
       </c>
       <c r="N125" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="O125" t="n">
-        <v>15977.1</v>
+        <v>16386.5</v>
       </c>
       <c r="P125" t="n">
         <v>15977.1</v>
       </c>
       <c r="Q125" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="R125" t="n">
         <v>52200</v>
@@ -9372,31 +9372,31 @@
         <v>0</v>
       </c>
       <c r="I126" t="n">
-        <v>3939.3</v>
+        <v>3834.8</v>
       </c>
       <c r="J126" t="n">
         <v>4474.9</v>
       </c>
       <c r="K126" t="n">
-        <v>-12</v>
+        <v>-14.3</v>
       </c>
       <c r="L126" t="n">
-        <v>6195.9</v>
+        <v>6089.3</v>
       </c>
       <c r="M126" t="n">
         <v>6539.1</v>
       </c>
       <c r="N126" t="n">
-        <v>-5.2</v>
+        <v>-6.9</v>
       </c>
       <c r="O126" t="n">
-        <v>7649.1</v>
+        <v>7599.1</v>
       </c>
       <c r="P126" t="n">
         <v>8019.2</v>
       </c>
       <c r="Q126" t="n">
-        <v>-4.6</v>
+        <v>-5.2</v>
       </c>
       <c r="R126" t="n">
         <v>127300</v>
@@ -9660,31 +9660,31 @@
         <v>0</v>
       </c>
       <c r="I130" t="n">
-        <v>15563.6</v>
+        <v>15130.3</v>
       </c>
       <c r="J130" t="n">
         <v>15563.6</v>
       </c>
       <c r="K130" t="n">
-        <v>0</v>
+        <v>-2.8</v>
       </c>
       <c r="L130" t="n">
-        <v>42293.6</v>
+        <v>42094.5</v>
       </c>
       <c r="M130" t="n">
         <v>42293.6</v>
       </c>
       <c r="N130" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="O130" t="n">
-        <v>57794.5</v>
+        <v>57719.8</v>
       </c>
       <c r="P130" t="n">
         <v>57794.5</v>
       </c>
       <c r="Q130" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="R130" t="n">
         <v>258000</v>
@@ -10164,31 +10164,31 @@
         <v>0</v>
       </c>
       <c r="I137" t="n">
-        <v>11021.2</v>
+        <v>10960.4</v>
       </c>
       <c r="J137" t="n">
         <v>11584.5</v>
       </c>
       <c r="K137" t="n">
-        <v>-4.9</v>
+        <v>-5.4</v>
       </c>
       <c r="L137" t="n">
-        <v>13777.4</v>
+        <v>13689.7</v>
       </c>
       <c r="M137" t="n">
         <v>15208.9</v>
       </c>
       <c r="N137" t="n">
-        <v>-9.4</v>
+        <v>-10</v>
       </c>
       <c r="O137" t="n">
-        <v>17340.5</v>
+        <v>17272.6</v>
       </c>
       <c r="P137" t="n">
         <v>18796.5</v>
       </c>
       <c r="Q137" t="n">
-        <v>-7.7</v>
+        <v>-8.1</v>
       </c>
       <c r="R137" t="n">
         <v>133700</v>
@@ -10227,40 +10227,40 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>1370</v>
+        <v>1377</v>
       </c>
       <c r="G138" t="n">
         <v>1377</v>
       </c>
       <c r="H138" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="I138" t="n">
-        <v>6015.2</v>
+        <v>5976.9</v>
       </c>
       <c r="J138" t="n">
         <v>6025.6</v>
       </c>
       <c r="K138" t="n">
-        <v>-0.2</v>
+        <v>-0.8</v>
       </c>
       <c r="L138" t="n">
-        <v>6838.7</v>
+        <v>6767.4</v>
       </c>
       <c r="M138" t="n">
         <v>6868.2</v>
       </c>
       <c r="N138" t="n">
-        <v>-0.4</v>
+        <v>-1.5</v>
       </c>
       <c r="O138" t="n">
-        <v>7643</v>
+        <v>7569.7</v>
       </c>
       <c r="P138" t="n">
         <v>7723.9</v>
       </c>
       <c r="Q138" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="R138" t="n">
         <v>62500</v>
@@ -10326,13 +10326,13 @@
         <v>0</v>
       </c>
       <c r="O139" t="n">
-        <v>2029.8</v>
+        <v>2036.2</v>
       </c>
       <c r="P139" t="n">
         <v>2029.8</v>
       </c>
       <c r="Q139" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="R139" t="n">
         <v>165500</v>
@@ -10380,31 +10380,31 @@
         <v>0</v>
       </c>
       <c r="I140" t="n">
-        <v>1092.8</v>
+        <v>1093.4</v>
       </c>
       <c r="J140" t="n">
         <v>1092.8</v>
       </c>
       <c r="K140" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L140" t="n">
-        <v>1215.6</v>
+        <v>1214.2</v>
       </c>
       <c r="M140" t="n">
         <v>1215.6</v>
       </c>
       <c r="N140" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="O140" t="n">
-        <v>1439.6</v>
+        <v>1437.6</v>
       </c>
       <c r="P140" t="n">
         <v>1439.6</v>
       </c>
       <c r="Q140" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="R140" t="n">
         <v>26500</v>
@@ -10452,31 +10452,31 @@
         <v>0</v>
       </c>
       <c r="I141" t="n">
-        <v>42384.2</v>
+        <v>45778.1</v>
       </c>
       <c r="J141" t="n">
         <v>42384.2</v>
       </c>
       <c r="K141" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L141" t="n">
-        <v>45628.6</v>
+        <v>47920.8</v>
       </c>
       <c r="M141" t="n">
         <v>45628.6</v>
       </c>
       <c r="N141" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="O141" t="n">
-        <v>55174.1</v>
+        <v>57864.5</v>
       </c>
       <c r="P141" t="n">
         <v>55174.1</v>
       </c>
       <c r="Q141" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="R141" t="n">
         <v>162100</v>
@@ -10740,7 +10740,7 @@
         <v>0</v>
       </c>
       <c r="I145" t="n">
-        <v>18478.3</v>
+        <v>18488.3</v>
       </c>
       <c r="J145" t="n">
         <v>17841.8</v>
@@ -10749,22 +10749,22 @@
         <v>3.6</v>
       </c>
       <c r="L145" t="n">
-        <v>21856.8</v>
+        <v>21876.8</v>
       </c>
       <c r="M145" t="n">
         <v>21006.4</v>
       </c>
       <c r="N145" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="O145" t="n">
-        <v>25471</v>
+        <v>25498.6</v>
       </c>
       <c r="P145" t="n">
         <v>24598.1</v>
       </c>
       <c r="Q145" t="n">
-        <v>3.5</v>
+        <v>3.7</v>
       </c>
       <c r="R145" t="n">
         <v>186700</v>
@@ -10884,31 +10884,31 @@
         <v>0</v>
       </c>
       <c r="I147" t="n">
-        <v>2335</v>
+        <v>2311</v>
       </c>
       <c r="J147" t="n">
         <v>2202</v>
       </c>
       <c r="K147" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L147" t="n">
-        <v>2506.3</v>
+        <v>2420.3</v>
       </c>
       <c r="M147" t="n">
         <v>2377</v>
       </c>
       <c r="N147" t="n">
-        <v>5.4</v>
+        <v>1.8</v>
       </c>
       <c r="O147" t="n">
-        <v>2967.4</v>
+        <v>2825.8</v>
       </c>
       <c r="P147" t="n">
         <v>3578.8</v>
       </c>
       <c r="Q147" t="n">
-        <v>-17.1</v>
+        <v>-21</v>
       </c>
       <c r="R147" t="n">
         <v>113800</v>
@@ -11172,31 +11172,31 @@
         <v>0</v>
       </c>
       <c r="I151" t="n">
-        <v>1517.2</v>
+        <v>1516.5</v>
       </c>
       <c r="J151" t="n">
         <v>1526.7</v>
       </c>
       <c r="K151" t="n">
-        <v>-0.6</v>
+        <v>-0.7</v>
       </c>
       <c r="L151" t="n">
-        <v>2058.2</v>
+        <v>2056.3</v>
       </c>
       <c r="M151" t="n">
         <v>2054.3</v>
       </c>
       <c r="N151" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="O151" t="n">
-        <v>2546.3</v>
+        <v>2542.2</v>
       </c>
       <c r="P151" t="n">
         <v>2545</v>
       </c>
       <c r="Q151" t="n">
-        <v>0.1</v>
+        <v>-0.1</v>
       </c>
       <c r="R151" t="n">
         <v>49450</v>
@@ -11244,31 +11244,31 @@
         <v>0</v>
       </c>
       <c r="I152" t="n">
-        <v>5922.1</v>
+        <v>6217.2</v>
       </c>
       <c r="J152" t="n">
         <v>5891.4</v>
       </c>
       <c r="K152" t="n">
-        <v>0.5</v>
+        <v>5.5</v>
       </c>
       <c r="L152" t="n">
-        <v>6584.1</v>
+        <v>6596.8</v>
       </c>
       <c r="M152" t="n">
         <v>6323.3</v>
       </c>
       <c r="N152" t="n">
-        <v>4.1</v>
+        <v>4.3</v>
       </c>
       <c r="O152" t="n">
-        <v>7258</v>
+        <v>7427.8</v>
       </c>
       <c r="P152" t="n">
         <v>7160.8</v>
       </c>
       <c r="Q152" t="n">
-        <v>1.4</v>
+        <v>3.7</v>
       </c>
       <c r="R152" t="n">
         <v>7290</v>
@@ -11685,13 +11685,13 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="G159" t="n">
         <v>561</v>
       </c>
       <c r="H159" t="n">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="I159" t="n">
         <v>2389.6</v>
@@ -12234,31 +12234,31 @@
         <v>0</v>
       </c>
       <c r="I167" t="n">
-        <v>4650.4</v>
+        <v>4810.5</v>
       </c>
       <c r="J167" t="n">
         <v>4647</v>
       </c>
       <c r="K167" t="n">
-        <v>0.1</v>
+        <v>3.5</v>
       </c>
       <c r="L167" t="n">
-        <v>5283.9</v>
+        <v>5542.3</v>
       </c>
       <c r="M167" t="n">
         <v>5283.7</v>
       </c>
       <c r="N167" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="O167" t="n">
-        <v>5871</v>
+        <v>6265.4</v>
       </c>
       <c r="P167" t="n">
         <v>5883.9</v>
       </c>
       <c r="Q167" t="n">
-        <v>-0.2</v>
+        <v>6.5</v>
       </c>
       <c r="R167" t="n">
         <v>130000</v>
@@ -12639,31 +12639,31 @@
         <v>0</v>
       </c>
       <c r="I173" t="n">
-        <v>54601.8</v>
+        <v>80836</v>
       </c>
       <c r="J173" t="n">
         <v>54601.8</v>
       </c>
       <c r="K173" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="L173" t="n">
-        <v>34598.5</v>
+        <v>41223.6</v>
       </c>
       <c r="M173" t="n">
         <v>34598.5</v>
       </c>
       <c r="N173" t="n">
-        <v>0</v>
+        <v>19.1</v>
       </c>
       <c r="O173" t="n">
-        <v>40044.5</v>
+        <v>44949.8</v>
       </c>
       <c r="P173" t="n">
         <v>40044.5</v>
       </c>
       <c r="Q173" t="n">
-        <v>0</v>
+        <v>12.2</v>
       </c>
       <c r="R173" t="n">
         <v>110500</v>
@@ -12972,31 +12972,31 @@
         <v>0</v>
       </c>
       <c r="I178" t="n">
-        <v>3594.6</v>
+        <v>3573.2</v>
       </c>
       <c r="J178" t="n">
         <v>3594.6</v>
       </c>
       <c r="K178" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="L178" t="n">
-        <v>3524.8</v>
+        <v>3455.3</v>
       </c>
       <c r="M178" t="n">
         <v>3524.8</v>
       </c>
       <c r="N178" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="O178" t="n">
-        <v>3913</v>
+        <v>3744.2</v>
       </c>
       <c r="P178" t="n">
         <v>3913</v>
       </c>
       <c r="Q178" t="n">
-        <v>0</v>
+        <v>-4.3</v>
       </c>
       <c r="R178" t="n">
         <v>71200</v>
@@ -13737,31 +13737,31 @@
         <v>0</v>
       </c>
       <c r="I189" t="n">
-        <v>10318.9</v>
+        <v>10183.5</v>
       </c>
       <c r="J189" t="n">
         <v>10990.9</v>
       </c>
       <c r="K189" t="n">
-        <v>-6.1</v>
+        <v>-7.3</v>
       </c>
       <c r="L189" t="n">
-        <v>11341.3</v>
+        <v>11267.5</v>
       </c>
       <c r="M189" t="n">
         <v>11876.1</v>
       </c>
       <c r="N189" t="n">
-        <v>-4.5</v>
+        <v>-5.1</v>
       </c>
       <c r="O189" t="n">
-        <v>11964.7</v>
+        <v>11910</v>
       </c>
       <c r="P189" t="n">
         <v>12628.4</v>
       </c>
       <c r="Q189" t="n">
-        <v>-5.3</v>
+        <v>-5.7</v>
       </c>
       <c r="R189" t="n">
         <v>15170</v>
@@ -13809,31 +13809,31 @@
         <v>0</v>
       </c>
       <c r="I190" t="n">
-        <v>6264</v>
+        <v>6291.4</v>
       </c>
       <c r="J190" t="n">
         <v>6565.1</v>
       </c>
       <c r="K190" t="n">
-        <v>-4.6</v>
+        <v>-4.2</v>
       </c>
       <c r="L190" t="n">
-        <v>6842.7</v>
+        <v>6860.1</v>
       </c>
       <c r="M190" t="n">
         <v>7114.6</v>
       </c>
       <c r="N190" t="n">
-        <v>-3.8</v>
+        <v>-3.6</v>
       </c>
       <c r="O190" t="n">
-        <v>7201.9</v>
+        <v>7226.9</v>
       </c>
       <c r="P190" t="n">
         <v>7534.6</v>
       </c>
       <c r="Q190" t="n">
-        <v>-4.4</v>
+        <v>-4.1</v>
       </c>
       <c r="R190" t="n">
         <v>16950</v>
@@ -14637,31 +14637,31 @@
         <v>0</v>
       </c>
       <c r="I202" t="n">
-        <v>787.1</v>
+        <v>759</v>
       </c>
       <c r="J202" t="n">
         <v>787.1</v>
       </c>
       <c r="K202" t="n">
-        <v>0</v>
+        <v>-3.6</v>
       </c>
       <c r="L202" t="n">
-        <v>900.7</v>
+        <v>874</v>
       </c>
       <c r="M202" t="n">
         <v>900.7</v>
       </c>
       <c r="N202" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="O202" t="n">
-        <v>1019</v>
+        <v>995</v>
       </c>
       <c r="P202" t="n">
         <v>1019</v>
       </c>
       <c r="Q202" t="n">
-        <v>0</v>
+        <v>-2.4</v>
       </c>
       <c r="R202" t="n">
         <v>66900</v>
@@ -14700,40 +14700,40 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="G203" t="n">
         <v>80</v>
       </c>
       <c r="H203" t="n">
-        <v>0</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I203" t="n">
-        <v>384.3</v>
+        <v>389.9</v>
       </c>
       <c r="J203" t="n">
         <v>384.3</v>
       </c>
       <c r="K203" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="L203" t="n">
-        <v>595.9</v>
+        <v>598.4</v>
       </c>
       <c r="M203" t="n">
         <v>595.9</v>
       </c>
       <c r="N203" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O203" t="n">
-        <v>882.5</v>
+        <v>887.5</v>
       </c>
       <c r="P203" t="n">
         <v>882.5</v>
       </c>
       <c r="Q203" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="R203" t="n">
         <v>58200</v>
@@ -14925,31 +14925,31 @@
         <v>0</v>
       </c>
       <c r="I206" t="n">
-        <v>1305.5</v>
+        <v>1303.4</v>
       </c>
       <c r="J206" t="n">
         <v>1307.8</v>
       </c>
       <c r="K206" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="L206" t="n">
-        <v>1480.4</v>
+        <v>1477.5</v>
       </c>
       <c r="M206" t="n">
         <v>1471.7</v>
       </c>
       <c r="N206" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="O206" t="n">
-        <v>1670.2</v>
+        <v>1681</v>
       </c>
       <c r="P206" t="n">
         <v>1623.6</v>
       </c>
       <c r="Q206" t="n">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
       <c r="R206" t="n">
         <v>36100</v>
@@ -15069,31 +15069,31 @@
         <v>0</v>
       </c>
       <c r="I208" t="n">
-        <v>4022.1</v>
+        <v>4107.2</v>
       </c>
       <c r="J208" t="n">
         <v>4022.1</v>
       </c>
       <c r="K208" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="L208" t="n">
-        <v>4688.9</v>
+        <v>4696.1</v>
       </c>
       <c r="M208" t="n">
         <v>4688.9</v>
       </c>
       <c r="N208" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O208" t="n">
-        <v>5231.2</v>
+        <v>5287.3</v>
       </c>
       <c r="P208" t="n">
         <v>5231.2</v>
       </c>
       <c r="Q208" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="R208" t="n">
         <v>44700</v>
@@ -15141,31 +15141,31 @@
         <v>0</v>
       </c>
       <c r="I209" t="n">
-        <v>24193.1</v>
+        <v>24162.2</v>
       </c>
       <c r="J209" t="n">
         <v>24196.8</v>
       </c>
       <c r="K209" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="L209" t="n">
-        <v>28135.5</v>
+        <v>28197.6</v>
       </c>
       <c r="M209" t="n">
         <v>28253.4</v>
       </c>
       <c r="N209" t="n">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
       <c r="O209" t="n">
-        <v>31109.9</v>
+        <v>30980.9</v>
       </c>
       <c r="P209" t="n">
         <v>30972.1</v>
       </c>
       <c r="Q209" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="R209" t="n">
         <v>1485000</v>
@@ -15204,40 +15204,40 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="G210" t="n">
         <v>510</v>
       </c>
       <c r="H210" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="I210" t="n">
-        <v>2117.3</v>
+        <v>2107.1</v>
       </c>
       <c r="J210" t="n">
         <v>2117.3</v>
       </c>
       <c r="K210" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="L210" t="n">
-        <v>2826.9</v>
+        <v>2814</v>
       </c>
       <c r="M210" t="n">
         <v>2826.9</v>
       </c>
       <c r="N210" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="O210" t="n">
-        <v>3490.6</v>
+        <v>3480.9</v>
       </c>
       <c r="P210" t="n">
         <v>3490.6</v>
       </c>
       <c r="Q210" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="R210" t="n">
         <v>41150</v>
@@ -15501,22 +15501,22 @@
         <v>0</v>
       </c>
       <c r="I214" t="n">
-        <v>755.4</v>
+        <v>753.9</v>
       </c>
       <c r="J214" t="n">
         <v>789.7</v>
       </c>
       <c r="K214" t="n">
-        <v>-4.3</v>
+        <v>-4.5</v>
       </c>
       <c r="L214" t="n">
-        <v>1028.3</v>
+        <v>1027.6</v>
       </c>
       <c r="M214" t="n">
         <v>1065</v>
       </c>
       <c r="N214" t="n">
-        <v>-3.4</v>
+        <v>-3.5</v>
       </c>
       <c r="O214" t="n">
         <v>1343.7</v>
@@ -15780,40 +15780,40 @@
         </is>
       </c>
       <c r="F218" t="n">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="G218" t="n">
         <v>239</v>
       </c>
       <c r="H218" t="n">
-        <v>-0.8</v>
+        <v>0</v>
       </c>
       <c r="I218" t="n">
-        <v>1130.3</v>
+        <v>1085.9</v>
       </c>
       <c r="J218" t="n">
         <v>1136.3</v>
       </c>
       <c r="K218" t="n">
-        <v>-0.5</v>
+        <v>-4.4</v>
       </c>
       <c r="L218" t="n">
-        <v>2136.7</v>
+        <v>1947.2</v>
       </c>
       <c r="M218" t="n">
         <v>2111.3</v>
       </c>
       <c r="N218" t="n">
-        <v>1.2</v>
+        <v>-7.8</v>
       </c>
       <c r="O218" t="n">
-        <v>3558.3</v>
+        <v>3429.6</v>
       </c>
       <c r="P218" t="n">
         <v>3469</v>
       </c>
       <c r="Q218" t="n">
-        <v>2.6</v>
+        <v>-1.1</v>
       </c>
       <c r="R218" t="n">
         <v>103500</v>
@@ -15852,40 +15852,40 @@
         </is>
       </c>
       <c r="F219" t="n">
-        <v>884</v>
+        <v>861</v>
       </c>
       <c r="G219" t="n">
         <v>889</v>
       </c>
       <c r="H219" t="n">
-        <v>-0.6</v>
+        <v>-3.1</v>
       </c>
       <c r="I219" t="n">
-        <v>3517.8</v>
+        <v>3508.1</v>
       </c>
       <c r="J219" t="n">
         <v>3601.2</v>
       </c>
       <c r="K219" t="n">
-        <v>-2.3</v>
+        <v>-2.6</v>
       </c>
       <c r="L219" t="n">
-        <v>4126.4</v>
+        <v>4192</v>
       </c>
       <c r="M219" t="n">
         <v>4239.1</v>
       </c>
       <c r="N219" t="n">
-        <v>-2.7</v>
+        <v>-1.1</v>
       </c>
       <c r="O219" t="n">
-        <v>4303.6</v>
+        <v>4414</v>
       </c>
       <c r="P219" t="n">
         <v>4385.8</v>
       </c>
       <c r="Q219" t="n">
-        <v>-1.9</v>
+        <v>0.6</v>
       </c>
       <c r="R219" t="n">
         <v>38300</v>
@@ -16149,31 +16149,31 @@
         <v>0</v>
       </c>
       <c r="I223" t="n">
-        <v>14488.1</v>
+        <v>14592.8</v>
       </c>
       <c r="J223" t="n">
         <v>14855.6</v>
       </c>
       <c r="K223" t="n">
-        <v>-2.5</v>
+        <v>-1.8</v>
       </c>
       <c r="L223" t="n">
-        <v>15738.2</v>
+        <v>15949.3</v>
       </c>
       <c r="M223" t="n">
         <v>15923.4</v>
       </c>
       <c r="N223" t="n">
-        <v>-1.2</v>
+        <v>0.2</v>
       </c>
       <c r="O223" t="n">
-        <v>16836.6</v>
+        <v>16935.4</v>
       </c>
       <c r="P223" t="n">
         <v>17431.9</v>
       </c>
       <c r="Q223" t="n">
-        <v>-3.4</v>
+        <v>-2.8</v>
       </c>
       <c r="R223" t="n">
         <v>243000</v>
@@ -16284,13 +16284,13 @@
         </is>
       </c>
       <c r="F225" t="n">
-        <v>22197</v>
+        <v>20915</v>
       </c>
       <c r="G225" t="n">
         <v>20915</v>
       </c>
       <c r="H225" t="n">
-        <v>6.1</v>
+        <v>0</v>
       </c>
       <c r="I225" t="n">
         <v>91376.2</v>
@@ -16527,13 +16527,13 @@
         <v>0</v>
       </c>
       <c r="O228" t="n">
-        <v>7564.6</v>
+        <v>7562.3</v>
       </c>
       <c r="P228" t="n">
         <v>7564.6</v>
       </c>
       <c r="Q228" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="R228" t="n">
         <v>131800</v>
@@ -16644,40 +16644,40 @@
         </is>
       </c>
       <c r="F230" t="n">
-        <v>-707</v>
+        <v>-655</v>
       </c>
       <c r="G230" t="n">
         <v>-707</v>
       </c>
       <c r="H230" t="n">
-        <v>0</v>
+        <v>7.4</v>
       </c>
       <c r="I230" t="n">
-        <v>-344.5</v>
+        <v>-297</v>
       </c>
       <c r="J230" t="n">
         <v>-344.5</v>
       </c>
       <c r="K230" t="n">
-        <v>0</v>
+        <v>13.8</v>
       </c>
       <c r="L230" t="n">
-        <v>835.2</v>
+        <v>799</v>
       </c>
       <c r="M230" t="n">
         <v>835.2</v>
       </c>
       <c r="N230" t="n">
-        <v>0</v>
+        <v>-4.3</v>
       </c>
       <c r="O230" t="n">
-        <v>1157.4</v>
+        <v>1236</v>
       </c>
       <c r="P230" t="n">
         <v>1157.4</v>
       </c>
       <c r="Q230" t="n">
-        <v>0</v>
+        <v>6.8</v>
       </c>
       <c r="R230" t="n">
         <v>5200</v>
@@ -17211,13 +17211,13 @@
         </is>
       </c>
       <c r="F238" t="n">
-        <v>2907</v>
+        <v>2812</v>
       </c>
       <c r="G238" t="n">
         <v>2812</v>
       </c>
       <c r="H238" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="I238" t="n">
         <v>10928</v>
@@ -17292,31 +17292,31 @@
         <v>0</v>
       </c>
       <c r="I239" t="n">
-        <v>2160.7</v>
+        <v>2341.8</v>
       </c>
       <c r="J239" t="n">
         <v>2200.4</v>
       </c>
       <c r="K239" t="n">
-        <v>-1.8</v>
+        <v>6.4</v>
       </c>
       <c r="L239" t="n">
-        <v>2614.3</v>
+        <v>2688.2</v>
       </c>
       <c r="M239" t="n">
         <v>2696.6</v>
       </c>
       <c r="N239" t="n">
-        <v>-3.1</v>
+        <v>-0.3</v>
       </c>
       <c r="O239" t="n">
-        <v>2810.7</v>
+        <v>2873</v>
       </c>
       <c r="P239" t="n">
         <v>2854.4</v>
       </c>
       <c r="Q239" t="n">
-        <v>-1.5</v>
+        <v>0.7</v>
       </c>
       <c r="R239" t="n">
         <v>160800</v>
@@ -17643,31 +17643,31 @@
         <v>0</v>
       </c>
       <c r="I244" t="n">
-        <v>2808.3</v>
+        <v>2805.4</v>
       </c>
       <c r="J244" t="n">
         <v>2738</v>
       </c>
       <c r="K244" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="L244" t="n">
-        <v>3555.2</v>
+        <v>3500.2</v>
       </c>
       <c r="M244" t="n">
         <v>3653.6</v>
       </c>
       <c r="N244" t="n">
-        <v>-2.7</v>
+        <v>-4.2</v>
       </c>
       <c r="O244" t="n">
-        <v>4469.2</v>
+        <v>4478.6</v>
       </c>
       <c r="P244" t="n">
         <v>4585.7</v>
       </c>
       <c r="Q244" t="n">
-        <v>-2.5</v>
+        <v>-2.3</v>
       </c>
       <c r="R244" t="n">
         <v>364500</v>
@@ -18066,31 +18066,31 @@
         <v>0</v>
       </c>
       <c r="I250" t="n">
-        <v>40062</v>
+        <v>40238.8</v>
       </c>
       <c r="J250" t="n">
         <v>38876</v>
       </c>
       <c r="K250" t="n">
-        <v>3.1</v>
+        <v>3.5</v>
       </c>
       <c r="L250" t="n">
-        <v>46975.6</v>
+        <v>46858.8</v>
       </c>
       <c r="M250" t="n">
         <v>45739.8</v>
       </c>
       <c r="N250" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="O250" t="n">
-        <v>54196.9</v>
+        <v>54155.1</v>
       </c>
       <c r="P250" t="n">
         <v>52641.7</v>
       </c>
       <c r="Q250" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="R250" t="n">
         <v>481000</v>
@@ -18138,31 +18138,31 @@
         <v>0</v>
       </c>
       <c r="I251" t="n">
-        <v>2934.4</v>
+        <v>2864.8</v>
       </c>
       <c r="J251" t="n">
         <v>2750.3</v>
       </c>
       <c r="K251" t="n">
-        <v>6.7</v>
+        <v>4.2</v>
       </c>
       <c r="L251" t="n">
-        <v>4920.5</v>
+        <v>4903.3</v>
       </c>
       <c r="M251" t="n">
         <v>4937.1</v>
       </c>
       <c r="N251" t="n">
-        <v>-0.3</v>
+        <v>-0.7</v>
       </c>
       <c r="O251" t="n">
-        <v>5606.9</v>
+        <v>5518.4</v>
       </c>
       <c r="P251" t="n">
         <v>5399.4</v>
       </c>
       <c r="Q251" t="n">
-        <v>3.8</v>
+        <v>2.2</v>
       </c>
       <c r="R251" t="n">
         <v>168800</v>
@@ -18210,31 +18210,31 @@
         <v>0</v>
       </c>
       <c r="I252" t="n">
-        <v>2550.6</v>
+        <v>2584.8</v>
       </c>
       <c r="J252" t="n">
         <v>2550.6</v>
       </c>
       <c r="K252" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="L252" t="n">
-        <v>3642.6</v>
+        <v>3713.6</v>
       </c>
       <c r="M252" t="n">
         <v>3642.6</v>
       </c>
       <c r="N252" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="O252" t="n">
-        <v>4513.6</v>
+        <v>4621.8</v>
       </c>
       <c r="P252" t="n">
         <v>4513.6</v>
       </c>
       <c r="Q252" t="n">
-        <v>0</v>
+        <v>2.4</v>
       </c>
       <c r="R252" t="n">
         <v>96800</v>
@@ -18354,31 +18354,31 @@
         <v>0</v>
       </c>
       <c r="I254" t="n">
-        <v>-2448.4</v>
+        <v>-2511.6</v>
       </c>
       <c r="J254" t="n">
         <v>-2448.4</v>
       </c>
       <c r="K254" t="n">
-        <v>0</v>
+        <v>-2.6</v>
       </c>
       <c r="L254" t="n">
-        <v>-938</v>
+        <v>-981.6</v>
       </c>
       <c r="M254" t="n">
         <v>-938</v>
       </c>
       <c r="N254" t="n">
-        <v>0</v>
+        <v>-4.6</v>
       </c>
       <c r="O254" t="n">
-        <v>203.6</v>
+        <v>178.5</v>
       </c>
       <c r="P254" t="n">
         <v>203.6</v>
       </c>
       <c r="Q254" t="n">
-        <v>0</v>
+        <v>-12.3</v>
       </c>
       <c r="R254" t="n">
         <v>13260</v>
@@ -18426,31 +18426,31 @@
         <v>0</v>
       </c>
       <c r="I255" t="n">
-        <v>11337.5</v>
+        <v>9459.6</v>
       </c>
       <c r="J255" t="n">
         <v>11337.5</v>
       </c>
       <c r="K255" t="n">
-        <v>0</v>
+        <v>-16.6</v>
       </c>
       <c r="L255" t="n">
-        <v>39777.8</v>
+        <v>39260.5</v>
       </c>
       <c r="M255" t="n">
         <v>39777.8</v>
       </c>
       <c r="N255" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="O255" t="n">
-        <v>61996.8</v>
+        <v>61218.4</v>
       </c>
       <c r="P255" t="n">
         <v>61996.8</v>
       </c>
       <c r="Q255" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="R255" t="n">
         <v>328000</v>
@@ -18498,31 +18498,31 @@
         <v>0</v>
       </c>
       <c r="I256" t="n">
-        <v>5272.2</v>
+        <v>5744.6</v>
       </c>
       <c r="J256" t="n">
         <v>5272.2</v>
       </c>
       <c r="K256" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L256" t="n">
-        <v>5624.7</v>
+        <v>5756.8</v>
       </c>
       <c r="M256" t="n">
         <v>5624.7</v>
       </c>
       <c r="N256" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
       <c r="O256" t="n">
-        <v>6119.8</v>
+        <v>6461.5</v>
       </c>
       <c r="P256" t="n">
         <v>6119.8</v>
       </c>
       <c r="Q256" t="n">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="R256" t="n">
         <v>58500</v>
@@ -18984,40 +18984,40 @@
         </is>
       </c>
       <c r="F264" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="G264" t="n">
         <v>49</v>
       </c>
       <c r="H264" t="n">
-        <v>0</v>
+        <v>12.2</v>
       </c>
       <c r="I264" t="n">
-        <v>291.8</v>
+        <v>297.4</v>
       </c>
       <c r="J264" t="n">
         <v>291.8</v>
       </c>
       <c r="K264" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="L264" t="n">
-        <v>833</v>
+        <v>836</v>
       </c>
       <c r="M264" t="n">
         <v>833</v>
       </c>
       <c r="N264" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O264" t="n">
-        <v>764</v>
+        <v>798</v>
       </c>
       <c r="P264" t="n">
         <v>764</v>
       </c>
       <c r="Q264" t="n">
-        <v>0</v>
+        <v>4.5</v>
       </c>
       <c r="R264" t="n">
         <v>103500</v>
@@ -19065,31 +19065,31 @@
         <v>0</v>
       </c>
       <c r="I265" t="n">
-        <v>3666.2</v>
+        <v>3646.8</v>
       </c>
       <c r="J265" t="n">
         <v>3670.6</v>
       </c>
       <c r="K265" t="n">
-        <v>-0.1</v>
+        <v>-0.6</v>
       </c>
       <c r="L265" t="n">
-        <v>3728.8</v>
+        <v>3739.2</v>
       </c>
       <c r="M265" t="n">
         <v>3828.1</v>
       </c>
       <c r="N265" t="n">
-        <v>-2.6</v>
+        <v>-2.3</v>
       </c>
       <c r="O265" t="n">
-        <v>4268.8</v>
+        <v>4253.5</v>
       </c>
       <c r="P265" t="n">
         <v>4209</v>
       </c>
       <c r="Q265" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="R265" t="n">
         <v>50100</v>
@@ -19227,13 +19227,13 @@
         <v>-1.6</v>
       </c>
       <c r="O267" t="n">
-        <v>6638.8</v>
+        <v>6713.7</v>
       </c>
       <c r="P267" t="n">
         <v>6676.8</v>
       </c>
       <c r="Q267" t="n">
-        <v>-0.6</v>
+        <v>0.6</v>
       </c>
       <c r="R267" t="n">
         <v>184000</v>
@@ -19353,31 +19353,31 @@
         <v>0</v>
       </c>
       <c r="I269" t="n">
-        <v>1167</v>
+        <v>1234.7</v>
       </c>
       <c r="J269" t="n">
         <v>1015.3</v>
       </c>
       <c r="K269" t="n">
-        <v>14.9</v>
+        <v>21.6</v>
       </c>
       <c r="L269" t="n">
-        <v>1477.5</v>
+        <v>1485</v>
       </c>
       <c r="M269" t="n">
         <v>1305.3</v>
       </c>
       <c r="N269" t="n">
-        <v>13.2</v>
+        <v>13.8</v>
       </c>
       <c r="O269" t="n">
-        <v>1637.5</v>
+        <v>1601.7</v>
       </c>
       <c r="P269" t="n">
         <v>1408.7</v>
       </c>
       <c r="Q269" t="n">
-        <v>16.2</v>
+        <v>13.7</v>
       </c>
       <c r="R269" t="n">
         <v>9010</v>
@@ -19641,31 +19641,31 @@
         <v>0</v>
       </c>
       <c r="I273" t="n">
-        <v>1854</v>
+        <v>1924</v>
       </c>
       <c r="J273" t="n">
         <v>1854</v>
       </c>
       <c r="K273" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="L273" t="n">
-        <v>2817</v>
+        <v>2897</v>
       </c>
       <c r="M273" t="n">
         <v>2817</v>
       </c>
       <c r="N273" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="O273" t="n">
-        <v>3774</v>
+        <v>3880.7</v>
       </c>
       <c r="P273" t="n">
         <v>3774</v>
       </c>
       <c r="Q273" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="R273" t="n">
         <v>42000</v>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-08-14
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -696,13 +696,13 @@
         <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>83100</v>
+        <v>83700</v>
       </c>
       <c r="S4" t="n">
         <v>80600</v>
       </c>
       <c r="T4" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="5">
@@ -768,13 +768,13 @@
         <v>-2</v>
       </c>
       <c r="R5" t="n">
-        <v>75700</v>
+        <v>77200</v>
       </c>
       <c r="S5" t="n">
         <v>79000</v>
       </c>
       <c r="T5" t="n">
-        <v>-4.2</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="6">
@@ -840,13 +840,13 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>1227000</v>
+        <v>1276000</v>
       </c>
       <c r="S6" t="n">
         <v>1191000</v>
       </c>
       <c r="T6" t="n">
-        <v>3</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="7">
@@ -912,13 +912,13 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>51500</v>
+        <v>51900</v>
       </c>
       <c r="S7" t="n">
         <v>50900</v>
       </c>
       <c r="T7" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -957,13 +957,13 @@
         <v>5340</v>
       </c>
       <c r="R8" t="n">
-        <v>25750</v>
+        <v>26250</v>
       </c>
       <c r="S8" t="n">
         <v>25850</v>
       </c>
       <c r="T8" t="n">
-        <v>-0.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="9">
@@ -1029,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>140100</v>
+        <v>141700</v>
       </c>
       <c r="S9" t="n">
         <v>134900</v>
       </c>
       <c r="T9" t="n">
-        <v>3.9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1101,13 +1101,13 @@
         <v>2.4</v>
       </c>
       <c r="R10" t="n">
-        <v>92000</v>
+        <v>93000</v>
       </c>
       <c r="S10" t="n">
         <v>89000</v>
       </c>
       <c r="T10" t="n">
-        <v>3.4</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="11">
@@ -1245,13 +1245,13 @@
         <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>113300</v>
+        <v>115800</v>
       </c>
       <c r="S12" t="n">
         <v>109900</v>
       </c>
       <c r="T12" t="n">
-        <v>3.1</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="13">
@@ -1317,13 +1317,13 @@
         <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>618000</v>
+        <v>615000</v>
       </c>
       <c r="S13" t="n">
         <v>645000</v>
       </c>
       <c r="T13" t="n">
-        <v>-4.2</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="14">
@@ -1461,13 +1461,13 @@
         <v>0.5</v>
       </c>
       <c r="R15" t="n">
-        <v>100300</v>
+        <v>102800</v>
       </c>
       <c r="S15" t="n">
         <v>84100</v>
       </c>
       <c r="T15" t="n">
-        <v>19.3</v>
+        <v>22.2</v>
       </c>
     </row>
     <row r="16">
@@ -1533,13 +1533,13 @@
         <v>0</v>
       </c>
       <c r="R16" t="n">
-        <v>134300</v>
+        <v>138100</v>
       </c>
       <c r="S16" t="n">
         <v>145700</v>
       </c>
       <c r="T16" t="n">
-        <v>-7.8</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="17">
@@ -1605,13 +1605,13 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>44200</v>
+        <v>45000</v>
       </c>
       <c r="S17" t="n">
         <v>41600</v>
       </c>
       <c r="T17" t="n">
-        <v>6.2</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="18">
@@ -1677,13 +1677,13 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>29050</v>
+        <v>29950</v>
       </c>
       <c r="S18" t="n">
         <v>27100</v>
       </c>
       <c r="T18" t="n">
-        <v>7.2</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="19">
@@ -1740,13 +1740,13 @@
         <v>0</v>
       </c>
       <c r="R19" t="n">
-        <v>44900</v>
+        <v>45350</v>
       </c>
       <c r="S19" t="n">
         <v>39300</v>
       </c>
       <c r="T19" t="n">
-        <v>14.2</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="20">
@@ -1812,13 +1812,13 @@
         <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>18130</v>
+        <v>18370</v>
       </c>
       <c r="S20" t="n">
         <v>18550</v>
       </c>
       <c r="T20" t="n">
-        <v>-2.3</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="21">
@@ -1938,13 +1938,13 @@
         <v>-1.5</v>
       </c>
       <c r="R22" t="n">
-        <v>6580</v>
+        <v>6730</v>
       </c>
       <c r="S22" t="n">
         <v>6550</v>
       </c>
       <c r="T22" t="n">
-        <v>0.5</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="23">
@@ -2010,13 +2010,13 @@
         <v>0</v>
       </c>
       <c r="R23" t="n">
-        <v>451000</v>
+        <v>465500</v>
       </c>
       <c r="S23" t="n">
         <v>442000</v>
       </c>
       <c r="T23" t="n">
-        <v>2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="24">
@@ -2082,13 +2082,13 @@
         <v>0</v>
       </c>
       <c r="R24" t="n">
-        <v>13310</v>
+        <v>13400</v>
       </c>
       <c r="S24" t="n">
         <v>9770</v>
       </c>
       <c r="T24" t="n">
-        <v>36.2</v>
+        <v>37.2</v>
       </c>
     </row>
     <row r="25">
@@ -2154,13 +2154,13 @@
         <v>0</v>
       </c>
       <c r="R25" t="n">
-        <v>109100</v>
+        <v>108000</v>
       </c>
       <c r="S25" t="n">
         <v>114500</v>
       </c>
       <c r="T25" t="n">
-        <v>-4.7</v>
+        <v>-5.7</v>
       </c>
     </row>
     <row r="26">
@@ -2226,13 +2226,13 @@
         <v>-4.3</v>
       </c>
       <c r="R26" t="n">
-        <v>10340</v>
+        <v>10240</v>
       </c>
       <c r="S26" t="n">
         <v>8950</v>
       </c>
       <c r="T26" t="n">
-        <v>15.5</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="27">
@@ -2289,13 +2289,13 @@
         <v>0</v>
       </c>
       <c r="R27" t="n">
-        <v>7940</v>
+        <v>7960</v>
       </c>
       <c r="S27" t="n">
         <v>8160</v>
       </c>
       <c r="T27" t="n">
-        <v>-2.7</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="28">
@@ -2361,13 +2361,13 @@
         <v>0</v>
       </c>
       <c r="R28" t="n">
-        <v>1273000</v>
+        <v>1270000</v>
       </c>
       <c r="S28" t="n">
         <v>1306000</v>
       </c>
       <c r="T28" t="n">
-        <v>-2.5</v>
+        <v>-2.8</v>
       </c>
     </row>
     <row r="29">
@@ -2433,13 +2433,13 @@
         <v>0</v>
       </c>
       <c r="R29" t="n">
-        <v>26250</v>
+        <v>26300</v>
       </c>
       <c r="S29" t="n">
         <v>27150</v>
       </c>
       <c r="T29" t="n">
-        <v>-3.3</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="30">
@@ -2505,13 +2505,13 @@
         <v>-8</v>
       </c>
       <c r="R30" t="n">
-        <v>116900</v>
+        <v>120000</v>
       </c>
       <c r="S30" t="n">
         <v>108100</v>
       </c>
       <c r="T30" t="n">
-        <v>8.1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="31">
@@ -2577,13 +2577,13 @@
         <v>-0.6</v>
       </c>
       <c r="R31" t="n">
-        <v>163200</v>
+        <v>170500</v>
       </c>
       <c r="S31" t="n">
         <v>155800</v>
       </c>
       <c r="T31" t="n">
-        <v>4.7</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="32">
@@ -2649,13 +2649,13 @@
         <v>0</v>
       </c>
       <c r="R32" t="n">
-        <v>46600</v>
+        <v>47100</v>
       </c>
       <c r="S32" t="n">
         <v>48550</v>
       </c>
       <c r="T32" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="33">
@@ -2721,13 +2721,13 @@
         <v>0.9</v>
       </c>
       <c r="R33" t="n">
-        <v>29150</v>
+        <v>29900</v>
       </c>
       <c r="S33" t="n">
         <v>28300</v>
       </c>
       <c r="T33" t="n">
-        <v>3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="34">
@@ -2793,13 +2793,13 @@
         <v>1.8</v>
       </c>
       <c r="R34" t="n">
-        <v>419500</v>
+        <v>427000</v>
       </c>
       <c r="S34" t="n">
         <v>420000</v>
       </c>
       <c r="T34" t="n">
-        <v>-0.1</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="35">
@@ -2865,13 +2865,13 @@
         <v>0</v>
       </c>
       <c r="R35" t="n">
-        <v>431000</v>
+        <v>437500</v>
       </c>
       <c r="S35" t="n">
         <v>405000</v>
       </c>
       <c r="T35" t="n">
-        <v>6.4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="R36" t="n">
-        <v>24050</v>
+        <v>24300</v>
       </c>
       <c r="S36" t="n">
         <v>23700</v>
       </c>
       <c r="T36" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="37">
@@ -3009,13 +3009,13 @@
         <v>0</v>
       </c>
       <c r="R37" t="n">
-        <v>101400</v>
+        <v>101700</v>
       </c>
       <c r="S37" t="n">
         <v>102600</v>
       </c>
       <c r="T37" t="n">
-        <v>-1.2</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="38">
@@ -3081,13 +3081,13 @@
         <v>-0.1</v>
       </c>
       <c r="R38" t="n">
-        <v>443500</v>
+        <v>453000</v>
       </c>
       <c r="S38" t="n">
         <v>395500</v>
       </c>
       <c r="T38" t="n">
-        <v>12.1</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="39">
@@ -3153,13 +3153,13 @@
         <v>0</v>
       </c>
       <c r="R39" t="n">
-        <v>328500</v>
+        <v>334000</v>
       </c>
       <c r="S39" t="n">
         <v>331000</v>
       </c>
       <c r="T39" t="n">
-        <v>-0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="40">
@@ -3225,13 +3225,13 @@
         <v>0</v>
       </c>
       <c r="R40" t="n">
-        <v>172100</v>
+        <v>176800</v>
       </c>
       <c r="S40" t="n">
         <v>165900</v>
       </c>
       <c r="T40" t="n">
-        <v>3.7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="41">
@@ -3297,13 +3297,13 @@
         <v>0</v>
       </c>
       <c r="R41" t="n">
-        <v>60000</v>
+        <v>61600</v>
       </c>
       <c r="S41" t="n">
         <v>55200</v>
       </c>
       <c r="T41" t="n">
-        <v>8.699999999999999</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="42">
@@ -3369,13 +3369,13 @@
         <v>-2.2</v>
       </c>
       <c r="R42" t="n">
-        <v>267500</v>
+        <v>274500</v>
       </c>
       <c r="S42" t="n">
         <v>231000</v>
       </c>
       <c r="T42" t="n">
-        <v>15.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="43">
@@ -3441,13 +3441,13 @@
         <v>0</v>
       </c>
       <c r="R43" t="n">
-        <v>28400</v>
+        <v>28750</v>
       </c>
       <c r="S43" t="n">
         <v>27800</v>
       </c>
       <c r="T43" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="44">
@@ -3513,13 +3513,13 @@
         <v>0.4</v>
       </c>
       <c r="R44" t="n">
-        <v>37650</v>
+        <v>37550</v>
       </c>
       <c r="S44" t="n">
         <v>37750</v>
       </c>
       <c r="T44" t="n">
-        <v>-0.3</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="45">
@@ -3585,13 +3585,13 @@
         <v>0</v>
       </c>
       <c r="R45" t="n">
-        <v>307500</v>
+        <v>323500</v>
       </c>
       <c r="S45" t="n">
         <v>317000</v>
       </c>
       <c r="T45" t="n">
-        <v>-3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="46">
@@ -3657,13 +3657,13 @@
         <v>0</v>
       </c>
       <c r="R46" t="n">
-        <v>128600</v>
+        <v>129200</v>
       </c>
       <c r="S46" t="n">
         <v>129900</v>
       </c>
       <c r="T46" t="n">
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="47">
@@ -3729,13 +3729,13 @@
         <v>0.3</v>
       </c>
       <c r="R47" t="n">
-        <v>34300</v>
+        <v>35350</v>
       </c>
       <c r="S47" t="n">
         <v>31650</v>
       </c>
       <c r="T47" t="n">
-        <v>8.4</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="48">
@@ -3801,13 +3801,13 @@
         <v>-0</v>
       </c>
       <c r="R48" t="n">
-        <v>495000</v>
+        <v>516000</v>
       </c>
       <c r="S48" t="n">
         <v>459000</v>
       </c>
       <c r="T48" t="n">
-        <v>7.8</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="49">
@@ -3873,13 +3873,13 @@
         <v>0</v>
       </c>
       <c r="R49" t="n">
-        <v>90400</v>
+        <v>91400</v>
       </c>
       <c r="S49" t="n">
         <v>93700</v>
       </c>
       <c r="T49" t="n">
-        <v>-3.5</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="50">
@@ -3945,13 +3945,13 @@
         <v>-0.5</v>
       </c>
       <c r="R50" t="n">
-        <v>37000</v>
+        <v>37650</v>
       </c>
       <c r="S50" t="n">
         <v>33900</v>
       </c>
       <c r="T50" t="n">
-        <v>9.1</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="51">
@@ -4017,13 +4017,13 @@
         <v>6.9</v>
       </c>
       <c r="R51" t="n">
-        <v>27750</v>
+        <v>27700</v>
       </c>
       <c r="S51" t="n">
         <v>28350</v>
       </c>
       <c r="T51" t="n">
-        <v>-2.1</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="52">
@@ -4089,13 +4089,13 @@
         <v>8.800000000000001</v>
       </c>
       <c r="R52" t="n">
-        <v>50300</v>
+        <v>58900</v>
       </c>
       <c r="S52" t="n">
         <v>47600</v>
       </c>
       <c r="T52" t="n">
-        <v>5.7</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="53">
@@ -4161,13 +4161,13 @@
         <v>0</v>
       </c>
       <c r="R53" t="n">
-        <v>90100</v>
+        <v>95600</v>
       </c>
       <c r="S53" t="n">
         <v>82300</v>
       </c>
       <c r="T53" t="n">
-        <v>9.5</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="54">
@@ -4233,13 +4233,13 @@
         <v>0</v>
       </c>
       <c r="R54" t="n">
-        <v>64200</v>
+        <v>63100</v>
       </c>
       <c r="S54" t="n">
         <v>55700</v>
       </c>
       <c r="T54" t="n">
-        <v>15.3</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="55">
@@ -4296,13 +4296,13 @@
         <v>0</v>
       </c>
       <c r="R55" t="n">
-        <v>14640</v>
+        <v>15090</v>
       </c>
       <c r="S55" t="n">
         <v>14840</v>
       </c>
       <c r="T55" t="n">
-        <v>-1.3</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="56">
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="R56" t="n">
-        <v>44800</v>
+        <v>45400</v>
       </c>
       <c r="S56" t="n">
         <v>42700</v>
       </c>
       <c r="T56" t="n">
-        <v>4.9</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="57">
@@ -4440,13 +4440,13 @@
         <v>0</v>
       </c>
       <c r="R57" t="n">
-        <v>1531000</v>
+        <v>1558000</v>
       </c>
       <c r="S57" t="n">
         <v>1278000</v>
       </c>
       <c r="T57" t="n">
-        <v>19.8</v>
+        <v>21.9</v>
       </c>
     </row>
     <row r="58">
@@ -4512,13 +4512,13 @@
         <v>-8.199999999999999</v>
       </c>
       <c r="R58" t="n">
-        <v>39700</v>
+        <v>40500</v>
       </c>
       <c r="S58" t="n">
         <v>40850</v>
       </c>
       <c r="T58" t="n">
-        <v>-2.8</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="59">
@@ -4584,13 +4584,13 @@
         <v>0</v>
       </c>
       <c r="R59" t="n">
-        <v>58200</v>
+        <v>59700</v>
       </c>
       <c r="S59" t="n">
         <v>54100</v>
       </c>
       <c r="T59" t="n">
-        <v>7.6</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="60">
@@ -4656,13 +4656,13 @@
         <v>-1.8</v>
       </c>
       <c r="R60" t="n">
-        <v>384500</v>
+        <v>386000</v>
       </c>
       <c r="S60" t="n">
         <v>398500</v>
       </c>
       <c r="T60" t="n">
-        <v>-3.5</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="61">
@@ -4728,13 +4728,13 @@
         <v>1.3</v>
       </c>
       <c r="R61" t="n">
-        <v>34950</v>
+        <v>35400</v>
       </c>
       <c r="S61" t="n">
         <v>33900</v>
       </c>
       <c r="T61" t="n">
-        <v>3.1</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="62">
@@ -4800,13 +4800,13 @@
         <v>0</v>
       </c>
       <c r="R62" t="n">
-        <v>267000</v>
+        <v>279000</v>
       </c>
       <c r="S62" t="n">
         <v>272500</v>
       </c>
       <c r="T62" t="n">
-        <v>-2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="63">
@@ -4872,13 +4872,13 @@
         <v>0</v>
       </c>
       <c r="R63" t="n">
-        <v>203500</v>
+        <v>206500</v>
       </c>
       <c r="S63" t="n">
         <v>201000</v>
       </c>
       <c r="T63" t="n">
-        <v>1.2</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="64">
@@ -4944,13 +4944,13 @@
         <v>-10</v>
       </c>
       <c r="R64" t="n">
-        <v>1184000</v>
+        <v>1196000</v>
       </c>
       <c r="S64" t="n">
         <v>1106000</v>
       </c>
       <c r="T64" t="n">
-        <v>7.1</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="65">
@@ -5016,13 +5016,13 @@
         <v>0</v>
       </c>
       <c r="R65" t="n">
-        <v>22350</v>
+        <v>22300</v>
       </c>
       <c r="S65" t="n">
         <v>22050</v>
       </c>
       <c r="T65" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="66">
@@ -5088,13 +5088,13 @@
         <v>-2.5</v>
       </c>
       <c r="R66" t="n">
-        <v>16090</v>
+        <v>16730</v>
       </c>
       <c r="S66" t="n">
         <v>19230</v>
       </c>
       <c r="T66" t="n">
-        <v>-16.3</v>
+        <v>-13</v>
       </c>
     </row>
     <row r="67">
@@ -5160,13 +5160,13 @@
         <v>0.7</v>
       </c>
       <c r="R67" t="n">
-        <v>143400</v>
+        <v>147600</v>
       </c>
       <c r="S67" t="n">
         <v>137600</v>
       </c>
       <c r="T67" t="n">
-        <v>4.2</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="68">
@@ -5232,13 +5232,13 @@
         <v>0</v>
       </c>
       <c r="R68" t="n">
-        <v>625000</v>
+        <v>654000</v>
       </c>
       <c r="S68" t="n">
         <v>552000</v>
       </c>
       <c r="T68" t="n">
-        <v>13.2</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="69">
@@ -5304,13 +5304,13 @@
         <v>-18.9</v>
       </c>
       <c r="R69" t="n">
-        <v>56900</v>
+        <v>57200</v>
       </c>
       <c r="S69" t="n">
         <v>61000</v>
       </c>
       <c r="T69" t="n">
-        <v>-6.7</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="70">
@@ -5376,13 +5376,13 @@
         <v>0</v>
       </c>
       <c r="R70" t="n">
-        <v>21050</v>
+        <v>21250</v>
       </c>
       <c r="S70" t="n">
         <v>21800</v>
       </c>
       <c r="T70" t="n">
-        <v>-3.4</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="71">
@@ -5448,13 +5448,13 @@
         <v>0</v>
       </c>
       <c r="R71" t="n">
-        <v>66800</v>
+        <v>67800</v>
       </c>
       <c r="S71" t="n">
         <v>62500</v>
       </c>
       <c r="T71" t="n">
-        <v>6.9</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="72">
@@ -5520,13 +5520,13 @@
         <v>-1</v>
       </c>
       <c r="R72" t="n">
-        <v>130000</v>
+        <v>130600</v>
       </c>
       <c r="S72" t="n">
         <v>129600</v>
       </c>
       <c r="T72" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="73">
@@ -5592,13 +5592,13 @@
         <v>0</v>
       </c>
       <c r="R73" t="n">
-        <v>87200</v>
+        <v>89800</v>
       </c>
       <c r="S73" t="n">
         <v>81200</v>
       </c>
       <c r="T73" t="n">
-        <v>7.4</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="74">
@@ -5664,13 +5664,13 @@
         <v>0</v>
       </c>
       <c r="R74" t="n">
-        <v>16520</v>
+        <v>16890</v>
       </c>
       <c r="S74" t="n">
         <v>15140</v>
       </c>
       <c r="T74" t="n">
-        <v>9.1</v>
+        <v>11.6</v>
       </c>
     </row>
     <row r="75">
@@ -5736,13 +5736,13 @@
         <v>0</v>
       </c>
       <c r="R75" t="n">
-        <v>532000</v>
+        <v>547000</v>
       </c>
       <c r="S75" t="n">
         <v>496500</v>
       </c>
       <c r="T75" t="n">
-        <v>7.2</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="76">
@@ -5808,13 +5808,13 @@
         <v>0</v>
       </c>
       <c r="R76" t="n">
-        <v>1148000</v>
+        <v>1160000</v>
       </c>
       <c r="S76" t="n">
         <v>1097000</v>
       </c>
       <c r="T76" t="n">
-        <v>4.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="77">
@@ -5880,13 +5880,13 @@
         <v>0.2</v>
       </c>
       <c r="R77" t="n">
-        <v>77200</v>
+        <v>77700</v>
       </c>
       <c r="S77" t="n">
         <v>76600</v>
       </c>
       <c r="T77" t="n">
-        <v>0.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="78">
@@ -5943,13 +5943,13 @@
         <v>0</v>
       </c>
       <c r="R78" t="n">
-        <v>20900</v>
+        <v>21600</v>
       </c>
       <c r="S78" t="n">
         <v>19940</v>
       </c>
       <c r="T78" t="n">
-        <v>4.8</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="79">
@@ -6015,13 +6015,13 @@
         <v>5.1</v>
       </c>
       <c r="R79" t="n">
-        <v>26450</v>
+        <v>26050</v>
       </c>
       <c r="S79" t="n">
         <v>26650</v>
       </c>
       <c r="T79" t="n">
-        <v>-0.8</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="80">
@@ -6087,13 +6087,13 @@
         <v>0.8</v>
       </c>
       <c r="R80" t="n">
-        <v>212000</v>
+        <v>218500</v>
       </c>
       <c r="S80" t="n">
         <v>222500</v>
       </c>
       <c r="T80" t="n">
-        <v>-4.7</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="81">
@@ -6159,13 +6159,13 @@
         <v>0</v>
       </c>
       <c r="R81" t="n">
-        <v>2505</v>
+        <v>2575</v>
       </c>
       <c r="S81" t="n">
         <v>2480</v>
       </c>
       <c r="T81" t="n">
-        <v>1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="82">
@@ -6231,13 +6231,13 @@
         <v>-8.699999999999999</v>
       </c>
       <c r="R82" t="n">
-        <v>32850</v>
+        <v>33250</v>
       </c>
       <c r="S82" t="n">
         <v>35600</v>
       </c>
       <c r="T82" t="n">
-        <v>-7.7</v>
+        <v>-6.6</v>
       </c>
     </row>
     <row r="83">
@@ -6303,13 +6303,13 @@
         <v>-0.5</v>
       </c>
       <c r="R83" t="n">
-        <v>92100</v>
+        <v>93000</v>
       </c>
       <c r="S83" t="n">
         <v>91000</v>
       </c>
       <c r="T83" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="84">
@@ -6375,13 +6375,13 @@
         <v>0.5</v>
       </c>
       <c r="R84" t="n">
-        <v>100000</v>
+        <v>100500</v>
       </c>
       <c r="S84" t="n">
         <v>88200</v>
       </c>
       <c r="T84" t="n">
-        <v>13.4</v>
+        <v>13.9</v>
       </c>
     </row>
     <row r="85">
@@ -6519,13 +6519,13 @@
         <v>0</v>
       </c>
       <c r="R86" t="n">
-        <v>24500</v>
+        <v>25150</v>
       </c>
       <c r="S86" t="n">
         <v>23100</v>
       </c>
       <c r="T86" t="n">
-        <v>6.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="87">
@@ -6591,13 +6591,13 @@
         <v>-0.5</v>
       </c>
       <c r="R87" t="n">
-        <v>234500</v>
+        <v>243500</v>
       </c>
       <c r="S87" t="n">
         <v>221500</v>
       </c>
       <c r="T87" t="n">
-        <v>5.9</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="88">
@@ -6663,13 +6663,13 @@
         <v>-0.5</v>
       </c>
       <c r="R88" t="n">
-        <v>3785</v>
+        <v>3820</v>
       </c>
       <c r="S88" t="n">
         <v>3625</v>
       </c>
       <c r="T88" t="n">
-        <v>4.4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="89">
@@ -6735,13 +6735,13 @@
         <v>3.9</v>
       </c>
       <c r="R89" t="n">
-        <v>98700</v>
+        <v>98200</v>
       </c>
       <c r="S89" t="n">
         <v>95700</v>
       </c>
       <c r="T89" t="n">
-        <v>3.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="90">
@@ -6807,13 +6807,13 @@
         <v>0</v>
       </c>
       <c r="R90" t="n">
-        <v>23250</v>
+        <v>23200</v>
       </c>
       <c r="S90" t="n">
         <v>23150</v>
       </c>
       <c r="T90" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="91">
@@ -6879,13 +6879,13 @@
         <v>-1</v>
       </c>
       <c r="R91" t="n">
-        <v>102000</v>
+        <v>102900</v>
       </c>
       <c r="S91" t="n">
         <v>99700</v>
       </c>
       <c r="T91" t="n">
-        <v>2.3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="92">
@@ -6951,13 +6951,13 @@
         <v>0</v>
       </c>
       <c r="R92" t="n">
-        <v>20250</v>
+        <v>20400</v>
       </c>
       <c r="S92" t="n">
         <v>20750</v>
       </c>
       <c r="T92" t="n">
-        <v>-2.4</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="93">
@@ -7023,13 +7023,13 @@
         <v>0</v>
       </c>
       <c r="R93" t="n">
-        <v>48900</v>
+        <v>49800</v>
       </c>
       <c r="S93" t="n">
         <v>48100</v>
       </c>
       <c r="T93" t="n">
-        <v>1.7</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="94">
@@ -7095,13 +7095,13 @@
         <v>0</v>
       </c>
       <c r="R94" t="n">
-        <v>362500</v>
+        <v>369000</v>
       </c>
       <c r="S94" t="n">
         <v>336500</v>
       </c>
       <c r="T94" t="n">
-        <v>7.7</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="95">
@@ -7167,13 +7167,13 @@
         <v>0.4</v>
       </c>
       <c r="R95" t="n">
-        <v>5690</v>
+        <v>5790</v>
       </c>
       <c r="S95" t="n">
         <v>6040</v>
       </c>
       <c r="T95" t="n">
-        <v>-5.8</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="96">
@@ -7239,13 +7239,13 @@
         <v>0</v>
       </c>
       <c r="R96" t="n">
-        <v>47950</v>
+        <v>48550</v>
       </c>
       <c r="S96" t="n">
         <v>47850</v>
       </c>
       <c r="T96" t="n">
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="97">
@@ -7311,7 +7311,7 @@
         <v>0</v>
       </c>
       <c r="R97" t="n">
-        <v>18970</v>
+        <v>18980</v>
       </c>
       <c r="S97" t="n">
         <v>19170</v>
@@ -7383,13 +7383,13 @@
         <v>-1.4</v>
       </c>
       <c r="R98" t="n">
-        <v>53800</v>
+        <v>53400</v>
       </c>
       <c r="S98" t="n">
         <v>53300</v>
       </c>
       <c r="T98" t="n">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="99">
@@ -7455,13 +7455,13 @@
         <v>0</v>
       </c>
       <c r="R99" t="n">
-        <v>100800</v>
+        <v>111200</v>
       </c>
       <c r="S99" t="n">
         <v>94000</v>
       </c>
       <c r="T99" t="n">
-        <v>7.2</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="100">
@@ -7500,13 +7500,13 @@
         <v>0</v>
       </c>
       <c r="R100" t="n">
-        <v>13780</v>
+        <v>13760</v>
       </c>
       <c r="S100" t="n">
         <v>13030</v>
       </c>
       <c r="T100" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="101">
@@ -7572,13 +7572,13 @@
         <v>2</v>
       </c>
       <c r="R101" t="n">
-        <v>14890</v>
+        <v>15060</v>
       </c>
       <c r="S101" t="n">
         <v>14960</v>
       </c>
       <c r="T101" t="n">
-        <v>-0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="102">
@@ -7644,13 +7644,13 @@
         <v>0</v>
       </c>
       <c r="R102" t="n">
-        <v>298000</v>
+        <v>301000</v>
       </c>
       <c r="S102" t="n">
         <v>275500</v>
       </c>
       <c r="T102" t="n">
-        <v>8.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="103">
@@ -7707,13 +7707,13 @@
         <v>0</v>
       </c>
       <c r="R103" t="n">
-        <v>17170</v>
+        <v>17350</v>
       </c>
       <c r="S103" t="n">
         <v>17000</v>
       </c>
       <c r="T103" t="n">
-        <v>1</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="104">
@@ -7779,13 +7779,13 @@
         <v>1.7</v>
       </c>
       <c r="R104" t="n">
-        <v>176700</v>
+        <v>176000</v>
       </c>
       <c r="S104" t="n">
         <v>188800</v>
       </c>
       <c r="T104" t="n">
-        <v>-6.4</v>
+        <v>-6.8</v>
       </c>
     </row>
     <row r="105">
@@ -7851,13 +7851,13 @@
         <v>0</v>
       </c>
       <c r="R105" t="n">
-        <v>81400</v>
+        <v>82600</v>
       </c>
       <c r="S105" t="n">
         <v>77100</v>
       </c>
       <c r="T105" t="n">
-        <v>5.6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="106">
@@ -7923,13 +7923,13 @@
         <v>0</v>
       </c>
       <c r="R106" t="n">
-        <v>9970</v>
+        <v>10270</v>
       </c>
       <c r="S106" t="n">
         <v>9770</v>
       </c>
       <c r="T106" t="n">
-        <v>2</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="107">
@@ -7995,13 +7995,13 @@
         <v>0.3</v>
       </c>
       <c r="R107" t="n">
-        <v>9780</v>
+        <v>9890</v>
       </c>
       <c r="S107" t="n">
         <v>10100</v>
       </c>
       <c r="T107" t="n">
-        <v>-3.2</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="108">
@@ -8067,13 +8067,13 @@
         <v>7.1</v>
       </c>
       <c r="R108" t="n">
-        <v>566000</v>
+        <v>585000</v>
       </c>
       <c r="S108" t="n">
         <v>508000</v>
       </c>
       <c r="T108" t="n">
-        <v>11.4</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="109">
@@ -8139,13 +8139,13 @@
         <v>-0</v>
       </c>
       <c r="R109" t="n">
-        <v>14720</v>
+        <v>14590</v>
       </c>
       <c r="S109" t="n">
         <v>14690</v>
       </c>
       <c r="T109" t="n">
-        <v>0.2</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="110">
@@ -8211,13 +8211,13 @@
         <v>-5.1</v>
       </c>
       <c r="R110" t="n">
-        <v>225500</v>
+        <v>228000</v>
       </c>
       <c r="S110" t="n">
         <v>210000</v>
       </c>
       <c r="T110" t="n">
-        <v>7.4</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="111">
@@ -8283,13 +8283,13 @@
         <v>7</v>
       </c>
       <c r="R111" t="n">
-        <v>39700</v>
+        <v>40000</v>
       </c>
       <c r="S111" t="n">
         <v>39900</v>
       </c>
       <c r="T111" t="n">
-        <v>-0.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="112">
@@ -8355,13 +8355,13 @@
         <v>2.3</v>
       </c>
       <c r="R112" t="n">
-        <v>34750</v>
+        <v>34400</v>
       </c>
       <c r="S112" t="n">
         <v>35450</v>
       </c>
       <c r="T112" t="n">
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="113">
@@ -8499,13 +8499,13 @@
         <v>0</v>
       </c>
       <c r="R114" t="n">
-        <v>8590</v>
+        <v>8760</v>
       </c>
       <c r="S114" t="n">
         <v>7510</v>
       </c>
       <c r="T114" t="n">
-        <v>14.4</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="115">
@@ -8571,13 +8571,13 @@
         <v>10</v>
       </c>
       <c r="R115" t="n">
-        <v>36450</v>
+        <v>36600</v>
       </c>
       <c r="S115" t="n">
         <v>35750</v>
       </c>
       <c r="T115" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="116">
@@ -8643,13 +8643,13 @@
         <v>6.3</v>
       </c>
       <c r="R116" t="n">
-        <v>242500</v>
+        <v>247500</v>
       </c>
       <c r="S116" t="n">
         <v>248500</v>
       </c>
       <c r="T116" t="n">
-        <v>-2.4</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="117">
@@ -8715,13 +8715,13 @@
         <v>0</v>
       </c>
       <c r="R117" t="n">
-        <v>173500</v>
+        <v>177800</v>
       </c>
       <c r="S117" t="n">
         <v>127800</v>
       </c>
       <c r="T117" t="n">
-        <v>35.8</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="118">
@@ -8787,13 +8787,13 @@
         <v>0</v>
       </c>
       <c r="R118" t="n">
-        <v>390000</v>
+        <v>404000</v>
       </c>
       <c r="S118" t="n">
         <v>324500</v>
       </c>
       <c r="T118" t="n">
-        <v>20.2</v>
+        <v>24.5</v>
       </c>
     </row>
     <row r="119">
@@ -8859,13 +8859,13 @@
         <v>-1.3</v>
       </c>
       <c r="R119" t="n">
-        <v>32450</v>
+        <v>32700</v>
       </c>
       <c r="S119" t="n">
         <v>31500</v>
       </c>
       <c r="T119" t="n">
-        <v>3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="120">
@@ -8931,13 +8931,13 @@
         <v>0</v>
       </c>
       <c r="R120" t="n">
-        <v>23450</v>
+        <v>23700</v>
       </c>
       <c r="S120" t="n">
         <v>21150</v>
       </c>
       <c r="T120" t="n">
-        <v>10.9</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="121">
@@ -9003,13 +9003,13 @@
         <v>-0.3</v>
       </c>
       <c r="R121" t="n">
-        <v>296000</v>
+        <v>300500</v>
       </c>
       <c r="S121" t="n">
         <v>277500</v>
       </c>
       <c r="T121" t="n">
-        <v>6.7</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="122">
@@ -9057,13 +9057,13 @@
         <v>-2.2</v>
       </c>
       <c r="R122" t="n">
-        <v>12230</v>
+        <v>12290</v>
       </c>
       <c r="S122" t="n">
         <v>12570</v>
       </c>
       <c r="T122" t="n">
-        <v>-2.7</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="123">
@@ -9129,13 +9129,13 @@
         <v>1.4</v>
       </c>
       <c r="R123" t="n">
-        <v>72800</v>
+        <v>73400</v>
       </c>
       <c r="S123" t="n">
         <v>75600</v>
       </c>
       <c r="T123" t="n">
-        <v>-3.7</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="124">
@@ -9201,13 +9201,13 @@
         <v>0</v>
       </c>
       <c r="R124" t="n">
-        <v>94000</v>
+        <v>95800</v>
       </c>
       <c r="S124" t="n">
         <v>89400</v>
       </c>
       <c r="T124" t="n">
-        <v>5.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="125">
@@ -9273,13 +9273,13 @@
         <v>0</v>
       </c>
       <c r="R125" t="n">
-        <v>224500</v>
+        <v>229000</v>
       </c>
       <c r="S125" t="n">
         <v>192300</v>
       </c>
       <c r="T125" t="n">
-        <v>16.7</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="126">
@@ -9345,13 +9345,13 @@
         <v>-0.3</v>
       </c>
       <c r="R126" t="n">
-        <v>17570</v>
+        <v>18010</v>
       </c>
       <c r="S126" t="n">
         <v>16410</v>
       </c>
       <c r="T126" t="n">
-        <v>7.1</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="127">
@@ -9417,13 +9417,13 @@
         <v>0</v>
       </c>
       <c r="R127" t="n">
-        <v>53100</v>
+        <v>53300</v>
       </c>
       <c r="S127" t="n">
         <v>58000</v>
       </c>
       <c r="T127" t="n">
-        <v>-8.4</v>
+        <v>-8.1</v>
       </c>
     </row>
     <row r="128">
@@ -9489,13 +9489,13 @@
         <v>-1.2</v>
       </c>
       <c r="R128" t="n">
-        <v>146800</v>
+        <v>146400</v>
       </c>
       <c r="S128" t="n">
         <v>154200</v>
       </c>
       <c r="T128" t="n">
-        <v>-4.8</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="129">
@@ -9561,13 +9561,13 @@
         <v>-0.4</v>
       </c>
       <c r="R129" t="n">
-        <v>24600</v>
+        <v>24850</v>
       </c>
       <c r="S129" t="n">
         <v>23450</v>
       </c>
       <c r="T129" t="n">
-        <v>4.9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="130">
@@ -9633,13 +9633,13 @@
         <v>-2.7</v>
       </c>
       <c r="R130" t="n">
-        <v>46050</v>
+        <v>46350</v>
       </c>
       <c r="S130" t="n">
         <v>47250</v>
       </c>
       <c r="T130" t="n">
-        <v>-2.5</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="131">
@@ -9777,13 +9777,13 @@
         <v>0</v>
       </c>
       <c r="R132" t="n">
-        <v>274500</v>
+        <v>280500</v>
       </c>
       <c r="S132" t="n">
         <v>276000</v>
       </c>
       <c r="T132" t="n">
-        <v>-0.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="133">
@@ -9849,13 +9849,13 @@
         <v>-10.3</v>
       </c>
       <c r="R133" t="n">
-        <v>100300</v>
+        <v>101000</v>
       </c>
       <c r="S133" t="n">
         <v>101900</v>
       </c>
       <c r="T133" t="n">
-        <v>-1.6</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="134">
@@ -9921,13 +9921,13 @@
         <v>0</v>
       </c>
       <c r="R134" t="n">
-        <v>107300</v>
+        <v>107400</v>
       </c>
       <c r="S134" t="n">
         <v>110000</v>
       </c>
       <c r="T134" t="n">
-        <v>-2.5</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="135">
@@ -9993,13 +9993,13 @@
         <v>2</v>
       </c>
       <c r="R135" t="n">
-        <v>71000</v>
+        <v>70800</v>
       </c>
       <c r="S135" t="n">
         <v>65700</v>
       </c>
       <c r="T135" t="n">
-        <v>8.1</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="136">
@@ -10065,13 +10065,13 @@
         <v>0</v>
       </c>
       <c r="R136" t="n">
-        <v>120000</v>
+        <v>118600</v>
       </c>
       <c r="S136" t="n">
         <v>101700</v>
       </c>
       <c r="T136" t="n">
-        <v>18</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="137">
@@ -10137,13 +10137,13 @@
         <v>0</v>
       </c>
       <c r="R137" t="n">
-        <v>41200</v>
+        <v>41100</v>
       </c>
       <c r="S137" t="n">
         <v>39100</v>
       </c>
       <c r="T137" t="n">
-        <v>5.4</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="138">
@@ -10209,13 +10209,13 @@
         <v>1</v>
       </c>
       <c r="R138" t="n">
-        <v>175200</v>
+        <v>182500</v>
       </c>
       <c r="S138" t="n">
         <v>157300</v>
       </c>
       <c r="T138" t="n">
-        <v>11.4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="139">
@@ -10281,13 +10281,13 @@
         <v>-1.9</v>
       </c>
       <c r="R139" t="n">
-        <v>144800</v>
+        <v>146900</v>
       </c>
       <c r="S139" t="n">
         <v>146900</v>
       </c>
       <c r="T139" t="n">
-        <v>-1.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140">
@@ -10353,13 +10353,13 @@
         <v>-0.6</v>
       </c>
       <c r="R140" t="n">
-        <v>77600</v>
+        <v>79900</v>
       </c>
       <c r="S140" t="n">
         <v>72600</v>
       </c>
       <c r="T140" t="n">
-        <v>6.9</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="141">
@@ -10425,13 +10425,13 @@
         <v>1.8</v>
       </c>
       <c r="R141" t="n">
-        <v>232000</v>
+        <v>244000</v>
       </c>
       <c r="S141" t="n">
         <v>167300</v>
       </c>
       <c r="T141" t="n">
-        <v>38.7</v>
+        <v>45.8</v>
       </c>
     </row>
     <row r="142">
@@ -10488,13 +10488,13 @@
         <v>0</v>
       </c>
       <c r="R142" t="n">
-        <v>28700</v>
+        <v>28450</v>
       </c>
       <c r="S142" t="n">
         <v>27350</v>
       </c>
       <c r="T142" t="n">
-        <v>4.9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="143">
@@ -10560,13 +10560,13 @@
         <v>0.9</v>
       </c>
       <c r="R143" t="n">
-        <v>207000</v>
+        <v>215000</v>
       </c>
       <c r="S143" t="n">
         <v>185000</v>
       </c>
       <c r="T143" t="n">
-        <v>11.9</v>
+        <v>16.2</v>
       </c>
     </row>
     <row r="144">
@@ -10632,13 +10632,13 @@
         <v>-2</v>
       </c>
       <c r="R144" t="n">
-        <v>103700</v>
+        <v>109700</v>
       </c>
       <c r="S144" t="n">
         <v>90200</v>
       </c>
       <c r="T144" t="n">
-        <v>15</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="145">
@@ -10704,13 +10704,13 @@
         <v>0</v>
       </c>
       <c r="R145" t="n">
-        <v>42050</v>
+        <v>41500</v>
       </c>
       <c r="S145" t="n">
         <v>43300</v>
       </c>
       <c r="T145" t="n">
-        <v>-2.9</v>
+        <v>-4.2</v>
       </c>
     </row>
     <row r="146">
@@ -10776,13 +10776,13 @@
         <v>0</v>
       </c>
       <c r="R146" t="n">
-        <v>35750</v>
+        <v>36600</v>
       </c>
       <c r="S146" t="n">
         <v>30000</v>
       </c>
       <c r="T146" t="n">
-        <v>19.2</v>
+        <v>22</v>
       </c>
     </row>
     <row r="147">
@@ -10848,13 +10848,13 @@
         <v>0.8</v>
       </c>
       <c r="R147" t="n">
-        <v>200500</v>
+        <v>201000</v>
       </c>
       <c r="S147" t="n">
         <v>199300</v>
       </c>
       <c r="T147" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="148">
@@ -10920,13 +10920,13 @@
         <v>0</v>
       </c>
       <c r="R148" t="n">
-        <v>16260</v>
+        <v>16350</v>
       </c>
       <c r="S148" t="n">
         <v>16450</v>
       </c>
       <c r="T148" t="n">
-        <v>-1.2</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="149">
@@ -11064,13 +11064,13 @@
         <v>-0.5</v>
       </c>
       <c r="R150" t="n">
-        <v>101800</v>
+        <v>102200</v>
       </c>
       <c r="S150" t="n">
         <v>101800</v>
       </c>
       <c r="T150" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="151">
@@ -11136,13 +11136,13 @@
         <v>2.1</v>
       </c>
       <c r="R151" t="n">
-        <v>200500</v>
+        <v>204000</v>
       </c>
       <c r="S151" t="n">
         <v>188000</v>
       </c>
       <c r="T151" t="n">
-        <v>6.6</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="152">
@@ -11208,13 +11208,13 @@
         <v>-7.4</v>
       </c>
       <c r="R152" t="n">
-        <v>74800</v>
+        <v>76400</v>
       </c>
       <c r="S152" t="n">
         <v>64500</v>
       </c>
       <c r="T152" t="n">
-        <v>16</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="153">
@@ -11280,13 +11280,13 @@
         <v>2.4</v>
       </c>
       <c r="R153" t="n">
-        <v>57500</v>
+        <v>58200</v>
       </c>
       <c r="S153" t="n">
         <v>55200</v>
       </c>
       <c r="T153" t="n">
-        <v>4.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="154">
@@ -11352,13 +11352,13 @@
         <v>0</v>
       </c>
       <c r="R154" t="n">
-        <v>8030</v>
+        <v>8140</v>
       </c>
       <c r="S154" t="n">
         <v>7810</v>
       </c>
       <c r="T154" t="n">
-        <v>2.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="155">
@@ -11469,13 +11469,13 @@
         <v>0</v>
       </c>
       <c r="R156" t="n">
-        <v>28450</v>
+        <v>28400</v>
       </c>
       <c r="S156" t="n">
         <v>27050</v>
       </c>
       <c r="T156" t="n">
-        <v>5.2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="157">
@@ -11541,13 +11541,13 @@
         <v>2.4</v>
       </c>
       <c r="R157" t="n">
-        <v>114900</v>
+        <v>117000</v>
       </c>
       <c r="S157" t="n">
         <v>98900</v>
       </c>
       <c r="T157" t="n">
-        <v>16.2</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="158">
@@ -11613,13 +11613,13 @@
         <v>2.4</v>
       </c>
       <c r="R158" t="n">
-        <v>811000</v>
+        <v>815000</v>
       </c>
       <c r="S158" t="n">
         <v>741000</v>
       </c>
       <c r="T158" t="n">
-        <v>9.4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="159">
@@ -11658,13 +11658,13 @@
         <v>0</v>
       </c>
       <c r="R159" t="n">
-        <v>9110</v>
+        <v>9200</v>
       </c>
       <c r="S159" t="n">
         <v>8920</v>
       </c>
       <c r="T159" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="160">
@@ -11730,13 +11730,13 @@
         <v>0</v>
       </c>
       <c r="R160" t="n">
-        <v>42900</v>
+        <v>42500</v>
       </c>
       <c r="S160" t="n">
         <v>46600</v>
       </c>
       <c r="T160" t="n">
-        <v>-7.9</v>
+        <v>-8.800000000000001</v>
       </c>
     </row>
     <row r="161">
@@ -11802,13 +11802,13 @@
         <v>0</v>
       </c>
       <c r="R161" t="n">
-        <v>47750</v>
+        <v>49050</v>
       </c>
       <c r="S161" t="n">
         <v>42500</v>
       </c>
       <c r="T161" t="n">
-        <v>12.4</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="162">
@@ -11850,7 +11850,7 @@
         <v>1928.3</v>
       </c>
       <c r="R162" t="n">
-        <v>57600</v>
+        <v>61300</v>
       </c>
     </row>
     <row r="163">
@@ -11916,13 +11916,13 @@
         <v>0</v>
       </c>
       <c r="R163" t="n">
-        <v>124900</v>
+        <v>131100</v>
       </c>
       <c r="S163" t="n">
         <v>111200</v>
       </c>
       <c r="T163" t="n">
-        <v>12.3</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="164">
@@ -11988,13 +11988,13 @@
         <v>0</v>
       </c>
       <c r="R164" t="n">
-        <v>206500</v>
+        <v>211000</v>
       </c>
       <c r="S164" t="n">
         <v>207500</v>
       </c>
       <c r="T164" t="n">
-        <v>-0.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="165">
@@ -12060,13 +12060,13 @@
         <v>0</v>
       </c>
       <c r="R165" t="n">
-        <v>133200</v>
+        <v>133000</v>
       </c>
       <c r="S165" t="n">
         <v>134700</v>
       </c>
       <c r="T165" t="n">
-        <v>-1.1</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="166">
@@ -12123,13 +12123,13 @@
         <v>14.6</v>
       </c>
       <c r="R166" t="n">
-        <v>5365</v>
+        <v>5630</v>
       </c>
       <c r="S166" t="n">
         <v>4555</v>
       </c>
       <c r="T166" t="n">
-        <v>17.8</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="167">
@@ -12168,13 +12168,13 @@
         <v>0</v>
       </c>
       <c r="R167" t="n">
-        <v>48300</v>
+        <v>49250</v>
       </c>
       <c r="S167" t="n">
         <v>43350</v>
       </c>
       <c r="T167" t="n">
-        <v>11.4</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="168">
@@ -12240,13 +12240,13 @@
         <v>-1.1</v>
       </c>
       <c r="R168" t="n">
-        <v>43300</v>
+        <v>45000</v>
       </c>
       <c r="S168" t="n">
         <v>40400</v>
       </c>
       <c r="T168" t="n">
-        <v>7.2</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="169">
@@ -12312,13 +12312,13 @@
         <v>0</v>
       </c>
       <c r="R169" t="n">
-        <v>65200</v>
+        <v>68200</v>
       </c>
       <c r="S169" t="n">
         <v>60500</v>
       </c>
       <c r="T169" t="n">
-        <v>7.8</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="170">
@@ -12384,13 +12384,13 @@
         <v>0</v>
       </c>
       <c r="R170" t="n">
-        <v>135600</v>
+        <v>135700</v>
       </c>
       <c r="S170" t="n">
         <v>141800</v>
       </c>
       <c r="T170" t="n">
-        <v>-4.4</v>
+        <v>-4.3</v>
       </c>
     </row>
     <row r="171">
@@ -12429,13 +12429,13 @@
         <v>0</v>
       </c>
       <c r="R171" t="n">
-        <v>12370</v>
+        <v>12400</v>
       </c>
       <c r="S171" t="n">
         <v>9940</v>
       </c>
       <c r="T171" t="n">
-        <v>24.4</v>
+        <v>24.7</v>
       </c>
     </row>
     <row r="172">
@@ -12501,13 +12501,13 @@
         <v>0</v>
       </c>
       <c r="R172" t="n">
-        <v>158900</v>
+        <v>161300</v>
       </c>
       <c r="S172" t="n">
         <v>131000</v>
       </c>
       <c r="T172" t="n">
-        <v>21.3</v>
+        <v>23.1</v>
       </c>
     </row>
     <row r="173">
@@ -12573,13 +12573,13 @@
         <v>0.3</v>
       </c>
       <c r="R173" t="n">
-        <v>140700</v>
+        <v>147500</v>
       </c>
       <c r="S173" t="n">
         <v>124600</v>
       </c>
       <c r="T173" t="n">
-        <v>12.9</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="174">
@@ -12645,13 +12645,13 @@
         <v>-30</v>
       </c>
       <c r="R174" t="n">
-        <v>18870</v>
+        <v>19100</v>
       </c>
       <c r="S174" t="n">
         <v>19280</v>
       </c>
       <c r="T174" t="n">
-        <v>-2.1</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="175">
@@ -12717,13 +12717,13 @@
         <v>-1.2</v>
       </c>
       <c r="R175" t="n">
-        <v>32500</v>
+        <v>32150</v>
       </c>
       <c r="S175" t="n">
         <v>28900</v>
       </c>
       <c r="T175" t="n">
-        <v>12.5</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="176">
@@ -12789,13 +12789,13 @@
         <v>0</v>
       </c>
       <c r="R176" t="n">
-        <v>126800</v>
+        <v>128700</v>
       </c>
       <c r="S176" t="n">
         <v>120300</v>
       </c>
       <c r="T176" t="n">
-        <v>5.4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="177">
@@ -12861,13 +12861,13 @@
         <v>-2</v>
       </c>
       <c r="R177" t="n">
-        <v>186700</v>
+        <v>185400</v>
       </c>
       <c r="S177" t="n">
         <v>204500</v>
       </c>
       <c r="T177" t="n">
-        <v>-8.699999999999999</v>
+        <v>-9.300000000000001</v>
       </c>
     </row>
     <row r="178">
@@ -12906,13 +12906,13 @@
         <v>0</v>
       </c>
       <c r="R178" t="n">
-        <v>31400</v>
+        <v>32350</v>
       </c>
       <c r="S178" t="n">
         <v>29600</v>
       </c>
       <c r="T178" t="n">
-        <v>6.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="179">
@@ -12978,13 +12978,13 @@
         <v>0</v>
       </c>
       <c r="R179" t="n">
-        <v>18220</v>
+        <v>18460</v>
       </c>
       <c r="S179" t="n">
         <v>18400</v>
       </c>
       <c r="T179" t="n">
-        <v>-1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="180">
@@ -13050,13 +13050,13 @@
         <v>0</v>
       </c>
       <c r="R180" t="n">
-        <v>80700</v>
+        <v>81400</v>
       </c>
       <c r="S180" t="n">
         <v>74800</v>
       </c>
       <c r="T180" t="n">
-        <v>7.9</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="181">
@@ -13122,13 +13122,13 @@
         <v>0</v>
       </c>
       <c r="R181" t="n">
-        <v>81400</v>
+        <v>82000</v>
       </c>
       <c r="S181" t="n">
         <v>83600</v>
       </c>
       <c r="T181" t="n">
-        <v>-2.6</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="182">
@@ -13194,13 +13194,13 @@
         <v>0</v>
       </c>
       <c r="R182" t="n">
-        <v>168800</v>
+        <v>168500</v>
       </c>
       <c r="S182" t="n">
         <v>175800</v>
       </c>
       <c r="T182" t="n">
-        <v>-4</v>
+        <v>-4.2</v>
       </c>
     </row>
     <row r="183">
@@ -13266,13 +13266,13 @@
         <v>0</v>
       </c>
       <c r="R183" t="n">
-        <v>272000</v>
+        <v>280000</v>
       </c>
       <c r="S183" t="n">
         <v>229500</v>
       </c>
       <c r="T183" t="n">
-        <v>18.5</v>
+        <v>22</v>
       </c>
     </row>
     <row r="184">
@@ -13338,13 +13338,13 @@
         <v>0</v>
       </c>
       <c r="R184" t="n">
-        <v>85800</v>
+        <v>85900</v>
       </c>
       <c r="S184" t="n">
         <v>93400</v>
       </c>
       <c r="T184" t="n">
-        <v>-8.1</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="185">
@@ -13410,13 +13410,13 @@
         <v>-19</v>
       </c>
       <c r="R185" t="n">
-        <v>45450</v>
+        <v>46850</v>
       </c>
       <c r="S185" t="n">
         <v>43850</v>
       </c>
       <c r="T185" t="n">
-        <v>3.6</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="186">
@@ -13455,13 +13455,13 @@
         <v>0</v>
       </c>
       <c r="R186" t="n">
-        <v>9450</v>
+        <v>9400</v>
       </c>
       <c r="S186" t="n">
         <v>9500</v>
       </c>
       <c r="T186" t="n">
-        <v>-0.5</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="187">
@@ -13527,13 +13527,13 @@
         <v>5</v>
       </c>
       <c r="R187" t="n">
-        <v>55900</v>
+        <v>55300</v>
       </c>
       <c r="S187" t="n">
         <v>58600</v>
       </c>
       <c r="T187" t="n">
-        <v>-4.6</v>
+        <v>-5.6</v>
       </c>
     </row>
     <row r="188">
@@ -13599,13 +13599,13 @@
         <v>4.1</v>
       </c>
       <c r="R188" t="n">
-        <v>40650</v>
+        <v>41050</v>
       </c>
       <c r="S188" t="n">
         <v>41550</v>
       </c>
       <c r="T188" t="n">
-        <v>-2.2</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="189">
@@ -13671,13 +13671,13 @@
         <v>-3.2</v>
       </c>
       <c r="R189" t="n">
-        <v>392500</v>
+        <v>398500</v>
       </c>
       <c r="S189" t="n">
         <v>392500</v>
       </c>
       <c r="T189" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="190">
@@ -13743,13 +13743,13 @@
         <v>0</v>
       </c>
       <c r="R190" t="n">
-        <v>257500</v>
+        <v>260000</v>
       </c>
       <c r="S190" t="n">
         <v>207000</v>
       </c>
       <c r="T190" t="n">
-        <v>24.4</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="191">
@@ -13815,13 +13815,13 @@
         <v>-0.4</v>
       </c>
       <c r="R191" t="n">
-        <v>116100</v>
+        <v>116700</v>
       </c>
       <c r="S191" t="n">
         <v>126300</v>
       </c>
       <c r="T191" t="n">
-        <v>-8.1</v>
+        <v>-7.6</v>
       </c>
     </row>
     <row r="192">
@@ -13887,13 +13887,13 @@
         <v>0</v>
       </c>
       <c r="R192" t="n">
-        <v>15050</v>
+        <v>15130</v>
       </c>
       <c r="S192" t="n">
         <v>15150</v>
       </c>
       <c r="T192" t="n">
-        <v>-0.7</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="193">
@@ -13959,13 +13959,13 @@
         <v>0</v>
       </c>
       <c r="R193" t="n">
-        <v>17280</v>
+        <v>17470</v>
       </c>
       <c r="S193" t="n">
         <v>17870</v>
       </c>
       <c r="T193" t="n">
-        <v>-3.3</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="194">
@@ -14031,13 +14031,13 @@
         <v>0</v>
       </c>
       <c r="R194" t="n">
-        <v>77900</v>
+        <v>78900</v>
       </c>
       <c r="S194" t="n">
         <v>81600</v>
       </c>
       <c r="T194" t="n">
-        <v>-4.5</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="195">
@@ -14166,13 +14166,13 @@
         <v>0</v>
       </c>
       <c r="R196" t="n">
-        <v>112900</v>
+        <v>113900</v>
       </c>
       <c r="S196" t="n">
         <v>113200</v>
       </c>
       <c r="T196" t="n">
-        <v>-0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="197">
@@ -14238,13 +14238,13 @@
         <v>1.1</v>
       </c>
       <c r="R197" t="n">
-        <v>254500</v>
+        <v>256000</v>
       </c>
       <c r="S197" t="n">
         <v>273500</v>
       </c>
       <c r="T197" t="n">
-        <v>-6.9</v>
+        <v>-6.4</v>
       </c>
     </row>
     <row r="198">
@@ -14310,13 +14310,13 @@
         <v>-21.6</v>
       </c>
       <c r="R198" t="n">
-        <v>40300</v>
+        <v>40700</v>
       </c>
       <c r="S198" t="n">
         <v>41400</v>
       </c>
       <c r="T198" t="n">
-        <v>-2.7</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="199">
@@ -14355,13 +14355,13 @@
         <v>0</v>
       </c>
       <c r="R199" t="n">
-        <v>10160</v>
+        <v>10180</v>
       </c>
       <c r="S199" t="n">
         <v>9680</v>
       </c>
       <c r="T199" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="200">
@@ -14427,13 +14427,13 @@
         <v>1.1</v>
       </c>
       <c r="R200" t="n">
-        <v>70700</v>
+        <v>71600</v>
       </c>
       <c r="S200" t="n">
         <v>70500</v>
       </c>
       <c r="T200" t="n">
-        <v>0.3</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="201">
@@ -14499,13 +14499,13 @@
         <v>12.6</v>
       </c>
       <c r="R201" t="n">
-        <v>137300</v>
+        <v>136700</v>
       </c>
       <c r="S201" t="n">
         <v>106700</v>
       </c>
       <c r="T201" t="n">
-        <v>28.7</v>
+        <v>28.1</v>
       </c>
     </row>
     <row r="202">
@@ -14571,13 +14571,13 @@
         <v>1.4</v>
       </c>
       <c r="R202" t="n">
-        <v>38450</v>
+        <v>38500</v>
       </c>
       <c r="S202" t="n">
         <v>38250</v>
       </c>
       <c r="T202" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="203">
@@ -14643,13 +14643,13 @@
         <v>0</v>
       </c>
       <c r="R203" t="n">
-        <v>28150</v>
+        <v>28000</v>
       </c>
       <c r="S203" t="n">
         <v>28850</v>
       </c>
       <c r="T203" t="n">
-        <v>-2.4</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="204">
@@ -14706,13 +14706,13 @@
         <v>26.8</v>
       </c>
       <c r="R204" t="n">
-        <v>36350</v>
+        <v>36950</v>
       </c>
       <c r="S204" t="n">
         <v>34100</v>
       </c>
       <c r="T204" t="n">
-        <v>6.6</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="205">
@@ -14778,13 +14778,13 @@
         <v>0</v>
       </c>
       <c r="R205" t="n">
-        <v>68200</v>
+        <v>68300</v>
       </c>
       <c r="S205" t="n">
         <v>70500</v>
       </c>
       <c r="T205" t="n">
-        <v>-3.3</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="206">
@@ -14850,13 +14850,13 @@
         <v>0</v>
       </c>
       <c r="R206" t="n">
-        <v>77300</v>
+        <v>79000</v>
       </c>
       <c r="S206" t="n">
         <v>70600</v>
       </c>
       <c r="T206" t="n">
-        <v>9.5</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="207">
@@ -14922,13 +14922,13 @@
         <v>-3.1</v>
       </c>
       <c r="R207" t="n">
-        <v>61800</v>
+        <v>61600</v>
       </c>
       <c r="S207" t="n">
         <v>62300</v>
       </c>
       <c r="T207" t="n">
-        <v>-0.8</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="208">
@@ -14994,13 +14994,13 @@
         <v>15.4</v>
       </c>
       <c r="R208" t="n">
-        <v>249000</v>
+        <v>247500</v>
       </c>
       <c r="S208" t="n">
         <v>205500</v>
       </c>
       <c r="T208" t="n">
-        <v>21.2</v>
+        <v>20.4</v>
       </c>
     </row>
     <row r="209">
@@ -15066,13 +15066,13 @@
         <v>0</v>
       </c>
       <c r="R209" t="n">
-        <v>41400</v>
+        <v>41650</v>
       </c>
       <c r="S209" t="n">
         <v>41600</v>
       </c>
       <c r="T209" t="n">
-        <v>-0.5</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="210">
@@ -15138,13 +15138,13 @@
         <v>-2.4</v>
       </c>
       <c r="R210" t="n">
-        <v>313000</v>
+        <v>314000</v>
       </c>
       <c r="S210" t="n">
         <v>305000</v>
       </c>
       <c r="T210" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="211">
@@ -15210,13 +15210,13 @@
         <v>0.3</v>
       </c>
       <c r="R211" t="n">
-        <v>55300</v>
+        <v>57100</v>
       </c>
       <c r="S211" t="n">
         <v>50800</v>
       </c>
       <c r="T211" t="n">
-        <v>8.9</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="212">
@@ -15282,13 +15282,13 @@
         <v>0</v>
       </c>
       <c r="R212" t="n">
-        <v>1547000</v>
+        <v>1548000</v>
       </c>
       <c r="S212" t="n">
         <v>1556000</v>
       </c>
       <c r="T212" t="n">
-        <v>-0.6</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="213">
@@ -15354,13 +15354,13 @@
         <v>-5.3</v>
       </c>
       <c r="R213" t="n">
-        <v>38150</v>
+        <v>37500</v>
       </c>
       <c r="S213" t="n">
         <v>45900</v>
       </c>
       <c r="T213" t="n">
-        <v>-16.9</v>
+        <v>-18.3</v>
       </c>
     </row>
     <row r="214">
@@ -15426,13 +15426,13 @@
         <v>-0.8</v>
       </c>
       <c r="R214" t="n">
-        <v>401000</v>
+        <v>398000</v>
       </c>
       <c r="S214" t="n">
         <v>378500</v>
       </c>
       <c r="T214" t="n">
-        <v>5.9</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="215">
@@ -15498,13 +15498,13 @@
         <v>0</v>
       </c>
       <c r="R215" t="n">
-        <v>52100</v>
+        <v>53200</v>
       </c>
       <c r="S215" t="n">
         <v>48450</v>
       </c>
       <c r="T215" t="n">
-        <v>7.5</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="216">
@@ -15570,13 +15570,13 @@
         <v>2.7</v>
       </c>
       <c r="R216" t="n">
-        <v>104500</v>
+        <v>108700</v>
       </c>
       <c r="S216" t="n">
         <v>110000</v>
       </c>
       <c r="T216" t="n">
-        <v>-5</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="217">
@@ -15642,13 +15642,13 @@
         <v>0</v>
       </c>
       <c r="R217" t="n">
-        <v>105700</v>
+        <v>106400</v>
       </c>
       <c r="S217" t="n">
         <v>100100</v>
       </c>
       <c r="T217" t="n">
-        <v>5.6</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="218">
@@ -15714,13 +15714,13 @@
         <v>-2.4</v>
       </c>
       <c r="R218" t="n">
-        <v>111100</v>
+        <v>116600</v>
       </c>
       <c r="S218" t="n">
         <v>88300</v>
       </c>
       <c r="T218" t="n">
-        <v>25.8</v>
+        <v>32</v>
       </c>
     </row>
     <row r="219">
@@ -15786,13 +15786,13 @@
         <v>2.9</v>
       </c>
       <c r="R219" t="n">
-        <v>65100</v>
+        <v>66100</v>
       </c>
       <c r="S219" t="n">
         <v>63600</v>
       </c>
       <c r="T219" t="n">
-        <v>2.4</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="220">
@@ -15858,13 +15858,13 @@
         <v>10.9</v>
       </c>
       <c r="R220" t="n">
-        <v>129000</v>
+        <v>127200</v>
       </c>
       <c r="S220" t="n">
         <v>95900</v>
       </c>
       <c r="T220" t="n">
-        <v>34.5</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="221">
@@ -15930,13 +15930,13 @@
         <v>0</v>
       </c>
       <c r="R221" t="n">
-        <v>114000</v>
+        <v>116700</v>
       </c>
       <c r="S221" t="n">
         <v>107000</v>
       </c>
       <c r="T221" t="n">
-        <v>6.5</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="222">
@@ -16002,13 +16002,13 @@
         <v>-1.4</v>
       </c>
       <c r="R222" t="n">
-        <v>38850</v>
+        <v>39100</v>
       </c>
       <c r="S222" t="n">
         <v>40900</v>
       </c>
       <c r="T222" t="n">
-        <v>-5</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="223">
@@ -16074,13 +16074,13 @@
         <v>20.1</v>
       </c>
       <c r="R223" t="n">
-        <v>53100</v>
+        <v>53000</v>
       </c>
       <c r="S223" t="n">
         <v>49500</v>
       </c>
       <c r="T223" t="n">
-        <v>7.3</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="224">
@@ -16146,13 +16146,13 @@
         <v>1.3</v>
       </c>
       <c r="R224" t="n">
-        <v>23550</v>
+        <v>23600</v>
       </c>
       <c r="S224" t="n">
         <v>25200</v>
       </c>
       <c r="T224" t="n">
-        <v>-6.5</v>
+        <v>-6.3</v>
       </c>
     </row>
     <row r="225">
@@ -16218,13 +16218,13 @@
         <v>0.3</v>
       </c>
       <c r="R225" t="n">
-        <v>43950</v>
+        <v>42850</v>
       </c>
       <c r="S225" t="n">
         <v>39300</v>
       </c>
       <c r="T225" t="n">
-        <v>11.8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="226">
@@ -16290,13 +16290,13 @@
         <v>-0.2</v>
       </c>
       <c r="R226" t="n">
-        <v>237000</v>
+        <v>238000</v>
       </c>
       <c r="S226" t="n">
         <v>241500</v>
       </c>
       <c r="T226" t="n">
-        <v>-1.9</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="227">
@@ -16362,13 +16362,13 @@
         <v>-15.3</v>
       </c>
       <c r="R227" t="n">
-        <v>31400</v>
+        <v>31250</v>
       </c>
       <c r="S227" t="n">
         <v>35600</v>
       </c>
       <c r="T227" t="n">
-        <v>-11.8</v>
+        <v>-12.2</v>
       </c>
     </row>
     <row r="228">
@@ -16434,13 +16434,13 @@
         <v>3.6</v>
       </c>
       <c r="R228" t="n">
-        <v>236500</v>
+        <v>235500</v>
       </c>
       <c r="S228" t="n">
         <v>225000</v>
       </c>
       <c r="T228" t="n">
-        <v>5.1</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="229">
@@ -16506,13 +16506,13 @@
         <v>0</v>
       </c>
       <c r="R229" t="n">
-        <v>774000</v>
+        <v>803000</v>
       </c>
       <c r="S229" t="n">
         <v>762000</v>
       </c>
       <c r="T229" t="n">
-        <v>1.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="230">
@@ -16578,13 +16578,13 @@
         <v>0</v>
       </c>
       <c r="R230" t="n">
-        <v>135900</v>
+        <v>138600</v>
       </c>
       <c r="S230" t="n">
         <v>138100</v>
       </c>
       <c r="T230" t="n">
-        <v>-1.6</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="231">
@@ -16650,13 +16650,13 @@
         <v>0.1</v>
       </c>
       <c r="R231" t="n">
-        <v>135500</v>
+        <v>134000</v>
       </c>
       <c r="S231" t="n">
         <v>137600</v>
       </c>
       <c r="T231" t="n">
-        <v>-1.5</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="232">
@@ -16794,13 +16794,13 @@
         <v>0</v>
       </c>
       <c r="R233" t="n">
-        <v>5260</v>
+        <v>5320</v>
       </c>
       <c r="S233" t="n">
         <v>5380</v>
       </c>
       <c r="T233" t="n">
-        <v>-2.2</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="234">
@@ -16857,13 +16857,13 @@
         <v>0</v>
       </c>
       <c r="R234" t="n">
-        <v>496500</v>
+        <v>501000</v>
       </c>
       <c r="S234" t="n">
         <v>465000</v>
       </c>
       <c r="T234" t="n">
-        <v>6.8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="235">
@@ -16929,13 +16929,13 @@
         <v>0.8</v>
       </c>
       <c r="R235" t="n">
-        <v>393000</v>
+        <v>390500</v>
       </c>
       <c r="S235" t="n">
         <v>384500</v>
       </c>
       <c r="T235" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="236">
@@ -17001,13 +17001,13 @@
         <v>9.300000000000001</v>
       </c>
       <c r="R236" t="n">
-        <v>127500</v>
+        <v>129300</v>
       </c>
       <c r="S236" t="n">
         <v>116900</v>
       </c>
       <c r="T236" t="n">
-        <v>9.1</v>
+        <v>10.6</v>
       </c>
     </row>
     <row r="237">
@@ -17073,13 +17073,13 @@
         <v>4.6</v>
       </c>
       <c r="R237" t="n">
-        <v>147000</v>
+        <v>145200</v>
       </c>
       <c r="S237" t="n">
         <v>153100</v>
       </c>
       <c r="T237" t="n">
-        <v>-4</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="238">
@@ -17145,13 +17145,13 @@
         <v>0</v>
       </c>
       <c r="R238" t="n">
-        <v>50100</v>
+        <v>50000</v>
       </c>
       <c r="S238" t="n">
         <v>43650</v>
       </c>
       <c r="T238" t="n">
-        <v>14.8</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="239">
@@ -17217,13 +17217,13 @@
         <v>0</v>
       </c>
       <c r="R239" t="n">
-        <v>22000</v>
+        <v>22100</v>
       </c>
       <c r="S239" t="n">
         <v>22650</v>
       </c>
       <c r="T239" t="n">
-        <v>-2.9</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="240">
@@ -17289,13 +17289,13 @@
         <v>0</v>
       </c>
       <c r="R240" t="n">
-        <v>323000</v>
+        <v>330500</v>
       </c>
       <c r="S240" t="n">
         <v>339000</v>
       </c>
       <c r="T240" t="n">
-        <v>-4.7</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="241">
@@ -17361,13 +17361,13 @@
         <v>0</v>
       </c>
       <c r="R241" t="n">
-        <v>2865000</v>
+        <v>2954000</v>
       </c>
       <c r="S241" t="n">
         <v>2832000</v>
       </c>
       <c r="T241" t="n">
-        <v>1.2</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="242">
@@ -17433,13 +17433,13 @@
         <v>0</v>
       </c>
       <c r="R242" t="n">
-        <v>174700</v>
+        <v>177700</v>
       </c>
       <c r="S242" t="n">
         <v>183200</v>
       </c>
       <c r="T242" t="n">
-        <v>-4.6</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="243">
@@ -17496,13 +17496,13 @@
         <v>0</v>
       </c>
       <c r="R243" t="n">
-        <v>83500</v>
+        <v>84100</v>
       </c>
       <c r="S243" t="n">
         <v>86600</v>
       </c>
       <c r="T243" t="n">
-        <v>-3.6</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="244">
@@ -17568,13 +17568,13 @@
         <v>0</v>
       </c>
       <c r="R244" t="n">
-        <v>14770</v>
+        <v>14900</v>
       </c>
       <c r="S244" t="n">
         <v>14830</v>
       </c>
       <c r="T244" t="n">
-        <v>-0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="245">
@@ -17631,13 +17631,13 @@
         <v>-184.9</v>
       </c>
       <c r="R245" t="n">
-        <v>37300</v>
+        <v>37650</v>
       </c>
       <c r="S245" t="n">
         <v>36850</v>
       </c>
       <c r="T245" t="n">
-        <v>1.2</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="246">
@@ -17703,13 +17703,13 @@
         <v>0</v>
       </c>
       <c r="R246" t="n">
-        <v>131100</v>
+        <v>132800</v>
       </c>
       <c r="S246" t="n">
         <v>132000</v>
       </c>
       <c r="T246" t="n">
-        <v>-0.7</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="247">
@@ -17775,13 +17775,13 @@
         <v>0</v>
       </c>
       <c r="R247" t="n">
-        <v>473500</v>
+        <v>489500</v>
       </c>
       <c r="S247" t="n">
         <v>412000</v>
       </c>
       <c r="T247" t="n">
-        <v>14.9</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="248">
@@ -17847,13 +17847,13 @@
         <v>0</v>
       </c>
       <c r="R248" t="n">
-        <v>33350</v>
+        <v>33700</v>
       </c>
       <c r="S248" t="n">
         <v>34800</v>
       </c>
       <c r="T248" t="n">
-        <v>-4.2</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="249">
@@ -17913,13 +17913,13 @@
         <v>1043</v>
       </c>
       <c r="R249" t="n">
-        <v>9590</v>
+        <v>10030</v>
       </c>
       <c r="S249" t="n">
         <v>8320</v>
       </c>
       <c r="T249" t="n">
-        <v>15.3</v>
+        <v>20.6</v>
       </c>
     </row>
     <row r="250">
@@ -17985,13 +17985,13 @@
         <v>0</v>
       </c>
       <c r="R250" t="n">
-        <v>128000</v>
+        <v>134100</v>
       </c>
       <c r="S250" t="n">
         <v>118400</v>
       </c>
       <c r="T250" t="n">
-        <v>8.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="251">
@@ -18057,13 +18057,13 @@
         <v>-0.5</v>
       </c>
       <c r="R251" t="n">
-        <v>22150</v>
+        <v>22200</v>
       </c>
       <c r="S251" t="n">
         <v>22000</v>
       </c>
       <c r="T251" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="252">
@@ -18129,13 +18129,13 @@
         <v>0.1</v>
       </c>
       <c r="R252" t="n">
-        <v>86800</v>
+        <v>87300</v>
       </c>
       <c r="S252" t="n">
         <v>85400</v>
       </c>
       <c r="T252" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="253">
@@ -18201,13 +18201,13 @@
         <v>-0.9</v>
       </c>
       <c r="R253" t="n">
-        <v>507000</v>
+        <v>510000</v>
       </c>
       <c r="S253" t="n">
         <v>506000</v>
       </c>
       <c r="T253" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="254">
@@ -18273,13 +18273,13 @@
         <v>0</v>
       </c>
       <c r="R254" t="n">
-        <v>177600</v>
+        <v>179400</v>
       </c>
       <c r="S254" t="n">
         <v>185000</v>
       </c>
       <c r="T254" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="255">
@@ -18345,13 +18345,13 @@
         <v>0</v>
       </c>
       <c r="R255" t="n">
-        <v>116200</v>
+        <v>119100</v>
       </c>
       <c r="S255" t="n">
         <v>103800</v>
       </c>
       <c r="T255" t="n">
-        <v>11.9</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="256">
@@ -18417,13 +18417,13 @@
         <v>0</v>
       </c>
       <c r="R256" t="n">
-        <v>306000</v>
+        <v>322000</v>
       </c>
       <c r="S256" t="n">
         <v>295000</v>
       </c>
       <c r="T256" t="n">
-        <v>3.7</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="257">
@@ -18489,13 +18489,13 @@
         <v>-40.6</v>
       </c>
       <c r="R257" t="n">
-        <v>15260</v>
+        <v>15550</v>
       </c>
       <c r="S257" t="n">
         <v>14980</v>
       </c>
       <c r="T257" t="n">
-        <v>1.9</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="258">
@@ -18561,13 +18561,13 @@
         <v>0</v>
       </c>
       <c r="R258" t="n">
-        <v>361000</v>
+        <v>369500</v>
       </c>
       <c r="S258" t="n">
         <v>360000</v>
       </c>
       <c r="T258" t="n">
-        <v>0.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="259">
@@ -18633,13 +18633,13 @@
         <v>0</v>
       </c>
       <c r="R259" t="n">
-        <v>73400</v>
+        <v>73800</v>
       </c>
       <c r="S259" t="n">
         <v>72000</v>
       </c>
       <c r="T259" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="260">
@@ -18705,13 +18705,13 @@
         <v>-2.1</v>
       </c>
       <c r="R260" t="n">
-        <v>19750</v>
+        <v>19800</v>
       </c>
       <c r="S260" t="n">
         <v>19660</v>
       </c>
       <c r="T260" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="261">
@@ -18777,13 +18777,13 @@
         <v>-15.5</v>
       </c>
       <c r="R261" t="n">
-        <v>45450</v>
+        <v>45150</v>
       </c>
       <c r="S261" t="n">
         <v>42000</v>
       </c>
       <c r="T261" t="n">
-        <v>8.199999999999999</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="262">
@@ -18849,13 +18849,13 @@
         <v>0</v>
       </c>
       <c r="R262" t="n">
-        <v>67500</v>
+        <v>67000</v>
       </c>
       <c r="S262" t="n">
         <v>67000</v>
       </c>
       <c r="T262" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="263">
@@ -18894,13 +18894,13 @@
         <v>0</v>
       </c>
       <c r="R263" t="n">
-        <v>41550</v>
+        <v>41100</v>
       </c>
       <c r="S263" t="n">
         <v>33500</v>
       </c>
       <c r="T263" t="n">
-        <v>24</v>
+        <v>22.7</v>
       </c>
     </row>
     <row r="264">
@@ -18966,13 +18966,13 @@
         <v>0</v>
       </c>
       <c r="R264" t="n">
-        <v>1143000</v>
+        <v>1154000</v>
       </c>
       <c r="S264" t="n">
         <v>939000</v>
       </c>
       <c r="T264" t="n">
-        <v>21.7</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="265">
@@ -19011,13 +19011,13 @@
         <v>0</v>
       </c>
       <c r="R265" t="n">
-        <v>39550</v>
+        <v>40400</v>
       </c>
       <c r="S265" t="n">
         <v>34400</v>
       </c>
       <c r="T265" t="n">
-        <v>15</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="266">
@@ -19083,13 +19083,13 @@
         <v>0.9</v>
       </c>
       <c r="R266" t="n">
-        <v>116100</v>
+        <v>120100</v>
       </c>
       <c r="S266" t="n">
         <v>110300</v>
       </c>
       <c r="T266" t="n">
-        <v>5.3</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="267">
@@ -19155,13 +19155,13 @@
         <v>0</v>
       </c>
       <c r="R267" t="n">
-        <v>55500</v>
+        <v>54700</v>
       </c>
       <c r="S267" t="n">
         <v>49150</v>
       </c>
       <c r="T267" t="n">
-        <v>12.9</v>
+        <v>11.3</v>
       </c>
     </row>
     <row r="268">
@@ -19227,13 +19227,13 @@
         <v>0</v>
       </c>
       <c r="R268" t="n">
-        <v>65400</v>
+        <v>65500</v>
       </c>
       <c r="S268" t="n">
         <v>57100</v>
       </c>
       <c r="T268" t="n">
-        <v>14.5</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="269">
@@ -19299,13 +19299,13 @@
         <v>0</v>
       </c>
       <c r="R269" t="n">
-        <v>200500</v>
+        <v>196800</v>
       </c>
       <c r="S269" t="n">
         <v>196400</v>
       </c>
       <c r="T269" t="n">
-        <v>2.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="270">
@@ -19371,13 +19371,13 @@
         <v>0</v>
       </c>
       <c r="R270" t="n">
-        <v>79300</v>
+        <v>80900</v>
       </c>
       <c r="S270" t="n">
         <v>77400</v>
       </c>
       <c r="T270" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="271">
@@ -19443,13 +19443,13 @@
         <v>0</v>
       </c>
       <c r="R271" t="n">
-        <v>9800</v>
+        <v>9860</v>
       </c>
       <c r="S271" t="n">
         <v>9800</v>
       </c>
       <c r="T271" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="272">
@@ -19515,13 +19515,13 @@
         <v>-5.5</v>
       </c>
       <c r="R272" t="n">
-        <v>31200</v>
+        <v>31700</v>
       </c>
       <c r="S272" t="n">
         <v>32750</v>
       </c>
       <c r="T272" t="n">
-        <v>-4.7</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="273">
@@ -19587,13 +19587,13 @@
         <v>1.1</v>
       </c>
       <c r="R273" t="n">
-        <v>228000</v>
+        <v>228500</v>
       </c>
       <c r="S273" t="n">
         <v>246000</v>
       </c>
       <c r="T273" t="n">
-        <v>-7.3</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="274">
@@ -19659,13 +19659,13 @@
         <v>0</v>
       </c>
       <c r="R274" t="n">
-        <v>18030</v>
+        <v>17820</v>
       </c>
       <c r="S274" t="n">
         <v>16000</v>
       </c>
       <c r="T274" t="n">
-        <v>12.7</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="275">
@@ -19731,13 +19731,13 @@
         <v>-1</v>
       </c>
       <c r="R275" t="n">
-        <v>53200</v>
+        <v>53300</v>
       </c>
       <c r="S275" t="n">
         <v>48900</v>
       </c>
       <c r="T275" t="n">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
     </row>
     <row r="276">
@@ -19776,13 +19776,13 @@
         <v>0</v>
       </c>
       <c r="R276" t="n">
-        <v>45400</v>
+        <v>45900</v>
       </c>
       <c r="S276" t="n">
         <v>46200</v>
       </c>
       <c r="T276" t="n">
-        <v>-1.7</v>
+        <v>-0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-08-15
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -455,7 +455,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-08-14 · 전주 2026-08-07</t>
+          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-08-15 · 전주 2026-08-07</t>
         </is>
       </c>
     </row>
@@ -597,31 +597,31 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1913.1</v>
+        <v>1912.4</v>
       </c>
       <c r="J3" t="n">
         <v>1913.1</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="L3" t="n">
-        <v>2014.5</v>
+        <v>2027</v>
       </c>
       <c r="M3" t="n">
         <v>2014.5</v>
       </c>
       <c r="N3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="O3" t="n">
-        <v>2156.6</v>
+        <v>2164.2</v>
       </c>
       <c r="P3" t="n">
         <v>2156.6</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R3" t="n">
         <v>15850</v>
@@ -1290,31 +1290,31 @@
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>30987.2</v>
+        <v>31281.5</v>
       </c>
       <c r="J13" t="n">
         <v>30987.2</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L13" t="n">
-        <v>33793.2</v>
+        <v>36815.2</v>
       </c>
       <c r="M13" t="n">
         <v>33793.2</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>8.9</v>
       </c>
       <c r="O13" t="n">
-        <v>34047.1</v>
+        <v>37033.8</v>
       </c>
       <c r="P13" t="n">
         <v>34047.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="R13" t="n">
         <v>615000</v>
@@ -1713,31 +1713,31 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>10874.9</v>
+        <v>10934.2</v>
       </c>
       <c r="J19" t="n">
         <v>10874.9</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L19" t="n">
-        <v>12172.3</v>
+        <v>12243.7</v>
       </c>
       <c r="M19" t="n">
         <v>12172.3</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="O19" t="n">
-        <v>13312.2</v>
+        <v>13359.8</v>
       </c>
       <c r="P19" t="n">
         <v>13312.2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R19" t="n">
         <v>45350</v>
@@ -1911,7 +1911,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="n">
-        <v>1772.2</v>
+        <v>1771.6</v>
       </c>
       <c r="J22" t="n">
         <v>1776.7</v>
@@ -1920,7 +1920,7 @@
         <v>-0.3</v>
       </c>
       <c r="L22" t="n">
-        <v>2130.3</v>
+        <v>2132.2</v>
       </c>
       <c r="M22" t="n">
         <v>2139.9</v>
@@ -1929,7 +1929,7 @@
         <v>-0.4</v>
       </c>
       <c r="O22" t="n">
-        <v>2401.6</v>
+        <v>2400.2</v>
       </c>
       <c r="P22" t="n">
         <v>2437.2</v>
@@ -2478,31 +2478,31 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>15660.6</v>
+        <v>16363.9</v>
       </c>
       <c r="J30" t="n">
         <v>16388.5</v>
       </c>
       <c r="K30" t="n">
-        <v>-4.4</v>
+        <v>-0.2</v>
       </c>
       <c r="L30" t="n">
-        <v>18708.9</v>
+        <v>20311.2</v>
       </c>
       <c r="M30" t="n">
         <v>20712.2</v>
       </c>
       <c r="N30" t="n">
-        <v>-9.699999999999999</v>
+        <v>-1.9</v>
       </c>
       <c r="O30" t="n">
-        <v>20155.3</v>
+        <v>22126.9</v>
       </c>
       <c r="P30" t="n">
         <v>21913.1</v>
       </c>
       <c r="Q30" t="n">
-        <v>-8</v>
+        <v>1</v>
       </c>
       <c r="R30" t="n">
         <v>120000</v>
@@ -3198,31 +3198,31 @@
         <v>0</v>
       </c>
       <c r="I40" t="n">
-        <v>21369.8</v>
+        <v>23213.5</v>
       </c>
       <c r="J40" t="n">
         <v>21369.8</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>8.6</v>
       </c>
       <c r="L40" t="n">
-        <v>23187</v>
+        <v>23939.7</v>
       </c>
       <c r="M40" t="n">
         <v>23187</v>
       </c>
       <c r="N40" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="O40" t="n">
-        <v>24471.6</v>
+        <v>25246.5</v>
       </c>
       <c r="P40" t="n">
         <v>24471.6</v>
       </c>
       <c r="Q40" t="n">
-        <v>0</v>
+        <v>3.2</v>
       </c>
       <c r="R40" t="n">
         <v>176800</v>
@@ -3486,31 +3486,31 @@
         <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>5543</v>
+        <v>5742</v>
       </c>
       <c r="J44" t="n">
         <v>5491.8</v>
       </c>
       <c r="K44" t="n">
-        <v>0.9</v>
+        <v>4.6</v>
       </c>
       <c r="L44" t="n">
-        <v>5933</v>
+        <v>6005.3</v>
       </c>
       <c r="M44" t="n">
         <v>5863.2</v>
       </c>
       <c r="N44" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="O44" t="n">
-        <v>6040</v>
+        <v>6140</v>
       </c>
       <c r="P44" t="n">
         <v>6013</v>
       </c>
       <c r="Q44" t="n">
-        <v>0.4</v>
+        <v>2.1</v>
       </c>
       <c r="R44" t="n">
         <v>37550</v>
@@ -3918,31 +3918,31 @@
         <v>0</v>
       </c>
       <c r="I50" t="n">
-        <v>47527.2</v>
+        <v>47797.9</v>
       </c>
       <c r="J50" t="n">
         <v>42637.8</v>
       </c>
       <c r="K50" t="n">
-        <v>11.5</v>
+        <v>12.1</v>
       </c>
       <c r="L50" t="n">
-        <v>26108.4</v>
+        <v>26153.7</v>
       </c>
       <c r="M50" t="n">
         <v>26349.2</v>
       </c>
       <c r="N50" t="n">
-        <v>-0.9</v>
+        <v>-0.7</v>
       </c>
       <c r="O50" t="n">
-        <v>27025.7</v>
+        <v>27203.7</v>
       </c>
       <c r="P50" t="n">
         <v>27155.9</v>
       </c>
       <c r="Q50" t="n">
-        <v>-0.5</v>
+        <v>0.2</v>
       </c>
       <c r="R50" t="n">
         <v>37650</v>
@@ -4485,31 +4485,31 @@
         <v>0</v>
       </c>
       <c r="I58" t="n">
-        <v>383.2</v>
+        <v>389.2</v>
       </c>
       <c r="J58" t="n">
         <v>378.1</v>
       </c>
       <c r="K58" t="n">
-        <v>1.3</v>
+        <v>2.9</v>
       </c>
       <c r="L58" t="n">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="M58" t="n">
         <v>447.1</v>
       </c>
       <c r="N58" t="n">
-        <v>-3.8</v>
+        <v>-4.7</v>
       </c>
       <c r="O58" t="n">
-        <v>537.5</v>
+        <v>524.2</v>
       </c>
       <c r="P58" t="n">
         <v>585.4</v>
       </c>
       <c r="Q58" t="n">
-        <v>-8.199999999999999</v>
+        <v>-10.5</v>
       </c>
       <c r="R58" t="n">
         <v>40500</v>
@@ -5061,31 +5061,31 @@
         <v>0</v>
       </c>
       <c r="I66" t="n">
-        <v>1950.4</v>
+        <v>1768.2</v>
       </c>
       <c r="J66" t="n">
         <v>1998</v>
       </c>
       <c r="K66" t="n">
-        <v>-2.4</v>
+        <v>-11.5</v>
       </c>
       <c r="L66" t="n">
-        <v>2052</v>
+        <v>1935.2</v>
       </c>
       <c r="M66" t="n">
         <v>2174.8</v>
       </c>
       <c r="N66" t="n">
-        <v>-5.6</v>
+        <v>-11</v>
       </c>
       <c r="O66" t="n">
-        <v>3472.8</v>
+        <v>3376.5</v>
       </c>
       <c r="P66" t="n">
         <v>3560.6</v>
       </c>
       <c r="Q66" t="n">
-        <v>-2.5</v>
+        <v>-5.2</v>
       </c>
       <c r="R66" t="n">
         <v>16730</v>
@@ -5349,31 +5349,31 @@
         <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>14632.7</v>
+        <v>15670.8</v>
       </c>
       <c r="J70" t="n">
         <v>14632.7</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>7.1</v>
       </c>
       <c r="L70" t="n">
-        <v>10103.5</v>
+        <v>10170.2</v>
       </c>
       <c r="M70" t="n">
         <v>10103.5</v>
       </c>
       <c r="N70" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="O70" t="n">
-        <v>10048.4</v>
+        <v>8860.5</v>
       </c>
       <c r="P70" t="n">
         <v>10048.4</v>
       </c>
       <c r="Q70" t="n">
-        <v>0</v>
+        <v>-11.8</v>
       </c>
       <c r="R70" t="n">
         <v>21250</v>
@@ -6060,31 +6060,31 @@
         <v>0</v>
       </c>
       <c r="I80" t="n">
-        <v>1880</v>
+        <v>1880.4</v>
       </c>
       <c r="J80" t="n">
         <v>1879.4</v>
       </c>
       <c r="K80" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="L80" t="n">
-        <v>2387.1</v>
+        <v>2382.7</v>
       </c>
       <c r="M80" t="n">
         <v>2389</v>
       </c>
       <c r="N80" t="n">
-        <v>-0.1</v>
+        <v>-0.3</v>
       </c>
       <c r="O80" t="n">
-        <v>3114.2</v>
+        <v>3075</v>
       </c>
       <c r="P80" t="n">
         <v>3090.2</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.8</v>
+        <v>-0.5</v>
       </c>
       <c r="R80" t="n">
         <v>218500</v>
@@ -6204,31 +6204,31 @@
         <v>0</v>
       </c>
       <c r="I82" t="n">
-        <v>84649.3</v>
+        <v>81516.39999999999</v>
       </c>
       <c r="J82" t="n">
         <v>97891.39999999999</v>
       </c>
       <c r="K82" t="n">
-        <v>-13.5</v>
+        <v>-16.7</v>
       </c>
       <c r="L82" t="n">
-        <v>121459.2</v>
+        <v>118344.1</v>
       </c>
       <c r="M82" t="n">
         <v>137111.9</v>
       </c>
       <c r="N82" t="n">
-        <v>-11.4</v>
+        <v>-13.7</v>
       </c>
       <c r="O82" t="n">
-        <v>139310.8</v>
+        <v>139037.8</v>
       </c>
       <c r="P82" t="n">
         <v>152635.4</v>
       </c>
       <c r="Q82" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.9</v>
       </c>
       <c r="R82" t="n">
         <v>33250</v>
@@ -6780,31 +6780,31 @@
         <v>0</v>
       </c>
       <c r="I90" t="n">
-        <v>482</v>
+        <v>467.8</v>
       </c>
       <c r="J90" t="n">
         <v>482</v>
       </c>
       <c r="K90" t="n">
-        <v>0</v>
+        <v>-2.9</v>
       </c>
       <c r="L90" t="n">
-        <v>820</v>
+        <v>765.2</v>
       </c>
       <c r="M90" t="n">
         <v>820</v>
       </c>
       <c r="N90" t="n">
-        <v>0</v>
+        <v>-6.7</v>
       </c>
       <c r="O90" t="n">
-        <v>740.3</v>
+        <v>746.8</v>
       </c>
       <c r="P90" t="n">
         <v>740.3</v>
       </c>
       <c r="Q90" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="R90" t="n">
         <v>23200</v>
@@ -7130,15 +7130,6 @@
           <t>KOSPI200,커버리지</t>
         </is>
       </c>
-      <c r="F95" t="n">
-        <v>1557</v>
-      </c>
-      <c r="G95" t="n">
-        <v>1557</v>
-      </c>
-      <c r="H95" t="n">
-        <v>0</v>
-      </c>
       <c r="I95" t="n">
         <v>6781</v>
       </c>
@@ -7617,31 +7608,31 @@
         <v>0</v>
       </c>
       <c r="I102" t="n">
-        <v>33560.4</v>
+        <v>32159.5</v>
       </c>
       <c r="J102" t="n">
         <v>33471.6</v>
       </c>
       <c r="K102" t="n">
-        <v>0.3</v>
+        <v>-3.9</v>
       </c>
       <c r="L102" t="n">
-        <v>55259.8</v>
+        <v>68894.5</v>
       </c>
       <c r="M102" t="n">
         <v>55410.6</v>
       </c>
       <c r="N102" t="n">
-        <v>-0.3</v>
+        <v>24.3</v>
       </c>
       <c r="O102" t="n">
-        <v>33270.9</v>
+        <v>45521.6</v>
       </c>
       <c r="P102" t="n">
         <v>33270.9</v>
       </c>
       <c r="Q102" t="n">
-        <v>0</v>
+        <v>36.8</v>
       </c>
       <c r="R102" t="n">
         <v>301000</v>
@@ -8184,31 +8175,31 @@
         <v>-0.1</v>
       </c>
       <c r="I110" t="n">
-        <v>22425.2</v>
+        <v>22171.3</v>
       </c>
       <c r="J110" t="n">
         <v>23801.6</v>
       </c>
       <c r="K110" t="n">
-        <v>-5.8</v>
+        <v>-6.8</v>
       </c>
       <c r="L110" t="n">
-        <v>26076.1</v>
+        <v>25835.1</v>
       </c>
       <c r="M110" t="n">
         <v>27787.1</v>
       </c>
       <c r="N110" t="n">
-        <v>-6.2</v>
+        <v>-7</v>
       </c>
       <c r="O110" t="n">
-        <v>30354.1</v>
+        <v>30038.4</v>
       </c>
       <c r="P110" t="n">
         <v>31999.8</v>
       </c>
       <c r="Q110" t="n">
-        <v>-5.1</v>
+        <v>-6.1</v>
       </c>
       <c r="R110" t="n">
         <v>228000</v>
@@ -8400,31 +8391,31 @@
         <v>0</v>
       </c>
       <c r="I113" t="n">
-        <v>1541.9</v>
+        <v>1529.1</v>
       </c>
       <c r="J113" t="n">
         <v>1676.8</v>
       </c>
       <c r="K113" t="n">
-        <v>-8</v>
+        <v>-8.800000000000001</v>
       </c>
       <c r="L113" t="n">
-        <v>1702.5</v>
+        <v>1681.4</v>
       </c>
       <c r="M113" t="n">
         <v>1888.7</v>
       </c>
       <c r="N113" t="n">
-        <v>-9.9</v>
+        <v>-11</v>
       </c>
       <c r="O113" t="n">
-        <v>1734.1</v>
+        <v>1702.3</v>
       </c>
       <c r="P113" t="n">
         <v>1924.5</v>
       </c>
       <c r="Q113" t="n">
-        <v>-9.9</v>
+        <v>-11.5</v>
       </c>
       <c r="R113" t="n">
         <v>41050</v>
@@ -8562,13 +8553,13 @@
         <v>8.199999999999999</v>
       </c>
       <c r="O115" t="n">
-        <v>24280.4</v>
+        <v>24366.8</v>
       </c>
       <c r="P115" t="n">
         <v>22082.9</v>
       </c>
       <c r="Q115" t="n">
-        <v>10</v>
+        <v>10.3</v>
       </c>
       <c r="R115" t="n">
         <v>36600</v>
@@ -8832,31 +8823,31 @@
         <v>0</v>
       </c>
       <c r="I119" t="n">
-        <v>519.4</v>
+        <v>507.8</v>
       </c>
       <c r="J119" t="n">
         <v>525.4</v>
       </c>
       <c r="K119" t="n">
-        <v>-1.1</v>
+        <v>-3.3</v>
       </c>
       <c r="L119" t="n">
-        <v>678.8</v>
+        <v>651.2</v>
       </c>
       <c r="M119" t="n">
         <v>678.8</v>
       </c>
       <c r="N119" t="n">
-        <v>0</v>
+        <v>-4.1</v>
       </c>
       <c r="O119" t="n">
-        <v>756.8</v>
+        <v>723.5</v>
       </c>
       <c r="P119" t="n">
         <v>766.8</v>
       </c>
       <c r="Q119" t="n">
-        <v>-1.3</v>
+        <v>-5.6</v>
       </c>
       <c r="R119" t="n">
         <v>32700</v>
@@ -9164,15 +9155,6 @@
           <t>KOSPI200,커버리지</t>
         </is>
       </c>
-      <c r="F124" t="n">
-        <v>5335</v>
-      </c>
-      <c r="G124" t="n">
-        <v>5335</v>
-      </c>
-      <c r="H124" t="n">
-        <v>0</v>
-      </c>
       <c r="I124" t="n">
         <v>22530</v>
       </c>
@@ -9462,31 +9444,31 @@
         <v>0</v>
       </c>
       <c r="I128" t="n">
-        <v>3712.8</v>
+        <v>3653.6</v>
       </c>
       <c r="J128" t="n">
         <v>3849.6</v>
       </c>
       <c r="K128" t="n">
-        <v>-3.6</v>
+        <v>-5.1</v>
       </c>
       <c r="L128" t="n">
-        <v>5996.2</v>
+        <v>5956.6</v>
       </c>
       <c r="M128" t="n">
         <v>6069.3</v>
       </c>
       <c r="N128" t="n">
-        <v>-1.2</v>
+        <v>-1.9</v>
       </c>
       <c r="O128" t="n">
-        <v>7480.7</v>
+        <v>7433.4</v>
       </c>
       <c r="P128" t="n">
         <v>7572.3</v>
       </c>
       <c r="Q128" t="n">
-        <v>-1.2</v>
+        <v>-1.8</v>
       </c>
       <c r="R128" t="n">
         <v>146400</v>
@@ -11880,40 +11862,40 @@
         </is>
       </c>
       <c r="F163" t="n">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="G163" t="n">
         <v>249</v>
       </c>
       <c r="H163" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="I163" t="n">
-        <v>1027.3</v>
+        <v>1055.5</v>
       </c>
       <c r="J163" t="n">
         <v>1027.3</v>
       </c>
       <c r="K163" t="n">
-        <v>0</v>
+        <v>2.7</v>
       </c>
       <c r="L163" t="n">
-        <v>1319</v>
+        <v>1382</v>
       </c>
       <c r="M163" t="n">
         <v>1319</v>
       </c>
       <c r="N163" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="O163" t="n">
-        <v>1390</v>
+        <v>1350</v>
       </c>
       <c r="P163" t="n">
         <v>1390</v>
       </c>
       <c r="Q163" t="n">
-        <v>0</v>
+        <v>-2.9</v>
       </c>
       <c r="R163" t="n">
         <v>131100</v>
@@ -12546,31 +12528,31 @@
         <v>0</v>
       </c>
       <c r="I173" t="n">
-        <v>1018.8</v>
+        <v>1031.3</v>
       </c>
       <c r="J173" t="n">
         <v>1015.8</v>
       </c>
       <c r="K173" t="n">
-        <v>0.3</v>
+        <v>1.5</v>
       </c>
       <c r="L173" t="n">
-        <v>1375</v>
+        <v>1441</v>
       </c>
       <c r="M173" t="n">
         <v>1356.6</v>
       </c>
       <c r="N173" t="n">
-        <v>1.4</v>
+        <v>6.2</v>
       </c>
       <c r="O173" t="n">
-        <v>1823.4</v>
+        <v>1927.3</v>
       </c>
       <c r="P173" t="n">
         <v>1817.3</v>
       </c>
       <c r="Q173" t="n">
-        <v>0.3</v>
+        <v>6.1</v>
       </c>
       <c r="R173" t="n">
         <v>147500</v>
@@ -12618,22 +12600,22 @@
         <v>0</v>
       </c>
       <c r="I174" t="n">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="J174" t="n">
         <v>366.5</v>
       </c>
       <c r="K174" t="n">
-        <v>-4.5</v>
+        <v>-5.9</v>
       </c>
       <c r="L174" t="n">
-        <v>485.8</v>
+        <v>493.2</v>
       </c>
       <c r="M174" t="n">
         <v>473.4</v>
       </c>
       <c r="N174" t="n">
-        <v>2.6</v>
+        <v>4.2</v>
       </c>
       <c r="O174" t="n">
         <v>598.2</v>
@@ -12762,31 +12744,31 @@
         <v>0</v>
       </c>
       <c r="I176" t="n">
-        <v>80330.10000000001</v>
+        <v>84273.89999999999</v>
       </c>
       <c r="J176" t="n">
         <v>80330.10000000001</v>
       </c>
       <c r="K176" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="L176" t="n">
-        <v>40678.1</v>
+        <v>41287.8</v>
       </c>
       <c r="M176" t="n">
         <v>40678.1</v>
       </c>
       <c r="N176" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="O176" t="n">
-        <v>44043.8</v>
+        <v>43216.7</v>
       </c>
       <c r="P176" t="n">
         <v>44043.8</v>
       </c>
       <c r="Q176" t="n">
-        <v>0</v>
+        <v>-1.9</v>
       </c>
       <c r="R176" t="n">
         <v>128700</v>
@@ -13788,31 +13770,31 @@
         <v>0</v>
       </c>
       <c r="I191" t="n">
-        <v>32341.8</v>
+        <v>32423.4</v>
       </c>
       <c r="J191" t="n">
         <v>31480.7</v>
       </c>
       <c r="K191" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="L191" t="n">
-        <v>34098.8</v>
+        <v>34399</v>
       </c>
       <c r="M191" t="n">
         <v>33722</v>
       </c>
       <c r="N191" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="O191" t="n">
-        <v>35395.8</v>
+        <v>35646.6</v>
       </c>
       <c r="P191" t="n">
         <v>35539.5</v>
       </c>
       <c r="Q191" t="n">
-        <v>-0.4</v>
+        <v>0.3</v>
       </c>
       <c r="R191" t="n">
         <v>116700</v>
@@ -14004,31 +13986,31 @@
         <v>0</v>
       </c>
       <c r="I194" t="n">
-        <v>5200.8</v>
+        <v>4188.1</v>
       </c>
       <c r="J194" t="n">
         <v>5200.8</v>
       </c>
       <c r="K194" t="n">
-        <v>0</v>
+        <v>-19.5</v>
       </c>
       <c r="L194" t="n">
-        <v>6201.1</v>
+        <v>5619.9</v>
       </c>
       <c r="M194" t="n">
         <v>6201.1</v>
       </c>
       <c r="N194" t="n">
-        <v>0</v>
+        <v>-9.4</v>
       </c>
       <c r="O194" t="n">
-        <v>6784.5</v>
+        <v>6077.9</v>
       </c>
       <c r="P194" t="n">
         <v>6784.5</v>
       </c>
       <c r="Q194" t="n">
-        <v>0</v>
+        <v>-10.4</v>
       </c>
       <c r="R194" t="n">
         <v>78900</v>
@@ -14283,31 +14265,31 @@
         <v>0</v>
       </c>
       <c r="I198" t="n">
-        <v>783.3</v>
+        <v>768.8</v>
       </c>
       <c r="J198" t="n">
         <v>862.2</v>
       </c>
       <c r="K198" t="n">
-        <v>-9.199999999999999</v>
+        <v>-10.8</v>
       </c>
       <c r="L198" t="n">
-        <v>938</v>
+        <v>911</v>
       </c>
       <c r="M198" t="n">
         <v>1060.2</v>
       </c>
       <c r="N198" t="n">
-        <v>-11.5</v>
+        <v>-14.1</v>
       </c>
       <c r="O198" t="n">
-        <v>1175</v>
+        <v>1130</v>
       </c>
       <c r="P198" t="n">
         <v>1499</v>
       </c>
       <c r="Q198" t="n">
-        <v>-21.6</v>
+        <v>-24.6</v>
       </c>
       <c r="R198" t="n">
         <v>40700</v>
@@ -14895,16 +14877,16 @@
         <v>0</v>
       </c>
       <c r="I207" t="n">
-        <v>2836.8</v>
+        <v>2831</v>
       </c>
       <c r="J207" t="n">
         <v>2857.4</v>
       </c>
       <c r="K207" t="n">
-        <v>-0.7</v>
+        <v>-0.9</v>
       </c>
       <c r="L207" t="n">
-        <v>3094.6</v>
+        <v>3094.2</v>
       </c>
       <c r="M207" t="n">
         <v>3131.4</v>
@@ -15111,13 +15093,13 @@
         <v>5.2</v>
       </c>
       <c r="I210" t="n">
-        <v>2588.5</v>
+        <v>2641.5</v>
       </c>
       <c r="J210" t="n">
         <v>2573.5</v>
       </c>
       <c r="K210" t="n">
-        <v>0.6</v>
+        <v>2.6</v>
       </c>
       <c r="L210" t="n">
         <v>4463</v>
@@ -15327,31 +15309,31 @@
         <v>0</v>
       </c>
       <c r="I213" t="n">
-        <v>2006.2</v>
+        <v>1944.1</v>
       </c>
       <c r="J213" t="n">
         <v>2107.1</v>
       </c>
       <c r="K213" t="n">
-        <v>-4.8</v>
+        <v>-7.7</v>
       </c>
       <c r="L213" t="n">
-        <v>2665.9</v>
+        <v>2569.5</v>
       </c>
       <c r="M213" t="n">
         <v>2814</v>
       </c>
       <c r="N213" t="n">
-        <v>-5.3</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="O213" t="n">
-        <v>3295.3</v>
+        <v>3234</v>
       </c>
       <c r="P213" t="n">
         <v>3480.9</v>
       </c>
       <c r="Q213" t="n">
-        <v>-5.3</v>
+        <v>-7.1</v>
       </c>
       <c r="R213" t="n">
         <v>37500</v>
@@ -15399,31 +15381,31 @@
         <v>0</v>
       </c>
       <c r="I214" t="n">
-        <v>2709.2</v>
+        <v>2706.6</v>
       </c>
       <c r="J214" t="n">
         <v>2704.3</v>
       </c>
       <c r="K214" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L214" t="n">
-        <v>3369.9</v>
+        <v>3364.9</v>
       </c>
       <c r="M214" t="n">
         <v>3377.6</v>
       </c>
       <c r="N214" t="n">
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="O214" t="n">
-        <v>4047.7</v>
+        <v>4032.5</v>
       </c>
       <c r="P214" t="n">
         <v>4080.3</v>
       </c>
       <c r="Q214" t="n">
-        <v>-0.8</v>
+        <v>-1.2</v>
       </c>
       <c r="R214" t="n">
         <v>398000</v>
@@ -15543,31 +15525,31 @@
         <v>0</v>
       </c>
       <c r="I216" t="n">
-        <v>2381.4</v>
+        <v>2453.7</v>
       </c>
       <c r="J216" t="n">
         <v>2310.6</v>
       </c>
       <c r="K216" t="n">
-        <v>3.1</v>
+        <v>6.2</v>
       </c>
       <c r="L216" t="n">
-        <v>3986.6</v>
+        <v>4074.3</v>
       </c>
       <c r="M216" t="n">
         <v>3869.9</v>
       </c>
       <c r="N216" t="n">
-        <v>3</v>
+        <v>5.3</v>
       </c>
       <c r="O216" t="n">
-        <v>5005.4</v>
+        <v>5154.1</v>
       </c>
       <c r="P216" t="n">
         <v>4872.6</v>
       </c>
       <c r="Q216" t="n">
-        <v>2.7</v>
+        <v>5.8</v>
       </c>
       <c r="R216" t="n">
         <v>108700</v>
@@ -16191,31 +16173,31 @@
         <v>0</v>
       </c>
       <c r="I225" t="n">
-        <v>2784.7</v>
+        <v>2928.9</v>
       </c>
       <c r="J225" t="n">
         <v>2766.7</v>
       </c>
       <c r="K225" t="n">
-        <v>0.7</v>
+        <v>5.9</v>
       </c>
       <c r="L225" t="n">
-        <v>3498.9</v>
+        <v>3725</v>
       </c>
       <c r="M225" t="n">
         <v>3488.9</v>
       </c>
       <c r="N225" t="n">
-        <v>0.3</v>
+        <v>6.8</v>
       </c>
       <c r="O225" t="n">
-        <v>4209.2</v>
+        <v>4538.8</v>
       </c>
       <c r="P225" t="n">
         <v>4195.5</v>
       </c>
       <c r="Q225" t="n">
-        <v>0.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="R225" t="n">
         <v>42850</v>
@@ -16767,31 +16749,31 @@
         <v>0</v>
       </c>
       <c r="I233" t="n">
-        <v>-297</v>
+        <v>-302.4</v>
       </c>
       <c r="J233" t="n">
         <v>-297</v>
       </c>
       <c r="K233" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="L233" t="n">
-        <v>799</v>
+        <v>790.1</v>
       </c>
       <c r="M233" t="n">
         <v>799</v>
       </c>
       <c r="N233" t="n">
-        <v>0</v>
+        <v>-1.1</v>
       </c>
       <c r="O233" t="n">
-        <v>1236</v>
+        <v>1297.8</v>
       </c>
       <c r="P233" t="n">
         <v>1236</v>
       </c>
       <c r="Q233" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="R233" t="n">
         <v>5320</v>
@@ -17118,31 +17100,31 @@
         <v>0</v>
       </c>
       <c r="I238" t="n">
-        <v>78.5</v>
+        <v>587</v>
       </c>
       <c r="J238" t="n">
         <v>78.5</v>
       </c>
       <c r="K238" t="n">
-        <v>0</v>
+        <v>647.8</v>
       </c>
       <c r="L238" t="n">
-        <v>1154</v>
+        <v>1592</v>
       </c>
       <c r="M238" t="n">
         <v>1154</v>
       </c>
       <c r="N238" t="n">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="O238" t="n">
-        <v>1770</v>
+        <v>2230</v>
       </c>
       <c r="P238" t="n">
         <v>1770</v>
       </c>
       <c r="Q238" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="R238" t="n">
         <v>50000</v>
@@ -18462,31 +18444,31 @@
         <v>0</v>
       </c>
       <c r="I257" t="n">
-        <v>-2424.1</v>
+        <v>-2480.9</v>
       </c>
       <c r="J257" t="n">
         <v>-2433.7</v>
       </c>
       <c r="K257" t="n">
-        <v>0.4</v>
+        <v>-1.9</v>
       </c>
       <c r="L257" t="n">
-        <v>-1037.2</v>
+        <v>-1153.1</v>
       </c>
       <c r="M257" t="n">
         <v>-990.8</v>
       </c>
       <c r="N257" t="n">
-        <v>-4.7</v>
+        <v>-16.4</v>
       </c>
       <c r="O257" t="n">
-        <v>41.4</v>
+        <v>3</v>
       </c>
       <c r="P257" t="n">
         <v>69.7</v>
       </c>
       <c r="Q257" t="n">
-        <v>-40.6</v>
+        <v>-95.7</v>
       </c>
       <c r="R257" t="n">
         <v>15550</v>
@@ -19560,31 +19542,31 @@
         <v>0</v>
       </c>
       <c r="I273" t="n">
-        <v>1614.8</v>
+        <v>1628.2</v>
       </c>
       <c r="J273" t="n">
         <v>1615.7</v>
       </c>
       <c r="K273" t="n">
-        <v>-0.1</v>
+        <v>0.8</v>
       </c>
       <c r="L273" t="n">
-        <v>2195.4</v>
+        <v>2207.5</v>
       </c>
       <c r="M273" t="n">
         <v>2185.1</v>
       </c>
       <c r="N273" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O273" t="n">
-        <v>2782.4</v>
+        <v>2796</v>
       </c>
       <c r="P273" t="n">
         <v>2752.9</v>
       </c>
       <c r="Q273" t="n">
-        <v>1.1</v>
+        <v>1.6</v>
       </c>
       <c r="R273" t="n">
         <v>228500</v>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-08-24
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -455,7 +455,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-08-22 · 전주 2026-08-16</t>
+          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-08-24 · 전주 2026-08-16</t>
         </is>
       </c>
     </row>
@@ -615,13 +615,13 @@
         <v>-0.2</v>
       </c>
       <c r="R3" t="n">
-        <v>15240</v>
+        <v>15470</v>
       </c>
       <c r="S3" t="n">
         <v>15850</v>
       </c>
       <c r="T3" t="n">
-        <v>-3.8</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="4">
@@ -678,13 +678,13 @@
         <v>-2.3</v>
       </c>
       <c r="R4" t="n">
-        <v>82300</v>
+        <v>84500</v>
       </c>
       <c r="S4" t="n">
         <v>83700</v>
       </c>
       <c r="T4" t="n">
-        <v>-1.7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -813,13 +813,13 @@
         <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>1078000</v>
+        <v>1084000</v>
       </c>
       <c r="S6" t="n">
         <v>1276000</v>
       </c>
       <c r="T6" t="n">
-        <v>-15.5</v>
+        <v>-15</v>
       </c>
     </row>
     <row r="7">
@@ -885,13 +885,13 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>46700</v>
+        <v>46600</v>
       </c>
       <c r="S7" t="n">
         <v>51900</v>
       </c>
       <c r="T7" t="n">
-        <v>-10</v>
+        <v>-10.2</v>
       </c>
     </row>
     <row r="8">
@@ -948,13 +948,13 @@
         <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>23250</v>
+        <v>23775</v>
       </c>
       <c r="S8" t="n">
         <v>26250</v>
       </c>
       <c r="T8" t="n">
-        <v>-11.4</v>
+        <v>-9.4</v>
       </c>
     </row>
     <row r="9">
@@ -1020,13 +1020,13 @@
         <v>0.7</v>
       </c>
       <c r="R9" t="n">
-        <v>130900</v>
+        <v>130800</v>
       </c>
       <c r="S9" t="n">
         <v>141700</v>
       </c>
       <c r="T9" t="n">
-        <v>-7.6</v>
+        <v>-7.7</v>
       </c>
     </row>
     <row r="10">
@@ -1092,13 +1092,13 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>90000</v>
+        <v>92100</v>
       </c>
       <c r="S10" t="n">
         <v>93000</v>
       </c>
       <c r="T10" t="n">
-        <v>-3.2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="11">
@@ -1155,13 +1155,13 @@
         <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>1730000</v>
+        <v>1679000</v>
       </c>
       <c r="S11" t="n">
         <v>1645000</v>
       </c>
       <c r="T11" t="n">
-        <v>5.2</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="12">
@@ -1227,13 +1227,13 @@
         <v>-0.3</v>
       </c>
       <c r="R12" t="n">
-        <v>105600</v>
+        <v>104500</v>
       </c>
       <c r="S12" t="n">
         <v>115800</v>
       </c>
       <c r="T12" t="n">
-        <v>-8.800000000000001</v>
+        <v>-9.800000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -1299,13 +1299,13 @@
         <v>-1.2</v>
       </c>
       <c r="R13" t="n">
-        <v>661000</v>
+        <v>633000</v>
       </c>
       <c r="S13" t="n">
         <v>615000</v>
       </c>
       <c r="T13" t="n">
-        <v>7.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="14">
@@ -1434,13 +1434,13 @@
         <v>5.9</v>
       </c>
       <c r="R15" t="n">
-        <v>89700</v>
+        <v>87000</v>
       </c>
       <c r="S15" t="n">
         <v>102800</v>
       </c>
       <c r="T15" t="n">
-        <v>-12.7</v>
+        <v>-15.4</v>
       </c>
     </row>
     <row r="16">
@@ -1506,13 +1506,13 @@
         <v>1.1</v>
       </c>
       <c r="R16" t="n">
-        <v>121300</v>
+        <v>127200</v>
       </c>
       <c r="S16" t="n">
         <v>138100</v>
       </c>
       <c r="T16" t="n">
-        <v>-12.2</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="17">
@@ -1578,13 +1578,13 @@
         <v>0</v>
       </c>
       <c r="R17" t="n">
-        <v>39350</v>
+        <v>41900</v>
       </c>
       <c r="S17" t="n">
         <v>45000</v>
       </c>
       <c r="T17" t="n">
-        <v>-12.6</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="18">
@@ -1650,13 +1650,13 @@
         <v>0</v>
       </c>
       <c r="R18" t="n">
-        <v>26650</v>
+        <v>26600</v>
       </c>
       <c r="S18" t="n">
         <v>29950</v>
       </c>
       <c r="T18" t="n">
-        <v>-11</v>
+        <v>-11.2</v>
       </c>
     </row>
     <row r="19">
@@ -1713,13 +1713,13 @@
         <v>17.9</v>
       </c>
       <c r="R19" t="n">
-        <v>49750</v>
+        <v>50200</v>
       </c>
       <c r="S19" t="n">
         <v>45350</v>
       </c>
       <c r="T19" t="n">
-        <v>9.699999999999999</v>
+        <v>10.7</v>
       </c>
     </row>
     <row r="20">
@@ -1785,13 +1785,13 @@
         <v>0</v>
       </c>
       <c r="R20" t="n">
-        <v>17320</v>
+        <v>17990</v>
       </c>
       <c r="S20" t="n">
         <v>18370</v>
       </c>
       <c r="T20" t="n">
-        <v>-5.7</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="21">
@@ -1848,13 +1848,13 @@
         <v>0</v>
       </c>
       <c r="R21" t="n">
-        <v>6400</v>
+        <v>6550</v>
       </c>
       <c r="S21" t="n">
         <v>6730</v>
       </c>
       <c r="T21" t="n">
-        <v>-4.9</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="22">
@@ -1920,13 +1920,13 @@
         <v>-0.1</v>
       </c>
       <c r="R22" t="n">
-        <v>484000</v>
+        <v>450500</v>
       </c>
       <c r="S22" t="n">
         <v>465500</v>
       </c>
       <c r="T22" t="n">
-        <v>4</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="23">
@@ -1983,13 +1983,13 @@
         <v>17.4</v>
       </c>
       <c r="R23" t="n">
-        <v>14750</v>
+        <v>14880</v>
       </c>
       <c r="S23" t="n">
         <v>13400</v>
       </c>
       <c r="T23" t="n">
-        <v>10.1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24">
@@ -2055,13 +2055,13 @@
         <v>-21.5</v>
       </c>
       <c r="R24" t="n">
-        <v>100300</v>
+        <v>100500</v>
       </c>
       <c r="S24" t="n">
         <v>108000</v>
       </c>
       <c r="T24" t="n">
-        <v>-7.1</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="25">
@@ -2127,13 +2127,13 @@
         <v>0</v>
       </c>
       <c r="R25" t="n">
-        <v>9700</v>
+        <v>9690</v>
       </c>
       <c r="S25" t="n">
         <v>10240</v>
       </c>
       <c r="T25" t="n">
-        <v>-5.3</v>
+        <v>-5.4</v>
       </c>
     </row>
     <row r="26">
@@ -2190,13 +2190,13 @@
         <v>-30</v>
       </c>
       <c r="R26" t="n">
-        <v>7710</v>
+        <v>7810</v>
       </c>
       <c r="S26" t="n">
         <v>7960</v>
       </c>
       <c r="T26" t="n">
-        <v>-3.1</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="27">
@@ -2253,13 +2253,13 @@
         <v>1.1</v>
       </c>
       <c r="R27" t="n">
-        <v>1366000</v>
+        <v>1402000</v>
       </c>
       <c r="S27" t="n">
         <v>1270000</v>
       </c>
       <c r="T27" t="n">
-        <v>7.6</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="28">
@@ -2325,13 +2325,13 @@
         <v>-0.3</v>
       </c>
       <c r="R28" t="n">
-        <v>25800</v>
+        <v>26050</v>
       </c>
       <c r="S28" t="n">
         <v>26300</v>
       </c>
       <c r="T28" t="n">
-        <v>-1.9</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="29">
@@ -2397,13 +2397,13 @@
         <v>0.9</v>
       </c>
       <c r="R29" t="n">
-        <v>107700</v>
+        <v>112300</v>
       </c>
       <c r="S29" t="n">
         <v>120000</v>
       </c>
       <c r="T29" t="n">
-        <v>-10.2</v>
+        <v>-6.4</v>
       </c>
     </row>
     <row r="30">
@@ -2460,13 +2460,13 @@
         <v>0</v>
       </c>
       <c r="R30" t="n">
-        <v>154900</v>
+        <v>170700</v>
       </c>
       <c r="S30" t="n">
         <v>170500</v>
       </c>
       <c r="T30" t="n">
-        <v>-9.1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="31">
@@ -2523,13 +2523,13 @@
         <v>0</v>
       </c>
       <c r="R31" t="n">
-        <v>44150</v>
+        <v>45500</v>
       </c>
       <c r="S31" t="n">
         <v>47100</v>
       </c>
       <c r="T31" t="n">
-        <v>-6.3</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="32">
@@ -2595,13 +2595,13 @@
         <v>0</v>
       </c>
       <c r="R32" t="n">
-        <v>27000</v>
+        <v>27800</v>
       </c>
       <c r="S32" t="n">
         <v>29900</v>
       </c>
       <c r="T32" t="n">
-        <v>-9.699999999999999</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="33">
@@ -2658,13 +2658,13 @@
         <v>-0.7</v>
       </c>
       <c r="R33" t="n">
-        <v>400500</v>
+        <v>397500</v>
       </c>
       <c r="S33" t="n">
         <v>427000</v>
       </c>
       <c r="T33" t="n">
-        <v>-6.2</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="34">
@@ -2721,13 +2721,13 @@
         <v>5.8</v>
       </c>
       <c r="R34" t="n">
-        <v>432500</v>
+        <v>454500</v>
       </c>
       <c r="S34" t="n">
         <v>437500</v>
       </c>
       <c r="T34" t="n">
-        <v>-1.1</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="35">
@@ -2793,13 +2793,13 @@
         <v>0.8</v>
       </c>
       <c r="R35" t="n">
-        <v>22800</v>
+        <v>23050</v>
       </c>
       <c r="S35" t="n">
         <v>24300</v>
       </c>
       <c r="T35" t="n">
-        <v>-6.2</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="36">
@@ -2856,13 +2856,13 @@
         <v>0</v>
       </c>
       <c r="R36" t="n">
-        <v>96600</v>
+        <v>97700</v>
       </c>
       <c r="S36" t="n">
         <v>101700</v>
       </c>
       <c r="T36" t="n">
-        <v>-5</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="37">
@@ -2919,13 +2919,13 @@
         <v>0.1</v>
       </c>
       <c r="R37" t="n">
-        <v>415000</v>
+        <v>410500</v>
       </c>
       <c r="S37" t="n">
         <v>453000</v>
       </c>
       <c r="T37" t="n">
-        <v>-8.4</v>
+        <v>-9.4</v>
       </c>
     </row>
     <row r="38">
@@ -2982,13 +2982,13 @@
         <v>0</v>
       </c>
       <c r="R38" t="n">
-        <v>310000</v>
+        <v>326500</v>
       </c>
       <c r="S38" t="n">
         <v>334000</v>
       </c>
       <c r="T38" t="n">
-        <v>-7.2</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="39">
@@ -3054,13 +3054,13 @@
         <v>-0.8</v>
       </c>
       <c r="R39" t="n">
-        <v>177800</v>
+        <v>180400</v>
       </c>
       <c r="S39" t="n">
         <v>176800</v>
       </c>
       <c r="T39" t="n">
-        <v>0.6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
@@ -3126,13 +3126,13 @@
         <v>0.8</v>
       </c>
       <c r="R40" t="n">
-        <v>52400</v>
+        <v>53500</v>
       </c>
       <c r="S40" t="n">
         <v>61600</v>
       </c>
       <c r="T40" t="n">
-        <v>-14.9</v>
+        <v>-13.1</v>
       </c>
     </row>
     <row r="41">
@@ -3189,13 +3189,13 @@
         <v>0</v>
       </c>
       <c r="R41" t="n">
-        <v>281500</v>
+        <v>256750</v>
       </c>
       <c r="S41" t="n">
         <v>274500</v>
       </c>
       <c r="T41" t="n">
-        <v>2.6</v>
+        <v>-6.5</v>
       </c>
     </row>
     <row r="42">
@@ -3261,13 +3261,13 @@
         <v>0</v>
       </c>
       <c r="R42" t="n">
-        <v>26100</v>
+        <v>25900</v>
       </c>
       <c r="S42" t="n">
         <v>28750</v>
       </c>
       <c r="T42" t="n">
-        <v>-9.199999999999999</v>
+        <v>-9.9</v>
       </c>
     </row>
     <row r="43">
@@ -3324,13 +3324,13 @@
         <v>0</v>
       </c>
       <c r="R43" t="n">
-        <v>37750</v>
+        <v>38000</v>
       </c>
       <c r="S43" t="n">
         <v>37550</v>
       </c>
       <c r="T43" t="n">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="44">
@@ -3387,13 +3387,13 @@
         <v>11.7</v>
       </c>
       <c r="R44" t="n">
-        <v>293500</v>
+        <v>286000</v>
       </c>
       <c r="S44" t="n">
         <v>323500</v>
       </c>
       <c r="T44" t="n">
-        <v>-9.300000000000001</v>
+        <v>-11.6</v>
       </c>
     </row>
     <row r="45">
@@ -3459,13 +3459,13 @@
         <v>-0.6</v>
       </c>
       <c r="R45" t="n">
-        <v>122100</v>
+        <v>130600</v>
       </c>
       <c r="S45" t="n">
         <v>129200</v>
       </c>
       <c r="T45" t="n">
-        <v>-5.5</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="46">
@@ -3522,13 +3522,13 @@
         <v>0</v>
       </c>
       <c r="R46" t="n">
-        <v>33250</v>
+        <v>34150</v>
       </c>
       <c r="S46" t="n">
         <v>35350</v>
       </c>
       <c r="T46" t="n">
-        <v>-5.9</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="47">
@@ -3594,13 +3594,13 @@
         <v>0</v>
       </c>
       <c r="R47" t="n">
-        <v>478000</v>
+        <v>514000</v>
       </c>
       <c r="S47" t="n">
         <v>516000</v>
       </c>
       <c r="T47" t="n">
-        <v>-7.4</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="48">
@@ -3657,13 +3657,13 @@
         <v>0</v>
       </c>
       <c r="R48" t="n">
-        <v>80300</v>
+        <v>82700</v>
       </c>
       <c r="S48" t="n">
         <v>91400</v>
       </c>
       <c r="T48" t="n">
-        <v>-12.1</v>
+        <v>-9.5</v>
       </c>
     </row>
     <row r="49">
@@ -3729,13 +3729,13 @@
         <v>0</v>
       </c>
       <c r="R49" t="n">
-        <v>34500</v>
+        <v>34550</v>
       </c>
       <c r="S49" t="n">
         <v>37650</v>
       </c>
       <c r="T49" t="n">
-        <v>-8.4</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="50">
@@ -3792,13 +3792,13 @@
         <v>-0.6</v>
       </c>
       <c r="R50" t="n">
-        <v>25800</v>
+        <v>26800</v>
       </c>
       <c r="S50" t="n">
         <v>27700</v>
       </c>
       <c r="T50" t="n">
-        <v>-6.9</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="51">
@@ -3855,13 +3855,13 @@
         <v>8.800000000000001</v>
       </c>
       <c r="R51" t="n">
-        <v>44200</v>
+        <v>47950</v>
       </c>
       <c r="S51" t="n">
         <v>58900</v>
       </c>
       <c r="T51" t="n">
-        <v>-25</v>
+        <v>-18.6</v>
       </c>
     </row>
     <row r="52">
@@ -3927,13 +3927,13 @@
         <v>5.8</v>
       </c>
       <c r="R52" t="n">
-        <v>99300</v>
+        <v>101300</v>
       </c>
       <c r="S52" t="n">
         <v>95600</v>
       </c>
       <c r="T52" t="n">
-        <v>3.9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53">
@@ -3990,13 +3990,13 @@
         <v>-0.3</v>
       </c>
       <c r="R53" t="n">
-        <v>54600</v>
+        <v>55200</v>
       </c>
       <c r="S53" t="n">
         <v>63100</v>
       </c>
       <c r="T53" t="n">
-        <v>-13.5</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="54">
@@ -4053,13 +4053,13 @@
         <v>0</v>
       </c>
       <c r="R54" t="n">
-        <v>14860</v>
+        <v>15120</v>
       </c>
       <c r="S54" t="n">
         <v>15090</v>
       </c>
       <c r="T54" t="n">
-        <v>-1.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="55">
@@ -4116,13 +4116,13 @@
         <v>0</v>
       </c>
       <c r="R55" t="n">
-        <v>42300</v>
+        <v>42100</v>
       </c>
       <c r="S55" t="n">
         <v>45400</v>
       </c>
       <c r="T55" t="n">
-        <v>-6.8</v>
+        <v>-7.3</v>
       </c>
     </row>
     <row r="56">
@@ -4179,13 +4179,13 @@
         <v>0</v>
       </c>
       <c r="R56" t="n">
-        <v>1316000</v>
+        <v>1318000</v>
       </c>
       <c r="S56" t="n">
         <v>1558000</v>
       </c>
       <c r="T56" t="n">
-        <v>-15.5</v>
+        <v>-15.4</v>
       </c>
     </row>
     <row r="57">
@@ -4242,13 +4242,13 @@
         <v>-3.3</v>
       </c>
       <c r="R57" t="n">
-        <v>38050</v>
+        <v>39050</v>
       </c>
       <c r="S57" t="n">
         <v>40500</v>
       </c>
       <c r="T57" t="n">
-        <v>-6</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="58">
@@ -4287,13 +4287,13 @@
         <v>0</v>
       </c>
       <c r="R58" t="n">
-        <v>56500</v>
+        <v>60200</v>
       </c>
       <c r="S58" t="n">
         <v>59700</v>
       </c>
       <c r="T58" t="n">
-        <v>-5.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="59">
@@ -4350,13 +4350,13 @@
         <v>1.7</v>
       </c>
       <c r="R59" t="n">
-        <v>348500</v>
+        <v>351500</v>
       </c>
       <c r="S59" t="n">
         <v>386000</v>
       </c>
       <c r="T59" t="n">
-        <v>-9.699999999999999</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="60">
@@ -4413,13 +4413,13 @@
         <v>0</v>
       </c>
       <c r="R60" t="n">
-        <v>32050</v>
+        <v>31800</v>
       </c>
       <c r="S60" t="n">
         <v>35400</v>
       </c>
       <c r="T60" t="n">
-        <v>-9.5</v>
+        <v>-10.2</v>
       </c>
     </row>
     <row r="61">
@@ -4476,13 +4476,13 @@
         <v>0</v>
       </c>
       <c r="R61" t="n">
-        <v>265000</v>
+        <v>268000</v>
       </c>
       <c r="S61" t="n">
         <v>279000</v>
       </c>
       <c r="T61" t="n">
-        <v>-5</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="62">
@@ -4548,13 +4548,13 @@
         <v>0</v>
       </c>
       <c r="R62" t="n">
-        <v>187000</v>
+        <v>191300</v>
       </c>
       <c r="S62" t="n">
         <v>206500</v>
       </c>
       <c r="T62" t="n">
-        <v>-9.4</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="63">
@@ -4611,13 +4611,13 @@
         <v>5.3</v>
       </c>
       <c r="R63" t="n">
-        <v>1237000</v>
+        <v>1347000</v>
       </c>
       <c r="S63" t="n">
         <v>1196000</v>
       </c>
       <c r="T63" t="n">
-        <v>3.4</v>
+        <v>12.6</v>
       </c>
     </row>
     <row r="64">
@@ -4683,13 +4683,13 @@
         <v>0</v>
       </c>
       <c r="R64" t="n">
-        <v>20200</v>
+        <v>20050</v>
       </c>
       <c r="S64" t="n">
         <v>22300</v>
       </c>
       <c r="T64" t="n">
-        <v>-9.4</v>
+        <v>-10.1</v>
       </c>
     </row>
     <row r="65">
@@ -4746,13 +4746,13 @@
         <v>0</v>
       </c>
       <c r="R65" t="n">
-        <v>15060</v>
+        <v>16010</v>
       </c>
       <c r="S65" t="n">
         <v>16730</v>
       </c>
       <c r="T65" t="n">
-        <v>-10</v>
+        <v>-4.3</v>
       </c>
     </row>
     <row r="66">
@@ -4809,13 +4809,13 @@
         <v>0</v>
       </c>
       <c r="R66" t="n">
-        <v>141100</v>
+        <v>141200</v>
       </c>
       <c r="S66" t="n">
         <v>147600</v>
       </c>
       <c r="T66" t="n">
-        <v>-4.4</v>
+        <v>-4.3</v>
       </c>
     </row>
     <row r="67">
@@ -4872,13 +4872,13 @@
         <v>0</v>
       </c>
       <c r="R67" t="n">
-        <v>550000</v>
+        <v>571000</v>
       </c>
       <c r="S67" t="n">
         <v>654000</v>
       </c>
       <c r="T67" t="n">
-        <v>-15.9</v>
+        <v>-12.7</v>
       </c>
     </row>
     <row r="68">
@@ -4944,13 +4944,13 @@
         <v>0</v>
       </c>
       <c r="R68" t="n">
-        <v>54300</v>
+        <v>55000</v>
       </c>
       <c r="S68" t="n">
         <v>57200</v>
       </c>
       <c r="T68" t="n">
-        <v>-5.1</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="69">
@@ -5007,13 +5007,13 @@
         <v>-1.5</v>
       </c>
       <c r="R69" t="n">
-        <v>21600</v>
+        <v>22800</v>
       </c>
       <c r="S69" t="n">
         <v>21250</v>
       </c>
       <c r="T69" t="n">
-        <v>1.6</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="70">
@@ -5079,13 +5079,13 @@
         <v>-0.1</v>
       </c>
       <c r="R70" t="n">
-        <v>59400</v>
+        <v>60200</v>
       </c>
       <c r="S70" t="n">
         <v>67800</v>
       </c>
       <c r="T70" t="n">
-        <v>-12.4</v>
+        <v>-11.2</v>
       </c>
     </row>
     <row r="71">
@@ -5142,13 +5142,13 @@
         <v>-1.5</v>
       </c>
       <c r="R71" t="n">
-        <v>117200</v>
+        <v>119500</v>
       </c>
       <c r="S71" t="n">
         <v>130600</v>
       </c>
       <c r="T71" t="n">
-        <v>-10.3</v>
+        <v>-8.5</v>
       </c>
     </row>
     <row r="72">
@@ -5205,13 +5205,13 @@
         <v>0</v>
       </c>
       <c r="R72" t="n">
-        <v>83400</v>
+        <v>84500</v>
       </c>
       <c r="S72" t="n">
         <v>89800</v>
       </c>
       <c r="T72" t="n">
-        <v>-7.1</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="73">
@@ -5268,13 +5268,13 @@
         <v>0</v>
       </c>
       <c r="R73" t="n">
-        <v>496000</v>
+        <v>495500</v>
       </c>
       <c r="S73" t="n">
         <v>547000</v>
       </c>
       <c r="T73" t="n">
-        <v>-9.300000000000001</v>
+        <v>-9.4</v>
       </c>
     </row>
     <row r="74">
@@ -5331,13 +5331,13 @@
         <v>0.3</v>
       </c>
       <c r="R74" t="n">
-        <v>1085000</v>
+        <v>1107000</v>
       </c>
       <c r="S74" t="n">
         <v>1160000</v>
       </c>
       <c r="T74" t="n">
-        <v>-6.5</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="75">
@@ -5403,13 +5403,13 @@
         <v>0</v>
       </c>
       <c r="R75" t="n">
-        <v>76800</v>
+        <v>78900</v>
       </c>
       <c r="S75" t="n">
         <v>77700</v>
       </c>
       <c r="T75" t="n">
-        <v>-1.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="76">
@@ -5466,13 +5466,13 @@
         <v>0</v>
       </c>
       <c r="R76" t="n">
-        <v>22200</v>
+        <v>22000</v>
       </c>
       <c r="S76" t="n">
         <v>21600</v>
       </c>
       <c r="T76" t="n">
-        <v>2.8</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="77">
@@ -5538,13 +5538,13 @@
         <v>1.2</v>
       </c>
       <c r="R77" t="n">
-        <v>22950</v>
+        <v>24100</v>
       </c>
       <c r="S77" t="n">
         <v>26050</v>
       </c>
       <c r="T77" t="n">
-        <v>-11.9</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="78">
@@ -5601,13 +5601,13 @@
         <v>-3.3</v>
       </c>
       <c r="R78" t="n">
-        <v>201000</v>
+        <v>203000</v>
       </c>
       <c r="S78" t="n">
         <v>218500</v>
       </c>
       <c r="T78" t="n">
-        <v>-8</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="79">
@@ -5736,13 +5736,13 @@
         <v>-3.7</v>
       </c>
       <c r="R80" t="n">
-        <v>31750</v>
+        <v>31300</v>
       </c>
       <c r="S80" t="n">
         <v>33250</v>
       </c>
       <c r="T80" t="n">
-        <v>-4.5</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="81">
@@ -5808,13 +5808,13 @@
         <v>0</v>
       </c>
       <c r="R81" t="n">
-        <v>92000</v>
+        <v>86200</v>
       </c>
       <c r="S81" t="n">
         <v>93000</v>
       </c>
       <c r="T81" t="n">
-        <v>-1.1</v>
+        <v>-7.3</v>
       </c>
     </row>
     <row r="82">
@@ -5871,13 +5871,13 @@
         <v>0</v>
       </c>
       <c r="R82" t="n">
-        <v>102200</v>
+        <v>103300</v>
       </c>
       <c r="S82" t="n">
         <v>100500</v>
       </c>
       <c r="T82" t="n">
-        <v>1.7</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="83">
@@ -5943,13 +5943,13 @@
         <v>0</v>
       </c>
       <c r="R83" t="n">
-        <v>72200</v>
+        <v>73900</v>
       </c>
       <c r="S83" t="n">
         <v>72500</v>
       </c>
       <c r="T83" t="n">
-        <v>-0.4</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="84">
@@ -6006,13 +6006,13 @@
         <v>-0.2</v>
       </c>
       <c r="R84" t="n">
-        <v>22550</v>
+        <v>22700</v>
       </c>
       <c r="S84" t="n">
         <v>25150</v>
       </c>
       <c r="T84" t="n">
-        <v>-10.3</v>
+        <v>-9.699999999999999</v>
       </c>
     </row>
     <row r="85">
@@ -6069,13 +6069,13 @@
         <v>0</v>
       </c>
       <c r="R85" t="n">
-        <v>228000</v>
+        <v>226000</v>
       </c>
       <c r="S85" t="n">
         <v>243500</v>
       </c>
       <c r="T85" t="n">
-        <v>-6.4</v>
+        <v>-7.2</v>
       </c>
     </row>
     <row r="86">
@@ -6132,13 +6132,13 @@
         <v>0</v>
       </c>
       <c r="R86" t="n">
-        <v>3400</v>
+        <v>3515</v>
       </c>
       <c r="S86" t="n">
         <v>3820</v>
       </c>
       <c r="T86" t="n">
-        <v>-11</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="87">
@@ -6195,13 +6195,13 @@
         <v>0</v>
       </c>
       <c r="R87" t="n">
-        <v>95900</v>
+        <v>97000</v>
       </c>
       <c r="S87" t="n">
         <v>98200</v>
       </c>
       <c r="T87" t="n">
-        <v>-2.3</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="88">
@@ -6267,13 +6267,13 @@
         <v>0</v>
       </c>
       <c r="R88" t="n">
-        <v>20150</v>
+        <v>21250</v>
       </c>
       <c r="S88" t="n">
         <v>23200</v>
       </c>
       <c r="T88" t="n">
-        <v>-13.1</v>
+        <v>-8.4</v>
       </c>
     </row>
     <row r="89">
@@ -6330,13 +6330,13 @@
         <v>0</v>
       </c>
       <c r="R89" t="n">
-        <v>96700</v>
+        <v>95400</v>
       </c>
       <c r="S89" t="n">
         <v>102900</v>
       </c>
       <c r="T89" t="n">
-        <v>-6</v>
+        <v>-7.3</v>
       </c>
     </row>
     <row r="90">
@@ -6402,13 +6402,13 @@
         <v>0.3</v>
       </c>
       <c r="R90" t="n">
-        <v>20000</v>
+        <v>20200</v>
       </c>
       <c r="S90" t="n">
         <v>20400</v>
       </c>
       <c r="T90" t="n">
-        <v>-2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="91">
@@ -6474,13 +6474,13 @@
         <v>0</v>
       </c>
       <c r="R91" t="n">
-        <v>45150</v>
+        <v>44650</v>
       </c>
       <c r="S91" t="n">
         <v>49800</v>
       </c>
       <c r="T91" t="n">
-        <v>-9.300000000000001</v>
+        <v>-10.3</v>
       </c>
     </row>
     <row r="92">
@@ -6537,13 +6537,13 @@
         <v>0</v>
       </c>
       <c r="R92" t="n">
-        <v>395500</v>
+        <v>361500</v>
       </c>
       <c r="S92" t="n">
         <v>369000</v>
       </c>
       <c r="T92" t="n">
-        <v>7.2</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="93">
@@ -6600,13 +6600,13 @@
         <v>-0.4</v>
       </c>
       <c r="R93" t="n">
-        <v>5850</v>
+        <v>6380</v>
       </c>
       <c r="S93" t="n">
         <v>5790</v>
       </c>
       <c r="T93" t="n">
-        <v>1</v>
+        <v>10.2</v>
       </c>
     </row>
     <row r="94">
@@ -6672,13 +6672,13 @@
         <v>0</v>
       </c>
       <c r="R94" t="n">
-        <v>46150</v>
+        <v>46250</v>
       </c>
       <c r="S94" t="n">
         <v>48550</v>
       </c>
       <c r="T94" t="n">
-        <v>-4.9</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="95">
@@ -6735,13 +6735,13 @@
         <v>0</v>
       </c>
       <c r="R95" t="n">
-        <v>18900</v>
+        <v>19090</v>
       </c>
       <c r="S95" t="n">
         <v>18980</v>
       </c>
       <c r="T95" t="n">
-        <v>-0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="96">
@@ -6807,13 +6807,13 @@
         <v>0</v>
       </c>
       <c r="R96" t="n">
-        <v>52400</v>
+        <v>52600</v>
       </c>
       <c r="S96" t="n">
         <v>53400</v>
       </c>
       <c r="T96" t="n">
-        <v>-1.9</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="97">
@@ -6879,13 +6879,13 @@
         <v>0.2</v>
       </c>
       <c r="R97" t="n">
-        <v>107500</v>
+        <v>110800</v>
       </c>
       <c r="S97" t="n">
         <v>111200</v>
       </c>
       <c r="T97" t="n">
-        <v>-3.3</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="98">
@@ -7014,13 +7014,13 @@
         <v>0.5</v>
       </c>
       <c r="R99" t="n">
-        <v>328500</v>
+        <v>287000</v>
       </c>
       <c r="S99" t="n">
         <v>301000</v>
       </c>
       <c r="T99" t="n">
-        <v>9.1</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="100">
@@ -7077,13 +7077,13 @@
         <v>7.3</v>
       </c>
       <c r="R100" t="n">
-        <v>16700</v>
+        <v>17040</v>
       </c>
       <c r="S100" t="n">
         <v>17350</v>
       </c>
       <c r="T100" t="n">
-        <v>-3.7</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="101">
@@ -7149,13 +7149,13 @@
         <v>0</v>
       </c>
       <c r="R101" t="n">
-        <v>172300</v>
+        <v>172600</v>
       </c>
       <c r="S101" t="n">
         <v>176000</v>
       </c>
       <c r="T101" t="n">
-        <v>-2.1</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="102">
@@ -7221,13 +7221,13 @@
         <v>0</v>
       </c>
       <c r="R102" t="n">
-        <v>73300</v>
+        <v>72300</v>
       </c>
       <c r="S102" t="n">
         <v>82600</v>
       </c>
       <c r="T102" t="n">
-        <v>-11.3</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="103">
@@ -7284,13 +7284,13 @@
         <v>0</v>
       </c>
       <c r="R103" t="n">
-        <v>9500</v>
+        <v>9580</v>
       </c>
       <c r="S103" t="n">
         <v>10270</v>
       </c>
       <c r="T103" t="n">
-        <v>-7.5</v>
+        <v>-6.7</v>
       </c>
     </row>
     <row r="104">
@@ -7347,13 +7347,13 @@
         <v>0.2</v>
       </c>
       <c r="R104" t="n">
-        <v>9260</v>
+        <v>9430</v>
       </c>
       <c r="S104" t="n">
         <v>9890</v>
       </c>
       <c r="T104" t="n">
-        <v>-6.4</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="105">
@@ -7419,13 +7419,13 @@
         <v>-1</v>
       </c>
       <c r="R105" t="n">
-        <v>586000</v>
+        <v>544000</v>
       </c>
       <c r="S105" t="n">
         <v>585000</v>
       </c>
       <c r="T105" t="n">
-        <v>0.2</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="106">
@@ -7491,13 +7491,13 @@
         <v>0</v>
       </c>
       <c r="R106" t="n">
-        <v>14310</v>
+        <v>14460</v>
       </c>
       <c r="S106" t="n">
         <v>14590</v>
       </c>
       <c r="T106" t="n">
-        <v>-1.9</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="107">
@@ -7554,13 +7554,13 @@
         <v>0</v>
       </c>
       <c r="R107" t="n">
-        <v>222000</v>
+        <v>223500</v>
       </c>
       <c r="S107" t="n">
         <v>228000</v>
       </c>
       <c r="T107" t="n">
-        <v>-2.6</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="108">
@@ -7626,13 +7626,13 @@
         <v>0</v>
       </c>
       <c r="R108" t="n">
-        <v>35800</v>
+        <v>35750</v>
       </c>
       <c r="S108" t="n">
         <v>40000</v>
       </c>
       <c r="T108" t="n">
-        <v>-10.5</v>
+        <v>-10.6</v>
       </c>
     </row>
     <row r="109">
@@ -7698,13 +7698,13 @@
         <v>0</v>
       </c>
       <c r="R109" t="n">
-        <v>31800</v>
+        <v>32850</v>
       </c>
       <c r="S109" t="n">
         <v>34400</v>
       </c>
       <c r="T109" t="n">
-        <v>-7.6</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="110">
@@ -7770,13 +7770,13 @@
         <v>-1.4</v>
       </c>
       <c r="R110" t="n">
-        <v>38800</v>
+        <v>39550</v>
       </c>
       <c r="S110" t="n">
         <v>41050</v>
       </c>
       <c r="T110" t="n">
-        <v>-5.5</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="111">
@@ -7842,13 +7842,13 @@
         <v>0</v>
       </c>
       <c r="R111" t="n">
-        <v>9020</v>
+        <v>8830</v>
       </c>
       <c r="S111" t="n">
         <v>8760</v>
       </c>
       <c r="T111" t="n">
-        <v>3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="112">
@@ -7905,13 +7905,13 @@
         <v>0</v>
       </c>
       <c r="R112" t="n">
-        <v>35650</v>
+        <v>36350</v>
       </c>
       <c r="S112" t="n">
         <v>36600</v>
       </c>
       <c r="T112" t="n">
-        <v>-2.6</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="113">
@@ -7977,13 +7977,13 @@
         <v>0</v>
       </c>
       <c r="R113" t="n">
-        <v>224500</v>
+        <v>225500</v>
       </c>
       <c r="S113" t="n">
         <v>247500</v>
       </c>
       <c r="T113" t="n">
-        <v>-9.300000000000001</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="114">
@@ -8049,13 +8049,13 @@
         <v>0</v>
       </c>
       <c r="R114" t="n">
-        <v>168600</v>
+        <v>167100</v>
       </c>
       <c r="S114" t="n">
         <v>177800</v>
       </c>
       <c r="T114" t="n">
-        <v>-5.2</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="115">
@@ -8121,13 +8121,13 @@
         <v>10.6</v>
       </c>
       <c r="R115" t="n">
-        <v>404500</v>
+        <v>388500</v>
       </c>
       <c r="S115" t="n">
         <v>404000</v>
       </c>
       <c r="T115" t="n">
-        <v>0.1</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="116">
@@ -8184,13 +8184,13 @@
         <v>0</v>
       </c>
       <c r="R116" t="n">
-        <v>31200</v>
+        <v>32000</v>
       </c>
       <c r="S116" t="n">
         <v>32700</v>
       </c>
       <c r="T116" t="n">
-        <v>-4.6</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="117">
@@ -8229,13 +8229,13 @@
         <v>0</v>
       </c>
       <c r="R117" t="n">
-        <v>19900</v>
+        <v>19290</v>
       </c>
       <c r="S117" t="n">
         <v>23700</v>
       </c>
       <c r="T117" t="n">
-        <v>-16</v>
+        <v>-18.6</v>
       </c>
     </row>
     <row r="118">
@@ -8301,13 +8301,13 @@
         <v>0</v>
       </c>
       <c r="R118" t="n">
-        <v>268000</v>
+        <v>266000</v>
       </c>
       <c r="S118" t="n">
         <v>300500</v>
       </c>
       <c r="T118" t="n">
-        <v>-10.8</v>
+        <v>-11.5</v>
       </c>
     </row>
     <row r="119">
@@ -8352,13 +8352,13 @@
         <v>350</v>
       </c>
       <c r="R119" t="n">
-        <v>11620</v>
+        <v>11200</v>
       </c>
       <c r="S119" t="n">
         <v>12290</v>
       </c>
       <c r="T119" t="n">
-        <v>-5.5</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="120">
@@ -8424,13 +8424,13 @@
         <v>0</v>
       </c>
       <c r="R120" t="n">
-        <v>71300</v>
+        <v>72000</v>
       </c>
       <c r="S120" t="n">
         <v>73400</v>
       </c>
       <c r="T120" t="n">
-        <v>-2.9</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="121">
@@ -8487,13 +8487,13 @@
         <v>0</v>
       </c>
       <c r="R121" t="n">
-        <v>84200</v>
+        <v>83000</v>
       </c>
       <c r="S121" t="n">
         <v>95800</v>
       </c>
       <c r="T121" t="n">
-        <v>-12.1</v>
+        <v>-13.4</v>
       </c>
     </row>
     <row r="122">
@@ -8550,13 +8550,13 @@
         <v>0</v>
       </c>
       <c r="R122" t="n">
-        <v>213500</v>
+        <v>209500</v>
       </c>
       <c r="S122" t="n">
         <v>229000</v>
       </c>
       <c r="T122" t="n">
-        <v>-6.8</v>
+        <v>-8.5</v>
       </c>
     </row>
     <row r="123">
@@ -8613,13 +8613,13 @@
         <v>0</v>
       </c>
       <c r="R123" t="n">
-        <v>15930</v>
+        <v>15640</v>
       </c>
       <c r="S123" t="n">
         <v>18010</v>
       </c>
       <c r="T123" t="n">
-        <v>-11.5</v>
+        <v>-13.2</v>
       </c>
     </row>
     <row r="124">
@@ -8676,13 +8676,13 @@
         <v>0</v>
       </c>
       <c r="R124" t="n">
-        <v>50600</v>
+        <v>53400</v>
       </c>
       <c r="S124" t="n">
         <v>53300</v>
       </c>
       <c r="T124" t="n">
-        <v>-5.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="125">
@@ -8739,13 +8739,13 @@
         <v>0</v>
       </c>
       <c r="R125" t="n">
-        <v>130000</v>
+        <v>129600</v>
       </c>
       <c r="S125" t="n">
         <v>146400</v>
       </c>
       <c r="T125" t="n">
-        <v>-11.2</v>
+        <v>-11.5</v>
       </c>
     </row>
     <row r="126">
@@ -8811,13 +8811,13 @@
         <v>0</v>
       </c>
       <c r="R126" t="n">
-        <v>23350</v>
+        <v>24000</v>
       </c>
       <c r="S126" t="n">
         <v>24850</v>
       </c>
       <c r="T126" t="n">
-        <v>-6</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="127">
@@ -8874,13 +8874,13 @@
         <v>-0.4</v>
       </c>
       <c r="R127" t="n">
-        <v>43800</v>
+        <v>43900</v>
       </c>
       <c r="S127" t="n">
         <v>46350</v>
       </c>
       <c r="T127" t="n">
-        <v>-5.5</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="128">
@@ -8946,13 +8946,13 @@
         <v>0</v>
       </c>
       <c r="R128" t="n">
-        <v>313000</v>
+        <v>317000</v>
       </c>
       <c r="S128" t="n">
         <v>307500</v>
       </c>
       <c r="T128" t="n">
-        <v>1.8</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="129">
@@ -9018,13 +9018,13 @@
         <v>0</v>
       </c>
       <c r="R129" t="n">
-        <v>252500</v>
+        <v>270000</v>
       </c>
       <c r="S129" t="n">
         <v>280500</v>
       </c>
       <c r="T129" t="n">
-        <v>-10</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="130">
@@ -9081,13 +9081,13 @@
         <v>0.8</v>
       </c>
       <c r="R130" t="n">
-        <v>91500</v>
+        <v>89700</v>
       </c>
       <c r="S130" t="n">
         <v>101000</v>
       </c>
       <c r="T130" t="n">
-        <v>-9.4</v>
+        <v>-11.2</v>
       </c>
     </row>
     <row r="131">
@@ -9153,13 +9153,13 @@
         <v>0</v>
       </c>
       <c r="R131" t="n">
-        <v>104100</v>
+        <v>103600</v>
       </c>
       <c r="S131" t="n">
         <v>107400</v>
       </c>
       <c r="T131" t="n">
-        <v>-3.1</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="132">
@@ -9216,13 +9216,13 @@
         <v>-4.3</v>
       </c>
       <c r="R132" t="n">
-        <v>65700</v>
+        <v>64700</v>
       </c>
       <c r="S132" t="n">
         <v>70800</v>
       </c>
       <c r="T132" t="n">
-        <v>-7.2</v>
+        <v>-8.6</v>
       </c>
     </row>
     <row r="133">
@@ -9288,13 +9288,13 @@
         <v>16.6</v>
       </c>
       <c r="R133" t="n">
-        <v>95500</v>
+        <v>93700</v>
       </c>
       <c r="S133" t="n">
         <v>118600</v>
       </c>
       <c r="T133" t="n">
-        <v>-19.5</v>
+        <v>-21</v>
       </c>
     </row>
     <row r="134">
@@ -9360,13 +9360,13 @@
         <v>25</v>
       </c>
       <c r="R134" t="n">
-        <v>38650</v>
+        <v>39500</v>
       </c>
       <c r="S134" t="n">
         <v>41100</v>
       </c>
       <c r="T134" t="n">
-        <v>-6</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="135">
@@ -9432,13 +9432,13 @@
         <v>0</v>
       </c>
       <c r="R135" t="n">
-        <v>164800</v>
+        <v>164900</v>
       </c>
       <c r="S135" t="n">
         <v>182500</v>
       </c>
       <c r="T135" t="n">
-        <v>-9.699999999999999</v>
+        <v>-9.6</v>
       </c>
     </row>
     <row r="136">
@@ -9495,13 +9495,13 @@
         <v>0</v>
       </c>
       <c r="R136" t="n">
-        <v>130100</v>
+        <v>133400</v>
       </c>
       <c r="S136" t="n">
         <v>146900</v>
       </c>
       <c r="T136" t="n">
-        <v>-11.4</v>
+        <v>-9.199999999999999</v>
       </c>
     </row>
     <row r="137">
@@ -9558,13 +9558,13 @@
         <v>0</v>
       </c>
       <c r="R137" t="n">
-        <v>71600</v>
+        <v>71900</v>
       </c>
       <c r="S137" t="n">
         <v>79900</v>
       </c>
       <c r="T137" t="n">
-        <v>-10.4</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="138">
@@ -9630,13 +9630,13 @@
         <v>1.4</v>
       </c>
       <c r="R138" t="n">
-        <v>225500</v>
+        <v>227500</v>
       </c>
       <c r="S138" t="n">
         <v>244000</v>
       </c>
       <c r="T138" t="n">
-        <v>-7.6</v>
+        <v>-6.8</v>
       </c>
     </row>
     <row r="139">
@@ -9693,13 +9693,13 @@
         <v>0</v>
       </c>
       <c r="R139" t="n">
-        <v>26100</v>
+        <v>26450</v>
       </c>
       <c r="S139" t="n">
         <v>28450</v>
       </c>
       <c r="T139" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="140">
@@ -9756,13 +9756,13 @@
         <v>3.1</v>
       </c>
       <c r="R140" t="n">
-        <v>194500</v>
+        <v>199100</v>
       </c>
       <c r="S140" t="n">
         <v>215000</v>
       </c>
       <c r="T140" t="n">
-        <v>-9.5</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="141">
@@ -9819,13 +9819,13 @@
         <v>0</v>
       </c>
       <c r="R141" t="n">
-        <v>104500</v>
+        <v>122500</v>
       </c>
       <c r="S141" t="n">
         <v>109700</v>
       </c>
       <c r="T141" t="n">
-        <v>-4.7</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="142">
@@ -9891,13 +9891,13 @@
         <v>0</v>
       </c>
       <c r="R142" t="n">
-        <v>37650</v>
+        <v>38100</v>
       </c>
       <c r="S142" t="n">
         <v>41500</v>
       </c>
       <c r="T142" t="n">
-        <v>-9.300000000000001</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="143">
@@ -9963,13 +9963,13 @@
         <v>5.3</v>
       </c>
       <c r="R143" t="n">
-        <v>35000</v>
+        <v>34350</v>
       </c>
       <c r="S143" t="n">
         <v>36600</v>
       </c>
       <c r="T143" t="n">
-        <v>-4.4</v>
+        <v>-6.1</v>
       </c>
     </row>
     <row r="144">
@@ -10035,13 +10035,13 @@
         <v>-0.3</v>
       </c>
       <c r="R144" t="n">
-        <v>192300</v>
+        <v>193700</v>
       </c>
       <c r="S144" t="n">
         <v>201000</v>
       </c>
       <c r="T144" t="n">
-        <v>-4.3</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="145">
@@ -10098,13 +10098,13 @@
         <v>0</v>
       </c>
       <c r="R145" t="n">
-        <v>15730</v>
+        <v>15940</v>
       </c>
       <c r="S145" t="n">
         <v>16350</v>
       </c>
       <c r="T145" t="n">
-        <v>-3.8</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="146">
@@ -10161,13 +10161,13 @@
         <v>0</v>
       </c>
       <c r="R146" t="n">
-        <v>119500</v>
+        <v>124500</v>
       </c>
       <c r="S146" t="n">
         <v>124600</v>
       </c>
       <c r="T146" t="n">
-        <v>-4.1</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="147">
@@ -10224,13 +10224,13 @@
         <v>-0.6</v>
       </c>
       <c r="R147" t="n">
-        <v>93400</v>
+        <v>93500</v>
       </c>
       <c r="S147" t="n">
         <v>102200</v>
       </c>
       <c r="T147" t="n">
-        <v>-8.6</v>
+        <v>-8.5</v>
       </c>
     </row>
     <row r="148">
@@ -10296,13 +10296,13 @@
         <v>0.5</v>
       </c>
       <c r="R148" t="n">
-        <v>184500</v>
+        <v>183100</v>
       </c>
       <c r="S148" t="n">
         <v>204000</v>
       </c>
       <c r="T148" t="n">
-        <v>-9.6</v>
+        <v>-10.2</v>
       </c>
     </row>
     <row r="149">
@@ -10359,13 +10359,13 @@
         <v>0</v>
       </c>
       <c r="R149" t="n">
-        <v>72500</v>
+        <v>72600</v>
       </c>
       <c r="S149" t="n">
         <v>76400</v>
       </c>
       <c r="T149" t="n">
-        <v>-5.1</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="150">
@@ -10422,13 +10422,13 @@
         <v>0</v>
       </c>
       <c r="R150" t="n">
-        <v>49700</v>
+        <v>50100</v>
       </c>
       <c r="S150" t="n">
         <v>58200</v>
       </c>
       <c r="T150" t="n">
-        <v>-14.6</v>
+        <v>-13.9</v>
       </c>
     </row>
     <row r="151">
@@ -10485,13 +10485,13 @@
         <v>0</v>
       </c>
       <c r="R151" t="n">
-        <v>7250</v>
+        <v>7160</v>
       </c>
       <c r="S151" t="n">
         <v>8140</v>
       </c>
       <c r="T151" t="n">
-        <v>-10.9</v>
+        <v>-12</v>
       </c>
     </row>
     <row r="152">
@@ -10548,13 +10548,13 @@
         <v>-0.1</v>
       </c>
       <c r="R152" t="n">
-        <v>23450</v>
+        <v>23400</v>
       </c>
       <c r="S152" t="n">
         <v>28400</v>
       </c>
       <c r="T152" t="n">
-        <v>-17.4</v>
+        <v>-17.6</v>
       </c>
     </row>
     <row r="153">
@@ -10611,13 +10611,13 @@
         <v>1.5</v>
       </c>
       <c r="R153" t="n">
-        <v>116200</v>
+        <v>114600</v>
       </c>
       <c r="S153" t="n">
         <v>117000</v>
       </c>
       <c r="T153" t="n">
-        <v>-0.7</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="154">
@@ -10683,13 +10683,13 @@
         <v>0</v>
       </c>
       <c r="R154" t="n">
-        <v>695000</v>
+        <v>712000</v>
       </c>
       <c r="S154" t="n">
         <v>815000</v>
       </c>
       <c r="T154" t="n">
-        <v>-14.7</v>
+        <v>-12.6</v>
       </c>
     </row>
     <row r="155">
@@ -10728,13 +10728,13 @@
         <v>0</v>
       </c>
       <c r="R155" t="n">
-        <v>8730</v>
+        <v>8970</v>
       </c>
       <c r="S155" t="n">
         <v>9200</v>
       </c>
       <c r="T155" t="n">
-        <v>-5.1</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="156">
@@ -10791,13 +10791,13 @@
         <v>1.8</v>
       </c>
       <c r="R156" t="n">
-        <v>41750</v>
+        <v>42150</v>
       </c>
       <c r="S156" t="n">
         <v>42500</v>
       </c>
       <c r="T156" t="n">
-        <v>-1.8</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="157">
@@ -10863,13 +10863,13 @@
         <v>0</v>
       </c>
       <c r="R157" t="n">
-        <v>44100</v>
+        <v>45050</v>
       </c>
       <c r="S157" t="n">
         <v>49050</v>
       </c>
       <c r="T157" t="n">
-        <v>-10.1</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="158">
@@ -10935,13 +10935,13 @@
         <v>15.3</v>
       </c>
       <c r="R158" t="n">
-        <v>56500</v>
+        <v>55900</v>
       </c>
       <c r="S158" t="n">
         <v>61300</v>
       </c>
       <c r="T158" t="n">
-        <v>-7.8</v>
+        <v>-8.800000000000001</v>
       </c>
     </row>
     <row r="159">
@@ -11007,13 +11007,13 @@
         <v>33.3</v>
       </c>
       <c r="R159" t="n">
-        <v>128500</v>
+        <v>136300</v>
       </c>
       <c r="S159" t="n">
         <v>131100</v>
       </c>
       <c r="T159" t="n">
-        <v>-2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="160">
@@ -11070,13 +11070,13 @@
         <v>-0.8</v>
       </c>
       <c r="R160" t="n">
-        <v>196700</v>
+        <v>198600</v>
       </c>
       <c r="S160" t="n">
         <v>211000</v>
       </c>
       <c r="T160" t="n">
-        <v>-6.8</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="161">
@@ -11142,13 +11142,13 @@
         <v>0</v>
       </c>
       <c r="R161" t="n">
-        <v>128800</v>
+        <v>127900</v>
       </c>
       <c r="S161" t="n">
         <v>133000</v>
       </c>
       <c r="T161" t="n">
-        <v>-3.2</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="162">
@@ -11205,13 +11205,13 @@
         <v>-0.6</v>
       </c>
       <c r="R162" t="n">
-        <v>5470</v>
+        <v>5230</v>
       </c>
       <c r="S162" t="n">
         <v>5630</v>
       </c>
       <c r="T162" t="n">
-        <v>-2.8</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="163">
@@ -11250,13 +11250,13 @@
         <v>0</v>
       </c>
       <c r="R163" t="n">
-        <v>48400</v>
+        <v>46650</v>
       </c>
       <c r="S163" t="n">
         <v>49250</v>
       </c>
       <c r="T163" t="n">
-        <v>-1.7</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="164">
@@ -11322,13 +11322,13 @@
         <v>0</v>
       </c>
       <c r="R164" t="n">
-        <v>45900</v>
+        <v>46100</v>
       </c>
       <c r="S164" t="n">
         <v>45000</v>
       </c>
       <c r="T164" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="165">
@@ -11385,13 +11385,13 @@
         <v>0.6</v>
       </c>
       <c r="R165" t="n">
-        <v>58100</v>
+        <v>58400</v>
       </c>
       <c r="S165" t="n">
         <v>68200</v>
       </c>
       <c r="T165" t="n">
-        <v>-14.8</v>
+        <v>-14.4</v>
       </c>
     </row>
     <row r="166">
@@ -11457,13 +11457,13 @@
         <v>0</v>
       </c>
       <c r="R166" t="n">
-        <v>138000</v>
+        <v>139100</v>
       </c>
       <c r="S166" t="n">
         <v>135700</v>
       </c>
       <c r="T166" t="n">
-        <v>1.7</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="167">
@@ -11529,13 +11529,13 @@
         <v>0</v>
       </c>
       <c r="R167" t="n">
-        <v>154300</v>
+        <v>153400</v>
       </c>
       <c r="S167" t="n">
         <v>161300</v>
       </c>
       <c r="T167" t="n">
-        <v>-4.3</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="168">
@@ -11592,13 +11592,13 @@
         <v>-2.9</v>
       </c>
       <c r="R168" t="n">
-        <v>132900</v>
+        <v>133500</v>
       </c>
       <c r="S168" t="n">
         <v>147500</v>
       </c>
       <c r="T168" t="n">
-        <v>-9.9</v>
+        <v>-9.5</v>
       </c>
     </row>
     <row r="169">
@@ -11664,13 +11664,13 @@
         <v>2.4</v>
       </c>
       <c r="R169" t="n">
-        <v>17790</v>
+        <v>18200</v>
       </c>
       <c r="S169" t="n">
         <v>19100</v>
       </c>
       <c r="T169" t="n">
-        <v>-6.9</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="170">
@@ -11736,13 +11736,13 @@
         <v>0</v>
       </c>
       <c r="R170" t="n">
-        <v>30500</v>
+        <v>32050</v>
       </c>
       <c r="S170" t="n">
         <v>32150</v>
       </c>
       <c r="T170" t="n">
-        <v>-5.1</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="171">
@@ -11808,13 +11808,13 @@
         <v>0</v>
       </c>
       <c r="R171" t="n">
-        <v>124800</v>
+        <v>129100</v>
       </c>
       <c r="S171" t="n">
         <v>128700</v>
       </c>
       <c r="T171" t="n">
-        <v>-3</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="172">
@@ -11871,13 +11871,13 @@
         <v>0</v>
       </c>
       <c r="R172" t="n">
-        <v>184000</v>
+        <v>189800</v>
       </c>
       <c r="S172" t="n">
         <v>185400</v>
       </c>
       <c r="T172" t="n">
-        <v>-0.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="173">
@@ -11916,13 +11916,13 @@
         <v>0</v>
       </c>
       <c r="R173" t="n">
-        <v>28300</v>
+        <v>27200</v>
       </c>
       <c r="S173" t="n">
         <v>32350</v>
       </c>
       <c r="T173" t="n">
-        <v>-12.5</v>
+        <v>-15.9</v>
       </c>
     </row>
     <row r="174">
@@ -11988,13 +11988,13 @@
         <v>0</v>
       </c>
       <c r="R174" t="n">
-        <v>17500</v>
+        <v>17900</v>
       </c>
       <c r="S174" t="n">
         <v>18460</v>
       </c>
       <c r="T174" t="n">
-        <v>-5.2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="175">
@@ -12051,13 +12051,13 @@
         <v>0</v>
       </c>
       <c r="R175" t="n">
-        <v>69400</v>
+        <v>70500</v>
       </c>
       <c r="S175" t="n">
         <v>81400</v>
       </c>
       <c r="T175" t="n">
-        <v>-14.7</v>
+        <v>-13.4</v>
       </c>
     </row>
     <row r="176">
@@ -12123,13 +12123,13 @@
         <v>0</v>
       </c>
       <c r="R176" t="n">
-        <v>77800</v>
+        <v>81900</v>
       </c>
       <c r="S176" t="n">
         <v>82000</v>
       </c>
       <c r="T176" t="n">
-        <v>-5.1</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="177">
@@ -12195,13 +12195,13 @@
         <v>0</v>
       </c>
       <c r="R177" t="n">
-        <v>164300</v>
+        <v>162500</v>
       </c>
       <c r="S177" t="n">
         <v>168500</v>
       </c>
       <c r="T177" t="n">
-        <v>-2.5</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="178">
@@ -12267,13 +12267,13 @@
         <v>-7</v>
       </c>
       <c r="R178" t="n">
-        <v>254000</v>
+        <v>245500</v>
       </c>
       <c r="S178" t="n">
         <v>280000</v>
       </c>
       <c r="T178" t="n">
-        <v>-9.300000000000001</v>
+        <v>-12.3</v>
       </c>
     </row>
     <row r="179">
@@ -12339,13 +12339,13 @@
         <v>-0.1</v>
       </c>
       <c r="R179" t="n">
-        <v>74700</v>
+        <v>75400</v>
       </c>
       <c r="S179" t="n">
         <v>85900</v>
       </c>
       <c r="T179" t="n">
-        <v>-13</v>
+        <v>-12.2</v>
       </c>
     </row>
     <row r="180">
@@ -12402,13 +12402,13 @@
         <v>0</v>
       </c>
       <c r="R180" t="n">
-        <v>46550</v>
+        <v>46900</v>
       </c>
       <c r="S180" t="n">
         <v>46850</v>
       </c>
       <c r="T180" t="n">
-        <v>-0.6</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="181">
@@ -12465,13 +12465,13 @@
         <v>3.4</v>
       </c>
       <c r="R181" t="n">
-        <v>49650</v>
+        <v>50000</v>
       </c>
       <c r="S181" t="n">
         <v>55300</v>
       </c>
       <c r="T181" t="n">
-        <v>-10.2</v>
+        <v>-9.6</v>
       </c>
     </row>
     <row r="182">
@@ -12537,13 +12537,13 @@
         <v>0</v>
       </c>
       <c r="R182" t="n">
-        <v>39100</v>
+        <v>39350</v>
       </c>
       <c r="S182" t="n">
         <v>41050</v>
       </c>
       <c r="T182" t="n">
-        <v>-4.8</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="183">
@@ -12609,13 +12609,13 @@
         <v>0</v>
       </c>
       <c r="R183" t="n">
-        <v>415500</v>
+        <v>540000</v>
       </c>
       <c r="S183" t="n">
         <v>398500</v>
       </c>
       <c r="T183" t="n">
-        <v>4.3</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="184">
@@ -12681,13 +12681,13 @@
         <v>15.1</v>
       </c>
       <c r="R184" t="n">
-        <v>222000</v>
+        <v>245500</v>
       </c>
       <c r="S184" t="n">
         <v>260000</v>
       </c>
       <c r="T184" t="n">
-        <v>-14.6</v>
+        <v>-5.6</v>
       </c>
     </row>
     <row r="185">
@@ -12753,13 +12753,13 @@
         <v>0</v>
       </c>
       <c r="R185" t="n">
-        <v>115400</v>
+        <v>114800</v>
       </c>
       <c r="S185" t="n">
         <v>116700</v>
       </c>
       <c r="T185" t="n">
-        <v>-1.1</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="186">
@@ -12825,13 +12825,13 @@
         <v>0</v>
       </c>
       <c r="R186" t="n">
-        <v>14310</v>
+        <v>14300</v>
       </c>
       <c r="S186" t="n">
         <v>15130</v>
       </c>
       <c r="T186" t="n">
-        <v>-5.4</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="187">
@@ -12897,13 +12897,13 @@
         <v>0.5</v>
       </c>
       <c r="R187" t="n">
-        <v>17180</v>
+        <v>17100</v>
       </c>
       <c r="S187" t="n">
         <v>17470</v>
       </c>
       <c r="T187" t="n">
-        <v>-1.7</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="188">
@@ -12969,13 +12969,13 @@
         <v>-0.4</v>
       </c>
       <c r="R188" t="n">
-        <v>71900</v>
+        <v>72600</v>
       </c>
       <c r="S188" t="n">
         <v>78900</v>
       </c>
       <c r="T188" t="n">
-        <v>-8.9</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="189">
@@ -13041,13 +13041,13 @@
         <v>-8</v>
       </c>
       <c r="R189" t="n">
-        <v>259500</v>
+        <v>265500</v>
       </c>
       <c r="S189" t="n">
         <v>279500</v>
       </c>
       <c r="T189" t="n">
-        <v>-7.2</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="190">
@@ -13104,13 +13104,13 @@
         <v>0</v>
       </c>
       <c r="R190" t="n">
-        <v>100000</v>
+        <v>102500</v>
       </c>
       <c r="S190" t="n">
         <v>113900</v>
       </c>
       <c r="T190" t="n">
-        <v>-12.2</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="191">
@@ -13176,13 +13176,13 @@
         <v>-0</v>
       </c>
       <c r="R191" t="n">
-        <v>245000</v>
+        <v>252000</v>
       </c>
       <c r="S191" t="n">
         <v>256000</v>
       </c>
       <c r="T191" t="n">
-        <v>-4.3</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="192">
@@ -13239,13 +13239,13 @@
         <v>-6.2</v>
       </c>
       <c r="R192" t="n">
-        <v>36350</v>
+        <v>36850</v>
       </c>
       <c r="S192" t="n">
         <v>40700</v>
       </c>
       <c r="T192" t="n">
-        <v>-10.7</v>
+        <v>-9.5</v>
       </c>
     </row>
     <row r="193">
@@ -13284,13 +13284,13 @@
         <v>0</v>
       </c>
       <c r="R193" t="n">
-        <v>9680</v>
+        <v>9620</v>
       </c>
       <c r="S193" t="n">
         <v>10180</v>
       </c>
       <c r="T193" t="n">
-        <v>-4.9</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="194">
@@ -13347,13 +13347,13 @@
         <v>0</v>
       </c>
       <c r="R194" t="n">
-        <v>66000</v>
+        <v>66400</v>
       </c>
       <c r="S194" t="n">
         <v>71600</v>
       </c>
       <c r="T194" t="n">
-        <v>-7.8</v>
+        <v>-7.3</v>
       </c>
     </row>
     <row r="195">
@@ -13419,13 +13419,13 @@
         <v>0</v>
       </c>
       <c r="R195" t="n">
-        <v>136700</v>
+        <v>143300</v>
       </c>
       <c r="S195" t="n">
         <v>136700</v>
       </c>
       <c r="T195" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="196">
@@ -13491,13 +13491,13 @@
         <v>0</v>
       </c>
       <c r="R196" t="n">
-        <v>37050</v>
+        <v>37750</v>
       </c>
       <c r="S196" t="n">
         <v>38500</v>
       </c>
       <c r="T196" t="n">
-        <v>-3.8</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="197">
@@ -13563,13 +13563,13 @@
         <v>0.1</v>
       </c>
       <c r="R197" t="n">
-        <v>26600</v>
+        <v>27250</v>
       </c>
       <c r="S197" t="n">
         <v>28000</v>
       </c>
       <c r="T197" t="n">
-        <v>-5</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="198">
@@ -13629,13 +13629,13 @@
         <v>4450</v>
       </c>
       <c r="R198" t="n">
-        <v>36250</v>
+        <v>38200</v>
       </c>
       <c r="S198" t="n">
         <v>36950</v>
       </c>
       <c r="T198" t="n">
-        <v>-1.9</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="199">
@@ -13701,13 +13701,13 @@
         <v>0</v>
       </c>
       <c r="R199" t="n">
-        <v>66900</v>
+        <v>68800</v>
       </c>
       <c r="S199" t="n">
         <v>68300</v>
       </c>
       <c r="T199" t="n">
-        <v>-2</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="200">
@@ -13773,13 +13773,13 @@
         <v>3.9</v>
       </c>
       <c r="R200" t="n">
-        <v>62900</v>
+        <v>65600</v>
       </c>
       <c r="S200" t="n">
         <v>79000</v>
       </c>
       <c r="T200" t="n">
-        <v>-20.4</v>
+        <v>-17</v>
       </c>
     </row>
     <row r="201">
@@ -13836,13 +13836,13 @@
         <v>0</v>
       </c>
       <c r="R201" t="n">
-        <v>59400</v>
+        <v>58700</v>
       </c>
       <c r="S201" t="n">
         <v>61600</v>
       </c>
       <c r="T201" t="n">
-        <v>-3.6</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="202">
@@ -13899,13 +13899,13 @@
         <v>0</v>
       </c>
       <c r="R202" t="n">
-        <v>271000</v>
+        <v>287000</v>
       </c>
       <c r="S202" t="n">
         <v>247500</v>
       </c>
       <c r="T202" t="n">
-        <v>9.5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="203">
@@ -13971,13 +13971,13 @@
         <v>0</v>
       </c>
       <c r="R203" t="n">
-        <v>41000</v>
+        <v>44150</v>
       </c>
       <c r="S203" t="n">
         <v>41650</v>
       </c>
       <c r="T203" t="n">
-        <v>-1.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="204">
@@ -14043,13 +14043,13 @@
         <v>0</v>
       </c>
       <c r="R204" t="n">
-        <v>320000</v>
+        <v>320500</v>
       </c>
       <c r="S204" t="n">
         <v>314000</v>
       </c>
       <c r="T204" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="205">
@@ -14106,13 +14106,13 @@
         <v>0</v>
       </c>
       <c r="R205" t="n">
-        <v>51500</v>
+        <v>50900</v>
       </c>
       <c r="S205" t="n">
         <v>57100</v>
       </c>
       <c r="T205" t="n">
-        <v>-9.800000000000001</v>
+        <v>-10.9</v>
       </c>
     </row>
     <row r="206">
@@ -14169,13 +14169,13 @@
         <v>0</v>
       </c>
       <c r="R206" t="n">
-        <v>1551000</v>
+        <v>1567000</v>
       </c>
       <c r="S206" t="n">
         <v>1548000</v>
       </c>
       <c r="T206" t="n">
-        <v>0.2</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="207">
@@ -14241,13 +14241,13 @@
         <v>-1.2</v>
       </c>
       <c r="R207" t="n">
-        <v>32150</v>
+        <v>33300</v>
       </c>
       <c r="S207" t="n">
         <v>37500</v>
       </c>
       <c r="T207" t="n">
-        <v>-14.3</v>
+        <v>-11.2</v>
       </c>
     </row>
     <row r="208">
@@ -14313,13 +14313,13 @@
         <v>0.7</v>
       </c>
       <c r="R208" t="n">
-        <v>400500</v>
+        <v>416000</v>
       </c>
       <c r="S208" t="n">
         <v>398000</v>
       </c>
       <c r="T208" t="n">
-        <v>0.6</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="209">
@@ -14376,13 +14376,13 @@
         <v>0</v>
       </c>
       <c r="R209" t="n">
-        <v>47150</v>
+        <v>46350</v>
       </c>
       <c r="S209" t="n">
         <v>53200</v>
       </c>
       <c r="T209" t="n">
-        <v>-11.4</v>
+        <v>-12.9</v>
       </c>
     </row>
     <row r="210">
@@ -14439,13 +14439,13 @@
         <v>0</v>
       </c>
       <c r="R210" t="n">
-        <v>99700</v>
+        <v>105500</v>
       </c>
       <c r="S210" t="n">
         <v>108700</v>
       </c>
       <c r="T210" t="n">
-        <v>-8.300000000000001</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="211">
@@ -14511,13 +14511,13 @@
         <v>-0.6</v>
       </c>
       <c r="R211" t="n">
-        <v>99700</v>
+        <v>110700</v>
       </c>
       <c r="S211" t="n">
         <v>106400</v>
       </c>
       <c r="T211" t="n">
-        <v>-6.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="212">
@@ -14583,13 +14583,13 @@
         <v>0</v>
       </c>
       <c r="R212" t="n">
-        <v>107900</v>
+        <v>106800</v>
       </c>
       <c r="S212" t="n">
         <v>116600</v>
       </c>
       <c r="T212" t="n">
-        <v>-7.5</v>
+        <v>-8.4</v>
       </c>
     </row>
     <row r="213">
@@ -14646,13 +14646,13 @@
         <v>0</v>
       </c>
       <c r="R213" t="n">
-        <v>57900</v>
+        <v>60000</v>
       </c>
       <c r="S213" t="n">
         <v>66100</v>
       </c>
       <c r="T213" t="n">
-        <v>-12.4</v>
+        <v>-9.199999999999999</v>
       </c>
     </row>
     <row r="214">
@@ -14718,13 +14718,13 @@
         <v>1.8</v>
       </c>
       <c r="R214" t="n">
-        <v>137300</v>
+        <v>139900</v>
       </c>
       <c r="S214" t="n">
         <v>127200</v>
       </c>
       <c r="T214" t="n">
-        <v>7.9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="215">
@@ -14790,13 +14790,13 @@
         <v>-10.6</v>
       </c>
       <c r="R215" t="n">
-        <v>105600</v>
+        <v>117000</v>
       </c>
       <c r="S215" t="n">
         <v>116700</v>
       </c>
       <c r="T215" t="n">
-        <v>-9.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="216">
@@ -14862,13 +14862,13 @@
         <v>0</v>
       </c>
       <c r="R216" t="n">
-        <v>37050</v>
+        <v>37750</v>
       </c>
       <c r="S216" t="n">
         <v>39100</v>
       </c>
       <c r="T216" t="n">
-        <v>-5.2</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="217">
@@ -14934,13 +14934,13 @@
         <v>0.5</v>
       </c>
       <c r="R217" t="n">
-        <v>59800</v>
+        <v>63000</v>
       </c>
       <c r="S217" t="n">
         <v>53000</v>
       </c>
       <c r="T217" t="n">
-        <v>12.8</v>
+        <v>18.9</v>
       </c>
     </row>
     <row r="218">
@@ -15006,13 +15006,13 @@
         <v>0</v>
       </c>
       <c r="R218" t="n">
-        <v>21150</v>
+        <v>21450</v>
       </c>
       <c r="S218" t="n">
         <v>23600</v>
       </c>
       <c r="T218" t="n">
-        <v>-10.4</v>
+        <v>-9.1</v>
       </c>
     </row>
     <row r="219">
@@ -15078,13 +15078,13 @@
         <v>0.4</v>
       </c>
       <c r="R219" t="n">
-        <v>47650</v>
+        <v>49450</v>
       </c>
       <c r="S219" t="n">
         <v>42850</v>
       </c>
       <c r="T219" t="n">
-        <v>11.2</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="220">
@@ -15150,13 +15150,13 @@
         <v>0</v>
       </c>
       <c r="R220" t="n">
-        <v>222000</v>
+        <v>223500</v>
       </c>
       <c r="S220" t="n">
         <v>238000</v>
       </c>
       <c r="T220" t="n">
-        <v>-6.7</v>
+        <v>-6.1</v>
       </c>
     </row>
     <row r="221">
@@ -15222,13 +15222,13 @@
         <v>0</v>
       </c>
       <c r="R221" t="n">
-        <v>32200</v>
+        <v>32050</v>
       </c>
       <c r="S221" t="n">
         <v>31250</v>
       </c>
       <c r="T221" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="222">
@@ -15294,13 +15294,13 @@
         <v>2.2</v>
       </c>
       <c r="R222" t="n">
-        <v>213000</v>
+        <v>210500</v>
       </c>
       <c r="S222" t="n">
         <v>235500</v>
       </c>
       <c r="T222" t="n">
-        <v>-9.6</v>
+        <v>-10.6</v>
       </c>
     </row>
     <row r="223">
@@ -15357,13 +15357,13 @@
         <v>0</v>
       </c>
       <c r="R223" t="n">
-        <v>718000</v>
+        <v>716000</v>
       </c>
       <c r="S223" t="n">
         <v>803000</v>
       </c>
       <c r="T223" t="n">
-        <v>-10.6</v>
+        <v>-10.8</v>
       </c>
     </row>
     <row r="224">
@@ -15420,13 +15420,13 @@
         <v>0</v>
       </c>
       <c r="R224" t="n">
-        <v>115500</v>
+        <v>126900</v>
       </c>
       <c r="S224" t="n">
         <v>138600</v>
       </c>
       <c r="T224" t="n">
-        <v>-16.7</v>
+        <v>-8.4</v>
       </c>
     </row>
     <row r="225">
@@ -15483,13 +15483,13 @@
         <v>-0.2</v>
       </c>
       <c r="R225" t="n">
-        <v>125400</v>
+        <v>128000</v>
       </c>
       <c r="S225" t="n">
         <v>134000</v>
       </c>
       <c r="T225" t="n">
-        <v>-6.4</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="226">
@@ -15546,13 +15546,13 @@
         <v>-1.6</v>
       </c>
       <c r="R226" t="n">
-        <v>70300</v>
+        <v>69300</v>
       </c>
       <c r="S226" t="n">
         <v>80300</v>
       </c>
       <c r="T226" t="n">
-        <v>-12.5</v>
+        <v>-13.7</v>
       </c>
     </row>
     <row r="227">
@@ -15609,13 +15609,13 @@
         <v>-1.9</v>
       </c>
       <c r="R227" t="n">
-        <v>5170</v>
+        <v>5720</v>
       </c>
       <c r="S227" t="n">
         <v>5320</v>
       </c>
       <c r="T227" t="n">
-        <v>-2.8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="228">
@@ -15672,13 +15672,13 @@
         <v>254.1</v>
       </c>
       <c r="R228" t="n">
-        <v>454000</v>
+        <v>443000</v>
       </c>
       <c r="S228" t="n">
         <v>501000</v>
       </c>
       <c r="T228" t="n">
-        <v>-9.4</v>
+        <v>-11.6</v>
       </c>
     </row>
     <row r="229">
@@ -15744,13 +15744,13 @@
         <v>0</v>
       </c>
       <c r="R229" t="n">
-        <v>385000</v>
+        <v>407000</v>
       </c>
       <c r="S229" t="n">
         <v>390500</v>
       </c>
       <c r="T229" t="n">
-        <v>-1.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="230">
@@ -15807,13 +15807,13 @@
         <v>0.2</v>
       </c>
       <c r="R230" t="n">
-        <v>128300</v>
+        <v>130700</v>
       </c>
       <c r="S230" t="n">
         <v>129300</v>
       </c>
       <c r="T230" t="n">
-        <v>-0.8</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="231">
@@ -15870,13 +15870,13 @@
         <v>-0.2</v>
       </c>
       <c r="R231" t="n">
-        <v>141400</v>
+        <v>145600</v>
       </c>
       <c r="S231" t="n">
         <v>145200</v>
       </c>
       <c r="T231" t="n">
-        <v>-2.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="232">
@@ -15933,13 +15933,13 @@
         <v>0</v>
       </c>
       <c r="R232" t="n">
-        <v>49600</v>
+        <v>50000</v>
       </c>
       <c r="S232" t="n">
         <v>50000</v>
       </c>
       <c r="T232" t="n">
-        <v>-0.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="233">
@@ -16005,13 +16005,13 @@
         <v>0</v>
       </c>
       <c r="R233" t="n">
-        <v>21600</v>
+        <v>22000</v>
       </c>
       <c r="S233" t="n">
         <v>22100</v>
       </c>
       <c r="T233" t="n">
-        <v>-2.3</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="234">
@@ -16068,13 +16068,13 @@
         <v>0</v>
       </c>
       <c r="R234" t="n">
-        <v>312000</v>
+        <v>314000</v>
       </c>
       <c r="S234" t="n">
         <v>330500</v>
       </c>
       <c r="T234" t="n">
-        <v>-5.6</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="235">
@@ -16131,13 +16131,13 @@
         <v>0</v>
       </c>
       <c r="R235" t="n">
-        <v>2721000</v>
+        <v>2770000</v>
       </c>
       <c r="S235" t="n">
         <v>2954000</v>
       </c>
       <c r="T235" t="n">
-        <v>-7.9</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="236">
@@ -16203,13 +16203,13 @@
         <v>0</v>
       </c>
       <c r="R236" t="n">
-        <v>160600</v>
+        <v>165900</v>
       </c>
       <c r="S236" t="n">
         <v>177700</v>
       </c>
       <c r="T236" t="n">
-        <v>-9.6</v>
+        <v>-6.6</v>
       </c>
     </row>
     <row r="237">
@@ -16266,13 +16266,13 @@
         <v>0</v>
       </c>
       <c r="R237" t="n">
-        <v>75200</v>
+        <v>75600</v>
       </c>
       <c r="S237" t="n">
         <v>84100</v>
       </c>
       <c r="T237" t="n">
-        <v>-10.6</v>
+        <v>-10.1</v>
       </c>
     </row>
     <row r="238">
@@ -16329,13 +16329,13 @@
         <v>4.8</v>
       </c>
       <c r="R238" t="n">
-        <v>15520</v>
+        <v>16220</v>
       </c>
       <c r="S238" t="n">
         <v>14900</v>
       </c>
       <c r="T238" t="n">
-        <v>4.2</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="239">
@@ -16392,13 +16392,13 @@
         <v>-26.3</v>
       </c>
       <c r="R239" t="n">
-        <v>36500</v>
+        <v>38200</v>
       </c>
       <c r="S239" t="n">
         <v>37650</v>
       </c>
       <c r="T239" t="n">
-        <v>-3.1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="240">
@@ -16464,13 +16464,13 @@
         <v>4.6</v>
       </c>
       <c r="R240" t="n">
-        <v>138500</v>
+        <v>137800</v>
       </c>
       <c r="S240" t="n">
         <v>132800</v>
       </c>
       <c r="T240" t="n">
-        <v>4.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="241">
@@ -16527,13 +16527,13 @@
         <v>0</v>
       </c>
       <c r="R241" t="n">
-        <v>448000</v>
+        <v>458000</v>
       </c>
       <c r="S241" t="n">
         <v>489500</v>
       </c>
       <c r="T241" t="n">
-        <v>-8.5</v>
+        <v>-6.4</v>
       </c>
     </row>
     <row r="242">
@@ -16599,13 +16599,13 @@
         <v>0</v>
       </c>
       <c r="R242" t="n">
-        <v>31750</v>
+        <v>31850</v>
       </c>
       <c r="S242" t="n">
         <v>33700</v>
       </c>
       <c r="T242" t="n">
-        <v>-5.8</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="243">
@@ -16662,13 +16662,13 @@
         <v>0</v>
       </c>
       <c r="R243" t="n">
-        <v>10020</v>
+        <v>10260</v>
       </c>
       <c r="S243" t="n">
         <v>10030</v>
       </c>
       <c r="T243" t="n">
-        <v>-0.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="244">
@@ -16734,13 +16734,13 @@
         <v>-3.4</v>
       </c>
       <c r="R244" t="n">
-        <v>122200</v>
+        <v>125800</v>
       </c>
       <c r="S244" t="n">
         <v>134100</v>
       </c>
       <c r="T244" t="n">
-        <v>-8.9</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="245">
@@ -16806,13 +16806,13 @@
         <v>0</v>
       </c>
       <c r="R245" t="n">
-        <v>21300</v>
+        <v>21550</v>
       </c>
       <c r="S245" t="n">
         <v>22200</v>
       </c>
       <c r="T245" t="n">
-        <v>-4.1</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="246">
@@ -16869,13 +16869,13 @@
         <v>1.1</v>
       </c>
       <c r="R246" t="n">
-        <v>83700</v>
+        <v>86000</v>
       </c>
       <c r="S246" t="n">
         <v>87300</v>
       </c>
       <c r="T246" t="n">
-        <v>-4.1</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="247">
@@ -16932,13 +16932,13 @@
         <v>0.4</v>
       </c>
       <c r="R247" t="n">
-        <v>453000</v>
+        <v>455000</v>
       </c>
       <c r="S247" t="n">
         <v>510000</v>
       </c>
       <c r="T247" t="n">
-        <v>-11.2</v>
+        <v>-10.8</v>
       </c>
     </row>
     <row r="248">
@@ -17004,13 +17004,13 @@
         <v>0</v>
       </c>
       <c r="R248" t="n">
-        <v>167900</v>
+        <v>174400</v>
       </c>
       <c r="S248" t="n">
         <v>179400</v>
       </c>
       <c r="T248" t="n">
-        <v>-6.4</v>
+        <v>-2.8</v>
       </c>
     </row>
     <row r="249">
@@ -17067,13 +17067,13 @@
         <v>0</v>
       </c>
       <c r="R249" t="n">
-        <v>104300</v>
+        <v>104500</v>
       </c>
       <c r="S249" t="n">
         <v>119100</v>
       </c>
       <c r="T249" t="n">
-        <v>-12.4</v>
+        <v>-12.3</v>
       </c>
     </row>
     <row r="250">
@@ -17139,13 +17139,13 @@
         <v>1.1</v>
       </c>
       <c r="R250" t="n">
-        <v>326000</v>
+        <v>330500</v>
       </c>
       <c r="S250" t="n">
         <v>322000</v>
       </c>
       <c r="T250" t="n">
-        <v>1.2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="251">
@@ -17202,13 +17202,13 @@
         <v>-4450</v>
       </c>
       <c r="R251" t="n">
-        <v>13950</v>
+        <v>15340</v>
       </c>
       <c r="S251" t="n">
         <v>15550</v>
       </c>
       <c r="T251" t="n">
-        <v>-10.3</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="252">
@@ -17265,13 +17265,13 @@
         <v>0</v>
       </c>
       <c r="R252" t="n">
-        <v>343500</v>
+        <v>361000</v>
       </c>
       <c r="S252" t="n">
         <v>369500</v>
       </c>
       <c r="T252" t="n">
-        <v>-7</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="253">
@@ -17337,13 +17337,13 @@
         <v>0</v>
       </c>
       <c r="R253" t="n">
-        <v>68200</v>
+        <v>68300</v>
       </c>
       <c r="S253" t="n">
         <v>73800</v>
       </c>
       <c r="T253" t="n">
-        <v>-7.6</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="254">
@@ -17409,13 +17409,13 @@
         <v>-1.5</v>
       </c>
       <c r="R254" t="n">
-        <v>18170</v>
+        <v>18340</v>
       </c>
       <c r="S254" t="n">
         <v>19800</v>
       </c>
       <c r="T254" t="n">
-        <v>-8.199999999999999</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="255">
@@ -17481,13 +17481,13 @@
         <v>0</v>
       </c>
       <c r="R255" t="n">
-        <v>42500</v>
+        <v>44800</v>
       </c>
       <c r="S255" t="n">
         <v>45150</v>
       </c>
       <c r="T255" t="n">
-        <v>-5.9</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="256">
@@ -17553,13 +17553,13 @@
         <v>0</v>
       </c>
       <c r="R256" t="n">
-        <v>62200</v>
+        <v>63100</v>
       </c>
       <c r="S256" t="n">
         <v>67000</v>
       </c>
       <c r="T256" t="n">
-        <v>-7.2</v>
+        <v>-5.8</v>
       </c>
     </row>
     <row r="257">
@@ -17598,13 +17598,13 @@
         <v>0</v>
       </c>
       <c r="R257" t="n">
-        <v>35500</v>
+        <v>36700</v>
       </c>
       <c r="S257" t="n">
         <v>41100</v>
       </c>
       <c r="T257" t="n">
-        <v>-13.6</v>
+        <v>-10.7</v>
       </c>
     </row>
     <row r="258">
@@ -17661,13 +17661,13 @@
         <v>0.7</v>
       </c>
       <c r="R258" t="n">
-        <v>1123000</v>
+        <v>1068000</v>
       </c>
       <c r="S258" t="n">
         <v>1154000</v>
       </c>
       <c r="T258" t="n">
-        <v>-2.7</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="259">
@@ -17706,13 +17706,13 @@
         <v>0</v>
       </c>
       <c r="R259" t="n">
-        <v>44900</v>
+        <v>44000</v>
       </c>
       <c r="S259" t="n">
         <v>40400</v>
       </c>
       <c r="T259" t="n">
-        <v>11.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="260">
@@ -17778,13 +17778,13 @@
         <v>5.1</v>
       </c>
       <c r="R260" t="n">
-        <v>105300</v>
+        <v>104700</v>
       </c>
       <c r="S260" t="n">
         <v>120100</v>
       </c>
       <c r="T260" t="n">
-        <v>-12.3</v>
+        <v>-12.8</v>
       </c>
     </row>
     <row r="261">
@@ -17841,13 +17841,13 @@
         <v>0</v>
       </c>
       <c r="R261" t="n">
-        <v>49050</v>
+        <v>48750</v>
       </c>
       <c r="S261" t="n">
         <v>54700</v>
       </c>
       <c r="T261" t="n">
-        <v>-10.3</v>
+        <v>-10.9</v>
       </c>
     </row>
     <row r="262">
@@ -17904,13 +17904,13 @@
         <v>9.800000000000001</v>
       </c>
       <c r="R262" t="n">
-        <v>61900</v>
+        <v>61700</v>
       </c>
       <c r="S262" t="n">
         <v>65500</v>
       </c>
       <c r="T262" t="n">
-        <v>-5.5</v>
+        <v>-5.8</v>
       </c>
     </row>
     <row r="263">
@@ -17967,13 +17967,13 @@
         <v>0</v>
       </c>
       <c r="R263" t="n">
-        <v>197700</v>
+        <v>207000</v>
       </c>
       <c r="S263" t="n">
         <v>196800</v>
       </c>
       <c r="T263" t="n">
-        <v>0.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="264">
@@ -18093,13 +18093,13 @@
         <v>0</v>
       </c>
       <c r="R265" t="n">
-        <v>9140</v>
+        <v>9260</v>
       </c>
       <c r="S265" t="n">
         <v>9860</v>
       </c>
       <c r="T265" t="n">
-        <v>-7.3</v>
+        <v>-6.1</v>
       </c>
     </row>
     <row r="266">
@@ -18156,13 +18156,13 @@
         <v>3.6</v>
       </c>
       <c r="R266" t="n">
-        <v>31800</v>
+        <v>31750</v>
       </c>
       <c r="S266" t="n">
         <v>31700</v>
       </c>
       <c r="T266" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="267">
@@ -18219,13 +18219,13 @@
         <v>-0.2</v>
       </c>
       <c r="R267" t="n">
-        <v>216500</v>
+        <v>232500</v>
       </c>
       <c r="S267" t="n">
         <v>228500</v>
       </c>
       <c r="T267" t="n">
-        <v>-5.3</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="268">
@@ -18282,13 +18282,13 @@
         <v>0</v>
       </c>
       <c r="R268" t="n">
-        <v>15140</v>
+        <v>15230</v>
       </c>
       <c r="S268" t="n">
         <v>17820</v>
       </c>
       <c r="T268" t="n">
-        <v>-15</v>
+        <v>-14.5</v>
       </c>
     </row>
     <row r="269">
@@ -18345,13 +18345,13 @@
         <v>0</v>
       </c>
       <c r="R269" t="n">
-        <v>51200</v>
+        <v>50100</v>
       </c>
       <c r="S269" t="n">
         <v>53300</v>
       </c>
       <c r="T269" t="n">
-        <v>-3.9</v>
+        <v>-6</v>
       </c>
     </row>
     <row r="270">
@@ -18390,13 +18390,13 @@
         <v>0</v>
       </c>
       <c r="R270" t="n">
-        <v>33450</v>
+        <v>35000</v>
       </c>
       <c r="S270" t="n">
         <v>45900</v>
       </c>
       <c r="T270" t="n">
-        <v>-27.1</v>
+        <v>-23.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-09-04
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -458,7 +458,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-09-03 · 전주 2026-08-30</t>
+          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-09-04 · 전주 2026-08-30</t>
         </is>
       </c>
     </row>
@@ -642,13 +642,13 @@
         <v>0</v>
       </c>
       <c r="U3" t="n">
-        <v>15590</v>
+        <v>15540</v>
       </c>
       <c r="V3" t="n">
         <v>15720</v>
       </c>
       <c r="W3" t="n">
-        <v>-0.8</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="4">
@@ -786,13 +786,13 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>73500</v>
+        <v>73400</v>
       </c>
       <c r="V5" t="n">
         <v>74700</v>
       </c>
       <c r="W5" t="n">
-        <v>-1.6</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="6">
@@ -858,13 +858,13 @@
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>1125000</v>
+        <v>1142000</v>
       </c>
       <c r="V6" t="n">
         <v>1238000</v>
       </c>
       <c r="W6" t="n">
-        <v>-9.1</v>
+        <v>-7.8</v>
       </c>
     </row>
     <row r="7">
@@ -930,13 +930,13 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>55000</v>
+        <v>53600</v>
       </c>
       <c r="V7" t="n">
         <v>50000</v>
       </c>
       <c r="W7" t="n">
-        <v>10</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="8">
@@ -1002,13 +1002,13 @@
         <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>24400</v>
+        <v>24550</v>
       </c>
       <c r="V8" t="n">
         <v>24750</v>
       </c>
       <c r="W8" t="n">
-        <v>-1.4</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="9">
@@ -1074,13 +1074,13 @@
         <v>-0.4</v>
       </c>
       <c r="U9" t="n">
-        <v>127400</v>
+        <v>126500</v>
       </c>
       <c r="V9" t="n">
         <v>128000</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.5</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="10">
@@ -1146,13 +1146,13 @@
         <v>0</v>
       </c>
       <c r="U10" t="n">
-        <v>94000</v>
+        <v>92600</v>
       </c>
       <c r="V10" t="n">
         <v>96000</v>
       </c>
       <c r="W10" t="n">
-        <v>-2.1</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="11">
@@ -1182,13 +1182,13 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>787166</v>
+        <v>788035</v>
       </c>
       <c r="G11" t="n">
         <v>788035</v>
       </c>
       <c r="H11" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="L11" t="n">
         <v>2664365</v>
@@ -1218,13 +1218,13 @@
         <v>1.9</v>
       </c>
       <c r="U11" t="n">
-        <v>1596000</v>
+        <v>1647000</v>
       </c>
       <c r="V11" t="n">
         <v>1653000</v>
       </c>
       <c r="W11" t="n">
-        <v>-3.4</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="12">
@@ -1290,13 +1290,13 @@
         <v>0</v>
       </c>
       <c r="U12" t="n">
-        <v>119500</v>
+        <v>119700</v>
       </c>
       <c r="V12" t="n">
         <v>128900</v>
       </c>
       <c r="W12" t="n">
-        <v>-7.3</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="13">
@@ -1353,13 +1353,13 @@
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>702000</v>
+        <v>663000</v>
       </c>
       <c r="V13" t="n">
         <v>687000</v>
       </c>
       <c r="W13" t="n">
-        <v>2.2</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="14">
@@ -1425,13 +1425,13 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>133700</v>
+        <v>137400</v>
       </c>
       <c r="V14" t="n">
         <v>134900</v>
       </c>
       <c r="W14" t="n">
-        <v>-0.9</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="15">
@@ -1497,13 +1497,13 @@
         <v>0</v>
       </c>
       <c r="U15" t="n">
-        <v>88100</v>
+        <v>89900</v>
       </c>
       <c r="V15" t="n">
         <v>93900</v>
       </c>
       <c r="W15" t="n">
-        <v>-6.2</v>
+        <v>-4.3</v>
       </c>
     </row>
     <row r="16">
@@ -1569,13 +1569,13 @@
         <v>-4.1</v>
       </c>
       <c r="U16" t="n">
-        <v>128500</v>
+        <v>131400</v>
       </c>
       <c r="V16" t="n">
         <v>130500</v>
       </c>
       <c r="W16" t="n">
-        <v>-1.5</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="17">
@@ -1641,13 +1641,13 @@
         <v>1.1</v>
       </c>
       <c r="U17" t="n">
-        <v>40400</v>
+        <v>42350</v>
       </c>
       <c r="V17" t="n">
         <v>42600</v>
       </c>
       <c r="W17" t="n">
-        <v>-5.2</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="18">
@@ -1713,13 +1713,13 @@
         <v>0</v>
       </c>
       <c r="U18" t="n">
-        <v>26950</v>
+        <v>27400</v>
       </c>
       <c r="V18" t="n">
         <v>29700</v>
       </c>
       <c r="W18" t="n">
-        <v>-9.300000000000001</v>
+        <v>-7.7</v>
       </c>
     </row>
     <row r="19">
@@ -1776,13 +1776,13 @@
         <v>0</v>
       </c>
       <c r="U19" t="n">
-        <v>53500</v>
+        <v>51100</v>
       </c>
       <c r="V19" t="n">
         <v>52400</v>
       </c>
       <c r="W19" t="n">
-        <v>2.1</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="20">
@@ -1839,13 +1839,13 @@
         <v>-0.8</v>
       </c>
       <c r="U20" t="n">
-        <v>19050</v>
+        <v>19210</v>
       </c>
       <c r="V20" t="n">
         <v>18200</v>
       </c>
       <c r="W20" t="n">
-        <v>4.7</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="21">
@@ -1887,13 +1887,13 @@
         <v>6750</v>
       </c>
       <c r="U21" t="n">
-        <v>25300</v>
+        <v>25550</v>
       </c>
       <c r="V21" t="n">
         <v>26200</v>
       </c>
       <c r="W21" t="n">
-        <v>-3.4</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="22">
@@ -2031,13 +2031,13 @@
         <v>-0.2</v>
       </c>
       <c r="U23" t="n">
-        <v>485000</v>
+        <v>482000</v>
       </c>
       <c r="V23" t="n">
         <v>473500</v>
       </c>
       <c r="W23" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="24">
@@ -2103,13 +2103,13 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>16510</v>
+        <v>16090</v>
       </c>
       <c r="V24" t="n">
         <v>17020</v>
       </c>
       <c r="W24" t="n">
-        <v>-3</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="25">
@@ -2175,13 +2175,13 @@
         <v>0</v>
       </c>
       <c r="U25" t="n">
-        <v>104300</v>
+        <v>103000</v>
       </c>
       <c r="V25" t="n">
         <v>103400</v>
       </c>
       <c r="W25" t="n">
-        <v>0.9</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="26">
@@ -2247,13 +2247,13 @@
         <v>0</v>
       </c>
       <c r="U26" t="n">
-        <v>9440</v>
+        <v>9350</v>
       </c>
       <c r="V26" t="n">
         <v>9920</v>
       </c>
       <c r="W26" t="n">
-        <v>-4.8</v>
+        <v>-5.7</v>
       </c>
     </row>
     <row r="27">
@@ -2319,13 +2319,13 @@
         <v>0</v>
       </c>
       <c r="U27" t="n">
-        <v>7990</v>
+        <v>8070</v>
       </c>
       <c r="V27" t="n">
         <v>7880</v>
       </c>
       <c r="W27" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="28">
@@ -2391,13 +2391,13 @@
         <v>0.1</v>
       </c>
       <c r="U28" t="n">
-        <v>1424000</v>
+        <v>1417000</v>
       </c>
       <c r="V28" t="n">
         <v>1547000</v>
       </c>
       <c r="W28" t="n">
-        <v>-8</v>
+        <v>-8.4</v>
       </c>
     </row>
     <row r="29">
@@ -2463,13 +2463,13 @@
         <v>0</v>
       </c>
       <c r="U29" t="n">
-        <v>29150</v>
+        <v>30200</v>
       </c>
       <c r="V29" t="n">
         <v>28700</v>
       </c>
       <c r="W29" t="n">
-        <v>1.6</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="30">
@@ -2535,13 +2535,13 @@
         <v>1.2</v>
       </c>
       <c r="U30" t="n">
-        <v>118300</v>
+        <v>121100</v>
       </c>
       <c r="V30" t="n">
         <v>116300</v>
       </c>
       <c r="W30" t="n">
-        <v>1.7</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="31">
@@ -2607,13 +2607,13 @@
         <v>0</v>
       </c>
       <c r="U31" t="n">
-        <v>183800</v>
+        <v>183600</v>
       </c>
       <c r="V31" t="n">
         <v>186300</v>
       </c>
       <c r="W31" t="n">
-        <v>-1.3</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="32">
@@ -2679,13 +2679,13 @@
         <v>0</v>
       </c>
       <c r="U32" t="n">
-        <v>46100</v>
+        <v>45700</v>
       </c>
       <c r="V32" t="n">
         <v>48350</v>
       </c>
       <c r="W32" t="n">
-        <v>-4.7</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="33">
@@ -2751,13 +2751,13 @@
         <v>-0.9</v>
       </c>
       <c r="U33" t="n">
-        <v>31650</v>
+        <v>31500</v>
       </c>
       <c r="V33" t="n">
         <v>31000</v>
       </c>
       <c r="W33" t="n">
-        <v>2.1</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="34">
@@ -2823,13 +2823,13 @@
         <v>0</v>
       </c>
       <c r="U34" t="n">
-        <v>379500</v>
+        <v>382500</v>
       </c>
       <c r="V34" t="n">
         <v>405500</v>
       </c>
       <c r="W34" t="n">
-        <v>-6.4</v>
+        <v>-5.7</v>
       </c>
     </row>
     <row r="35">
@@ -2895,13 +2895,13 @@
         <v>0</v>
       </c>
       <c r="U35" t="n">
-        <v>430500</v>
+        <v>430000</v>
       </c>
       <c r="V35" t="n">
         <v>450500</v>
       </c>
       <c r="W35" t="n">
-        <v>-4.4</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="36">
@@ -2931,49 +2931,49 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2015</v>
+        <v>1920</v>
       </c>
       <c r="G36" t="n">
         <v>2015</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>-4.7</v>
       </c>
       <c r="L36" t="n">
-        <v>3676.7</v>
+        <v>3528.7</v>
       </c>
       <c r="M36" t="n">
         <v>3676.7</v>
       </c>
       <c r="N36" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="O36" t="n">
-        <v>4756.7</v>
+        <v>4472.7</v>
       </c>
       <c r="P36" t="n">
         <v>4756.7</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="R36" t="n">
-        <v>8550</v>
+        <v>5370</v>
       </c>
       <c r="S36" t="n">
         <v>8550</v>
       </c>
       <c r="T36" t="n">
-        <v>0</v>
+        <v>-37.2</v>
       </c>
       <c r="U36" t="n">
-        <v>24850</v>
+        <v>24750</v>
       </c>
       <c r="V36" t="n">
         <v>24150</v>
       </c>
       <c r="W36" t="n">
-        <v>2.9</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="37">
@@ -3183,13 +3183,13 @@
         <v>0.3</v>
       </c>
       <c r="U39" t="n">
-        <v>342000</v>
+        <v>337000</v>
       </c>
       <c r="V39" t="n">
         <v>337500</v>
       </c>
       <c r="W39" t="n">
-        <v>1.3</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="40">
@@ -3219,40 +3219,40 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>23905.3</v>
+        <v>23716.6</v>
       </c>
       <c r="M40" t="n">
         <v>23581.9</v>
       </c>
       <c r="N40" t="n">
-        <v>1.4</v>
+        <v>0.6</v>
       </c>
       <c r="O40" t="n">
-        <v>23943.7</v>
+        <v>23553.1</v>
       </c>
       <c r="P40" t="n">
         <v>23706.5</v>
       </c>
       <c r="Q40" t="n">
-        <v>1</v>
+        <v>-0.6</v>
       </c>
       <c r="R40" t="n">
-        <v>25222.9</v>
+        <v>24819.6</v>
       </c>
       <c r="S40" t="n">
         <v>25033.1</v>
       </c>
       <c r="T40" t="n">
-        <v>0.8</v>
+        <v>-0.9</v>
       </c>
       <c r="U40" t="n">
-        <v>203000</v>
+        <v>195700</v>
       </c>
       <c r="V40" t="n">
         <v>187400</v>
       </c>
       <c r="W40" t="n">
-        <v>8.300000000000001</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="41">
@@ -3318,13 +3318,13 @@
         <v>-3.4</v>
       </c>
       <c r="U41" t="n">
-        <v>50800</v>
+        <v>51400</v>
       </c>
       <c r="V41" t="n">
         <v>52400</v>
       </c>
       <c r="W41" t="n">
-        <v>-3.1</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="42">
@@ -3354,13 +3354,13 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1149671</v>
+        <v>1145149</v>
       </c>
       <c r="G42" t="n">
         <v>1145149</v>
       </c>
       <c r="H42" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="L42" t="n">
         <v>3933478.7</v>
@@ -3390,13 +3390,13 @@
         <v>3</v>
       </c>
       <c r="U42" t="n">
-        <v>250000</v>
+        <v>255500</v>
       </c>
       <c r="V42" t="n">
         <v>257000</v>
       </c>
       <c r="W42" t="n">
-        <v>-2.7</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="43">
@@ -3453,13 +3453,13 @@
         <v>0</v>
       </c>
       <c r="U43" t="n">
-        <v>26300</v>
+        <v>26650</v>
       </c>
       <c r="V43" t="n">
         <v>26650</v>
       </c>
       <c r="W43" t="n">
-        <v>-1.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44">
@@ -3525,13 +3525,13 @@
         <v>0</v>
       </c>
       <c r="U44" t="n">
-        <v>37850</v>
+        <v>38100</v>
       </c>
       <c r="V44" t="n">
         <v>38650</v>
       </c>
       <c r="W44" t="n">
-        <v>-2.1</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="45">
@@ -3597,13 +3597,13 @@
         <v>0</v>
       </c>
       <c r="U45" t="n">
-        <v>292000</v>
+        <v>299500</v>
       </c>
       <c r="V45" t="n">
         <v>313000</v>
       </c>
       <c r="W45" t="n">
-        <v>-6.7</v>
+        <v>-4.3</v>
       </c>
     </row>
     <row r="46">
@@ -3669,13 +3669,13 @@
         <v>0</v>
       </c>
       <c r="U46" t="n">
-        <v>127000</v>
+        <v>127600</v>
       </c>
       <c r="V46" t="n">
         <v>130500</v>
       </c>
       <c r="W46" t="n">
-        <v>-2.7</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="47">
@@ -3741,13 +3741,13 @@
         <v>0</v>
       </c>
       <c r="U47" t="n">
-        <v>33600</v>
+        <v>34250</v>
       </c>
       <c r="V47" t="n">
         <v>37150</v>
       </c>
       <c r="W47" t="n">
-        <v>-9.6</v>
+        <v>-7.8</v>
       </c>
     </row>
     <row r="48">
@@ -3813,13 +3813,13 @@
         <v>1.7</v>
       </c>
       <c r="U48" t="n">
-        <v>539000</v>
+        <v>548000</v>
       </c>
       <c r="V48" t="n">
         <v>571000</v>
       </c>
       <c r="W48" t="n">
-        <v>-5.6</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="49">
@@ -3885,13 +3885,13 @@
         <v>0</v>
       </c>
       <c r="U49" t="n">
-        <v>96400</v>
+        <v>96700</v>
       </c>
       <c r="V49" t="n">
         <v>95800</v>
       </c>
       <c r="W49" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="50">
@@ -3948,13 +3948,13 @@
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>33200</v>
+        <v>34450</v>
       </c>
       <c r="V50" t="n">
         <v>36150</v>
       </c>
       <c r="W50" t="n">
-        <v>-8.199999999999999</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="51">
@@ -4020,13 +4020,13 @@
         <v>0</v>
       </c>
       <c r="U51" t="n">
-        <v>25650</v>
+        <v>25400</v>
       </c>
       <c r="V51" t="n">
         <v>26650</v>
       </c>
       <c r="W51" t="n">
-        <v>-3.8</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="52">
@@ -4092,13 +4092,13 @@
         <v>0</v>
       </c>
       <c r="U52" t="n">
-        <v>46000</v>
+        <v>45100</v>
       </c>
       <c r="V52" t="n">
         <v>47200</v>
       </c>
       <c r="W52" t="n">
-        <v>-2.5</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="53">
@@ -4164,13 +4164,13 @@
         <v>0</v>
       </c>
       <c r="U53" t="n">
-        <v>106000</v>
+        <v>111100</v>
       </c>
       <c r="V53" t="n">
         <v>112800</v>
       </c>
       <c r="W53" t="n">
-        <v>-6</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="54">
@@ -4200,49 +4200,49 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>275</v>
+        <v>172</v>
       </c>
       <c r="G54" t="n">
         <v>338</v>
       </c>
       <c r="H54" t="n">
-        <v>-18.6</v>
+        <v>-49.1</v>
       </c>
       <c r="L54" t="n">
-        <v>1350.3</v>
+        <v>1197.3</v>
       </c>
       <c r="M54" t="n">
         <v>1421.8</v>
       </c>
       <c r="N54" t="n">
-        <v>-5</v>
+        <v>-15.8</v>
       </c>
       <c r="O54" t="n">
-        <v>2081.3</v>
+        <v>1920.3</v>
       </c>
       <c r="P54" t="n">
         <v>2222.2</v>
       </c>
       <c r="Q54" t="n">
-        <v>-6.3</v>
+        <v>-13.6</v>
       </c>
       <c r="R54" t="n">
-        <v>2772.7</v>
+        <v>2429</v>
       </c>
       <c r="S54" t="n">
         <v>2924.5</v>
       </c>
       <c r="T54" t="n">
-        <v>-5.2</v>
+        <v>-16.9</v>
       </c>
       <c r="U54" t="n">
-        <v>51400</v>
+        <v>51000</v>
       </c>
       <c r="V54" t="n">
         <v>60100</v>
       </c>
       <c r="W54" t="n">
-        <v>-14.5</v>
+        <v>-15.1</v>
       </c>
     </row>
     <row r="55">
@@ -4299,13 +4299,13 @@
         <v>0</v>
       </c>
       <c r="U55" t="n">
-        <v>16490</v>
+        <v>16260</v>
       </c>
       <c r="V55" t="n">
         <v>16800</v>
       </c>
       <c r="W55" t="n">
-        <v>-1.8</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="56">
@@ -4371,13 +4371,13 @@
         <v>0</v>
       </c>
       <c r="U56" t="n">
-        <v>41800</v>
+        <v>42200</v>
       </c>
       <c r="V56" t="n">
         <v>43000</v>
       </c>
       <c r="W56" t="n">
-        <v>-2.8</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="57">
@@ -4407,49 +4407,49 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>5960</v>
+        <v>5972</v>
       </c>
       <c r="G57" t="n">
         <v>5913</v>
       </c>
       <c r="H57" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>19445.5</v>
+        <v>19468</v>
       </c>
       <c r="M57" t="n">
         <v>19307</v>
       </c>
       <c r="N57" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="O57" t="n">
-        <v>37303</v>
+        <v>37338.5</v>
       </c>
       <c r="P57" t="n">
         <v>37111</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="R57" t="n">
-        <v>58720</v>
+        <v>58742.2</v>
       </c>
       <c r="S57" t="n">
         <v>58230.6</v>
       </c>
       <c r="T57" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="U57" t="n">
-        <v>1348000</v>
+        <v>1401000</v>
       </c>
       <c r="V57" t="n">
         <v>1421000</v>
       </c>
       <c r="W57" t="n">
-        <v>-5.1</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="58">
@@ -4515,13 +4515,13 @@
         <v>0</v>
       </c>
       <c r="U58" t="n">
-        <v>37000</v>
+        <v>37400</v>
       </c>
       <c r="V58" t="n">
         <v>39700</v>
       </c>
       <c r="W58" t="n">
-        <v>-6.8</v>
+        <v>-5.8</v>
       </c>
     </row>
     <row r="59">
@@ -4587,13 +4587,13 @@
         <v>0</v>
       </c>
       <c r="U59" t="n">
-        <v>344000</v>
+        <v>348500</v>
       </c>
       <c r="V59" t="n">
         <v>354500</v>
       </c>
       <c r="W59" t="n">
-        <v>-3</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="60">
@@ -4659,13 +4659,13 @@
         <v>5.5</v>
       </c>
       <c r="U60" t="n">
-        <v>29900</v>
+        <v>30050</v>
       </c>
       <c r="V60" t="n">
         <v>33750</v>
       </c>
       <c r="W60" t="n">
-        <v>-11.4</v>
+        <v>-11</v>
       </c>
     </row>
     <row r="61">
@@ -4803,13 +4803,13 @@
         <v>0</v>
       </c>
       <c r="U62" t="n">
-        <v>192100</v>
+        <v>195300</v>
       </c>
       <c r="V62" t="n">
         <v>214500</v>
       </c>
       <c r="W62" t="n">
-        <v>-10.4</v>
+        <v>-9</v>
       </c>
     </row>
     <row r="63">
@@ -4875,13 +4875,13 @@
         <v>0</v>
       </c>
       <c r="U63" t="n">
-        <v>1224000</v>
+        <v>1222000</v>
       </c>
       <c r="V63" t="n">
         <v>1375000</v>
       </c>
       <c r="W63" t="n">
-        <v>-11</v>
+        <v>-11.1</v>
       </c>
     </row>
     <row r="64">
@@ -4947,13 +4947,13 @@
         <v>0</v>
       </c>
       <c r="U64" t="n">
-        <v>21650</v>
+        <v>21400</v>
       </c>
       <c r="V64" t="n">
         <v>21200</v>
       </c>
       <c r="W64" t="n">
-        <v>2.1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="65">
@@ -4986,13 +4986,13 @@
         <v>59</v>
       </c>
       <c r="U65" t="n">
-        <v>12850</v>
+        <v>13010</v>
       </c>
       <c r="V65" t="n">
         <v>14310</v>
       </c>
       <c r="W65" t="n">
-        <v>-10.2</v>
+        <v>-9.1</v>
       </c>
     </row>
     <row r="66">
@@ -5058,13 +5058,13 @@
         <v>0</v>
       </c>
       <c r="U66" t="n">
-        <v>15670</v>
+        <v>15740</v>
       </c>
       <c r="V66" t="n">
         <v>16340</v>
       </c>
       <c r="W66" t="n">
-        <v>-4.1</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="67">
@@ -5130,13 +5130,13 @@
         <v>0</v>
       </c>
       <c r="U67" t="n">
-        <v>147900</v>
+        <v>157300</v>
       </c>
       <c r="V67" t="n">
         <v>149200</v>
       </c>
       <c r="W67" t="n">
-        <v>-0.9</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="68">
@@ -5202,13 +5202,13 @@
         <v>0.9</v>
       </c>
       <c r="U68" t="n">
-        <v>556000</v>
+        <v>562000</v>
       </c>
       <c r="V68" t="n">
         <v>611000</v>
       </c>
       <c r="W68" t="n">
-        <v>-9</v>
+        <v>-8</v>
       </c>
     </row>
     <row r="69">
@@ -5274,13 +5274,13 @@
         <v>0</v>
       </c>
       <c r="U69" t="n">
-        <v>61000</v>
+        <v>60000</v>
       </c>
       <c r="V69" t="n">
         <v>59500</v>
       </c>
       <c r="W69" t="n">
-        <v>2.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="70">
@@ -5346,13 +5346,13 @@
         <v>0</v>
       </c>
       <c r="U70" t="n">
-        <v>21350</v>
+        <v>21050</v>
       </c>
       <c r="V70" t="n">
         <v>21700</v>
       </c>
       <c r="W70" t="n">
-        <v>-1.6</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="71">
@@ -5418,13 +5418,13 @@
         <v>0</v>
       </c>
       <c r="U71" t="n">
-        <v>57200</v>
+        <v>57600</v>
       </c>
       <c r="V71" t="n">
         <v>59700</v>
       </c>
       <c r="W71" t="n">
-        <v>-4.2</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="72">
@@ -5490,13 +5490,13 @@
         <v>0</v>
       </c>
       <c r="U72" t="n">
-        <v>133100</v>
+        <v>125900</v>
       </c>
       <c r="V72" t="n">
         <v>125900</v>
       </c>
       <c r="W72" t="n">
-        <v>5.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -5562,13 +5562,13 @@
         <v>0</v>
       </c>
       <c r="U73" t="n">
-        <v>83900</v>
+        <v>84300</v>
       </c>
       <c r="V73" t="n">
         <v>91300</v>
       </c>
       <c r="W73" t="n">
-        <v>-8.1</v>
+        <v>-7.7</v>
       </c>
     </row>
     <row r="74">
@@ -5634,13 +5634,13 @@
         <v>0</v>
       </c>
       <c r="U74" t="n">
-        <v>15880</v>
+        <v>16110</v>
       </c>
       <c r="V74" t="n">
         <v>16910</v>
       </c>
       <c r="W74" t="n">
-        <v>-6.1</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="75">
@@ -5706,13 +5706,13 @@
         <v>-0.1</v>
       </c>
       <c r="U75" t="n">
-        <v>423500</v>
+        <v>422000</v>
       </c>
       <c r="V75" t="n">
         <v>450500</v>
       </c>
       <c r="W75" t="n">
-        <v>-6</v>
+        <v>-6.3</v>
       </c>
     </row>
     <row r="76">
@@ -5778,13 +5778,13 @@
         <v>0.4</v>
       </c>
       <c r="U76" t="n">
-        <v>1047000</v>
+        <v>1055000</v>
       </c>
       <c r="V76" t="n">
         <v>1157000</v>
       </c>
       <c r="W76" t="n">
-        <v>-9.5</v>
+        <v>-8.800000000000001</v>
       </c>
     </row>
     <row r="77">
@@ -5850,13 +5850,13 @@
         <v>0</v>
       </c>
       <c r="U77" t="n">
-        <v>80300</v>
+        <v>79200</v>
       </c>
       <c r="V77" t="n">
         <v>83500</v>
       </c>
       <c r="W77" t="n">
-        <v>-3.8</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="78">
@@ -5922,13 +5922,13 @@
         <v>0</v>
       </c>
       <c r="U78" t="n">
-        <v>30400</v>
+        <v>30850</v>
       </c>
       <c r="V78" t="n">
         <v>31850</v>
       </c>
       <c r="W78" t="n">
-        <v>-4.6</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="79">
@@ -5994,13 +5994,13 @@
         <v>0</v>
       </c>
       <c r="U79" t="n">
-        <v>192500</v>
+        <v>193100</v>
       </c>
       <c r="V79" t="n">
         <v>203000</v>
       </c>
       <c r="W79" t="n">
-        <v>-5.2</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="80">
@@ -6129,13 +6129,13 @@
         <v>0</v>
       </c>
       <c r="U81" t="n">
-        <v>32450</v>
+        <v>32150</v>
       </c>
       <c r="V81" t="n">
         <v>32550</v>
       </c>
       <c r="W81" t="n">
-        <v>-0.3</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="82">
@@ -6192,13 +6192,13 @@
         <v>0</v>
       </c>
       <c r="U82" t="n">
-        <v>86600</v>
+        <v>86800</v>
       </c>
       <c r="V82" t="n">
         <v>88500</v>
       </c>
       <c r="W82" t="n">
-        <v>-2.1</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="83">
@@ -6264,13 +6264,13 @@
         <v>0.2</v>
       </c>
       <c r="U83" t="n">
-        <v>89000</v>
+        <v>92500</v>
       </c>
       <c r="V83" t="n">
         <v>98600</v>
       </c>
       <c r="W83" t="n">
-        <v>-9.699999999999999</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="84">
@@ -6336,13 +6336,13 @@
         <v>0</v>
       </c>
       <c r="U84" t="n">
-        <v>74700</v>
+        <v>74900</v>
       </c>
       <c r="V84" t="n">
         <v>75600</v>
       </c>
       <c r="W84" t="n">
-        <v>-1.2</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="85">
@@ -6408,13 +6408,13 @@
         <v>1.5</v>
       </c>
       <c r="U85" t="n">
-        <v>22350</v>
+        <v>22550</v>
       </c>
       <c r="V85" t="n">
         <v>24950</v>
       </c>
       <c r="W85" t="n">
-        <v>-10.4</v>
+        <v>-9.6</v>
       </c>
     </row>
     <row r="86">
@@ -6480,13 +6480,13 @@
         <v>-0.4</v>
       </c>
       <c r="U86" t="n">
-        <v>226000</v>
+        <v>238000</v>
       </c>
       <c r="V86" t="n">
         <v>243000</v>
       </c>
       <c r="W86" t="n">
-        <v>-7</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="87">
@@ -6552,13 +6552,13 @@
         <v>-0.2</v>
       </c>
       <c r="U87" t="n">
-        <v>3495</v>
+        <v>3525</v>
       </c>
       <c r="V87" t="n">
         <v>3490</v>
       </c>
       <c r="W87" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88">
@@ -6624,13 +6624,13 @@
         <v>0</v>
       </c>
       <c r="U88" t="n">
-        <v>98200</v>
+        <v>99400</v>
       </c>
       <c r="V88" t="n">
         <v>100400</v>
       </c>
       <c r="W88" t="n">
-        <v>-2.2</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="89">
@@ -6696,13 +6696,13 @@
         <v>0</v>
       </c>
       <c r="U89" t="n">
-        <v>21400</v>
+        <v>21650</v>
       </c>
       <c r="V89" t="n">
         <v>21400</v>
       </c>
       <c r="W89" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="90">
@@ -6768,13 +6768,13 @@
         <v>0</v>
       </c>
       <c r="U90" t="n">
-        <v>25800</v>
+        <v>26150</v>
       </c>
       <c r="V90" t="n">
         <v>26600</v>
       </c>
       <c r="W90" t="n">
-        <v>-3</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="91">
@@ -6840,13 +6840,13 @@
         <v>0</v>
       </c>
       <c r="U91" t="n">
-        <v>105300</v>
+        <v>107500</v>
       </c>
       <c r="V91" t="n">
         <v>102100</v>
       </c>
       <c r="W91" t="n">
-        <v>3.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="92">
@@ -6906,13 +6906,13 @@
         <v>0</v>
       </c>
       <c r="U92" t="n">
-        <v>21150</v>
+        <v>20700</v>
       </c>
       <c r="V92" t="n">
         <v>20850</v>
       </c>
       <c r="W92" t="n">
-        <v>1.4</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="93">
@@ -6978,13 +6978,13 @@
         <v>0</v>
       </c>
       <c r="U93" t="n">
-        <v>46100</v>
+        <v>45850</v>
       </c>
       <c r="V93" t="n">
         <v>48750</v>
       </c>
       <c r="W93" t="n">
-        <v>-5.4</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="94">
@@ -7050,13 +7050,13 @@
         <v>0.1</v>
       </c>
       <c r="U94" t="n">
-        <v>372000</v>
+        <v>367000</v>
       </c>
       <c r="V94" t="n">
         <v>375000</v>
       </c>
       <c r="W94" t="n">
-        <v>-0.8</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="95">
@@ -7122,13 +7122,13 @@
         <v>0</v>
       </c>
       <c r="U95" t="n">
-        <v>5940</v>
+        <v>5960</v>
       </c>
       <c r="V95" t="n">
         <v>5790</v>
       </c>
       <c r="W95" t="n">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="96">
@@ -7185,13 +7185,13 @@
         <v>0</v>
       </c>
       <c r="U96" t="n">
-        <v>46600</v>
+        <v>46150</v>
       </c>
       <c r="V96" t="n">
         <v>47300</v>
       </c>
       <c r="W96" t="n">
-        <v>-1.5</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="97">
@@ -7257,7 +7257,7 @@
         <v>0</v>
       </c>
       <c r="U97" t="n">
-        <v>18940</v>
+        <v>18930</v>
       </c>
       <c r="V97" t="n">
         <v>19340</v>
@@ -7329,13 +7329,13 @@
         <v>0</v>
       </c>
       <c r="U98" t="n">
-        <v>53800</v>
+        <v>54300</v>
       </c>
       <c r="V98" t="n">
         <v>54500</v>
       </c>
       <c r="W98" t="n">
-        <v>-1.3</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="99">
@@ -7401,13 +7401,13 @@
         <v>0</v>
       </c>
       <c r="U99" t="n">
-        <v>129500</v>
+        <v>144000</v>
       </c>
       <c r="V99" t="n">
         <v>120100</v>
       </c>
       <c r="W99" t="n">
-        <v>7.8</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="100">
@@ -7446,13 +7446,13 @@
         <v>-1.1</v>
       </c>
       <c r="U100" t="n">
-        <v>12560</v>
+        <v>12530</v>
       </c>
       <c r="V100" t="n">
         <v>13250</v>
       </c>
       <c r="W100" t="n">
-        <v>-5.2</v>
+        <v>-5.4</v>
       </c>
     </row>
     <row r="101">
@@ -7518,13 +7518,13 @@
         <v>0</v>
       </c>
       <c r="U101" t="n">
-        <v>14810</v>
+        <v>14760</v>
       </c>
       <c r="V101" t="n">
         <v>15020</v>
       </c>
       <c r="W101" t="n">
-        <v>-1.4</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="102">
@@ -7581,13 +7581,13 @@
         <v>0</v>
       </c>
       <c r="U102" t="n">
-        <v>303000</v>
+        <v>297500</v>
       </c>
       <c r="V102" t="n">
         <v>310000</v>
       </c>
       <c r="W102" t="n">
-        <v>-2.3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="103">
@@ -7647,13 +7647,13 @@
         <v>1565</v>
       </c>
       <c r="U103" t="n">
-        <v>17030</v>
+        <v>17160</v>
       </c>
       <c r="V103" t="n">
         <v>18360</v>
       </c>
       <c r="W103" t="n">
-        <v>-7.2</v>
+        <v>-6.5</v>
       </c>
     </row>
     <row r="104">
@@ -7719,13 +7719,13 @@
         <v>0</v>
       </c>
       <c r="U104" t="n">
-        <v>174700</v>
+        <v>172500</v>
       </c>
       <c r="V104" t="n">
         <v>176300</v>
       </c>
       <c r="W104" t="n">
-        <v>-0.9</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="105">
@@ -7863,13 +7863,13 @@
         <v>0</v>
       </c>
       <c r="U106" t="n">
-        <v>9040</v>
+        <v>9130</v>
       </c>
       <c r="V106" t="n">
         <v>9620</v>
       </c>
       <c r="W106" t="n">
-        <v>-6</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="107">
@@ -7935,13 +7935,13 @@
         <v>0</v>
       </c>
       <c r="U107" t="n">
-        <v>9820</v>
+        <v>10090</v>
       </c>
       <c r="V107" t="n">
         <v>10030</v>
       </c>
       <c r="W107" t="n">
-        <v>-2.1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="108">
@@ -8007,13 +8007,13 @@
         <v>-3.9</v>
       </c>
       <c r="U108" t="n">
-        <v>545000</v>
+        <v>573000</v>
       </c>
       <c r="V108" t="n">
         <v>543000</v>
       </c>
       <c r="W108" t="n">
-        <v>0.4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="109">
@@ -8079,13 +8079,13 @@
         <v>0.5</v>
       </c>
       <c r="U109" t="n">
-        <v>14720</v>
+        <v>14750</v>
       </c>
       <c r="V109" t="n">
         <v>14790</v>
       </c>
       <c r="W109" t="n">
-        <v>-0.5</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="110">
@@ -8151,13 +8151,13 @@
         <v>0.1</v>
       </c>
       <c r="U110" t="n">
-        <v>207500</v>
+        <v>213500</v>
       </c>
       <c r="V110" t="n">
         <v>220500</v>
       </c>
       <c r="W110" t="n">
-        <v>-5.9</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="111">
@@ -8223,13 +8223,13 @@
         <v>0.4</v>
       </c>
       <c r="U111" t="n">
-        <v>35350</v>
+        <v>36200</v>
       </c>
       <c r="V111" t="n">
         <v>36850</v>
       </c>
       <c r="W111" t="n">
-        <v>-4.1</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="112">
@@ -8295,13 +8295,13 @@
         <v>0</v>
       </c>
       <c r="U112" t="n">
-        <v>32200</v>
+        <v>33050</v>
       </c>
       <c r="V112" t="n">
         <v>32850</v>
       </c>
       <c r="W112" t="n">
-        <v>-2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="113">
@@ -8367,13 +8367,13 @@
         <v>0</v>
       </c>
       <c r="U113" t="n">
-        <v>38500</v>
+        <v>39300</v>
       </c>
       <c r="V113" t="n">
         <v>40100</v>
       </c>
       <c r="W113" t="n">
-        <v>-4</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="114">
@@ -8439,13 +8439,13 @@
         <v>0</v>
       </c>
       <c r="U114" t="n">
-        <v>8790</v>
+        <v>8910</v>
       </c>
       <c r="V114" t="n">
         <v>8870</v>
       </c>
       <c r="W114" t="n">
-        <v>-0.9</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="115">
@@ -8511,13 +8511,13 @@
         <v>0</v>
       </c>
       <c r="U115" t="n">
-        <v>37700</v>
+        <v>35100</v>
       </c>
       <c r="V115" t="n">
         <v>37100</v>
       </c>
       <c r="W115" t="n">
-        <v>1.6</v>
+        <v>-5.4</v>
       </c>
     </row>
     <row r="116">
@@ -8583,13 +8583,13 @@
         <v>3.1</v>
       </c>
       <c r="U116" t="n">
-        <v>217000</v>
+        <v>222000</v>
       </c>
       <c r="V116" t="n">
         <v>225000</v>
       </c>
       <c r="W116" t="n">
-        <v>-3.6</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="117">
@@ -8655,13 +8655,13 @@
         <v>0</v>
       </c>
       <c r="U117" t="n">
-        <v>168000</v>
+        <v>178300</v>
       </c>
       <c r="V117" t="n">
         <v>176800</v>
       </c>
       <c r="W117" t="n">
-        <v>-5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="118">
@@ -8727,13 +8727,13 @@
         <v>0</v>
       </c>
       <c r="U118" t="n">
-        <v>418000</v>
+        <v>443000</v>
       </c>
       <c r="V118" t="n">
         <v>398500</v>
       </c>
       <c r="W118" t="n">
-        <v>4.9</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="119">
@@ -8799,13 +8799,13 @@
         <v>0</v>
       </c>
       <c r="U119" t="n">
-        <v>32450</v>
+        <v>32500</v>
       </c>
       <c r="V119" t="n">
         <v>32900</v>
       </c>
       <c r="W119" t="n">
-        <v>-1.4</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="120">
@@ -8862,13 +8862,13 @@
         <v>0</v>
       </c>
       <c r="U120" t="n">
-        <v>268500</v>
+        <v>270500</v>
       </c>
       <c r="V120" t="n">
         <v>278500</v>
       </c>
       <c r="W120" t="n">
-        <v>-3.6</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="121">
@@ -8934,13 +8934,13 @@
         <v>0</v>
       </c>
       <c r="U121" t="n">
-        <v>11010</v>
+        <v>10910</v>
       </c>
       <c r="V121" t="n">
         <v>11100</v>
       </c>
       <c r="W121" t="n">
-        <v>-0.8</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="122">
@@ -9006,13 +9006,13 @@
         <v>0</v>
       </c>
       <c r="U122" t="n">
-        <v>75300</v>
+        <v>79000</v>
       </c>
       <c r="V122" t="n">
         <v>75800</v>
       </c>
       <c r="W122" t="n">
-        <v>-0.7</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="123">
@@ -9078,13 +9078,13 @@
         <v>0</v>
       </c>
       <c r="U123" t="n">
-        <v>86500</v>
+        <v>86800</v>
       </c>
       <c r="V123" t="n">
         <v>88500</v>
       </c>
       <c r="W123" t="n">
-        <v>-2.3</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="124">
@@ -9150,13 +9150,13 @@
         <v>0</v>
       </c>
       <c r="U124" t="n">
-        <v>210500</v>
+        <v>230000</v>
       </c>
       <c r="V124" t="n">
         <v>219500</v>
       </c>
       <c r="W124" t="n">
-        <v>-4.1</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="125">
@@ -9222,13 +9222,13 @@
         <v>0</v>
       </c>
       <c r="U125" t="n">
-        <v>16750</v>
+        <v>16850</v>
       </c>
       <c r="V125" t="n">
         <v>19690</v>
       </c>
       <c r="W125" t="n">
-        <v>-14.9</v>
+        <v>-14.4</v>
       </c>
     </row>
     <row r="126">
@@ -9294,13 +9294,13 @@
         <v>0</v>
       </c>
       <c r="U126" t="n">
-        <v>55500</v>
+        <v>54700</v>
       </c>
       <c r="V126" t="n">
         <v>52700</v>
       </c>
       <c r="W126" t="n">
-        <v>5.3</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="127">
@@ -9366,13 +9366,13 @@
         <v>0</v>
       </c>
       <c r="U127" t="n">
-        <v>125000</v>
+        <v>126500</v>
       </c>
       <c r="V127" t="n">
         <v>133100</v>
       </c>
       <c r="W127" t="n">
-        <v>-6.1</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="128">
@@ -9432,13 +9432,13 @@
         <v>0</v>
       </c>
       <c r="U128" t="n">
-        <v>23600</v>
+        <v>23700</v>
       </c>
       <c r="V128" t="n">
         <v>24200</v>
       </c>
       <c r="W128" t="n">
-        <v>-2.5</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="129">
@@ -9504,13 +9504,13 @@
         <v>0</v>
       </c>
       <c r="U129" t="n">
-        <v>45300</v>
+        <v>45800</v>
       </c>
       <c r="V129" t="n">
         <v>47050</v>
       </c>
       <c r="W129" t="n">
-        <v>-3.7</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="130">
@@ -9576,13 +9576,13 @@
         <v>0</v>
       </c>
       <c r="U130" t="n">
-        <v>291500</v>
+        <v>294000</v>
       </c>
       <c r="V130" t="n">
         <v>318000</v>
       </c>
       <c r="W130" t="n">
-        <v>-8.300000000000001</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="131">
@@ -9648,13 +9648,13 @@
         <v>0</v>
       </c>
       <c r="U131" t="n">
-        <v>287000</v>
+        <v>282000</v>
       </c>
       <c r="V131" t="n">
         <v>277000</v>
       </c>
       <c r="W131" t="n">
-        <v>3.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="132">
@@ -9720,13 +9720,13 @@
         <v>0</v>
       </c>
       <c r="U132" t="n">
-        <v>107400</v>
+        <v>107600</v>
       </c>
       <c r="V132" t="n">
         <v>122400</v>
       </c>
       <c r="W132" t="n">
-        <v>-12.3</v>
+        <v>-12.1</v>
       </c>
     </row>
     <row r="133">
@@ -9786,13 +9786,13 @@
         <v>0</v>
       </c>
       <c r="U133" t="n">
-        <v>114500</v>
+        <v>110300</v>
       </c>
       <c r="V133" t="n">
         <v>109700</v>
       </c>
       <c r="W133" t="n">
-        <v>4.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="134">
@@ -9858,13 +9858,13 @@
         <v>1.7</v>
       </c>
       <c r="U134" t="n">
-        <v>64300</v>
+        <v>66600</v>
       </c>
       <c r="V134" t="n">
         <v>66800</v>
       </c>
       <c r="W134" t="n">
-        <v>-3.7</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="135">
@@ -9924,13 +9924,13 @@
         <v>0</v>
       </c>
       <c r="U135" t="n">
-        <v>83800</v>
+        <v>94200</v>
       </c>
       <c r="V135" t="n">
         <v>92700</v>
       </c>
       <c r="W135" t="n">
-        <v>-9.6</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="136">
@@ -9987,13 +9987,13 @@
         <v>0</v>
       </c>
       <c r="U136" t="n">
-        <v>39750</v>
+        <v>40150</v>
       </c>
       <c r="V136" t="n">
         <v>40500</v>
       </c>
       <c r="W136" t="n">
-        <v>-1.9</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="137">
@@ -10059,13 +10059,13 @@
         <v>0</v>
       </c>
       <c r="U137" t="n">
-        <v>186500</v>
+        <v>191700</v>
       </c>
       <c r="V137" t="n">
         <v>202500</v>
       </c>
       <c r="W137" t="n">
-        <v>-7.9</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="138">
@@ -10131,13 +10131,13 @@
         <v>-2.1</v>
       </c>
       <c r="U138" t="n">
-        <v>126400</v>
+        <v>126800</v>
       </c>
       <c r="V138" t="n">
         <v>139100</v>
       </c>
       <c r="W138" t="n">
-        <v>-9.1</v>
+        <v>-8.800000000000001</v>
       </c>
     </row>
     <row r="139">
@@ -10203,13 +10203,13 @@
         <v>0.2</v>
       </c>
       <c r="U139" t="n">
-        <v>72500</v>
+        <v>74100</v>
       </c>
       <c r="V139" t="n">
         <v>75800</v>
       </c>
       <c r="W139" t="n">
-        <v>-4.4</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="140">
@@ -10248,40 +10248,40 @@
         <v>0</v>
       </c>
       <c r="L140" t="n">
-        <v>1236.5</v>
+        <v>1234.1</v>
       </c>
       <c r="M140" t="n">
         <v>1236.5</v>
       </c>
       <c r="N140" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="O140" t="n">
-        <v>1677.2</v>
+        <v>1666.1</v>
       </c>
       <c r="P140" t="n">
         <v>1677.2</v>
       </c>
       <c r="Q140" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="R140" t="n">
-        <v>2108.8</v>
+        <v>2046.1</v>
       </c>
       <c r="S140" t="n">
         <v>2108.8</v>
       </c>
       <c r="T140" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="U140" t="n">
-        <v>240500</v>
+        <v>252000</v>
       </c>
       <c r="V140" t="n">
         <v>238500</v>
       </c>
       <c r="W140" t="n">
-        <v>0.8</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="141">
@@ -10347,13 +10347,13 @@
         <v>-3.3</v>
       </c>
       <c r="U141" t="n">
-        <v>26800</v>
+        <v>26250</v>
       </c>
       <c r="V141" t="n">
         <v>25850</v>
       </c>
       <c r="W141" t="n">
-        <v>3.7</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="142">
@@ -10419,13 +10419,13 @@
         <v>0</v>
       </c>
       <c r="U142" t="n">
-        <v>199700</v>
+        <v>201500</v>
       </c>
       <c r="V142" t="n">
         <v>201500</v>
       </c>
       <c r="W142" t="n">
-        <v>-0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -10491,13 +10491,13 @@
         <v>0</v>
       </c>
       <c r="U143" t="n">
-        <v>120900</v>
+        <v>121300</v>
       </c>
       <c r="V143" t="n">
         <v>134800</v>
       </c>
       <c r="W143" t="n">
-        <v>-10.3</v>
+        <v>-10</v>
       </c>
     </row>
     <row r="144">
@@ -10563,13 +10563,13 @@
         <v>0</v>
       </c>
       <c r="U144" t="n">
-        <v>37700</v>
+        <v>38050</v>
       </c>
       <c r="V144" t="n">
         <v>39500</v>
       </c>
       <c r="W144" t="n">
-        <v>-4.6</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="145">
@@ -10635,13 +10635,13 @@
         <v>0</v>
       </c>
       <c r="U145" t="n">
-        <v>34700</v>
+        <v>34850</v>
       </c>
       <c r="V145" t="n">
         <v>35350</v>
       </c>
       <c r="W145" t="n">
-        <v>-1.8</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="146">
@@ -10707,13 +10707,13 @@
         <v>0</v>
       </c>
       <c r="U146" t="n">
-        <v>187100</v>
+        <v>188100</v>
       </c>
       <c r="V146" t="n">
         <v>190700</v>
       </c>
       <c r="W146" t="n">
-        <v>-1.9</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="147">
@@ -10827,7 +10827,7 @@
         <v>-0</v>
       </c>
       <c r="U148" t="n">
-        <v>16330</v>
+        <v>16320</v>
       </c>
       <c r="V148" t="n">
         <v>16390</v>
@@ -10899,13 +10899,13 @@
         <v>0</v>
       </c>
       <c r="U149" t="n">
-        <v>114800</v>
+        <v>116100</v>
       </c>
       <c r="V149" t="n">
         <v>128800</v>
       </c>
       <c r="W149" t="n">
-        <v>-10.9</v>
+        <v>-9.9</v>
       </c>
     </row>
     <row r="150">
@@ -10971,13 +10971,13 @@
         <v>0.4</v>
       </c>
       <c r="U150" t="n">
-        <v>94600</v>
+        <v>96200</v>
       </c>
       <c r="V150" t="n">
         <v>93400</v>
       </c>
       <c r="W150" t="n">
-        <v>1.3</v>
+        <v>3</v>
       </c>
     </row>
     <row r="151">
@@ -11006,6 +11006,9 @@
           <t>KOSPI200</t>
         </is>
       </c>
+      <c r="F151" t="n">
+        <v>9012</v>
+      </c>
       <c r="L151" t="n">
         <v>40740.8</v>
       </c>
@@ -11034,13 +11037,13 @@
         <v>0</v>
       </c>
       <c r="U151" t="n">
-        <v>186600</v>
+        <v>188800</v>
       </c>
       <c r="V151" t="n">
         <v>191300</v>
       </c>
       <c r="W151" t="n">
-        <v>-2.5</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="152">
@@ -11106,13 +11109,13 @@
         <v>0</v>
       </c>
       <c r="U152" t="n">
-        <v>76500</v>
+        <v>75600</v>
       </c>
       <c r="V152" t="n">
         <v>74800</v>
       </c>
       <c r="W152" t="n">
-        <v>2.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="153">
@@ -11178,13 +11181,13 @@
         <v>0</v>
       </c>
       <c r="U153" t="n">
-        <v>49500</v>
+        <v>50200</v>
       </c>
       <c r="V153" t="n">
         <v>53100</v>
       </c>
       <c r="W153" t="n">
-        <v>-6.8</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="154">
@@ -11250,13 +11253,13 @@
         <v>0</v>
       </c>
       <c r="U154" t="n">
-        <v>7120</v>
+        <v>7180</v>
       </c>
       <c r="V154" t="n">
         <v>7360</v>
       </c>
       <c r="W154" t="n">
-        <v>-3.3</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="155">
@@ -11289,13 +11292,13 @@
         <v>230</v>
       </c>
       <c r="U155" t="n">
-        <v>10190</v>
+        <v>10280</v>
       </c>
       <c r="V155" t="n">
         <v>10660</v>
       </c>
       <c r="W155" t="n">
-        <v>-4.4</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="156">
@@ -11334,13 +11337,13 @@
         <v>4.5</v>
       </c>
       <c r="U156" t="n">
-        <v>9700</v>
+        <v>10060</v>
       </c>
       <c r="V156" t="n">
         <v>9850</v>
       </c>
       <c r="W156" t="n">
-        <v>-1.5</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="157">
@@ -11406,13 +11409,13 @@
         <v>0</v>
       </c>
       <c r="U157" t="n">
-        <v>23450</v>
+        <v>23550</v>
       </c>
       <c r="V157" t="n">
         <v>25300</v>
       </c>
       <c r="W157" t="n">
-        <v>-7.3</v>
+        <v>-6.9</v>
       </c>
     </row>
     <row r="158">
@@ -11478,13 +11481,13 @@
         <v>0</v>
       </c>
       <c r="U158" t="n">
-        <v>118900</v>
+        <v>123900</v>
       </c>
       <c r="V158" t="n">
         <v>129200</v>
       </c>
       <c r="W158" t="n">
-        <v>-8</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="159">
@@ -11550,13 +11553,13 @@
         <v>0</v>
       </c>
       <c r="U159" t="n">
-        <v>665000</v>
+        <v>652000</v>
       </c>
       <c r="V159" t="n">
         <v>734000</v>
       </c>
       <c r="W159" t="n">
-        <v>-9.4</v>
+        <v>-11.2</v>
       </c>
     </row>
     <row r="160">
@@ -11589,13 +11592,13 @@
         <v>10</v>
       </c>
       <c r="U160" t="n">
-        <v>8860</v>
+        <v>8970</v>
       </c>
       <c r="V160" t="n">
         <v>9150</v>
       </c>
       <c r="W160" t="n">
-        <v>-3.2</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="161">
@@ -11661,13 +11664,13 @@
         <v>0</v>
       </c>
       <c r="U161" t="n">
-        <v>40900</v>
+        <v>41400</v>
       </c>
       <c r="V161" t="n">
         <v>41350</v>
       </c>
       <c r="W161" t="n">
-        <v>-1.1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="162">
@@ -11805,13 +11808,13 @@
         <v>0</v>
       </c>
       <c r="U163" t="n">
-        <v>59300</v>
+        <v>60000</v>
       </c>
       <c r="V163" t="n">
         <v>65400</v>
       </c>
       <c r="W163" t="n">
-        <v>-9.300000000000001</v>
+        <v>-8.300000000000001</v>
       </c>
     </row>
     <row r="164">
@@ -11877,13 +11880,13 @@
         <v>0</v>
       </c>
       <c r="U164" t="n">
-        <v>130800</v>
+        <v>136500</v>
       </c>
       <c r="V164" t="n">
         <v>134000</v>
       </c>
       <c r="W164" t="n">
-        <v>-2.4</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="165">
@@ -11949,13 +11952,13 @@
         <v>0</v>
       </c>
       <c r="U165" t="n">
-        <v>202000</v>
+        <v>206000</v>
       </c>
       <c r="V165" t="n">
         <v>205000</v>
       </c>
       <c r="W165" t="n">
-        <v>-1.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="166">
@@ -12015,13 +12018,13 @@
         <v>-0</v>
       </c>
       <c r="U166" t="n">
-        <v>139500</v>
+        <v>134300</v>
       </c>
       <c r="V166" t="n">
         <v>136000</v>
       </c>
       <c r="W166" t="n">
-        <v>2.6</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="167">
@@ -12078,13 +12081,13 @@
         <v>0</v>
       </c>
       <c r="U167" t="n">
-        <v>6110</v>
+        <v>5740</v>
       </c>
       <c r="V167" t="n">
         <v>5950</v>
       </c>
       <c r="W167" t="n">
-        <v>2.7</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="168">
@@ -12150,13 +12153,13 @@
         <v>0.1</v>
       </c>
       <c r="U168" t="n">
-        <v>50400</v>
+        <v>50900</v>
       </c>
       <c r="V168" t="n">
         <v>47700</v>
       </c>
       <c r="W168" t="n">
-        <v>5.7</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="169">
@@ -12222,13 +12225,13 @@
         <v>0</v>
       </c>
       <c r="U169" t="n">
-        <v>51900</v>
+        <v>52800</v>
       </c>
       <c r="V169" t="n">
         <v>58000</v>
       </c>
       <c r="W169" t="n">
-        <v>-10.5</v>
+        <v>-9</v>
       </c>
     </row>
     <row r="170">
@@ -12294,13 +12297,13 @@
         <v>0.9</v>
       </c>
       <c r="U170" t="n">
-        <v>142500</v>
+        <v>143300</v>
       </c>
       <c r="V170" t="n">
         <v>150600</v>
       </c>
       <c r="W170" t="n">
-        <v>-5.4</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="171">
@@ -12339,13 +12342,13 @@
         <v>0</v>
       </c>
       <c r="U171" t="n">
-        <v>12250</v>
+        <v>12500</v>
       </c>
       <c r="V171" t="n">
         <v>12520</v>
       </c>
       <c r="W171" t="n">
-        <v>-2.2</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="172">
@@ -12405,13 +12408,13 @@
         <v>2.6</v>
       </c>
       <c r="U172" t="n">
-        <v>171700</v>
+        <v>182000</v>
       </c>
       <c r="V172" t="n">
         <v>173400</v>
       </c>
       <c r="W172" t="n">
-        <v>-1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="173">
@@ -12477,13 +12480,13 @@
         <v>0</v>
       </c>
       <c r="U173" t="n">
-        <v>133900</v>
+        <v>146800</v>
       </c>
       <c r="V173" t="n">
         <v>142700</v>
       </c>
       <c r="W173" t="n">
-        <v>-6.2</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="174">
@@ -12549,13 +12552,13 @@
         <v>6.1</v>
       </c>
       <c r="U174" t="n">
-        <v>17550</v>
+        <v>17910</v>
       </c>
       <c r="V174" t="n">
         <v>18470</v>
       </c>
       <c r="W174" t="n">
-        <v>-5</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="175">
@@ -12621,13 +12624,13 @@
         <v>0</v>
       </c>
       <c r="U175" t="n">
-        <v>31550</v>
+        <v>31900</v>
       </c>
       <c r="V175" t="n">
         <v>35650</v>
       </c>
       <c r="W175" t="n">
-        <v>-11.5</v>
+        <v>-10.5</v>
       </c>
     </row>
     <row r="176">
@@ -12693,13 +12696,13 @@
         <v>0</v>
       </c>
       <c r="U176" t="n">
-        <v>130800</v>
+        <v>138300</v>
       </c>
       <c r="V176" t="n">
         <v>116900</v>
       </c>
       <c r="W176" t="n">
-        <v>11.9</v>
+        <v>18.3</v>
       </c>
     </row>
     <row r="177">
@@ -12765,13 +12768,13 @@
         <v>0</v>
       </c>
       <c r="U177" t="n">
-        <v>185900</v>
+        <v>183400</v>
       </c>
       <c r="V177" t="n">
         <v>189300</v>
       </c>
       <c r="W177" t="n">
-        <v>-1.8</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="178">
@@ -12804,13 +12807,13 @@
         <v>151</v>
       </c>
       <c r="U178" t="n">
-        <v>27550</v>
+        <v>27900</v>
       </c>
       <c r="V178" t="n">
         <v>28700</v>
       </c>
       <c r="W178" t="n">
-        <v>-4</v>
+        <v>-2.8</v>
       </c>
     </row>
     <row r="179">
@@ -12948,13 +12951,13 @@
         <v>0</v>
       </c>
       <c r="U180" t="n">
-        <v>67400</v>
+        <v>70700</v>
       </c>
       <c r="V180" t="n">
         <v>74500</v>
       </c>
       <c r="W180" t="n">
-        <v>-9.5</v>
+        <v>-5.1</v>
       </c>
     </row>
     <row r="181">
@@ -13020,13 +13023,13 @@
         <v>0</v>
       </c>
       <c r="U181" t="n">
-        <v>78600</v>
+        <v>78400</v>
       </c>
       <c r="V181" t="n">
         <v>86400</v>
       </c>
       <c r="W181" t="n">
-        <v>-9</v>
+        <v>-9.300000000000001</v>
       </c>
     </row>
     <row r="182">
@@ -13086,13 +13089,13 @@
         <v>0</v>
       </c>
       <c r="U182" t="n">
-        <v>177900</v>
+        <v>172000</v>
       </c>
       <c r="V182" t="n">
         <v>171600</v>
       </c>
       <c r="W182" t="n">
-        <v>3.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="183">
@@ -13158,13 +13161,13 @@
         <v>-0.1</v>
       </c>
       <c r="U183" t="n">
-        <v>248500</v>
+        <v>304500</v>
       </c>
       <c r="V183" t="n">
         <v>242000</v>
       </c>
       <c r="W183" t="n">
-        <v>2.7</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="184">
@@ -13230,13 +13233,13 @@
         <v>0</v>
       </c>
       <c r="U184" t="n">
-        <v>75600</v>
+        <v>75000</v>
       </c>
       <c r="V184" t="n">
         <v>74300</v>
       </c>
       <c r="W184" t="n">
-        <v>1.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="185">
@@ -13302,13 +13305,13 @@
         <v>0</v>
       </c>
       <c r="U185" t="n">
-        <v>45900</v>
+        <v>46950</v>
       </c>
       <c r="V185" t="n">
         <v>49400</v>
       </c>
       <c r="W185" t="n">
-        <v>-7.1</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="186">
@@ -13347,13 +13350,13 @@
         <v>1.1</v>
       </c>
       <c r="U186" t="n">
-        <v>9390</v>
+        <v>9580</v>
       </c>
       <c r="V186" t="n">
         <v>9610</v>
       </c>
       <c r="W186" t="n">
-        <v>-2.3</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="187">
@@ -13419,13 +13422,13 @@
         <v>0</v>
       </c>
       <c r="U187" t="n">
-        <v>58200</v>
+        <v>55800</v>
       </c>
       <c r="V187" t="n">
         <v>56500</v>
       </c>
       <c r="W187" t="n">
-        <v>3</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="188">
@@ -13491,13 +13494,13 @@
         <v>0.1</v>
       </c>
       <c r="U188" t="n">
-        <v>40650</v>
+        <v>41950</v>
       </c>
       <c r="V188" t="n">
         <v>40450</v>
       </c>
       <c r="W188" t="n">
-        <v>0.5</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="189">
@@ -13563,13 +13566,13 @@
         <v>0</v>
       </c>
       <c r="U189" t="n">
-        <v>460500</v>
+        <v>473500</v>
       </c>
       <c r="V189" t="n">
         <v>509000</v>
       </c>
       <c r="W189" t="n">
-        <v>-9.5</v>
+        <v>-7</v>
       </c>
     </row>
     <row r="190">
@@ -13635,13 +13638,13 @@
         <v>0</v>
       </c>
       <c r="U190" t="n">
-        <v>224000</v>
+        <v>236500</v>
       </c>
       <c r="V190" t="n">
         <v>238500</v>
       </c>
       <c r="W190" t="n">
-        <v>-6.1</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="191">
@@ -13670,6 +13673,9 @@
           <t>KOSPI200</t>
         </is>
       </c>
+      <c r="F191" t="n">
+        <v>8497</v>
+      </c>
       <c r="L191" t="n">
         <v>32423.4</v>
       </c>
@@ -13698,13 +13704,13 @@
         <v>0</v>
       </c>
       <c r="U191" t="n">
-        <v>136900</v>
+        <v>135500</v>
       </c>
       <c r="V191" t="n">
         <v>122000</v>
       </c>
       <c r="W191" t="n">
-        <v>12.2</v>
+        <v>11.1</v>
       </c>
     </row>
     <row r="192">
@@ -13733,6 +13739,9 @@
           <t>KOSPI200</t>
         </is>
       </c>
+      <c r="F192" t="n">
+        <v>3418</v>
+      </c>
       <c r="L192" t="n">
         <v>10035.1</v>
       </c>
@@ -13761,13 +13770,13 @@
         <v>0</v>
       </c>
       <c r="U192" t="n">
-        <v>15820</v>
+        <v>15390</v>
       </c>
       <c r="V192" t="n">
         <v>15120</v>
       </c>
       <c r="W192" t="n">
-        <v>4.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="193">
@@ -13827,13 +13836,13 @@
         <v>0</v>
       </c>
       <c r="U193" t="n">
-        <v>19050</v>
+        <v>18120</v>
       </c>
       <c r="V193" t="n">
         <v>18120</v>
       </c>
       <c r="W193" t="n">
-        <v>5.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194">
@@ -13899,13 +13908,13 @@
         <v>0</v>
       </c>
       <c r="U194" t="n">
-        <v>73800</v>
+        <v>73500</v>
       </c>
       <c r="V194" t="n">
         <v>75100</v>
       </c>
       <c r="W194" t="n">
-        <v>-1.7</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="195">
@@ -13971,13 +13980,13 @@
         <v>0</v>
       </c>
       <c r="U195" t="n">
-        <v>254000</v>
+        <v>262500</v>
       </c>
       <c r="V195" t="n">
         <v>271000</v>
       </c>
       <c r="W195" t="n">
-        <v>-6.3</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="196">
@@ -14034,13 +14043,13 @@
         <v>-62.6</v>
       </c>
       <c r="U196" t="n">
-        <v>88300</v>
+        <v>92000</v>
       </c>
       <c r="V196" t="n">
         <v>101000</v>
       </c>
       <c r="W196" t="n">
-        <v>-12.6</v>
+        <v>-8.9</v>
       </c>
     </row>
     <row r="197">
@@ -14106,13 +14115,13 @@
         <v>0.1</v>
       </c>
       <c r="U197" t="n">
-        <v>240500</v>
+        <v>244000</v>
       </c>
       <c r="V197" t="n">
         <v>259000</v>
       </c>
       <c r="W197" t="n">
-        <v>-7.1</v>
+        <v>-5.8</v>
       </c>
     </row>
     <row r="198">
@@ -14178,13 +14187,13 @@
         <v>0</v>
       </c>
       <c r="U198" t="n">
-        <v>37250</v>
+        <v>37550</v>
       </c>
       <c r="V198" t="n">
         <v>38200</v>
       </c>
       <c r="W198" t="n">
-        <v>-2.5</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="199">
@@ -14217,13 +14226,13 @@
         <v>27</v>
       </c>
       <c r="U199" t="n">
-        <v>9360</v>
+        <v>9440</v>
       </c>
       <c r="V199" t="n">
         <v>9960</v>
       </c>
       <c r="W199" t="n">
-        <v>-6</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="200">
@@ -14289,13 +14298,13 @@
         <v>0</v>
       </c>
       <c r="U200" t="n">
-        <v>66500</v>
+        <v>65400</v>
       </c>
       <c r="V200" t="n">
         <v>66400</v>
       </c>
       <c r="W200" t="n">
-        <v>0.2</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="201">
@@ -14361,13 +14370,13 @@
         <v>0</v>
       </c>
       <c r="U201" t="n">
-        <v>150600</v>
+        <v>145800</v>
       </c>
       <c r="V201" t="n">
         <v>161700</v>
       </c>
       <c r="W201" t="n">
-        <v>-6.9</v>
+        <v>-9.800000000000001</v>
       </c>
     </row>
     <row r="202">
@@ -14433,13 +14442,13 @@
         <v>0</v>
       </c>
       <c r="U202" t="n">
-        <v>36900</v>
+        <v>36950</v>
       </c>
       <c r="V202" t="n">
         <v>38250</v>
       </c>
       <c r="W202" t="n">
-        <v>-3.5</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="203">
@@ -14468,6 +14477,9 @@
           <t>KOSPI200</t>
         </is>
       </c>
+      <c r="F203" t="n">
+        <v>3043</v>
+      </c>
       <c r="L203" t="n">
         <v>10225.2</v>
       </c>
@@ -14496,13 +14508,13 @@
         <v>0</v>
       </c>
       <c r="U203" t="n">
-        <v>31600</v>
+        <v>31000</v>
       </c>
       <c r="V203" t="n">
         <v>29050</v>
       </c>
       <c r="W203" t="n">
-        <v>8.800000000000001</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="204">
@@ -14568,13 +14580,13 @@
         <v>0</v>
       </c>
       <c r="U204" t="n">
-        <v>33200</v>
+        <v>33650</v>
       </c>
       <c r="V204" t="n">
         <v>38950</v>
       </c>
       <c r="W204" t="n">
-        <v>-14.8</v>
+        <v>-13.6</v>
       </c>
     </row>
     <row r="205">
@@ -14640,13 +14652,13 @@
         <v>0</v>
       </c>
       <c r="U205" t="n">
-        <v>68200</v>
+        <v>68000</v>
       </c>
       <c r="V205" t="n">
         <v>68500</v>
       </c>
       <c r="W205" t="n">
-        <v>-0.4</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="206">
@@ -14712,13 +14724,13 @@
         <v>0</v>
       </c>
       <c r="U206" t="n">
-        <v>60700</v>
+        <v>63100</v>
       </c>
       <c r="V206" t="n">
         <v>63800</v>
       </c>
       <c r="W206" t="n">
-        <v>-4.9</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="207">
@@ -14784,13 +14796,13 @@
         <v>-1.3</v>
       </c>
       <c r="U207" t="n">
-        <v>58000</v>
+        <v>57200</v>
       </c>
       <c r="V207" t="n">
         <v>59200</v>
       </c>
       <c r="W207" t="n">
-        <v>-2</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="208">
@@ -14856,13 +14868,13 @@
         <v>0</v>
       </c>
       <c r="U208" t="n">
-        <v>282000</v>
+        <v>275500</v>
       </c>
       <c r="V208" t="n">
         <v>303000</v>
       </c>
       <c r="W208" t="n">
-        <v>-6.9</v>
+        <v>-9.1</v>
       </c>
     </row>
     <row r="209">
@@ -14928,13 +14940,13 @@
         <v>0</v>
       </c>
       <c r="U209" t="n">
-        <v>41750</v>
+        <v>42050</v>
       </c>
       <c r="V209" t="n">
         <v>43650</v>
       </c>
       <c r="W209" t="n">
-        <v>-4.4</v>
+        <v>-3.7</v>
       </c>
     </row>
     <row r="210">
@@ -14973,40 +14985,40 @@
         <v>0</v>
       </c>
       <c r="L210" t="n">
-        <v>2641.5</v>
+        <v>2885.2</v>
       </c>
       <c r="M210" t="n">
         <v>2641.5</v>
       </c>
       <c r="N210" t="n">
-        <v>0</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O210" t="n">
-        <v>4463</v>
+        <v>4519.2</v>
       </c>
       <c r="P210" t="n">
         <v>4463</v>
       </c>
       <c r="Q210" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="R210" t="n">
-        <v>5872.8</v>
+        <v>6203</v>
       </c>
       <c r="S210" t="n">
         <v>5872.8</v>
       </c>
       <c r="T210" t="n">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="U210" t="n">
-        <v>283000</v>
+        <v>288500</v>
       </c>
       <c r="V210" t="n">
         <v>320000</v>
       </c>
       <c r="W210" t="n">
-        <v>-11.6</v>
+        <v>-9.800000000000001</v>
       </c>
     </row>
     <row r="211">
@@ -15072,13 +15084,13 @@
         <v>0</v>
       </c>
       <c r="U211" t="n">
-        <v>47650</v>
+        <v>48500</v>
       </c>
       <c r="V211" t="n">
         <v>50300</v>
       </c>
       <c r="W211" t="n">
-        <v>-5.3</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="212">
@@ -15144,13 +15156,13 @@
         <v>0</v>
       </c>
       <c r="U212" t="n">
-        <v>1477000</v>
+        <v>1447000</v>
       </c>
       <c r="V212" t="n">
         <v>1486000</v>
       </c>
       <c r="W212" t="n">
-        <v>-0.6</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="213">
@@ -15216,13 +15228,13 @@
         <v>0</v>
       </c>
       <c r="U213" t="n">
-        <v>31700</v>
+        <v>31800</v>
       </c>
       <c r="V213" t="n">
         <v>33250</v>
       </c>
       <c r="W213" t="n">
-        <v>-4.7</v>
+        <v>-4.4</v>
       </c>
     </row>
     <row r="214">
@@ -15288,13 +15300,13 @@
         <v>0.3</v>
       </c>
       <c r="U214" t="n">
-        <v>381000</v>
+        <v>386500</v>
       </c>
       <c r="V214" t="n">
         <v>461500</v>
       </c>
       <c r="W214" t="n">
-        <v>-17.4</v>
+        <v>-16.3</v>
       </c>
     </row>
     <row r="215">
@@ -15360,13 +15372,13 @@
         <v>0</v>
       </c>
       <c r="U215" t="n">
-        <v>46400</v>
+        <v>48300</v>
       </c>
       <c r="V215" t="n">
         <v>46800</v>
       </c>
       <c r="W215" t="n">
-        <v>-0.9</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="216">
@@ -15432,13 +15444,13 @@
         <v>0</v>
       </c>
       <c r="U216" t="n">
-        <v>117500</v>
+        <v>117900</v>
       </c>
       <c r="V216" t="n">
         <v>122800</v>
       </c>
       <c r="W216" t="n">
-        <v>-4.3</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="217">
@@ -15498,13 +15510,13 @@
         <v>0</v>
       </c>
       <c r="U217" t="n">
-        <v>99000</v>
+        <v>101200</v>
       </c>
       <c r="V217" t="n">
         <v>110200</v>
       </c>
       <c r="W217" t="n">
-        <v>-10.2</v>
+        <v>-8.199999999999999</v>
       </c>
     </row>
     <row r="218">
@@ -15570,13 +15582,13 @@
         <v>0</v>
       </c>
       <c r="U218" t="n">
-        <v>105000</v>
+        <v>114800</v>
       </c>
       <c r="V218" t="n">
         <v>111100</v>
       </c>
       <c r="W218" t="n">
-        <v>-5.5</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="219">
@@ -15714,13 +15726,13 @@
         <v>0</v>
       </c>
       <c r="U220" t="n">
-        <v>134200</v>
+        <v>134500</v>
       </c>
       <c r="V220" t="n">
         <v>153900</v>
       </c>
       <c r="W220" t="n">
-        <v>-12.8</v>
+        <v>-12.6</v>
       </c>
     </row>
     <row r="221">
@@ -15786,13 +15798,13 @@
         <v>0</v>
       </c>
       <c r="U221" t="n">
-        <v>106500</v>
+        <v>106000</v>
       </c>
       <c r="V221" t="n">
         <v>118200</v>
       </c>
       <c r="W221" t="n">
-        <v>-9.9</v>
+        <v>-10.3</v>
       </c>
     </row>
     <row r="222">
@@ -15858,13 +15870,13 @@
         <v>-3.4</v>
       </c>
       <c r="U222" t="n">
-        <v>36700</v>
+        <v>36300</v>
       </c>
       <c r="V222" t="n">
         <v>37450</v>
       </c>
       <c r="W222" t="n">
-        <v>-2</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="223">
@@ -15930,13 +15942,13 @@
         <v>0</v>
       </c>
       <c r="U223" t="n">
-        <v>57500</v>
+        <v>55300</v>
       </c>
       <c r="V223" t="n">
         <v>61700</v>
       </c>
       <c r="W223" t="n">
-        <v>-6.8</v>
+        <v>-10.4</v>
       </c>
     </row>
     <row r="224">
@@ -15996,13 +16008,13 @@
         <v>0</v>
       </c>
       <c r="U224" t="n">
-        <v>21200</v>
+        <v>21650</v>
       </c>
       <c r="V224" t="n">
         <v>22000</v>
       </c>
       <c r="W224" t="n">
-        <v>-3.6</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="225">
@@ -16068,13 +16080,13 @@
         <v>0</v>
       </c>
       <c r="U225" t="n">
-        <v>48500</v>
+        <v>48000</v>
       </c>
       <c r="V225" t="n">
         <v>53300</v>
       </c>
       <c r="W225" t="n">
-        <v>-9</v>
+        <v>-9.9</v>
       </c>
     </row>
     <row r="226">
@@ -16140,13 +16152,13 @@
         <v>-0.3</v>
       </c>
       <c r="U226" t="n">
-        <v>218000</v>
+        <v>216500</v>
       </c>
       <c r="V226" t="n">
         <v>222500</v>
       </c>
       <c r="W226" t="n">
-        <v>-2</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="227">
@@ -16206,13 +16218,13 @@
         <v>0</v>
       </c>
       <c r="U227" t="n">
-        <v>30950</v>
+        <v>34500</v>
       </c>
       <c r="V227" t="n">
         <v>32500</v>
       </c>
       <c r="W227" t="n">
-        <v>-4.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="228">
@@ -16278,13 +16290,13 @@
         <v>0</v>
       </c>
       <c r="U228" t="n">
-        <v>213500</v>
+        <v>240500</v>
       </c>
       <c r="V228" t="n">
         <v>218000</v>
       </c>
       <c r="W228" t="n">
-        <v>-2.1</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="229">
@@ -16350,13 +16362,13 @@
         <v>0</v>
       </c>
       <c r="U229" t="n">
-        <v>706000</v>
+        <v>714000</v>
       </c>
       <c r="V229" t="n">
         <v>814000</v>
       </c>
       <c r="W229" t="n">
-        <v>-13.3</v>
+        <v>-12.3</v>
       </c>
     </row>
     <row r="230">
@@ -16422,13 +16434,13 @@
         <v>0</v>
       </c>
       <c r="U230" t="n">
-        <v>135300</v>
+        <v>140000</v>
       </c>
       <c r="V230" t="n">
         <v>136600</v>
       </c>
       <c r="W230" t="n">
-        <v>-1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="231">
@@ -16494,13 +16506,13 @@
         <v>0</v>
       </c>
       <c r="U231" t="n">
-        <v>129300</v>
+        <v>126300</v>
       </c>
       <c r="V231" t="n">
         <v>129500</v>
       </c>
       <c r="W231" t="n">
-        <v>-0.2</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="232">
@@ -16566,13 +16578,13 @@
         <v>1</v>
       </c>
       <c r="U232" t="n">
-        <v>68000</v>
+        <v>68800</v>
       </c>
       <c r="V232" t="n">
         <v>75800</v>
       </c>
       <c r="W232" t="n">
-        <v>-10.3</v>
+        <v>-9.199999999999999</v>
       </c>
     </row>
     <row r="233">
@@ -16638,13 +16650,13 @@
         <v>0</v>
       </c>
       <c r="U233" t="n">
-        <v>5820</v>
+        <v>6140</v>
       </c>
       <c r="V233" t="n">
         <v>5910</v>
       </c>
       <c r="W233" t="n">
-        <v>-1.5</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="234">
@@ -16701,13 +16713,13 @@
         <v>0</v>
       </c>
       <c r="U234" t="n">
-        <v>436500</v>
+        <v>459000</v>
       </c>
       <c r="V234" t="n">
         <v>456000</v>
       </c>
       <c r="W234" t="n">
-        <v>-4.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="235">
@@ -16773,13 +16785,13 @@
         <v>0</v>
       </c>
       <c r="U235" t="n">
-        <v>406000</v>
+        <v>394000</v>
       </c>
       <c r="V235" t="n">
         <v>461500</v>
       </c>
       <c r="W235" t="n">
-        <v>-12</v>
+        <v>-14.6</v>
       </c>
     </row>
     <row r="236">
@@ -16845,13 +16857,13 @@
         <v>0.4</v>
       </c>
       <c r="U236" t="n">
-        <v>146600</v>
+        <v>145500</v>
       </c>
       <c r="V236" t="n">
         <v>146300</v>
       </c>
       <c r="W236" t="n">
-        <v>0.2</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="237">
@@ -16917,13 +16929,13 @@
         <v>0</v>
       </c>
       <c r="U237" t="n">
-        <v>150600</v>
+        <v>147600</v>
       </c>
       <c r="V237" t="n">
         <v>147000</v>
       </c>
       <c r="W237" t="n">
-        <v>2.4</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="238">
@@ -16989,13 +17001,13 @@
         <v>0</v>
       </c>
       <c r="U238" t="n">
-        <v>54900</v>
+        <v>55200</v>
       </c>
       <c r="V238" t="n">
         <v>54200</v>
       </c>
       <c r="W238" t="n">
-        <v>1.3</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="239">
@@ -17061,13 +17073,13 @@
         <v>0</v>
       </c>
       <c r="U239" t="n">
-        <v>23200</v>
+        <v>23300</v>
       </c>
       <c r="V239" t="n">
         <v>23150</v>
       </c>
       <c r="W239" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="240">
@@ -17133,13 +17145,13 @@
         <v>0</v>
       </c>
       <c r="U240" t="n">
-        <v>354500</v>
+        <v>347000</v>
       </c>
       <c r="V240" t="n">
         <v>346000</v>
       </c>
       <c r="W240" t="n">
-        <v>2.5</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="241">
@@ -17205,13 +17217,13 @@
         <v>0</v>
       </c>
       <c r="U241" t="n">
-        <v>2725000</v>
+        <v>2732000</v>
       </c>
       <c r="V241" t="n">
         <v>3153000</v>
       </c>
       <c r="W241" t="n">
-        <v>-13.6</v>
+        <v>-13.4</v>
       </c>
     </row>
     <row r="242">
@@ -17277,13 +17289,13 @@
         <v>0</v>
       </c>
       <c r="U242" t="n">
-        <v>175300</v>
+        <v>172800</v>
       </c>
       <c r="V242" t="n">
         <v>178800</v>
       </c>
       <c r="W242" t="n">
-        <v>-2</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="243">
@@ -17349,13 +17361,13 @@
         <v>0</v>
       </c>
       <c r="U243" t="n">
-        <v>16780</v>
+        <v>16670</v>
       </c>
       <c r="V243" t="n">
         <v>16950</v>
       </c>
       <c r="W243" t="n">
-        <v>-1</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="244">
@@ -17412,13 +17424,13 @@
         <v>0</v>
       </c>
       <c r="U244" t="n">
-        <v>37750</v>
+        <v>37900</v>
       </c>
       <c r="V244" t="n">
         <v>38950</v>
       </c>
       <c r="W244" t="n">
-        <v>-3.1</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="245">
@@ -17484,13 +17496,13 @@
         <v>-1.3</v>
       </c>
       <c r="U245" t="n">
-        <v>147500</v>
+        <v>144700</v>
       </c>
       <c r="V245" t="n">
         <v>139300</v>
       </c>
       <c r="W245" t="n">
-        <v>5.9</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="246">
@@ -17556,13 +17568,13 @@
         <v>0</v>
       </c>
       <c r="U246" t="n">
-        <v>384500</v>
+        <v>395000</v>
       </c>
       <c r="V246" t="n">
         <v>416000</v>
       </c>
       <c r="W246" t="n">
-        <v>-7.6</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="247">
@@ -17622,13 +17634,13 @@
         <v>0</v>
       </c>
       <c r="U247" t="n">
-        <v>34650</v>
+        <v>33200</v>
       </c>
       <c r="V247" t="n">
         <v>33900</v>
       </c>
       <c r="W247" t="n">
-        <v>2.2</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="248">
@@ -17694,13 +17706,13 @@
         <v>0</v>
       </c>
       <c r="U248" t="n">
-        <v>11240</v>
+        <v>11230</v>
       </c>
       <c r="V248" t="n">
         <v>11250</v>
       </c>
       <c r="W248" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="249">
@@ -17766,13 +17778,13 @@
         <v>0</v>
       </c>
       <c r="U249" t="n">
-        <v>122400</v>
+        <v>126500</v>
       </c>
       <c r="V249" t="n">
         <v>128600</v>
       </c>
       <c r="W249" t="n">
-        <v>-4.8</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="250">
@@ -17832,13 +17844,13 @@
         <v>0</v>
       </c>
       <c r="U250" t="n">
-        <v>21800</v>
+        <v>21950</v>
       </c>
       <c r="V250" t="n">
         <v>21850</v>
       </c>
       <c r="W250" t="n">
-        <v>-0.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="251">
@@ -17904,13 +17916,13 @@
         <v>0</v>
       </c>
       <c r="U251" t="n">
-        <v>86400</v>
+        <v>86600</v>
       </c>
       <c r="V251" t="n">
         <v>88000</v>
       </c>
       <c r="W251" t="n">
-        <v>-1.8</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="252">
@@ -17976,13 +17988,13 @@
         <v>0</v>
       </c>
       <c r="U252" t="n">
-        <v>435000</v>
+        <v>436500</v>
       </c>
       <c r="V252" t="n">
         <v>457000</v>
       </c>
       <c r="W252" t="n">
-        <v>-4.8</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="253">
@@ -18048,13 +18060,13 @@
         <v>0</v>
       </c>
       <c r="U253" t="n">
-        <v>176000</v>
+        <v>178500</v>
       </c>
       <c r="V253" t="n">
         <v>180000</v>
       </c>
       <c r="W253" t="n">
-        <v>-2.2</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="254">
@@ -18120,13 +18132,13 @@
         <v>-0.7</v>
       </c>
       <c r="U254" t="n">
-        <v>101600</v>
+        <v>99500</v>
       </c>
       <c r="V254" t="n">
         <v>107600</v>
       </c>
       <c r="W254" t="n">
-        <v>-5.6</v>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="255">
@@ -18192,13 +18204,13 @@
         <v>-2.3</v>
       </c>
       <c r="U255" t="n">
-        <v>319500</v>
+        <v>325000</v>
       </c>
       <c r="V255" t="n">
         <v>346500</v>
       </c>
       <c r="W255" t="n">
-        <v>-7.8</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="256">
@@ -18264,13 +18276,13 @@
         <v>0</v>
       </c>
       <c r="U256" t="n">
-        <v>15790</v>
+        <v>16280</v>
       </c>
       <c r="V256" t="n">
         <v>16680</v>
       </c>
       <c r="W256" t="n">
-        <v>-5.3</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="257">
@@ -18336,13 +18348,13 @@
         <v>0</v>
       </c>
       <c r="U257" t="n">
-        <v>365500</v>
+        <v>358500</v>
       </c>
       <c r="V257" t="n">
         <v>370000</v>
       </c>
       <c r="W257" t="n">
-        <v>-1.2</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="258">
@@ -18408,13 +18420,13 @@
         <v>0</v>
       </c>
       <c r="U258" t="n">
-        <v>72500</v>
+        <v>73400</v>
       </c>
       <c r="V258" t="n">
         <v>73300</v>
       </c>
       <c r="W258" t="n">
-        <v>-1.1</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="259">
@@ -18480,13 +18492,13 @@
         <v>0</v>
       </c>
       <c r="U259" t="n">
-        <v>17810</v>
+        <v>18060</v>
       </c>
       <c r="V259" t="n">
         <v>18910</v>
       </c>
       <c r="W259" t="n">
-        <v>-5.8</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="260">
@@ -18552,13 +18564,13 @@
         <v>0</v>
       </c>
       <c r="U260" t="n">
-        <v>44800</v>
+        <v>47300</v>
       </c>
       <c r="V260" t="n">
         <v>47350</v>
       </c>
       <c r="W260" t="n">
-        <v>-5.4</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="261">
@@ -18624,13 +18636,13 @@
         <v>0</v>
       </c>
       <c r="U261" t="n">
-        <v>66300</v>
+        <v>66900</v>
       </c>
       <c r="V261" t="n">
         <v>66900</v>
       </c>
       <c r="W261" t="n">
-        <v>-0.9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262">
@@ -18669,13 +18681,13 @@
         <v>0</v>
       </c>
       <c r="U262" t="n">
-        <v>34600</v>
+        <v>37750</v>
       </c>
       <c r="V262" t="n">
         <v>37900</v>
       </c>
       <c r="W262" t="n">
-        <v>-8.699999999999999</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="263">
@@ -18714,13 +18726,13 @@
         <v>-40</v>
       </c>
       <c r="U263" t="n">
-        <v>31100</v>
+        <v>31050</v>
       </c>
       <c r="V263" t="n">
         <v>33000</v>
       </c>
       <c r="W263" t="n">
-        <v>-5.8</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="264">
@@ -18780,13 +18792,13 @@
         <v>2.5</v>
       </c>
       <c r="U264" t="n">
-        <v>981000</v>
+        <v>1041000</v>
       </c>
       <c r="V264" t="n">
         <v>1028000</v>
       </c>
       <c r="W264" t="n">
-        <v>-4.6</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="265">
@@ -18816,22 +18828,22 @@
         </is>
       </c>
       <c r="F265" t="n">
-        <v>314</v>
+        <v>298</v>
       </c>
       <c r="G265" t="n">
         <v>314</v>
       </c>
       <c r="H265" t="n">
-        <v>0</v>
+        <v>-5.1</v>
       </c>
       <c r="U265" t="n">
-        <v>50200</v>
+        <v>50800</v>
       </c>
       <c r="V265" t="n">
         <v>51100</v>
       </c>
       <c r="W265" t="n">
-        <v>-1.8</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="266">
@@ -18897,13 +18909,13 @@
         <v>0</v>
       </c>
       <c r="U266" t="n">
-        <v>99900</v>
+        <v>101200</v>
       </c>
       <c r="V266" t="n">
         <v>109800</v>
       </c>
       <c r="W266" t="n">
-        <v>-9</v>
+        <v>-7.8</v>
       </c>
     </row>
     <row r="267">
@@ -18969,13 +18981,13 @@
         <v>0</v>
       </c>
       <c r="U267" t="n">
-        <v>46600</v>
+        <v>46950</v>
       </c>
       <c r="V267" t="n">
         <v>49000</v>
       </c>
       <c r="W267" t="n">
-        <v>-4.9</v>
+        <v>-4.2</v>
       </c>
     </row>
     <row r="268">
@@ -19041,13 +19053,13 @@
         <v>0</v>
       </c>
       <c r="U268" t="n">
-        <v>61500</v>
+        <v>67300</v>
       </c>
       <c r="V268" t="n">
         <v>63300</v>
       </c>
       <c r="W268" t="n">
-        <v>-2.8</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="269">
@@ -19113,13 +19125,13 @@
         <v>0</v>
       </c>
       <c r="U269" t="n">
-        <v>205500</v>
+        <v>210500</v>
       </c>
       <c r="V269" t="n">
         <v>221000</v>
       </c>
       <c r="W269" t="n">
-        <v>-7</v>
+        <v>-4.8</v>
       </c>
     </row>
     <row r="270">
@@ -19185,13 +19197,13 @@
         <v>0</v>
       </c>
       <c r="U270" t="n">
-        <v>79800</v>
+        <v>79300</v>
       </c>
       <c r="V270" t="n">
         <v>82000</v>
       </c>
       <c r="W270" t="n">
-        <v>-2.7</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="271">
@@ -19257,13 +19269,13 @@
         <v>0</v>
       </c>
       <c r="U271" t="n">
-        <v>10670</v>
+        <v>10510</v>
       </c>
       <c r="V271" t="n">
         <v>10380</v>
       </c>
       <c r="W271" t="n">
-        <v>2.8</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="272">
@@ -19329,13 +19341,13 @@
         <v>-3.8</v>
       </c>
       <c r="U272" t="n">
-        <v>32000</v>
+        <v>31850</v>
       </c>
       <c r="V272" t="n">
         <v>32900</v>
       </c>
       <c r="W272" t="n">
-        <v>-2.7</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="273">
@@ -19401,7 +19413,7 @@
         <v>0</v>
       </c>
       <c r="U273" t="n">
-        <v>190500</v>
+        <v>190600</v>
       </c>
       <c r="V273" t="n">
         <v>229000</v>
@@ -19437,49 +19449,49 @@
         </is>
       </c>
       <c r="F274" t="n">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="G274" t="n">
         <v>142</v>
       </c>
       <c r="H274" t="n">
-        <v>0</v>
+        <v>-14.1</v>
       </c>
       <c r="L274" t="n">
-        <v>636</v>
+        <v>571</v>
       </c>
       <c r="M274" t="n">
         <v>636</v>
       </c>
       <c r="N274" t="n">
-        <v>0</v>
+        <v>-10.2</v>
       </c>
       <c r="O274" t="n">
-        <v>847</v>
+        <v>733</v>
       </c>
       <c r="P274" t="n">
         <v>847</v>
       </c>
       <c r="Q274" t="n">
-        <v>0</v>
+        <v>-13.5</v>
       </c>
       <c r="R274" t="n">
-        <v>1111</v>
+        <v>948</v>
       </c>
       <c r="S274" t="n">
         <v>1111</v>
       </c>
       <c r="T274" t="n">
-        <v>0</v>
+        <v>-14.7</v>
       </c>
       <c r="U274" t="n">
-        <v>17280</v>
+        <v>16560</v>
       </c>
       <c r="V274" t="n">
         <v>15110</v>
       </c>
       <c r="W274" t="n">
-        <v>14.4</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="275">
@@ -19545,13 +19557,13 @@
         <v>0</v>
       </c>
       <c r="U275" t="n">
-        <v>48700</v>
+        <v>49400</v>
       </c>
       <c r="V275" t="n">
         <v>50200</v>
       </c>
       <c r="W275" t="n">
-        <v>-3</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="276">
@@ -19590,13 +19602,13 @@
         <v>0</v>
       </c>
       <c r="U276" t="n">
-        <v>33300</v>
+        <v>34500</v>
       </c>
       <c r="V276" t="n">
         <v>33450</v>
       </c>
       <c r="W276" t="n">
-        <v>-0.4</v>
+        <v>3.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-09-05
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -458,7 +458,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-09-04 · 전주 2026-08-30</t>
+          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-09-05 · 전주 2026-08-30</t>
         </is>
       </c>
     </row>
@@ -1325,6 +1325,9 @@
           <t>KOSPI200</t>
         </is>
       </c>
+      <c r="F13" t="n">
+        <v>7942</v>
+      </c>
       <c r="L13" t="n">
         <v>31986.2</v>
       </c>
@@ -1923,40 +1926,40 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="G22" t="n">
         <v>415</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="L22" t="n">
-        <v>1771.6</v>
+        <v>1757.7</v>
       </c>
       <c r="M22" t="n">
         <v>1771.6</v>
       </c>
       <c r="N22" t="n">
-        <v>0</v>
+        <v>-0.8</v>
       </c>
       <c r="O22" t="n">
-        <v>2132.2</v>
+        <v>2107.1</v>
       </c>
       <c r="P22" t="n">
         <v>2132.2</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="R22" t="n">
-        <v>2400.2</v>
+        <v>2357.9</v>
       </c>
       <c r="S22" t="n">
         <v>2400.2</v>
       </c>
       <c r="T22" t="n">
-        <v>0</v>
+        <v>-1.8</v>
       </c>
       <c r="U22" t="n">
         <v>6080</v>
@@ -3354,31 +3357,31 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1145149</v>
+        <v>1141888</v>
       </c>
       <c r="G42" t="n">
         <v>1145149</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="L42" t="n">
-        <v>3933478.7</v>
+        <v>3927530.9</v>
       </c>
       <c r="M42" t="n">
         <v>3917860.4</v>
       </c>
       <c r="N42" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="O42" t="n">
-        <v>5542251.7</v>
+        <v>5533556</v>
       </c>
       <c r="P42" t="n">
         <v>5433530.8</v>
       </c>
       <c r="Q42" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="R42" t="n">
         <v>5520887.9</v>
@@ -3777,25 +3780,25 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1014</v>
+        <v>1047</v>
       </c>
       <c r="G48" t="n">
         <v>995</v>
       </c>
       <c r="H48" t="n">
-        <v>1.9</v>
+        <v>5.2</v>
       </c>
       <c r="L48" t="n">
-        <v>3621.1</v>
+        <v>3662.4</v>
       </c>
       <c r="M48" t="n">
         <v>3521.7</v>
       </c>
       <c r="N48" t="n">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="O48" t="n">
-        <v>14400.7</v>
+        <v>14401.2</v>
       </c>
       <c r="P48" t="n">
         <v>14225.1</v>
@@ -7437,13 +7440,13 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="G100" t="n">
         <v>656</v>
       </c>
       <c r="H100" t="n">
-        <v>-1.1</v>
+        <v>-1.2</v>
       </c>
       <c r="U100" t="n">
         <v>12530</v>
@@ -7553,6 +7556,9 @@
           <t>KOSPI200</t>
         </is>
       </c>
+      <c r="F102" t="n">
+        <v>8596</v>
+      </c>
       <c r="L102" t="n">
         <v>34544.2</v>
       </c>
@@ -7908,22 +7914,22 @@
         <v>0</v>
       </c>
       <c r="L107" t="n">
-        <v>1651.7</v>
+        <v>1685.7</v>
       </c>
       <c r="M107" t="n">
         <v>1651.7</v>
       </c>
       <c r="N107" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="O107" t="n">
-        <v>2027.3</v>
+        <v>2065.2</v>
       </c>
       <c r="P107" t="n">
         <v>2027.3</v>
       </c>
       <c r="Q107" t="n">
-        <v>0</v>
+        <v>1.9</v>
       </c>
       <c r="R107" t="n">
         <v>2403.4</v>
@@ -8061,13 +8067,13 @@
         <v>-0.9</v>
       </c>
       <c r="O109" t="n">
-        <v>2218.8</v>
+        <v>2201</v>
       </c>
       <c r="P109" t="n">
         <v>2217.5</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.1</v>
+        <v>-0.7</v>
       </c>
       <c r="R109" t="n">
         <v>2580</v>
@@ -8340,22 +8346,22 @@
         <v>0</v>
       </c>
       <c r="L113" t="n">
-        <v>1529.1</v>
+        <v>1525.1</v>
       </c>
       <c r="M113" t="n">
         <v>1529.1</v>
       </c>
       <c r="N113" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="O113" t="n">
-        <v>1681.4</v>
+        <v>1673.1</v>
       </c>
       <c r="P113" t="n">
         <v>1681.4</v>
       </c>
       <c r="Q113" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="R113" t="n">
         <v>1679.3</v>
@@ -8979,13 +8985,13 @@
         <v>0</v>
       </c>
       <c r="L122" t="n">
-        <v>1886.6</v>
+        <v>1880.3</v>
       </c>
       <c r="M122" t="n">
         <v>1886.6</v>
       </c>
       <c r="N122" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="O122" t="n">
         <v>2167.6</v>
@@ -9330,13 +9336,13 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>895</v>
+        <v>872</v>
       </c>
       <c r="G127" t="n">
         <v>895</v>
       </c>
       <c r="H127" t="n">
-        <v>0</v>
+        <v>-2.6</v>
       </c>
       <c r="L127" t="n">
         <v>3569.9</v>
@@ -9612,40 +9618,40 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>2233</v>
+        <v>1906</v>
       </c>
       <c r="G131" t="n">
         <v>2233</v>
       </c>
       <c r="H131" t="n">
-        <v>0</v>
+        <v>-14.6</v>
       </c>
       <c r="L131" t="n">
-        <v>13021.5</v>
+        <v>12712.8</v>
       </c>
       <c r="M131" t="n">
         <v>13021.5</v>
       </c>
       <c r="N131" t="n">
-        <v>0</v>
+        <v>-2.4</v>
       </c>
       <c r="O131" t="n">
-        <v>39507.7</v>
+        <v>38502.2</v>
       </c>
       <c r="P131" t="n">
         <v>39507.7</v>
       </c>
       <c r="Q131" t="n">
-        <v>0</v>
+        <v>-2.5</v>
       </c>
       <c r="R131" t="n">
-        <v>55674.8</v>
+        <v>53851.1</v>
       </c>
       <c r="S131" t="n">
         <v>55674.8</v>
       </c>
       <c r="T131" t="n">
-        <v>0</v>
+        <v>-3.3</v>
       </c>
       <c r="U131" t="n">
         <v>282000</v>
@@ -11517,40 +11523,40 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>1054</v>
+        <v>1065</v>
       </c>
       <c r="G159" t="n">
         <v>1054</v>
       </c>
       <c r="H159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L159" t="n">
-        <v>4475.1</v>
+        <v>4486.7</v>
       </c>
       <c r="M159" t="n">
         <v>4475.1</v>
       </c>
       <c r="N159" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="O159" t="n">
-        <v>6270.8</v>
+        <v>6274.2</v>
       </c>
       <c r="P159" t="n">
         <v>6270.8</v>
       </c>
       <c r="Q159" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R159" t="n">
-        <v>8419.6</v>
+        <v>8410.1</v>
       </c>
       <c r="S159" t="n">
         <v>8419.6</v>
       </c>
       <c r="T159" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="U159" t="n">
         <v>652000</v>
@@ -12053,6 +12059,9 @@
           <t>KOSPI200</t>
         </is>
       </c>
+      <c r="F167" t="n">
+        <v>4601</v>
+      </c>
       <c r="L167" t="n">
         <v>9399.1</v>
       </c>
@@ -13476,13 +13485,13 @@
         <v>0</v>
       </c>
       <c r="O188" t="n">
-        <v>709.1</v>
+        <v>709.9</v>
       </c>
       <c r="P188" t="n">
         <v>709.2</v>
       </c>
       <c r="Q188" t="n">
-        <v>-0</v>
+        <v>0.1</v>
       </c>
       <c r="R188" t="n">
         <v>831.4</v>
@@ -14985,13 +14994,13 @@
         <v>0</v>
       </c>
       <c r="L210" t="n">
-        <v>2885.2</v>
+        <v>2886.2</v>
       </c>
       <c r="M210" t="n">
         <v>2641.5</v>
       </c>
       <c r="N210" t="n">
-        <v>9.199999999999999</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="O210" t="n">
         <v>4519.2</v>
@@ -15546,31 +15555,31 @@
         </is>
       </c>
       <c r="F218" t="n">
-        <v>695</v>
+        <v>709</v>
       </c>
       <c r="G218" t="n">
         <v>695</v>
       </c>
       <c r="H218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L218" t="n">
-        <v>1838.7</v>
+        <v>1794.3</v>
       </c>
       <c r="M218" t="n">
         <v>1838.7</v>
       </c>
       <c r="N218" t="n">
-        <v>0</v>
+        <v>-2.4</v>
       </c>
       <c r="O218" t="n">
-        <v>2755.7</v>
+        <v>2739.7</v>
       </c>
       <c r="P218" t="n">
         <v>2755.7</v>
       </c>
       <c r="Q218" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="R218" t="n">
         <v>3478.3</v>
@@ -15618,40 +15627,40 @@
         </is>
       </c>
       <c r="F219" t="n">
-        <v>1756</v>
+        <v>1851</v>
       </c>
       <c r="G219" t="n">
         <v>1756</v>
       </c>
       <c r="H219" t="n">
-        <v>0</v>
+        <v>5.4</v>
       </c>
       <c r="L219" t="n">
-        <v>8433.200000000001</v>
+        <v>8718</v>
       </c>
       <c r="M219" t="n">
         <v>8433.200000000001</v>
       </c>
       <c r="N219" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="O219" t="n">
-        <v>9515.799999999999</v>
+        <v>9654.4</v>
       </c>
       <c r="P219" t="n">
         <v>9515.799999999999</v>
       </c>
       <c r="Q219" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="R219" t="n">
-        <v>10663</v>
+        <v>10489.8</v>
       </c>
       <c r="S219" t="n">
         <v>10663</v>
       </c>
       <c r="T219" t="n">
-        <v>0</v>
+        <v>-1.6</v>
       </c>
       <c r="U219" t="n">
         <v>62800</v>
@@ -15843,31 +15852,31 @@
         <v>-1.1</v>
       </c>
       <c r="L222" t="n">
-        <v>3333.1</v>
+        <v>3272.2</v>
       </c>
       <c r="M222" t="n">
         <v>3346.9</v>
       </c>
       <c r="N222" t="n">
-        <v>-0.4</v>
+        <v>-2.2</v>
       </c>
       <c r="O222" t="n">
-        <v>3779.4</v>
+        <v>3717.2</v>
       </c>
       <c r="P222" t="n">
         <v>3866.4</v>
       </c>
       <c r="Q222" t="n">
-        <v>-2.3</v>
+        <v>-3.9</v>
       </c>
       <c r="R222" t="n">
-        <v>4067.6</v>
+        <v>3985.4</v>
       </c>
       <c r="S222" t="n">
         <v>4212</v>
       </c>
       <c r="T222" t="n">
-        <v>-3.4</v>
+        <v>-5.4</v>
       </c>
       <c r="U222" t="n">
         <v>36300</v>
@@ -15981,22 +15990,22 @@
         <v>136</v>
       </c>
       <c r="L224" t="n">
-        <v>476</v>
+        <v>474.2</v>
       </c>
       <c r="M224" t="n">
         <v>476</v>
       </c>
       <c r="N224" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="O224" t="n">
-        <v>591.5</v>
+        <v>589.8</v>
       </c>
       <c r="P224" t="n">
         <v>591.5</v>
       </c>
       <c r="Q224" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="R224" t="n">
         <v>686.1</v>
@@ -16044,40 +16053,40 @@
         </is>
       </c>
       <c r="F225" t="n">
-        <v>874</v>
+        <v>881</v>
       </c>
       <c r="G225" t="n">
         <v>874</v>
       </c>
       <c r="H225" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L225" t="n">
-        <v>2955.7</v>
+        <v>2959.7</v>
       </c>
       <c r="M225" t="n">
         <v>2955.7</v>
       </c>
       <c r="N225" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="O225" t="n">
-        <v>3766.7</v>
+        <v>3772.7</v>
       </c>
       <c r="P225" t="n">
         <v>3766.7</v>
       </c>
       <c r="Q225" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="R225" t="n">
-        <v>4587.8</v>
+        <v>4604.4</v>
       </c>
       <c r="S225" t="n">
         <v>4587.8</v>
       </c>
       <c r="T225" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="U225" t="n">
         <v>48000</v>
@@ -16398,40 +16407,40 @@
         </is>
       </c>
       <c r="F230" t="n">
-        <v>1864</v>
+        <v>1956</v>
       </c>
       <c r="G230" t="n">
         <v>1864</v>
       </c>
       <c r="H230" t="n">
-        <v>0</v>
+        <v>4.9</v>
       </c>
       <c r="L230" t="n">
-        <v>7602</v>
+        <v>7886.2</v>
       </c>
       <c r="M230" t="n">
         <v>7602</v>
       </c>
       <c r="N230" t="n">
-        <v>0</v>
+        <v>3.7</v>
       </c>
       <c r="O230" t="n">
-        <v>9271.200000000001</v>
+        <v>9327.299999999999</v>
       </c>
       <c r="P230" t="n">
         <v>9271.200000000001</v>
       </c>
       <c r="Q230" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="R230" t="n">
-        <v>10903.7</v>
+        <v>11424</v>
       </c>
       <c r="S230" t="n">
         <v>10903.7</v>
       </c>
       <c r="T230" t="n">
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="U230" t="n">
         <v>140000</v>
@@ -16542,40 +16551,40 @@
         </is>
       </c>
       <c r="F232" t="n">
-        <v>593</v>
+        <v>588</v>
       </c>
       <c r="G232" t="n">
         <v>593</v>
       </c>
       <c r="H232" t="n">
-        <v>0</v>
+        <v>-0.8</v>
       </c>
       <c r="L232" t="n">
-        <v>2485.8</v>
+        <v>2485.6</v>
       </c>
       <c r="M232" t="n">
         <v>2485.8</v>
       </c>
       <c r="N232" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="O232" t="n">
-        <v>4550.2</v>
+        <v>4530.6</v>
       </c>
       <c r="P232" t="n">
         <v>4550.2</v>
       </c>
       <c r="Q232" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="R232" t="n">
-        <v>5838.5</v>
+        <v>5778.4</v>
       </c>
       <c r="S232" t="n">
         <v>5779.9</v>
       </c>
       <c r="T232" t="n">
-        <v>1</v>
+        <v>-0</v>
       </c>
       <c r="U232" t="n">
         <v>68800</v>
@@ -17532,40 +17541,40 @@
         </is>
       </c>
       <c r="F246" t="n">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="G246" t="n">
         <v>777</v>
       </c>
       <c r="H246" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="L246" t="n">
-        <v>2823.7</v>
+        <v>2817.1</v>
       </c>
       <c r="M246" t="n">
         <v>2823.7</v>
       </c>
       <c r="N246" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="O246" t="n">
-        <v>3537</v>
+        <v>3535.8</v>
       </c>
       <c r="P246" t="n">
         <v>3537</v>
       </c>
       <c r="Q246" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="R246" t="n">
-        <v>4478.6</v>
+        <v>4487.9</v>
       </c>
       <c r="S246" t="n">
         <v>4478.6</v>
       </c>
       <c r="T246" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="U246" t="n">
         <v>395000</v>
@@ -18321,7 +18330,7 @@
         <v>-5</v>
       </c>
       <c r="L257" t="n">
-        <v>8298.799999999999</v>
+        <v>8298.6</v>
       </c>
       <c r="M257" t="n">
         <v>8254.1</v>
@@ -18330,7 +18339,7 @@
         <v>0.5</v>
       </c>
       <c r="O257" t="n">
-        <v>39816.5</v>
+        <v>39816.3</v>
       </c>
       <c r="P257" t="n">
         <v>38513.5</v>
@@ -18474,13 +18483,13 @@
         <v>0</v>
       </c>
       <c r="O259" t="n">
-        <v>438.4</v>
+        <v>447.6</v>
       </c>
       <c r="P259" t="n">
         <v>438.4</v>
       </c>
       <c r="Q259" t="n">
-        <v>0</v>
+        <v>2.1</v>
       </c>
       <c r="R259" t="n">
         <v>514.6</v>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-09-11
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -642,13 +642,13 @@
         <v>-1.7</v>
       </c>
       <c r="U3" t="n">
-        <v>15290</v>
+        <v>15320</v>
       </c>
       <c r="V3" t="n">
         <v>15540</v>
       </c>
       <c r="W3" t="n">
-        <v>-1.6</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="4">
@@ -714,13 +714,13 @@
         <v>0</v>
       </c>
       <c r="U4" t="n">
-        <v>78900</v>
+        <v>79400</v>
       </c>
       <c r="V4" t="n">
         <v>81400</v>
       </c>
       <c r="W4" t="n">
-        <v>-3.1</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="5">
@@ -786,13 +786,13 @@
         <v>0</v>
       </c>
       <c r="U5" t="n">
-        <v>71800</v>
+        <v>72200</v>
       </c>
       <c r="V5" t="n">
         <v>73400</v>
       </c>
       <c r="W5" t="n">
-        <v>-2.2</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="6">
@@ -858,13 +858,13 @@
         <v>0</v>
       </c>
       <c r="U6" t="n">
-        <v>1370000</v>
+        <v>1356000</v>
       </c>
       <c r="V6" t="n">
         <v>1142000</v>
       </c>
       <c r="W6" t="n">
-        <v>20</v>
+        <v>18.7</v>
       </c>
     </row>
     <row r="7">
@@ -930,13 +930,13 @@
         <v>0</v>
       </c>
       <c r="U7" t="n">
-        <v>55300</v>
+        <v>55000</v>
       </c>
       <c r="V7" t="n">
         <v>53600</v>
       </c>
       <c r="W7" t="n">
-        <v>3.2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="8">
@@ -1002,13 +1002,13 @@
         <v>0</v>
       </c>
       <c r="U8" t="n">
-        <v>24450</v>
+        <v>24500</v>
       </c>
       <c r="V8" t="n">
         <v>24550</v>
       </c>
       <c r="W8" t="n">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="9">
@@ -1074,13 +1074,13 @@
         <v>-0.4</v>
       </c>
       <c r="U9" t="n">
-        <v>126000</v>
+        <v>126600</v>
       </c>
       <c r="V9" t="n">
         <v>126500</v>
       </c>
       <c r="W9" t="n">
-        <v>-0.4</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="10">
@@ -1146,13 +1146,13 @@
         <v>0.1</v>
       </c>
       <c r="U10" t="n">
-        <v>90400</v>
+        <v>90700</v>
       </c>
       <c r="V10" t="n">
         <v>92600</v>
       </c>
       <c r="W10" t="n">
-        <v>-2.4</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="11">
@@ -1218,13 +1218,13 @@
         <v>0.4</v>
       </c>
       <c r="U11" t="n">
-        <v>1780000</v>
+        <v>1812000</v>
       </c>
       <c r="V11" t="n">
         <v>1647000</v>
       </c>
       <c r="W11" t="n">
-        <v>8.1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12">
@@ -1290,13 +1290,13 @@
         <v>0.2</v>
       </c>
       <c r="U12" t="n">
-        <v>135700</v>
+        <v>134900</v>
       </c>
       <c r="V12" t="n">
         <v>119700</v>
       </c>
       <c r="W12" t="n">
-        <v>13.4</v>
+        <v>12.7</v>
       </c>
     </row>
     <row r="13">
@@ -1362,13 +1362,13 @@
         <v>0</v>
       </c>
       <c r="U13" t="n">
-        <v>684000</v>
+        <v>686000</v>
       </c>
       <c r="V13" t="n">
         <v>663000</v>
       </c>
       <c r="W13" t="n">
-        <v>3.2</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="14">
@@ -1434,7 +1434,7 @@
         <v>0</v>
       </c>
       <c r="U14" t="n">
-        <v>137200</v>
+        <v>137300</v>
       </c>
       <c r="V14" t="n">
         <v>137400</v>
@@ -1506,13 +1506,13 @@
         <v>20</v>
       </c>
       <c r="U15" t="n">
-        <v>108600</v>
+        <v>105800</v>
       </c>
       <c r="V15" t="n">
         <v>89900</v>
       </c>
       <c r="W15" t="n">
-        <v>20.8</v>
+        <v>17.7</v>
       </c>
     </row>
     <row r="16">
@@ -1578,13 +1578,13 @@
         <v>0</v>
       </c>
       <c r="U16" t="n">
-        <v>126900</v>
+        <v>128300</v>
       </c>
       <c r="V16" t="n">
         <v>131400</v>
       </c>
       <c r="W16" t="n">
-        <v>-3.4</v>
+        <v>-2.4</v>
       </c>
     </row>
     <row r="17">
@@ -1650,13 +1650,13 @@
         <v>2.2</v>
       </c>
       <c r="U17" t="n">
-        <v>41200</v>
+        <v>41450</v>
       </c>
       <c r="V17" t="n">
         <v>42350</v>
       </c>
       <c r="W17" t="n">
-        <v>-2.7</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="18">
@@ -1722,13 +1722,13 @@
         <v>0</v>
       </c>
       <c r="U18" t="n">
-        <v>29150</v>
+        <v>29500</v>
       </c>
       <c r="V18" t="n">
         <v>27400</v>
       </c>
       <c r="W18" t="n">
-        <v>6.4</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="19">
@@ -1785,13 +1785,13 @@
         <v>0</v>
       </c>
       <c r="U19" t="n">
-        <v>50700</v>
+        <v>51300</v>
       </c>
       <c r="V19" t="n">
         <v>51100</v>
       </c>
       <c r="W19" t="n">
-        <v>-0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="20">
@@ -1839,13 +1839,13 @@
         <v>0</v>
       </c>
       <c r="U20" t="n">
-        <v>18780</v>
+        <v>18760</v>
       </c>
       <c r="V20" t="n">
         <v>19210</v>
       </c>
       <c r="W20" t="n">
-        <v>-2.2</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="21">
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="U22" t="n">
-        <v>5830</v>
+        <v>5800</v>
       </c>
       <c r="V22" t="n">
         <v>6080</v>
       </c>
       <c r="W22" t="n">
-        <v>-4.1</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="23">
@@ -2055,13 +2055,13 @@
         <v>0</v>
       </c>
       <c r="U23" t="n">
-        <v>483500</v>
+        <v>485500</v>
       </c>
       <c r="V23" t="n">
         <v>482000</v>
       </c>
       <c r="W23" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="24">
@@ -2127,13 +2127,13 @@
         <v>0</v>
       </c>
       <c r="U24" t="n">
-        <v>14910</v>
+        <v>14710</v>
       </c>
       <c r="V24" t="n">
         <v>16090</v>
       </c>
       <c r="W24" t="n">
-        <v>-7.3</v>
+        <v>-8.6</v>
       </c>
     </row>
     <row r="25">
@@ -2199,13 +2199,13 @@
         <v>0</v>
       </c>
       <c r="U25" t="n">
-        <v>106200</v>
+        <v>107100</v>
       </c>
       <c r="V25" t="n">
         <v>103000</v>
       </c>
       <c r="W25" t="n">
-        <v>3.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -2271,13 +2271,13 @@
         <v>0</v>
       </c>
       <c r="U26" t="n">
-        <v>9300</v>
+        <v>9260</v>
       </c>
       <c r="V26" t="n">
         <v>9350</v>
       </c>
       <c r="W26" t="n">
-        <v>-0.5</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="27">
@@ -2343,13 +2343,13 @@
         <v>0</v>
       </c>
       <c r="U27" t="n">
-        <v>8000</v>
+        <v>7970</v>
       </c>
       <c r="V27" t="n">
         <v>8070</v>
       </c>
       <c r="W27" t="n">
-        <v>-0.9</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="28">
@@ -2487,13 +2487,13 @@
         <v>-0.7</v>
       </c>
       <c r="U29" t="n">
-        <v>28650</v>
+        <v>28950</v>
       </c>
       <c r="V29" t="n">
         <v>30200</v>
       </c>
       <c r="W29" t="n">
-        <v>-5.1</v>
+        <v>-4.1</v>
       </c>
     </row>
     <row r="30">
@@ -2559,13 +2559,13 @@
         <v>0</v>
       </c>
       <c r="U30" t="n">
-        <v>112700</v>
+        <v>112500</v>
       </c>
       <c r="V30" t="n">
         <v>121100</v>
       </c>
       <c r="W30" t="n">
-        <v>-6.9</v>
+        <v>-7.1</v>
       </c>
     </row>
     <row r="31">
@@ -2631,13 +2631,13 @@
         <v>0</v>
       </c>
       <c r="U31" t="n">
-        <v>188200</v>
+        <v>185300</v>
       </c>
       <c r="V31" t="n">
         <v>183600</v>
       </c>
       <c r="W31" t="n">
-        <v>2.5</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="32">
@@ -2703,13 +2703,13 @@
         <v>0</v>
       </c>
       <c r="U32" t="n">
-        <v>45800</v>
+        <v>46150</v>
       </c>
       <c r="V32" t="n">
         <v>45700</v>
       </c>
       <c r="W32" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
@@ -2775,13 +2775,13 @@
         <v>-0.8</v>
       </c>
       <c r="U33" t="n">
-        <v>33550</v>
+        <v>33600</v>
       </c>
       <c r="V33" t="n">
         <v>31500</v>
       </c>
       <c r="W33" t="n">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="34">
@@ -2847,13 +2847,13 @@
         <v>0.4</v>
       </c>
       <c r="U34" t="n">
-        <v>385500</v>
+        <v>381000</v>
       </c>
       <c r="V34" t="n">
         <v>382500</v>
       </c>
       <c r="W34" t="n">
-        <v>0.8</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="35">
@@ -2919,13 +2919,13 @@
         <v>0.2</v>
       </c>
       <c r="U35" t="n">
-        <v>409500</v>
+        <v>414500</v>
       </c>
       <c r="V35" t="n">
         <v>430000</v>
       </c>
       <c r="W35" t="n">
-        <v>-4.8</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="36">
@@ -2991,13 +2991,13 @@
         <v>0</v>
       </c>
       <c r="U36" t="n">
-        <v>25000</v>
+        <v>25050</v>
       </c>
       <c r="V36" t="n">
         <v>24750</v>
       </c>
       <c r="W36" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="37">
@@ -3063,13 +3063,13 @@
         <v>-1.7</v>
       </c>
       <c r="U37" t="n">
-        <v>97200</v>
+        <v>97600</v>
       </c>
       <c r="V37" t="n">
         <v>98300</v>
       </c>
       <c r="W37" t="n">
-        <v>-1.1</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="38">
@@ -3135,13 +3135,13 @@
         <v>-0</v>
       </c>
       <c r="U38" t="n">
-        <v>381000</v>
+        <v>382500</v>
       </c>
       <c r="V38" t="n">
         <v>383500</v>
       </c>
       <c r="W38" t="n">
-        <v>-0.7</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="39">
@@ -3207,13 +3207,13 @@
         <v>0.6</v>
       </c>
       <c r="U39" t="n">
-        <v>332000</v>
+        <v>334000</v>
       </c>
       <c r="V39" t="n">
         <v>337000</v>
       </c>
       <c r="W39" t="n">
-        <v>-1.5</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="40">
@@ -3270,13 +3270,13 @@
         <v>0</v>
       </c>
       <c r="U40" t="n">
-        <v>189100</v>
+        <v>191700</v>
       </c>
       <c r="V40" t="n">
         <v>195700</v>
       </c>
       <c r="W40" t="n">
-        <v>-3.4</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="41">
@@ -3342,13 +3342,13 @@
         <v>0</v>
       </c>
       <c r="U41" t="n">
-        <v>52100</v>
+        <v>52200</v>
       </c>
       <c r="V41" t="n">
         <v>51400</v>
       </c>
       <c r="W41" t="n">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="42">
@@ -3414,13 +3414,13 @@
         <v>-0.1</v>
       </c>
       <c r="U42" t="n">
-        <v>257500</v>
+        <v>259500</v>
       </c>
       <c r="V42" t="n">
         <v>255500</v>
       </c>
       <c r="W42" t="n">
-        <v>0.8</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="43">
@@ -3480,13 +3480,13 @@
         <v>-0.4</v>
       </c>
       <c r="U43" t="n">
-        <v>26200</v>
+        <v>26300</v>
       </c>
       <c r="V43" t="n">
         <v>26650</v>
       </c>
       <c r="W43" t="n">
-        <v>-1.7</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="44">
@@ -3522,13 +3522,13 @@
         <v>932</v>
       </c>
       <c r="U44" t="n">
-        <v>8330</v>
+        <v>8240</v>
       </c>
       <c r="V44" t="n">
         <v>7520</v>
       </c>
       <c r="W44" t="n">
-        <v>10.8</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="45">
@@ -3666,13 +3666,13 @@
         <v>0</v>
       </c>
       <c r="U46" t="n">
-        <v>312000</v>
+        <v>319500</v>
       </c>
       <c r="V46" t="n">
         <v>299500</v>
       </c>
       <c r="W46" t="n">
-        <v>4.2</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="47">
@@ -3738,13 +3738,13 @@
         <v>0</v>
       </c>
       <c r="U47" t="n">
-        <v>129400</v>
+        <v>128300</v>
       </c>
       <c r="V47" t="n">
         <v>127600</v>
       </c>
       <c r="W47" t="n">
-        <v>1.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="48">
@@ -3810,13 +3810,13 @@
         <v>0</v>
       </c>
       <c r="U48" t="n">
-        <v>38250</v>
+        <v>38500</v>
       </c>
       <c r="V48" t="n">
         <v>34250</v>
       </c>
       <c r="W48" t="n">
-        <v>11.7</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="49">
@@ -3882,13 +3882,13 @@
         <v>0.7</v>
       </c>
       <c r="U49" t="n">
-        <v>548000</v>
+        <v>545000</v>
       </c>
       <c r="V49" t="n">
         <v>548000</v>
       </c>
       <c r="W49" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="50">
@@ -3954,13 +3954,13 @@
         <v>0</v>
       </c>
       <c r="U50" t="n">
-        <v>100600</v>
+        <v>102200</v>
       </c>
       <c r="V50" t="n">
         <v>96700</v>
       </c>
       <c r="W50" t="n">
-        <v>4</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="51">
@@ -4020,13 +4020,13 @@
         <v>1.2</v>
       </c>
       <c r="U51" t="n">
-        <v>33650</v>
+        <v>33450</v>
       </c>
       <c r="V51" t="n">
         <v>34450</v>
       </c>
       <c r="W51" t="n">
-        <v>-2.3</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="52">
@@ -4092,13 +4092,13 @@
         <v>0</v>
       </c>
       <c r="U52" t="n">
-        <v>24950</v>
+        <v>25050</v>
       </c>
       <c r="V52" t="n">
         <v>25400</v>
       </c>
       <c r="W52" t="n">
-        <v>-1.8</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="53">
@@ -4164,13 +4164,13 @@
         <v>0</v>
       </c>
       <c r="U53" t="n">
-        <v>46550</v>
+        <v>46800</v>
       </c>
       <c r="V53" t="n">
         <v>45100</v>
       </c>
       <c r="W53" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="54">
@@ -4236,13 +4236,13 @@
         <v>3.2</v>
       </c>
       <c r="U54" t="n">
-        <v>109700</v>
+        <v>109900</v>
       </c>
       <c r="V54" t="n">
         <v>111100</v>
       </c>
       <c r="W54" t="n">
-        <v>-1.3</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="55">
@@ -4308,13 +4308,13 @@
         <v>-22.7</v>
       </c>
       <c r="U55" t="n">
-        <v>50900</v>
+        <v>51100</v>
       </c>
       <c r="V55" t="n">
         <v>51000</v>
       </c>
       <c r="W55" t="n">
-        <v>-0.2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="56">
@@ -4380,13 +4380,13 @@
         <v>0.5</v>
       </c>
       <c r="U56" t="n">
-        <v>41250</v>
+        <v>41100</v>
       </c>
       <c r="V56" t="n">
         <v>42200</v>
       </c>
       <c r="W56" t="n">
-        <v>-2.3</v>
+        <v>-2.6</v>
       </c>
     </row>
     <row r="57">
@@ -4452,13 +4452,13 @@
         <v>0</v>
       </c>
       <c r="U57" t="n">
-        <v>1387000</v>
+        <v>1400000</v>
       </c>
       <c r="V57" t="n">
         <v>1401000</v>
       </c>
       <c r="W57" t="n">
-        <v>-1</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="58">
@@ -4524,13 +4524,13 @@
         <v>0</v>
       </c>
       <c r="U58" t="n">
-        <v>39400</v>
+        <v>39350</v>
       </c>
       <c r="V58" t="n">
         <v>37400</v>
       </c>
       <c r="W58" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="59">
@@ -4596,13 +4596,13 @@
         <v>0</v>
       </c>
       <c r="U59" t="n">
-        <v>363000</v>
+        <v>365500</v>
       </c>
       <c r="V59" t="n">
         <v>348500</v>
       </c>
       <c r="W59" t="n">
-        <v>4.2</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="60">
@@ -4668,13 +4668,13 @@
         <v>0</v>
       </c>
       <c r="U60" t="n">
-        <v>30100</v>
+        <v>29800</v>
       </c>
       <c r="V60" t="n">
         <v>30050</v>
       </c>
       <c r="W60" t="n">
-        <v>0.2</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="61">
@@ -4740,13 +4740,13 @@
         <v>0</v>
       </c>
       <c r="U61" t="n">
-        <v>218000</v>
+        <v>218500</v>
       </c>
       <c r="V61" t="n">
         <v>227500</v>
       </c>
       <c r="W61" t="n">
-        <v>-4.2</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="62">
@@ -4812,13 +4812,13 @@
         <v>1.2</v>
       </c>
       <c r="U62" t="n">
-        <v>202500</v>
+        <v>204500</v>
       </c>
       <c r="V62" t="n">
         <v>195300</v>
       </c>
       <c r="W62" t="n">
-        <v>3.7</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="63">
@@ -4884,13 +4884,13 @@
         <v>0</v>
       </c>
       <c r="U63" t="n">
-        <v>1181000</v>
+        <v>1179000</v>
       </c>
       <c r="V63" t="n">
         <v>1222000</v>
       </c>
       <c r="W63" t="n">
-        <v>-3.4</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="64">
@@ -5028,13 +5028,13 @@
         <v>-1.9</v>
       </c>
       <c r="U65" t="n">
-        <v>15850</v>
+        <v>15770</v>
       </c>
       <c r="V65" t="n">
         <v>15740</v>
       </c>
       <c r="W65" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="66">
@@ -5100,13 +5100,13 @@
         <v>1.6</v>
       </c>
       <c r="U66" t="n">
-        <v>152800</v>
+        <v>150000</v>
       </c>
       <c r="V66" t="n">
         <v>157300</v>
       </c>
       <c r="W66" t="n">
-        <v>-2.9</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="67">
@@ -5172,13 +5172,13 @@
         <v>0</v>
       </c>
       <c r="U67" t="n">
-        <v>540000</v>
+        <v>543000</v>
       </c>
       <c r="V67" t="n">
         <v>562000</v>
       </c>
       <c r="W67" t="n">
-        <v>-3.9</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="68">
@@ -5244,13 +5244,13 @@
         <v>0</v>
       </c>
       <c r="U68" t="n">
-        <v>63800</v>
+        <v>65500</v>
       </c>
       <c r="V68" t="n">
         <v>60000</v>
       </c>
       <c r="W68" t="n">
-        <v>6.3</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="69">
@@ -5316,13 +5316,13 @@
         <v>0</v>
       </c>
       <c r="U69" t="n">
-        <v>20700</v>
+        <v>20850</v>
       </c>
       <c r="V69" t="n">
         <v>21050</v>
       </c>
       <c r="W69" t="n">
-        <v>-1.7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="70">
@@ -5388,13 +5388,13 @@
         <v>0</v>
       </c>
       <c r="U70" t="n">
-        <v>57200</v>
+        <v>57400</v>
       </c>
       <c r="V70" t="n">
         <v>57600</v>
       </c>
       <c r="W70" t="n">
-        <v>-0.7</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="71">
@@ -5460,13 +5460,13 @@
         <v>0</v>
       </c>
       <c r="U71" t="n">
-        <v>124300</v>
+        <v>124900</v>
       </c>
       <c r="V71" t="n">
         <v>125900</v>
       </c>
       <c r="W71" t="n">
-        <v>-1.3</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="72">
@@ -5532,13 +5532,13 @@
         <v>0</v>
       </c>
       <c r="U72" t="n">
-        <v>89500</v>
+        <v>89600</v>
       </c>
       <c r="V72" t="n">
         <v>84300</v>
       </c>
       <c r="W72" t="n">
-        <v>6.2</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="73">
@@ -5604,13 +5604,13 @@
         <v>0</v>
       </c>
       <c r="U73" t="n">
-        <v>16460</v>
+        <v>16180</v>
       </c>
       <c r="V73" t="n">
         <v>16110</v>
       </c>
       <c r="W73" t="n">
-        <v>2.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="74">
@@ -5676,13 +5676,13 @@
         <v>0</v>
       </c>
       <c r="U74" t="n">
-        <v>417000</v>
+        <v>415500</v>
       </c>
       <c r="V74" t="n">
         <v>422000</v>
       </c>
       <c r="W74" t="n">
-        <v>-1.2</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="75">
@@ -5748,13 +5748,13 @@
         <v>0</v>
       </c>
       <c r="U75" t="n">
-        <v>1071000</v>
+        <v>1081000</v>
       </c>
       <c r="V75" t="n">
         <v>1055000</v>
       </c>
       <c r="W75" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="76">
@@ -5820,13 +5820,13 @@
         <v>0</v>
       </c>
       <c r="U76" t="n">
-        <v>81600</v>
+        <v>81400</v>
       </c>
       <c r="V76" t="n">
         <v>79200</v>
       </c>
       <c r="W76" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="77">
@@ -5892,13 +5892,13 @@
         <v>0</v>
       </c>
       <c r="U77" t="n">
-        <v>35325</v>
+        <v>34300</v>
       </c>
       <c r="V77" t="n">
         <v>30850</v>
       </c>
       <c r="W77" t="n">
-        <v>14.5</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="78">
@@ -5964,13 +5964,13 @@
         <v>-0.9</v>
       </c>
       <c r="U78" t="n">
-        <v>198000</v>
+        <v>200000</v>
       </c>
       <c r="V78" t="n">
         <v>193100</v>
       </c>
       <c r="W78" t="n">
-        <v>2.5</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="79">
@@ -6027,13 +6027,13 @@
         <v>0</v>
       </c>
       <c r="U79" t="n">
-        <v>2515</v>
+        <v>2530</v>
       </c>
       <c r="V79" t="n">
         <v>2555</v>
       </c>
       <c r="W79" t="n">
-        <v>-1.6</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="80">
@@ -6099,13 +6099,13 @@
         <v>-1.8</v>
       </c>
       <c r="U80" t="n">
-        <v>33350</v>
+        <v>33100</v>
       </c>
       <c r="V80" t="n">
         <v>32150</v>
       </c>
       <c r="W80" t="n">
-        <v>3.7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="81">
@@ -6165,13 +6165,13 @@
         <v>0.3</v>
       </c>
       <c r="U81" t="n">
-        <v>87300</v>
+        <v>87400</v>
       </c>
       <c r="V81" t="n">
         <v>86800</v>
       </c>
       <c r="W81" t="n">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="82">
@@ -6237,13 +6237,13 @@
         <v>0</v>
       </c>
       <c r="U82" t="n">
-        <v>90600</v>
+        <v>90900</v>
       </c>
       <c r="V82" t="n">
         <v>92500</v>
       </c>
       <c r="W82" t="n">
-        <v>-2.1</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="83">
@@ -6309,13 +6309,13 @@
         <v>0</v>
       </c>
       <c r="U83" t="n">
-        <v>74500</v>
+        <v>74300</v>
       </c>
       <c r="V83" t="n">
         <v>74900</v>
       </c>
       <c r="W83" t="n">
-        <v>-0.5</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="84">
@@ -6381,13 +6381,13 @@
         <v>0</v>
       </c>
       <c r="U84" t="n">
-        <v>21850</v>
+        <v>21700</v>
       </c>
       <c r="V84" t="n">
         <v>22550</v>
       </c>
       <c r="W84" t="n">
-        <v>-3.1</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="85">
@@ -6453,13 +6453,13 @@
         <v>0</v>
       </c>
       <c r="U85" t="n">
-        <v>221750</v>
+        <v>222500</v>
       </c>
       <c r="V85" t="n">
         <v>238000</v>
       </c>
       <c r="W85" t="n">
-        <v>-6.8</v>
+        <v>-6.5</v>
       </c>
     </row>
     <row r="86">
@@ -6525,13 +6525,13 @@
         <v>0</v>
       </c>
       <c r="U86" t="n">
-        <v>3465</v>
+        <v>3520</v>
       </c>
       <c r="V86" t="n">
         <v>3525</v>
       </c>
       <c r="W86" t="n">
-        <v>-1.7</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="87">
@@ -6597,13 +6597,13 @@
         <v>0</v>
       </c>
       <c r="U87" t="n">
-        <v>95400</v>
+        <v>95200</v>
       </c>
       <c r="V87" t="n">
         <v>99400</v>
       </c>
       <c r="W87" t="n">
-        <v>-4</v>
+        <v>-4.2</v>
       </c>
     </row>
     <row r="88">
@@ -6669,13 +6669,13 @@
         <v>0</v>
       </c>
       <c r="U88" t="n">
-        <v>21650</v>
+        <v>22150</v>
       </c>
       <c r="V88" t="n">
         <v>21650</v>
       </c>
       <c r="W88" t="n">
-        <v>0</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="89">
@@ -6741,13 +6741,13 @@
         <v>0</v>
       </c>
       <c r="U89" t="n">
-        <v>28700</v>
+        <v>28300</v>
       </c>
       <c r="V89" t="n">
         <v>26150</v>
       </c>
       <c r="W89" t="n">
-        <v>9.800000000000001</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="90">
@@ -6813,13 +6813,13 @@
         <v>0.4</v>
       </c>
       <c r="U90" t="n">
-        <v>112900</v>
+        <v>112000</v>
       </c>
       <c r="V90" t="n">
         <v>107500</v>
       </c>
       <c r="W90" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="91">
@@ -6885,13 +6885,13 @@
         <v>0</v>
       </c>
       <c r="U91" t="n">
-        <v>20700</v>
+        <v>20850</v>
       </c>
       <c r="V91" t="n">
         <v>20700</v>
       </c>
       <c r="W91" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="92">
@@ -6957,13 +6957,13 @@
         <v>0</v>
       </c>
       <c r="U92" t="n">
-        <v>50900</v>
+        <v>51000</v>
       </c>
       <c r="V92" t="n">
         <v>45850</v>
       </c>
       <c r="W92" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
     </row>
     <row r="93">
@@ -7029,13 +7029,13 @@
         <v>0</v>
       </c>
       <c r="U93" t="n">
-        <v>366000</v>
+        <v>367000</v>
       </c>
       <c r="V93" t="n">
         <v>367000</v>
       </c>
       <c r="W93" t="n">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -7101,13 +7101,13 @@
         <v>0</v>
       </c>
       <c r="U94" t="n">
-        <v>6100</v>
+        <v>6030</v>
       </c>
       <c r="V94" t="n">
         <v>5960</v>
       </c>
       <c r="W94" t="n">
-        <v>2.3</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="95">
@@ -7167,13 +7167,13 @@
         <v>0</v>
       </c>
       <c r="U95" t="n">
-        <v>45450</v>
+        <v>45500</v>
       </c>
       <c r="V95" t="n">
         <v>46150</v>
       </c>
       <c r="W95" t="n">
-        <v>-1.5</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="96">
@@ -7239,13 +7239,13 @@
         <v>0</v>
       </c>
       <c r="U96" t="n">
-        <v>18970</v>
+        <v>18910</v>
       </c>
       <c r="V96" t="n">
         <v>18930</v>
       </c>
       <c r="W96" t="n">
-        <v>0.2</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="97">
@@ -7311,13 +7311,13 @@
         <v>0.5</v>
       </c>
       <c r="U97" t="n">
-        <v>52600</v>
+        <v>52700</v>
       </c>
       <c r="V97" t="n">
         <v>54300</v>
       </c>
       <c r="W97" t="n">
-        <v>-3.1</v>
+        <v>-2.9</v>
       </c>
     </row>
     <row r="98">
@@ -7356,13 +7356,13 @@
         <v>-2.3</v>
       </c>
       <c r="U98" t="n">
-        <v>12150</v>
+        <v>12050</v>
       </c>
       <c r="V98" t="n">
         <v>12530</v>
       </c>
       <c r="W98" t="n">
-        <v>-3</v>
+        <v>-3.8</v>
       </c>
     </row>
     <row r="99">
@@ -7428,13 +7428,13 @@
         <v>0</v>
       </c>
       <c r="U99" t="n">
-        <v>14740</v>
+        <v>14890</v>
       </c>
       <c r="V99" t="n">
         <v>14760</v>
       </c>
       <c r="W99" t="n">
-        <v>-0.1</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="100">
@@ -7500,13 +7500,13 @@
         <v>0</v>
       </c>
       <c r="U100" t="n">
-        <v>304500</v>
+        <v>307500</v>
       </c>
       <c r="V100" t="n">
         <v>297500</v>
       </c>
       <c r="W100" t="n">
-        <v>2.4</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="101">
@@ -7572,13 +7572,13 @@
         <v>0</v>
       </c>
       <c r="U101" t="n">
-        <v>17000</v>
+        <v>16790</v>
       </c>
       <c r="V101" t="n">
         <v>17160</v>
       </c>
       <c r="W101" t="n">
-        <v>-0.9</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="102">
@@ -7644,13 +7644,13 @@
         <v>-0.2</v>
       </c>
       <c r="U102" t="n">
-        <v>171100</v>
+        <v>171800</v>
       </c>
       <c r="V102" t="n">
         <v>172500</v>
       </c>
       <c r="W102" t="n">
-        <v>-0.8</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="103">
@@ -7716,13 +7716,13 @@
         <v>0</v>
       </c>
       <c r="U103" t="n">
-        <v>89900</v>
+        <v>90800</v>
       </c>
       <c r="V103" t="n">
         <v>79200</v>
       </c>
       <c r="W103" t="n">
-        <v>13.5</v>
+        <v>14.6</v>
       </c>
     </row>
     <row r="104">
@@ -7788,13 +7788,13 @@
         <v>1.9</v>
       </c>
       <c r="U104" t="n">
-        <v>8810</v>
+        <v>8900</v>
       </c>
       <c r="V104" t="n">
         <v>9130</v>
       </c>
       <c r="W104" t="n">
-        <v>-3.5</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="105">
@@ -7860,13 +7860,13 @@
         <v>-0.1</v>
       </c>
       <c r="U105" t="n">
-        <v>9780</v>
+        <v>9930</v>
       </c>
       <c r="V105" t="n">
         <v>10090</v>
       </c>
       <c r="W105" t="n">
-        <v>-3.1</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="106">
@@ -7932,13 +7932,13 @@
         <v>0</v>
       </c>
       <c r="U106" t="n">
-        <v>579000</v>
+        <v>585000</v>
       </c>
       <c r="V106" t="n">
         <v>573000</v>
       </c>
       <c r="W106" t="n">
-        <v>1</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="107">
@@ -8004,13 +8004,13 @@
         <v>5.2</v>
       </c>
       <c r="U107" t="n">
-        <v>14700</v>
+        <v>14800</v>
       </c>
       <c r="V107" t="n">
         <v>14750</v>
       </c>
       <c r="W107" t="n">
-        <v>-0.3</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="108">
@@ -8076,13 +8076,13 @@
         <v>-0</v>
       </c>
       <c r="U108" t="n">
-        <v>204500</v>
+        <v>206500</v>
       </c>
       <c r="V108" t="n">
         <v>213500</v>
       </c>
       <c r="W108" t="n">
-        <v>-4.2</v>
+        <v>-3.3</v>
       </c>
     </row>
     <row r="109">
@@ -8148,13 +8148,13 @@
         <v>0</v>
       </c>
       <c r="U109" t="n">
-        <v>34550</v>
+        <v>34500</v>
       </c>
       <c r="V109" t="n">
         <v>36200</v>
       </c>
       <c r="W109" t="n">
-        <v>-4.6</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="110">
@@ -8220,13 +8220,13 @@
         <v>0</v>
       </c>
       <c r="U110" t="n">
-        <v>34400</v>
+        <v>35000</v>
       </c>
       <c r="V110" t="n">
         <v>33050</v>
       </c>
       <c r="W110" t="n">
-        <v>4.1</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="111">
@@ -8292,13 +8292,13 @@
         <v>-0.1</v>
       </c>
       <c r="U111" t="n">
-        <v>39450</v>
+        <v>39350</v>
       </c>
       <c r="V111" t="n">
         <v>39300</v>
       </c>
       <c r="W111" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="112">
@@ -8364,13 +8364,13 @@
         <v>0</v>
       </c>
       <c r="U112" t="n">
-        <v>8980</v>
+        <v>9010</v>
       </c>
       <c r="V112" t="n">
         <v>8910</v>
       </c>
       <c r="W112" t="n">
-        <v>0.8</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="113">
@@ -8436,13 +8436,13 @@
         <v>-0.5</v>
       </c>
       <c r="U113" t="n">
-        <v>36550</v>
+        <v>37000</v>
       </c>
       <c r="V113" t="n">
         <v>35100</v>
       </c>
       <c r="W113" t="n">
-        <v>4.1</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="114">
@@ -8508,13 +8508,13 @@
         <v>-3.5</v>
       </c>
       <c r="U114" t="n">
-        <v>206500</v>
+        <v>205500</v>
       </c>
       <c r="V114" t="n">
         <v>222000</v>
       </c>
       <c r="W114" t="n">
-        <v>-7</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="115">
@@ -8580,13 +8580,13 @@
         <v>0</v>
       </c>
       <c r="U115" t="n">
-        <v>219500</v>
+        <v>209000</v>
       </c>
       <c r="V115" t="n">
         <v>178300</v>
       </c>
       <c r="W115" t="n">
-        <v>23.1</v>
+        <v>17.2</v>
       </c>
     </row>
     <row r="116">
@@ -8652,13 +8652,13 @@
         <v>0</v>
       </c>
       <c r="U116" t="n">
-        <v>33200</v>
+        <v>33250</v>
       </c>
       <c r="V116" t="n">
         <v>32500</v>
       </c>
       <c r="W116" t="n">
-        <v>2.2</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="117">
@@ -8718,13 +8718,13 @@
         <v>0.6</v>
       </c>
       <c r="U117" t="n">
-        <v>275500</v>
+        <v>278000</v>
       </c>
       <c r="V117" t="n">
         <v>270500</v>
       </c>
       <c r="W117" t="n">
-        <v>1.8</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="118">
@@ -8790,13 +8790,13 @@
         <v>0</v>
       </c>
       <c r="U118" t="n">
-        <v>10930</v>
+        <v>11110</v>
       </c>
       <c r="V118" t="n">
         <v>10910</v>
       </c>
       <c r="W118" t="n">
-        <v>0.2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="119">
@@ -8862,13 +8862,13 @@
         <v>0.1</v>
       </c>
       <c r="U119" t="n">
-        <v>83600</v>
+        <v>84000</v>
       </c>
       <c r="V119" t="n">
         <v>79000</v>
       </c>
       <c r="W119" t="n">
-        <v>5.8</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="120">
@@ -8934,13 +8934,13 @@
         <v>-0.1</v>
       </c>
       <c r="U120" t="n">
-        <v>85700</v>
+        <v>85600</v>
       </c>
       <c r="V120" t="n">
         <v>86800</v>
       </c>
       <c r="W120" t="n">
-        <v>-1.3</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="121">
@@ -9006,13 +9006,13 @@
         <v>0</v>
       </c>
       <c r="U121" t="n">
-        <v>232500</v>
+        <v>231000</v>
       </c>
       <c r="V121" t="n">
         <v>230000</v>
       </c>
       <c r="W121" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="122">
@@ -9078,13 +9078,13 @@
         <v>-1.4</v>
       </c>
       <c r="U122" t="n">
-        <v>19690</v>
+        <v>19890</v>
       </c>
       <c r="V122" t="n">
         <v>16850</v>
       </c>
       <c r="W122" t="n">
-        <v>16.9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="123">
@@ -9150,13 +9150,13 @@
         <v>0</v>
       </c>
       <c r="U123" t="n">
-        <v>57600</v>
+        <v>57700</v>
       </c>
       <c r="V123" t="n">
         <v>54700</v>
       </c>
       <c r="W123" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="124">
@@ -9222,13 +9222,13 @@
         <v>0</v>
       </c>
       <c r="U124" t="n">
-        <v>131500</v>
+        <v>130500</v>
       </c>
       <c r="V124" t="n">
         <v>126500</v>
       </c>
       <c r="W124" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="125">
@@ -9294,13 +9294,13 @@
         <v>-2.7</v>
       </c>
       <c r="U125" t="n">
-        <v>22950</v>
+        <v>22850</v>
       </c>
       <c r="V125" t="n">
         <v>23700</v>
       </c>
       <c r="W125" t="n">
-        <v>-3.2</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="126">
@@ -9366,13 +9366,13 @@
         <v>3.9</v>
       </c>
       <c r="U126" t="n">
-        <v>48800</v>
+        <v>49300</v>
       </c>
       <c r="V126" t="n">
         <v>45800</v>
       </c>
       <c r="W126" t="n">
-        <v>6.6</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="127">
@@ -9438,13 +9438,13 @@
         <v>0</v>
       </c>
       <c r="U127" t="n">
-        <v>292000</v>
+        <v>291000</v>
       </c>
       <c r="V127" t="n">
         <v>294000</v>
       </c>
       <c r="W127" t="n">
-        <v>-0.7</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="128">
@@ -9510,13 +9510,13 @@
         <v>0</v>
       </c>
       <c r="U128" t="n">
-        <v>270500</v>
+        <v>273000</v>
       </c>
       <c r="V128" t="n">
         <v>282000</v>
       </c>
       <c r="W128" t="n">
-        <v>-4.1</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="129">
@@ -9582,13 +9582,13 @@
         <v>-0.4</v>
       </c>
       <c r="U129" t="n">
-        <v>145900</v>
+        <v>152000</v>
       </c>
       <c r="V129" t="n">
         <v>107600</v>
       </c>
       <c r="W129" t="n">
-        <v>35.6</v>
+        <v>41.3</v>
       </c>
     </row>
     <row r="130">
@@ -9654,13 +9654,13 @@
         <v>0</v>
       </c>
       <c r="U130" t="n">
-        <v>112300</v>
+        <v>112900</v>
       </c>
       <c r="V130" t="n">
         <v>110300</v>
       </c>
       <c r="W130" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="131">
@@ -9726,13 +9726,13 @@
         <v>0</v>
       </c>
       <c r="U131" t="n">
-        <v>94200</v>
+        <v>96800</v>
       </c>
       <c r="V131" t="n">
         <v>94200</v>
       </c>
       <c r="W131" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="132">
@@ -9789,13 +9789,13 @@
         <v>0</v>
       </c>
       <c r="U132" t="n">
-        <v>40050</v>
+        <v>39900</v>
       </c>
       <c r="V132" t="n">
         <v>40150</v>
       </c>
       <c r="W132" t="n">
-        <v>-0.2</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="133">
@@ -9861,13 +9861,13 @@
         <v>0</v>
       </c>
       <c r="U133" t="n">
-        <v>194700</v>
+        <v>198600</v>
       </c>
       <c r="V133" t="n">
         <v>191700</v>
       </c>
       <c r="W133" t="n">
-        <v>1.6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="134">
@@ -9933,13 +9933,13 @@
         <v>0</v>
       </c>
       <c r="U134" t="n">
-        <v>123800</v>
+        <v>124100</v>
       </c>
       <c r="V134" t="n">
         <v>126800</v>
       </c>
       <c r="W134" t="n">
-        <v>-2.4</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="135">
@@ -10005,13 +10005,13 @@
         <v>0</v>
       </c>
       <c r="U135" t="n">
-        <v>71500</v>
+        <v>71900</v>
       </c>
       <c r="V135" t="n">
         <v>74100</v>
       </c>
       <c r="W135" t="n">
-        <v>-3.5</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="136">
@@ -10077,13 +10077,13 @@
         <v>0</v>
       </c>
       <c r="U136" t="n">
-        <v>26800</v>
+        <v>26850</v>
       </c>
       <c r="V136" t="n">
         <v>26250</v>
       </c>
       <c r="W136" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="137">
@@ -10149,7 +10149,7 @@
         <v>0</v>
       </c>
       <c r="U137" t="n">
-        <v>199550</v>
+        <v>199500</v>
       </c>
       <c r="V137" t="n">
         <v>201500</v>
@@ -10221,13 +10221,13 @@
         <v>0.3</v>
       </c>
       <c r="U138" t="n">
-        <v>120400</v>
+        <v>120000</v>
       </c>
       <c r="V138" t="n">
         <v>121300</v>
       </c>
       <c r="W138" t="n">
-        <v>-0.7</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="139">
@@ -10293,13 +10293,13 @@
         <v>0</v>
       </c>
       <c r="U139" t="n">
-        <v>37050</v>
+        <v>37100</v>
       </c>
       <c r="V139" t="n">
         <v>38050</v>
       </c>
       <c r="W139" t="n">
-        <v>-2.6</v>
+        <v>-2.5</v>
       </c>
     </row>
     <row r="140">
@@ -10437,13 +10437,13 @@
         <v>0</v>
       </c>
       <c r="U141" t="n">
-        <v>16460</v>
+        <v>16430</v>
       </c>
       <c r="V141" t="n">
         <v>16320</v>
       </c>
       <c r="W141" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="142">
@@ -10509,13 +10509,13 @@
         <v>0</v>
       </c>
       <c r="U142" t="n">
-        <v>111500</v>
+        <v>111900</v>
       </c>
       <c r="V142" t="n">
         <v>116100</v>
       </c>
       <c r="W142" t="n">
-        <v>-4</v>
+        <v>-3.6</v>
       </c>
     </row>
     <row r="143">
@@ -10581,13 +10581,13 @@
         <v>0.5</v>
       </c>
       <c r="U143" t="n">
-        <v>99600</v>
+        <v>99000</v>
       </c>
       <c r="V143" t="n">
         <v>96200</v>
       </c>
       <c r="W143" t="n">
-        <v>3.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="144">
@@ -10653,13 +10653,13 @@
         <v>-0.5</v>
       </c>
       <c r="U144" t="n">
-        <v>192400</v>
+        <v>193600</v>
       </c>
       <c r="V144" t="n">
         <v>188800</v>
       </c>
       <c r="W144" t="n">
-        <v>1.9</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="145">
@@ -10725,13 +10725,13 @@
         <v>0</v>
       </c>
       <c r="U145" t="n">
-        <v>74800</v>
+        <v>74700</v>
       </c>
       <c r="V145" t="n">
         <v>75600</v>
       </c>
       <c r="W145" t="n">
-        <v>-1.1</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="146">
@@ -10797,13 +10797,13 @@
         <v>0</v>
       </c>
       <c r="U146" t="n">
-        <v>53100</v>
+        <v>52500</v>
       </c>
       <c r="V146" t="n">
         <v>50200</v>
       </c>
       <c r="W146" t="n">
-        <v>5.8</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="147">
@@ -10869,13 +10869,13 @@
         <v>0.5</v>
       </c>
       <c r="U147" t="n">
-        <v>7400</v>
+        <v>7370</v>
       </c>
       <c r="V147" t="n">
         <v>7180</v>
       </c>
       <c r="W147" t="n">
-        <v>3.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="148">
@@ -10914,13 +10914,13 @@
         <v>0</v>
       </c>
       <c r="U148" t="n">
-        <v>10570</v>
+        <v>10390</v>
       </c>
       <c r="V148" t="n">
         <v>10280</v>
       </c>
       <c r="W148" t="n">
-        <v>2.8</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="149">
@@ -10959,13 +10959,13 @@
         <v>0</v>
       </c>
       <c r="U149" t="n">
-        <v>10170</v>
+        <v>10030</v>
       </c>
       <c r="V149" t="n">
         <v>10060</v>
       </c>
       <c r="W149" t="n">
-        <v>1.1</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="150">
@@ -11031,13 +11031,13 @@
         <v>0</v>
       </c>
       <c r="U150" t="n">
-        <v>25600</v>
+        <v>24800</v>
       </c>
       <c r="V150" t="n">
         <v>23550</v>
       </c>
       <c r="W150" t="n">
-        <v>8.699999999999999</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="151">
@@ -11103,13 +11103,13 @@
         <v>0</v>
       </c>
       <c r="U151" t="n">
-        <v>117400</v>
+        <v>119000</v>
       </c>
       <c r="V151" t="n">
         <v>123900</v>
       </c>
       <c r="W151" t="n">
-        <v>-5.2</v>
+        <v>-4</v>
       </c>
     </row>
     <row r="152">
@@ -11175,13 +11175,13 @@
         <v>0</v>
       </c>
       <c r="U152" t="n">
-        <v>679000</v>
+        <v>678000</v>
       </c>
       <c r="V152" t="n">
         <v>652000</v>
       </c>
       <c r="W152" t="n">
-        <v>4.1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="153">
@@ -11220,13 +11220,13 @@
         <v>0</v>
       </c>
       <c r="U153" t="n">
-        <v>9560</v>
+        <v>9480</v>
       </c>
       <c r="V153" t="n">
         <v>8970</v>
       </c>
       <c r="W153" t="n">
-        <v>6.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="154">
@@ -11292,13 +11292,13 @@
         <v>0.5</v>
       </c>
       <c r="U154" t="n">
-        <v>39600</v>
+        <v>39950</v>
       </c>
       <c r="V154" t="n">
         <v>41400</v>
       </c>
       <c r="W154" t="n">
-        <v>-4.3</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="155">
@@ -11364,13 +11364,13 @@
         <v>0</v>
       </c>
       <c r="U155" t="n">
-        <v>50100</v>
+        <v>50300</v>
       </c>
       <c r="V155" t="n">
         <v>45600</v>
       </c>
       <c r="W155" t="n">
-        <v>9.9</v>
+        <v>10.3</v>
       </c>
     </row>
     <row r="156">
@@ -11436,13 +11436,13 @@
         <v>0</v>
       </c>
       <c r="U156" t="n">
-        <v>206000</v>
+        <v>208500</v>
       </c>
       <c r="V156" t="n">
         <v>206000</v>
       </c>
       <c r="W156" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="157">
@@ -11508,13 +11508,13 @@
         <v>0</v>
       </c>
       <c r="U157" t="n">
-        <v>136900</v>
+        <v>137800</v>
       </c>
       <c r="V157" t="n">
         <v>134300</v>
       </c>
       <c r="W157" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="158">
@@ -11580,13 +11580,13 @@
         <v>0</v>
       </c>
       <c r="U158" t="n">
-        <v>5900</v>
+        <v>5990</v>
       </c>
       <c r="V158" t="n">
         <v>5740</v>
       </c>
       <c r="W158" t="n">
-        <v>2.8</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="159">
@@ -11652,13 +11652,13 @@
         <v>0</v>
       </c>
       <c r="U159" t="n">
-        <v>48900</v>
+        <v>49300</v>
       </c>
       <c r="V159" t="n">
         <v>50900</v>
       </c>
       <c r="W159" t="n">
-        <v>-3.9</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="160">
@@ -11724,13 +11724,13 @@
         <v>0</v>
       </c>
       <c r="U160" t="n">
-        <v>48700</v>
+        <v>48650</v>
       </c>
       <c r="V160" t="n">
         <v>52800</v>
       </c>
       <c r="W160" t="n">
-        <v>-7.8</v>
+        <v>-7.9</v>
       </c>
     </row>
     <row r="161">
@@ -11796,13 +11796,13 @@
         <v>0.2</v>
       </c>
       <c r="U161" t="n">
-        <v>137200</v>
+        <v>140500</v>
       </c>
       <c r="V161" t="n">
         <v>143300</v>
       </c>
       <c r="W161" t="n">
-        <v>-4.3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="162">
@@ -11841,13 +11841,13 @@
         <v>0</v>
       </c>
       <c r="U162" t="n">
-        <v>13420</v>
+        <v>13310</v>
       </c>
       <c r="V162" t="n">
         <v>12500</v>
       </c>
       <c r="W162" t="n">
-        <v>7.4</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="163">
@@ -11913,13 +11913,13 @@
         <v>-1.1</v>
       </c>
       <c r="U163" t="n">
-        <v>17790</v>
+        <v>17890</v>
       </c>
       <c r="V163" t="n">
         <v>17910</v>
       </c>
       <c r="W163" t="n">
-        <v>-0.7</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="164">
@@ -11985,13 +11985,13 @@
         <v>0</v>
       </c>
       <c r="U164" t="n">
-        <v>31300</v>
+        <v>31550</v>
       </c>
       <c r="V164" t="n">
         <v>31900</v>
       </c>
       <c r="W164" t="n">
-        <v>-1.9</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="165">
@@ -12057,13 +12057,13 @@
         <v>0</v>
       </c>
       <c r="U165" t="n">
-        <v>144200</v>
+        <v>144800</v>
       </c>
       <c r="V165" t="n">
         <v>138300</v>
       </c>
       <c r="W165" t="n">
-        <v>4.3</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="166">
@@ -12129,13 +12129,13 @@
         <v>-1.3</v>
       </c>
       <c r="U166" t="n">
-        <v>179200</v>
+        <v>179700</v>
       </c>
       <c r="V166" t="n">
         <v>183400</v>
       </c>
       <c r="W166" t="n">
-        <v>-2.3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="167">
@@ -12201,13 +12201,13 @@
         <v>0</v>
       </c>
       <c r="U167" t="n">
-        <v>16470</v>
+        <v>16550</v>
       </c>
       <c r="V167" t="n">
         <v>16470</v>
       </c>
       <c r="W167" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="168">
@@ -12273,13 +12273,13 @@
         <v>0</v>
       </c>
       <c r="U168" t="n">
-        <v>71100</v>
+        <v>70300</v>
       </c>
       <c r="V168" t="n">
         <v>70700</v>
       </c>
       <c r="W168" t="n">
-        <v>0.6</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="169">
@@ -12345,13 +12345,13 @@
         <v>0.6</v>
       </c>
       <c r="U169" t="n">
-        <v>77400</v>
+        <v>77500</v>
       </c>
       <c r="V169" t="n">
         <v>78400</v>
       </c>
       <c r="W169" t="n">
-        <v>-1.3</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="170">
@@ -12417,13 +12417,13 @@
         <v>0</v>
       </c>
       <c r="U170" t="n">
-        <v>177100</v>
+        <v>177900</v>
       </c>
       <c r="V170" t="n">
         <v>172000</v>
       </c>
       <c r="W170" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="171">
@@ -12489,13 +12489,13 @@
         <v>0</v>
       </c>
       <c r="U171" t="n">
-        <v>324000</v>
+        <v>323500</v>
       </c>
       <c r="V171" t="n">
         <v>304500</v>
       </c>
       <c r="W171" t="n">
-        <v>6.4</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="172">
@@ -12561,13 +12561,13 @@
         <v>0</v>
       </c>
       <c r="U172" t="n">
-        <v>72500</v>
+        <v>72900</v>
       </c>
       <c r="V172" t="n">
         <v>75000</v>
       </c>
       <c r="W172" t="n">
-        <v>-3.3</v>
+        <v>-2.8</v>
       </c>
     </row>
     <row r="173">
@@ -12633,13 +12633,13 @@
         <v>0</v>
       </c>
       <c r="U173" t="n">
-        <v>52500</v>
+        <v>52800</v>
       </c>
       <c r="V173" t="n">
         <v>46950</v>
       </c>
       <c r="W173" t="n">
-        <v>11.8</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="174">
@@ -12750,13 +12750,13 @@
         <v>0</v>
       </c>
       <c r="U175" t="n">
-        <v>57500</v>
+        <v>57400</v>
       </c>
       <c r="V175" t="n">
         <v>55800</v>
       </c>
       <c r="W175" t="n">
-        <v>3</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="176">
@@ -12822,13 +12822,13 @@
         <v>0.3</v>
       </c>
       <c r="U176" t="n">
-        <v>43500</v>
+        <v>43400</v>
       </c>
       <c r="V176" t="n">
         <v>41950</v>
       </c>
       <c r="W176" t="n">
-        <v>3.7</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="177">
@@ -12894,13 +12894,13 @@
         <v>0</v>
       </c>
       <c r="U177" t="n">
-        <v>462500</v>
+        <v>464000</v>
       </c>
       <c r="V177" t="n">
         <v>473500</v>
       </c>
       <c r="W177" t="n">
-        <v>-2.3</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="178">
@@ -12966,13 +12966,13 @@
         <v>0</v>
       </c>
       <c r="U178" t="n">
-        <v>129200</v>
+        <v>128400</v>
       </c>
       <c r="V178" t="n">
         <v>135500</v>
       </c>
       <c r="W178" t="n">
-        <v>-4.6</v>
+        <v>-5.2</v>
       </c>
     </row>
     <row r="179">
@@ -13038,13 +13038,13 @@
         <v>0</v>
       </c>
       <c r="U179" t="n">
-        <v>16120</v>
+        <v>15930</v>
       </c>
       <c r="V179" t="n">
         <v>15390</v>
       </c>
       <c r="W179" t="n">
-        <v>4.7</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="180">
@@ -13110,13 +13110,13 @@
         <v>0</v>
       </c>
       <c r="U180" t="n">
-        <v>18430</v>
+        <v>18450</v>
       </c>
       <c r="V180" t="n">
         <v>18120</v>
       </c>
       <c r="W180" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="181">
@@ -13182,13 +13182,13 @@
         <v>-0.2</v>
       </c>
       <c r="U181" t="n">
-        <v>73500</v>
+        <v>73700</v>
       </c>
       <c r="V181" t="n">
         <v>73500</v>
       </c>
       <c r="W181" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="182">
@@ -13245,13 +13245,13 @@
         <v>0</v>
       </c>
       <c r="U182" t="n">
-        <v>83900</v>
+        <v>85200</v>
       </c>
       <c r="V182" t="n">
         <v>92000</v>
       </c>
       <c r="W182" t="n">
-        <v>-8.800000000000001</v>
+        <v>-7.4</v>
       </c>
     </row>
     <row r="183">
@@ -13317,13 +13317,13 @@
         <v>0</v>
       </c>
       <c r="U183" t="n">
-        <v>231500</v>
+        <v>231000</v>
       </c>
       <c r="V183" t="n">
         <v>244000</v>
       </c>
       <c r="W183" t="n">
-        <v>-5.1</v>
+        <v>-5.3</v>
       </c>
     </row>
     <row r="184">
@@ -13389,13 +13389,13 @@
         <v>0</v>
       </c>
       <c r="U184" t="n">
-        <v>37250</v>
+        <v>37850</v>
       </c>
       <c r="V184" t="n">
         <v>37550</v>
       </c>
       <c r="W184" t="n">
-        <v>-0.8</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="185">
@@ -13434,13 +13434,13 @@
         <v>0</v>
       </c>
       <c r="U185" t="n">
-        <v>9010</v>
+        <v>8980</v>
       </c>
       <c r="V185" t="n">
         <v>9440</v>
       </c>
       <c r="W185" t="n">
-        <v>-4.6</v>
+        <v>-4.9</v>
       </c>
     </row>
     <row r="186">
@@ -13578,13 +13578,13 @@
         <v>0</v>
       </c>
       <c r="U187" t="n">
-        <v>140400</v>
+        <v>141300</v>
       </c>
       <c r="V187" t="n">
         <v>145800</v>
       </c>
       <c r="W187" t="n">
-        <v>-3.7</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="188">
@@ -13650,13 +13650,13 @@
         <v>0</v>
       </c>
       <c r="U188" t="n">
-        <v>35950</v>
+        <v>36250</v>
       </c>
       <c r="V188" t="n">
         <v>36950</v>
       </c>
       <c r="W188" t="n">
-        <v>-2.7</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="189">
@@ -13722,13 +13722,13 @@
         <v>0.5</v>
       </c>
       <c r="U189" t="n">
-        <v>31650</v>
+        <v>31750</v>
       </c>
       <c r="V189" t="n">
         <v>31000</v>
       </c>
       <c r="W189" t="n">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="190">
@@ -13866,13 +13866,13 @@
         <v>0</v>
       </c>
       <c r="U191" t="n">
-        <v>64600</v>
+        <v>63400</v>
       </c>
       <c r="V191" t="n">
         <v>63100</v>
       </c>
       <c r="W191" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="192">
@@ -13938,13 +13938,13 @@
         <v>0</v>
       </c>
       <c r="U192" t="n">
-        <v>57100</v>
+        <v>58100</v>
       </c>
       <c r="V192" t="n">
         <v>57200</v>
       </c>
       <c r="W192" t="n">
-        <v>-0.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="193">
@@ -14082,13 +14082,13 @@
         <v>0</v>
       </c>
       <c r="U194" t="n">
-        <v>40575</v>
+        <v>40700</v>
       </c>
       <c r="V194" t="n">
         <v>42050</v>
       </c>
       <c r="W194" t="n">
-        <v>-3.5</v>
+        <v>-3.2</v>
       </c>
     </row>
     <row r="195">
@@ -14154,13 +14154,13 @@
         <v>0</v>
       </c>
       <c r="U195" t="n">
-        <v>49550</v>
+        <v>49750</v>
       </c>
       <c r="V195" t="n">
         <v>48500</v>
       </c>
       <c r="W195" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="196">
@@ -14226,13 +14226,13 @@
         <v>0</v>
       </c>
       <c r="U196" t="n">
-        <v>1401000</v>
+        <v>1415000</v>
       </c>
       <c r="V196" t="n">
         <v>1447000</v>
       </c>
       <c r="W196" t="n">
-        <v>-3.2</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="197">
@@ -14298,13 +14298,13 @@
         <v>0</v>
       </c>
       <c r="U197" t="n">
-        <v>31850</v>
+        <v>32050</v>
       </c>
       <c r="V197" t="n">
         <v>31800</v>
       </c>
       <c r="W197" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="198">
@@ -14370,13 +14370,13 @@
         <v>0</v>
       </c>
       <c r="U198" t="n">
-        <v>339000</v>
+        <v>342000</v>
       </c>
       <c r="V198" t="n">
         <v>386500</v>
       </c>
       <c r="W198" t="n">
-        <v>-12.3</v>
+        <v>-11.5</v>
       </c>
     </row>
     <row r="199">
@@ -14442,13 +14442,13 @@
         <v>0</v>
       </c>
       <c r="U199" t="n">
-        <v>49450</v>
+        <v>48800</v>
       </c>
       <c r="V199" t="n">
         <v>48300</v>
       </c>
       <c r="W199" t="n">
-        <v>2.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="200">
@@ -14514,13 +14514,13 @@
         <v>0</v>
       </c>
       <c r="U200" t="n">
-        <v>89600</v>
+        <v>90000</v>
       </c>
       <c r="V200" t="n">
         <v>101200</v>
       </c>
       <c r="W200" t="n">
-        <v>-11.5</v>
+        <v>-11.1</v>
       </c>
     </row>
     <row r="201">
@@ -14586,13 +14586,13 @@
         <v>-1.3</v>
       </c>
       <c r="U201" t="n">
-        <v>61400</v>
+        <v>61600</v>
       </c>
       <c r="V201" t="n">
         <v>62800</v>
       </c>
       <c r="W201" t="n">
-        <v>-2.2</v>
+        <v>-1.9</v>
       </c>
     </row>
     <row r="202">
@@ -14730,13 +14730,13 @@
         <v>0</v>
       </c>
       <c r="U203" t="n">
-        <v>112600</v>
+        <v>110300</v>
       </c>
       <c r="V203" t="n">
         <v>106000</v>
       </c>
       <c r="W203" t="n">
-        <v>6.2</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="204">
@@ -14802,13 +14802,13 @@
         <v>0</v>
       </c>
       <c r="U204" t="n">
-        <v>34950</v>
+        <v>35200</v>
       </c>
       <c r="V204" t="n">
         <v>36300</v>
       </c>
       <c r="W204" t="n">
-        <v>-3.7</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="205">
@@ -14874,13 +14874,13 @@
         <v>0</v>
       </c>
       <c r="U205" t="n">
-        <v>53600</v>
+        <v>52800</v>
       </c>
       <c r="V205" t="n">
         <v>55300</v>
       </c>
       <c r="W205" t="n">
-        <v>-3.1</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="206">
@@ -14946,13 +14946,13 @@
         <v>0</v>
       </c>
       <c r="U206" t="n">
-        <v>21400</v>
+        <v>21450</v>
       </c>
       <c r="V206" t="n">
         <v>21650</v>
       </c>
       <c r="W206" t="n">
-        <v>-1.2</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="207">
@@ -15018,13 +15018,13 @@
         <v>-0.5</v>
       </c>
       <c r="U207" t="n">
-        <v>209500</v>
+        <v>212500</v>
       </c>
       <c r="V207" t="n">
         <v>216500</v>
       </c>
       <c r="W207" t="n">
-        <v>-3.2</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="208">
@@ -15090,13 +15090,13 @@
         <v>0</v>
       </c>
       <c r="U208" t="n">
-        <v>254000</v>
+        <v>247500</v>
       </c>
       <c r="V208" t="n">
         <v>240500</v>
       </c>
       <c r="W208" t="n">
-        <v>5.6</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="209">
@@ -15162,13 +15162,13 @@
         <v>-0</v>
       </c>
       <c r="U209" t="n">
-        <v>740000</v>
+        <v>747000</v>
       </c>
       <c r="V209" t="n">
         <v>714000</v>
       </c>
       <c r="W209" t="n">
-        <v>3.6</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="210">
@@ -15234,13 +15234,13 @@
         <v>0.3</v>
       </c>
       <c r="U210" t="n">
-        <v>141600</v>
+        <v>142500</v>
       </c>
       <c r="V210" t="n">
         <v>140000</v>
       </c>
       <c r="W210" t="n">
-        <v>1.1</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="211">
@@ -15306,13 +15306,13 @@
         <v>0</v>
       </c>
       <c r="U211" t="n">
-        <v>118800</v>
+        <v>119300</v>
       </c>
       <c r="V211" t="n">
         <v>126300</v>
       </c>
       <c r="W211" t="n">
-        <v>-5.9</v>
+        <v>-5.5</v>
       </c>
     </row>
     <row r="212">
@@ -15378,13 +15378,13 @@
         <v>0</v>
       </c>
       <c r="U212" t="n">
-        <v>71800</v>
+        <v>70900</v>
       </c>
       <c r="V212" t="n">
         <v>68800</v>
       </c>
       <c r="W212" t="n">
-        <v>4.4</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="213">
@@ -15450,13 +15450,13 @@
         <v>0</v>
       </c>
       <c r="U213" t="n">
-        <v>5990</v>
+        <v>5930</v>
       </c>
       <c r="V213" t="n">
         <v>6140</v>
       </c>
       <c r="W213" t="n">
-        <v>-2.4</v>
+        <v>-3.4</v>
       </c>
     </row>
     <row r="214">
@@ -15585,13 +15585,13 @@
         <v>0.1</v>
       </c>
       <c r="U215" t="n">
-        <v>365000</v>
+        <v>372000</v>
       </c>
       <c r="V215" t="n">
         <v>394000</v>
       </c>
       <c r="W215" t="n">
-        <v>-7.4</v>
+        <v>-5.6</v>
       </c>
     </row>
     <row r="216">
@@ -15657,13 +15657,13 @@
         <v>0</v>
       </c>
       <c r="U216" t="n">
-        <v>145700</v>
+        <v>142900</v>
       </c>
       <c r="V216" t="n">
         <v>145500</v>
       </c>
       <c r="W216" t="n">
-        <v>0.1</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="217">
@@ -15729,13 +15729,13 @@
         <v>0</v>
       </c>
       <c r="U217" t="n">
-        <v>143800</v>
+        <v>145000</v>
       </c>
       <c r="V217" t="n">
         <v>147600</v>
       </c>
       <c r="W217" t="n">
-        <v>-2.6</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="218">
@@ -15801,13 +15801,13 @@
         <v>0</v>
       </c>
       <c r="U218" t="n">
-        <v>53700</v>
+        <v>54100</v>
       </c>
       <c r="V218" t="n">
         <v>55200</v>
       </c>
       <c r="W218" t="n">
-        <v>-2.7</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="219">
@@ -15873,13 +15873,13 @@
         <v>0</v>
       </c>
       <c r="U219" t="n">
-        <v>24750</v>
+        <v>24850</v>
       </c>
       <c r="V219" t="n">
         <v>23300</v>
       </c>
       <c r="W219" t="n">
-        <v>6.2</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="220">
@@ -15945,13 +15945,13 @@
         <v>0</v>
       </c>
       <c r="U220" t="n">
-        <v>337000</v>
+        <v>341000</v>
       </c>
       <c r="V220" t="n">
         <v>347000</v>
       </c>
       <c r="W220" t="n">
-        <v>-2.9</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="221">
@@ -16017,13 +16017,13 @@
         <v>0.9</v>
       </c>
       <c r="U221" t="n">
-        <v>2809000</v>
+        <v>2854000</v>
       </c>
       <c r="V221" t="n">
         <v>2732000</v>
       </c>
       <c r="W221" t="n">
-        <v>2.8</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="222">
@@ -16089,13 +16089,13 @@
         <v>0</v>
       </c>
       <c r="U222" t="n">
-        <v>171200</v>
+        <v>172100</v>
       </c>
       <c r="V222" t="n">
         <v>172800</v>
       </c>
       <c r="W222" t="n">
-        <v>-0.9</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="223">
@@ -16161,13 +16161,13 @@
         <v>0.9</v>
       </c>
       <c r="U223" t="n">
-        <v>16660</v>
+        <v>16600</v>
       </c>
       <c r="V223" t="n">
         <v>16670</v>
       </c>
       <c r="W223" t="n">
-        <v>-0.1</v>
+        <v>-0.4</v>
       </c>
     </row>
     <row r="224">
@@ -16224,13 +16224,13 @@
         <v>0</v>
       </c>
       <c r="U224" t="n">
-        <v>37500</v>
+        <v>37250</v>
       </c>
       <c r="V224" t="n">
         <v>37900</v>
       </c>
       <c r="W224" t="n">
-        <v>-1.1</v>
+        <v>-1.7</v>
       </c>
     </row>
     <row r="225">
@@ -16296,13 +16296,13 @@
         <v>0</v>
       </c>
       <c r="U225" t="n">
-        <v>150200</v>
+        <v>150600</v>
       </c>
       <c r="V225" t="n">
         <v>144700</v>
       </c>
       <c r="W225" t="n">
-        <v>3.8</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="226">
@@ -16368,13 +16368,13 @@
         <v>-1.5</v>
       </c>
       <c r="U226" t="n">
-        <v>388500</v>
+        <v>390000</v>
       </c>
       <c r="V226" t="n">
         <v>395000</v>
       </c>
       <c r="W226" t="n">
-        <v>-1.6</v>
+        <v>-1.3</v>
       </c>
     </row>
     <row r="227">
@@ -16440,13 +16440,13 @@
         <v>0</v>
       </c>
       <c r="U227" t="n">
-        <v>34950</v>
+        <v>35100</v>
       </c>
       <c r="V227" t="n">
         <v>33200</v>
       </c>
       <c r="W227" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="228">
@@ -16512,13 +16512,13 @@
         <v>0</v>
       </c>
       <c r="U228" t="n">
-        <v>10750</v>
+        <v>11330</v>
       </c>
       <c r="V228" t="n">
         <v>11230</v>
       </c>
       <c r="W228" t="n">
-        <v>-4.3</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="229">
@@ -16584,13 +16584,13 @@
         <v>0</v>
       </c>
       <c r="U229" t="n">
-        <v>21450</v>
+        <v>21350</v>
       </c>
       <c r="V229" t="n">
         <v>21950</v>
       </c>
       <c r="W229" t="n">
-        <v>-2.3</v>
+        <v>-2.7</v>
       </c>
     </row>
     <row r="230">
@@ -16656,13 +16656,13 @@
         <v>0</v>
       </c>
       <c r="U230" t="n">
-        <v>78600</v>
+        <v>79400</v>
       </c>
       <c r="V230" t="n">
         <v>86600</v>
       </c>
       <c r="W230" t="n">
-        <v>-9.199999999999999</v>
+        <v>-8.300000000000001</v>
       </c>
     </row>
     <row r="231">
@@ -16728,13 +16728,13 @@
         <v>-0</v>
       </c>
       <c r="U231" t="n">
-        <v>479500</v>
+        <v>479000</v>
       </c>
       <c r="V231" t="n">
         <v>436500</v>
       </c>
       <c r="W231" t="n">
-        <v>9.9</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="232">
@@ -16800,7 +16800,7 @@
         <v>-0.7</v>
       </c>
       <c r="U232" t="n">
-        <v>172900</v>
+        <v>173000</v>
       </c>
       <c r="V232" t="n">
         <v>178500</v>
@@ -16872,13 +16872,13 @@
         <v>0</v>
       </c>
       <c r="U233" t="n">
-        <v>99000</v>
+        <v>100000</v>
       </c>
       <c r="V233" t="n">
         <v>99500</v>
       </c>
       <c r="W233" t="n">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="234">
@@ -16944,13 +16944,13 @@
         <v>0</v>
       </c>
       <c r="U234" t="n">
-        <v>16620</v>
+        <v>16690</v>
       </c>
       <c r="V234" t="n">
         <v>16280</v>
       </c>
       <c r="W234" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="235">
@@ -17016,13 +17016,13 @@
         <v>0</v>
       </c>
       <c r="U235" t="n">
-        <v>355500</v>
+        <v>360000</v>
       </c>
       <c r="V235" t="n">
         <v>358500</v>
       </c>
       <c r="W235" t="n">
-        <v>-0.8</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="236">
@@ -17088,13 +17088,13 @@
         <v>0</v>
       </c>
       <c r="U236" t="n">
-        <v>86100</v>
+        <v>85800</v>
       </c>
       <c r="V236" t="n">
         <v>73400</v>
       </c>
       <c r="W236" t="n">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
     </row>
     <row r="237">
@@ -17160,13 +17160,13 @@
         <v>-0.3</v>
       </c>
       <c r="U237" t="n">
-        <v>17940</v>
+        <v>17850</v>
       </c>
       <c r="V237" t="n">
         <v>18060</v>
       </c>
       <c r="W237" t="n">
-        <v>-0.7</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="238">
@@ -17232,13 +17232,13 @@
         <v>0</v>
       </c>
       <c r="U238" t="n">
-        <v>46300</v>
+        <v>46250</v>
       </c>
       <c r="V238" t="n">
         <v>47300</v>
       </c>
       <c r="W238" t="n">
-        <v>-2.1</v>
+        <v>-2.2</v>
       </c>
     </row>
     <row r="239">
@@ -17304,13 +17304,13 @@
         <v>0</v>
       </c>
       <c r="U239" t="n">
-        <v>64700</v>
+        <v>64800</v>
       </c>
       <c r="V239" t="n">
         <v>66900</v>
       </c>
       <c r="W239" t="n">
-        <v>-3.3</v>
+        <v>-3.1</v>
       </c>
     </row>
     <row r="240">
@@ -17349,13 +17349,13 @@
         <v>0</v>
       </c>
       <c r="U240" t="n">
-        <v>40750</v>
+        <v>40350</v>
       </c>
       <c r="V240" t="n">
         <v>37750</v>
       </c>
       <c r="W240" t="n">
-        <v>7.9</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="241">
@@ -17394,13 +17394,13 @@
         <v>0</v>
       </c>
       <c r="U241" t="n">
-        <v>28750</v>
+        <v>29500</v>
       </c>
       <c r="V241" t="n">
         <v>31050</v>
       </c>
       <c r="W241" t="n">
-        <v>-7.4</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="242">
@@ -17466,13 +17466,13 @@
         <v>0</v>
       </c>
       <c r="U242" t="n">
-        <v>1074000</v>
+        <v>1089000</v>
       </c>
       <c r="V242" t="n">
         <v>1041000</v>
       </c>
       <c r="W242" t="n">
-        <v>3.2</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="243">
@@ -17538,13 +17538,13 @@
         <v>0</v>
       </c>
       <c r="U243" t="n">
-        <v>92700</v>
+        <v>93800</v>
       </c>
       <c r="V243" t="n">
         <v>101200</v>
       </c>
       <c r="W243" t="n">
-        <v>-8.4</v>
+        <v>-7.3</v>
       </c>
     </row>
     <row r="244">
@@ -17610,13 +17610,13 @@
         <v>0</v>
       </c>
       <c r="U244" t="n">
-        <v>47950</v>
+        <v>47300</v>
       </c>
       <c r="V244" t="n">
         <v>46950</v>
       </c>
       <c r="W244" t="n">
-        <v>2.1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="245">
@@ -17682,13 +17682,13 @@
         <v>-2</v>
       </c>
       <c r="U245" t="n">
-        <v>248000</v>
+        <v>247000</v>
       </c>
       <c r="V245" t="n">
         <v>210500</v>
       </c>
       <c r="W245" t="n">
-        <v>17.8</v>
+        <v>17.3</v>
       </c>
     </row>
     <row r="246">
@@ -17754,13 +17754,13 @@
         <v>0</v>
       </c>
       <c r="U246" t="n">
-        <v>79000</v>
+        <v>80200</v>
       </c>
       <c r="V246" t="n">
         <v>79300</v>
       </c>
       <c r="W246" t="n">
-        <v>-0.4</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="247">
@@ -17826,13 +17826,13 @@
         <v>0</v>
       </c>
       <c r="U247" t="n">
-        <v>10400</v>
+        <v>10320</v>
       </c>
       <c r="V247" t="n">
         <v>10510</v>
       </c>
       <c r="W247" t="n">
-        <v>-1</v>
+        <v>-1.8</v>
       </c>
     </row>
     <row r="248">
@@ -17898,13 +17898,13 @@
         <v>0.2</v>
       </c>
       <c r="U248" t="n">
-        <v>31700</v>
+        <v>31400</v>
       </c>
       <c r="V248" t="n">
         <v>31850</v>
       </c>
       <c r="W248" t="n">
-        <v>-0.5</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="249">
@@ -17970,13 +17970,13 @@
         <v>0</v>
       </c>
       <c r="U249" t="n">
-        <v>167100</v>
+        <v>167600</v>
       </c>
       <c r="V249" t="n">
         <v>190600</v>
       </c>
       <c r="W249" t="n">
-        <v>-12.3</v>
+        <v>-12.1</v>
       </c>
     </row>
     <row r="250">
@@ -18042,13 +18042,13 @@
         <v>0</v>
       </c>
       <c r="U250" t="n">
-        <v>18360</v>
+        <v>17930</v>
       </c>
       <c r="V250" t="n">
         <v>16560</v>
       </c>
       <c r="W250" t="n">
-        <v>10.9</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="251">
@@ -18114,13 +18114,13 @@
         <v>0</v>
       </c>
       <c r="U251" t="n">
-        <v>47150</v>
+        <v>47200</v>
       </c>
       <c r="V251" t="n">
         <v>49400</v>
       </c>
       <c r="W251" t="n">
-        <v>-4.6</v>
+        <v>-4.5</v>
       </c>
     </row>
     <row r="252">
@@ -18159,13 +18159,13 @@
         <v>0</v>
       </c>
       <c r="U252" t="n">
-        <v>32450</v>
+        <v>32550</v>
       </c>
       <c r="V252" t="n">
         <v>34500</v>
       </c>
       <c r="W252" t="n">
-        <v>-5.9</v>
+        <v>-5.7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(consensus): 주간 컨센 스냅샷 2026-09-12
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/consensus_full.xlsx
+++ b/telegram_research_dashboard/static/consensus_full.xlsx
@@ -458,7 +458,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-09-11 · 전주 2026-09-05</t>
+          <t>영업이익 컨센(KOSPI200·KOSDAQ50·커버리지) · 기준일 2026-09-12 · 전주 2026-09-05</t>
         </is>
       </c>
     </row>
@@ -1326,40 +1326,40 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>7942</v>
+        <v>8076</v>
       </c>
       <c r="G13" t="n">
         <v>7942</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>1.7</v>
       </c>
       <c r="L13" t="n">
-        <v>31986.2</v>
+        <v>32316.9</v>
       </c>
       <c r="M13" t="n">
         <v>31986.2</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O13" t="n">
-        <v>37928.1</v>
+        <v>38353.5</v>
       </c>
       <c r="P13" t="n">
         <v>37928.1</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="R13" t="n">
-        <v>36586.3</v>
+        <v>37044</v>
       </c>
       <c r="S13" t="n">
         <v>36586.3</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="U13" t="n">
         <v>686000</v>
@@ -1758,31 +1758,31 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>13301.4</v>
+        <v>13355.3</v>
       </c>
       <c r="M19" t="n">
         <v>13301.4</v>
       </c>
       <c r="N19" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="O19" t="n">
-        <v>14411.4</v>
+        <v>14475.3</v>
       </c>
       <c r="P19" t="n">
         <v>14411.4</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R19" t="n">
-        <v>15783.6</v>
+        <v>15992.7</v>
       </c>
       <c r="S19" t="n">
         <v>15783.6</v>
       </c>
       <c r="T19" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="U19" t="n">
         <v>51300</v>
@@ -2811,16 +2811,16 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1820</v>
+        <v>1815</v>
       </c>
       <c r="G34" t="n">
         <v>1817</v>
       </c>
       <c r="H34" t="n">
-        <v>0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="L34" t="n">
-        <v>7910.7</v>
+        <v>7906</v>
       </c>
       <c r="M34" t="n">
         <v>7892.4</v>
@@ -2829,7 +2829,7 @@
         <v>0.2</v>
       </c>
       <c r="O34" t="n">
-        <v>8704.299999999999</v>
+        <v>8700.200000000001</v>
       </c>
       <c r="P34" t="n">
         <v>8712.799999999999</v>
@@ -2838,13 +2838,13 @@
         <v>-0.1</v>
       </c>
       <c r="R34" t="n">
-        <v>9361.200000000001</v>
+        <v>9352.4</v>
       </c>
       <c r="S34" t="n">
         <v>9323.9</v>
       </c>
       <c r="T34" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="U34" t="n">
         <v>381000</v>
@@ -3243,31 +3243,31 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>23716.6</v>
+        <v>23970.6</v>
       </c>
       <c r="M40" t="n">
         <v>23716.6</v>
       </c>
       <c r="N40" t="n">
-        <v>0</v>
+        <v>1.1</v>
       </c>
       <c r="O40" t="n">
-        <v>23553.1</v>
+        <v>24081.6</v>
       </c>
       <c r="P40" t="n">
         <v>23553.1</v>
       </c>
       <c r="Q40" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
       <c r="R40" t="n">
-        <v>24819.6</v>
+        <v>25469.6</v>
       </c>
       <c r="S40" t="n">
         <v>24819.6</v>
       </c>
       <c r="T40" t="n">
-        <v>0</v>
+        <v>2.6</v>
       </c>
       <c r="U40" t="n">
         <v>191700</v>
@@ -3630,40 +3630,40 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4936</v>
+        <v>4900</v>
       </c>
       <c r="G46" t="n">
         <v>4936</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>-0.7</v>
       </c>
       <c r="L46" t="n">
-        <v>19998.9</v>
+        <v>19996.3</v>
       </c>
       <c r="M46" t="n">
         <v>19998.9</v>
       </c>
       <c r="N46" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="O46" t="n">
-        <v>22439.8</v>
+        <v>22339.8</v>
       </c>
       <c r="P46" t="n">
         <v>22439.8</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="R46" t="n">
-        <v>25550.7</v>
+        <v>25700.6</v>
       </c>
       <c r="S46" t="n">
         <v>25550.7</v>
       </c>
       <c r="T46" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="U46" t="n">
         <v>319500</v>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>3373</v>
+        <v>3300</v>
       </c>
       <c r="L51" t="n">
-        <v>47821.3</v>
+        <v>47817.2</v>
       </c>
       <c r="M51" t="n">
         <v>47797.9</v>
@@ -4002,22 +4002,22 @@
         <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>26286.9</v>
+        <v>26232.4</v>
       </c>
       <c r="P51" t="n">
         <v>26153.7</v>
       </c>
       <c r="Q51" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="R51" t="n">
-        <v>27528.3</v>
+        <v>27610.4</v>
       </c>
       <c r="S51" t="n">
         <v>27203.7</v>
       </c>
       <c r="T51" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="U51" t="n">
         <v>33450</v>
@@ -4632,40 +4632,40 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>2085</v>
+        <v>2092</v>
       </c>
       <c r="G60" t="n">
         <v>2085</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="L60" t="n">
-        <v>8727.4</v>
+        <v>8899.700000000001</v>
       </c>
       <c r="M60" t="n">
         <v>8727.4</v>
       </c>
       <c r="N60" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O60" t="n">
-        <v>12809.5</v>
+        <v>12961.1</v>
       </c>
       <c r="P60" t="n">
         <v>12809.5</v>
       </c>
       <c r="Q60" t="n">
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="R60" t="n">
-        <v>14612.6</v>
+        <v>14572.8</v>
       </c>
       <c r="S60" t="n">
         <v>14612.6</v>
       </c>
       <c r="T60" t="n">
-        <v>0</v>
+        <v>-0.3</v>
       </c>
       <c r="U60" t="n">
         <v>29800</v>
@@ -6135,34 +6135,34 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>5558</v>
+        <v>5563</v>
       </c>
       <c r="L81" t="n">
-        <v>23139.6</v>
+        <v>23117.3</v>
       </c>
       <c r="M81" t="n">
         <v>23242.3</v>
       </c>
       <c r="N81" t="n">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
       <c r="O81" t="n">
-        <v>20886.3</v>
+        <v>21025.9</v>
       </c>
       <c r="P81" t="n">
         <v>20844.1</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="R81" t="n">
-        <v>21226.2</v>
+        <v>21395.8</v>
       </c>
       <c r="S81" t="n">
         <v>21165.2</v>
       </c>
       <c r="T81" t="n">
-        <v>0.3</v>
+        <v>1.1</v>
       </c>
       <c r="U81" t="n">
         <v>87400</v>
@@ -6777,40 +6777,40 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>1832</v>
+        <v>1823</v>
       </c>
       <c r="G90" t="n">
         <v>1830</v>
       </c>
       <c r="H90" t="n">
-        <v>0.1</v>
+        <v>-0.4</v>
       </c>
       <c r="L90" t="n">
-        <v>7995.5</v>
+        <v>7987.8</v>
       </c>
       <c r="M90" t="n">
         <v>8000.9</v>
       </c>
       <c r="N90" t="n">
-        <v>-0.1</v>
+        <v>-0.2</v>
       </c>
       <c r="O90" t="n">
-        <v>8680.799999999999</v>
+        <v>8679.299999999999</v>
       </c>
       <c r="P90" t="n">
         <v>8680</v>
       </c>
       <c r="Q90" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="R90" t="n">
-        <v>9374.700000000001</v>
+        <v>9373.200000000001</v>
       </c>
       <c r="S90" t="n">
         <v>9341.299999999999</v>
       </c>
       <c r="T90" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="U90" t="n">
         <v>112000</v>
@@ -8688,34 +8688,34 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>5293</v>
+        <v>5229</v>
       </c>
       <c r="L117" t="n">
-        <v>22944.8</v>
+        <v>22916.7</v>
       </c>
       <c r="M117" t="n">
         <v>22983.8</v>
       </c>
       <c r="N117" t="n">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
       <c r="O117" t="n">
-        <v>19125.1</v>
+        <v>19010.9</v>
       </c>
       <c r="P117" t="n">
         <v>19067.2</v>
       </c>
       <c r="Q117" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="R117" t="n">
-        <v>19634.6</v>
+        <v>19670.8</v>
       </c>
       <c r="S117" t="n">
         <v>19518.9</v>
       </c>
       <c r="T117" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="U117" t="n">
         <v>278000</v>
@@ -9051,7 +9051,7 @@
         <v>-1.9</v>
       </c>
       <c r="L122" t="n">
-        <v>8268.799999999999</v>
+        <v>8269.299999999999</v>
       </c>
       <c r="M122" t="n">
         <v>8310</v>
@@ -9060,22 +9060,22 @@
         <v>-0.5</v>
       </c>
       <c r="O122" t="n">
-        <v>8090.3</v>
+        <v>8120.3</v>
       </c>
       <c r="P122" t="n">
         <v>8159.2</v>
       </c>
       <c r="Q122" t="n">
-        <v>-0.8</v>
+        <v>-0.5</v>
       </c>
       <c r="R122" t="n">
-        <v>9053.799999999999</v>
+        <v>9066.200000000001</v>
       </c>
       <c r="S122" t="n">
         <v>9186.4</v>
       </c>
       <c r="T122" t="n">
-        <v>-1.4</v>
+        <v>-1.3</v>
       </c>
       <c r="U122" t="n">
         <v>19890</v>
@@ -9114,40 +9114,40 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>3776</v>
+        <v>3754</v>
       </c>
       <c r="G123" t="n">
         <v>3776</v>
       </c>
       <c r="H123" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="L123" t="n">
-        <v>14688.2</v>
+        <v>14652.1</v>
       </c>
       <c r="M123" t="n">
         <v>14688.2</v>
       </c>
       <c r="N123" t="n">
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="O123" t="n">
-        <v>15554.8</v>
+        <v>15480.2</v>
       </c>
       <c r="P123" t="n">
         <v>15554.8</v>
       </c>
       <c r="Q123" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="R123" t="n">
-        <v>16386.5</v>
+        <v>16311.2</v>
       </c>
       <c r="S123" t="n">
         <v>16386.5</v>
       </c>
       <c r="T123" t="n">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="U123" t="n">
         <v>57700</v>
@@ -9258,40 +9258,40 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="G125" t="n">
         <v>342</v>
       </c>
       <c r="H125" t="n">
-        <v>0</v>
+        <v>-2.3</v>
       </c>
       <c r="L125" t="n">
-        <v>1019.8</v>
+        <v>1006.1</v>
       </c>
       <c r="M125" t="n">
         <v>1019.8</v>
       </c>
       <c r="N125" t="n">
-        <v>0</v>
+        <v>-1.3</v>
       </c>
       <c r="O125" t="n">
-        <v>1160</v>
+        <v>1145.7</v>
       </c>
       <c r="P125" t="n">
         <v>1160</v>
       </c>
       <c r="Q125" t="n">
-        <v>0</v>
+        <v>-1.2</v>
       </c>
       <c r="R125" t="n">
-        <v>1255.7</v>
+        <v>1244.2</v>
       </c>
       <c r="S125" t="n">
         <v>1290.5</v>
       </c>
       <c r="T125" t="n">
-        <v>-2.7</v>
+        <v>-3.6</v>
       </c>
       <c r="U125" t="n">
         <v>22850</v>
@@ -10617,40 +10617,40 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>8771</v>
+        <v>8784</v>
       </c>
       <c r="G144" t="n">
         <v>9012</v>
       </c>
       <c r="H144" t="n">
-        <v>-2.7</v>
+        <v>-2.5</v>
       </c>
       <c r="L144" t="n">
-        <v>40568.7</v>
+        <v>40613.8</v>
       </c>
       <c r="M144" t="n">
         <v>40740.8</v>
       </c>
       <c r="N144" t="n">
-        <v>-0.4</v>
+        <v>-0.3</v>
       </c>
       <c r="O144" t="n">
-        <v>32676.4</v>
+        <v>32549.8</v>
       </c>
       <c r="P144" t="n">
         <v>32826.1</v>
       </c>
       <c r="Q144" t="n">
-        <v>-0.5</v>
+        <v>-0.8</v>
       </c>
       <c r="R144" t="n">
-        <v>33367.7</v>
+        <v>33383.2</v>
       </c>
       <c r="S144" t="n">
         <v>33520.6</v>
       </c>
       <c r="T144" t="n">
-        <v>-0.5</v>
+        <v>-0.4</v>
       </c>
       <c r="U144" t="n">
         <v>193600</v>
@@ -12309,40 +12309,40 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>1077</v>
+        <v>1086</v>
       </c>
       <c r="G169" t="n">
         <v>1083</v>
       </c>
       <c r="H169" t="n">
-        <v>-0.6</v>
+        <v>0.3</v>
       </c>
       <c r="L169" t="n">
-        <v>4242.3</v>
+        <v>4253.7</v>
       </c>
       <c r="M169" t="n">
         <v>4266.3</v>
       </c>
       <c r="N169" t="n">
-        <v>-0.6</v>
+        <v>-0.3</v>
       </c>
       <c r="O169" t="n">
-        <v>3878</v>
+        <v>3853.9</v>
       </c>
       <c r="P169" t="n">
         <v>3867.1</v>
       </c>
       <c r="Q169" t="n">
-        <v>0.3</v>
+        <v>-0.3</v>
       </c>
       <c r="R169" t="n">
-        <v>4169</v>
+        <v>4142.7</v>
       </c>
       <c r="S169" t="n">
         <v>4143.9</v>
       </c>
       <c r="T169" t="n">
-        <v>0.6</v>
+        <v>-0</v>
       </c>
       <c r="U169" t="n">
         <v>77500</v>
@@ -14046,40 +14046,40 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="G194" t="n">
         <v>314</v>
       </c>
       <c r="H194" t="n">
-        <v>0</v>
+        <v>-0.6</v>
       </c>
       <c r="L194" t="n">
-        <v>1304.1</v>
+        <v>1307.2</v>
       </c>
       <c r="M194" t="n">
         <v>1304.1</v>
       </c>
       <c r="N194" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="O194" t="n">
-        <v>1479.1</v>
+        <v>1480.5</v>
       </c>
       <c r="P194" t="n">
         <v>1479.1</v>
       </c>
       <c r="Q194" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="R194" t="n">
-        <v>1684.3</v>
+        <v>1688.6</v>
       </c>
       <c r="S194" t="n">
         <v>1684.3</v>
       </c>
       <c r="T194" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="U194" t="n">
         <v>40700</v>
@@ -15342,13 +15342,13 @@
         </is>
       </c>
       <c r="F212" t="n">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="G212" t="n">
         <v>588</v>
       </c>
       <c r="H212" t="n">
-        <v>0</v>
+        <v>0.7</v>
       </c>
       <c r="L212" t="n">
         <v>2485.5</v>
@@ -16692,40 +16692,40 @@
         </is>
       </c>
       <c r="F231" t="n">
-        <v>10073</v>
+        <v>10106</v>
       </c>
       <c r="G231" t="n">
         <v>10073</v>
       </c>
       <c r="H231" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="L231" t="n">
-        <v>40520</v>
+        <v>40491.8</v>
       </c>
       <c r="M231" t="n">
         <v>40521.2</v>
       </c>
       <c r="N231" t="n">
-        <v>-0</v>
+        <v>-0.1</v>
       </c>
       <c r="O231" t="n">
-        <v>47401.8</v>
+        <v>47253.1</v>
       </c>
       <c r="P231" t="n">
         <v>47403.9</v>
       </c>
       <c r="Q231" t="n">
-        <v>-0</v>
+        <v>-0.3</v>
       </c>
       <c r="R231" t="n">
-        <v>54806.5</v>
+        <v>55163</v>
       </c>
       <c r="S231" t="n">
         <v>54808.5</v>
       </c>
       <c r="T231" t="n">
-        <v>-0</v>
+        <v>0.6</v>
       </c>
       <c r="U231" t="n">
         <v>479000</v>
@@ -17655,7 +17655,7 @@
         <v>-1.5</v>
       </c>
       <c r="L245" t="n">
-        <v>4148.6</v>
+        <v>4149</v>
       </c>
       <c r="M245" t="n">
         <v>4184.6</v>
@@ -17664,22 +17664,22 @@
         <v>-0.9</v>
       </c>
       <c r="O245" t="n">
-        <v>5280.9</v>
+        <v>5281.3</v>
       </c>
       <c r="P245" t="n">
         <v>5358.9</v>
       </c>
       <c r="Q245" t="n">
-        <v>-1.5</v>
+        <v>-1.4</v>
       </c>
       <c r="R245" t="n">
-        <v>6579.7</v>
+        <v>6584.7</v>
       </c>
       <c r="S245" t="n">
         <v>6713.7</v>
       </c>
       <c r="T245" t="n">
-        <v>-2</v>
+        <v>-1.9</v>
       </c>
       <c r="U245" t="n">
         <v>247000</v>

</xml_diff>